<commit_message>
fix: stabilize PPV flow
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Hari.Prasad/jobbot/dazn-tests/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5DC1D45-CF0E-7B4E-AAF4-009E002E13FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D74F6815-8762-6143-9D97-3044B8672F8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17280" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Landing page" sheetId="1" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="182">
   <si>
     <t>Field</t>
   </si>
@@ -223,9 +223,6 @@
     <t>Event Name</t>
   </si>
   <si>
-    <t>{{PPV_NAME}} PPV</t>
-  </si>
-  <si>
     <t>PPV Price</t>
   </si>
   <si>
@@ -535,9 +532,6 @@
     <t>Upsell Plan Highlight</t>
   </si>
   <si>
-    <t>pay over time</t>
-  </si>
-  <si>
     <t>First Month Free Text</t>
   </si>
   <si>
@@ -553,9 +547,6 @@
     <t>Then</t>
   </si>
   <si>
-    <t>Then {{CURRENCY}}{{MONTHLY_PRICE}} /month for 11 months.</t>
-  </si>
-  <si>
     <t>Upsell Renewal Text</t>
   </si>
   <si>
@@ -602,6 +593,18 @@
   </si>
   <si>
     <t>Google Pay Option</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Then ₹{{ANNUAL_PRICE}} /month for {{ANNUAL_MONTHS}} months.</t>
+  </si>
+  <si>
+    <t>{{PPV_NAME}}.</t>
+  </si>
+  <si>
+    <t>Pay-per-views included at no extra cost. Minimum of 12 events per year including {{PPV_NAME}}.</t>
   </si>
 </sst>
 </file>
@@ -1001,7 +1004,7 @@
     </row>
     <row r="2" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B2" t="s">
         <v>19</v>
@@ -1009,7 +1012,7 @@
     </row>
     <row r="3" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
@@ -1017,15 +1020,15 @@
     </row>
     <row r="4" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B5" t="s">
         <v>19</v>
@@ -1123,7 +1126,7 @@
         <v>53</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>54</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1131,7 +1134,7 @@
         <v>45</v>
       </c>
       <c r="B8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>8</v>
@@ -1142,10 +1145,10 @@
         <v>45</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1153,7 +1156,7 @@
         <v>45</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C10" s="1" t="e" cm="1">
         <f t="array" ref="C10">+DAZN Standard</f>
@@ -1165,7 +1168,7 @@
         <v>45</v>
       </c>
       <c r="B11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>7</v>
@@ -1176,7 +1179,7 @@
         <v>45</v>
       </c>
       <c r="B12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>19</v>
@@ -1187,10 +1190,10 @@
         <v>45</v>
       </c>
       <c r="B13" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1198,7 +1201,7 @@
         <v>45</v>
       </c>
       <c r="B14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>19</v>
@@ -1209,7 +1212,7 @@
         <v>45</v>
       </c>
       <c r="B15" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>19</v>
@@ -1220,10 +1223,10 @@
         <v>45</v>
       </c>
       <c r="B16" t="s">
+        <v>63</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>64</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1234,7 +1237,7 @@
         <v>30</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1242,10 +1245,10 @@
         <v>45</v>
       </c>
       <c r="B18" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1256,7 +1259,7 @@
         <v>32</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1264,10 +1267,10 @@
         <v>45</v>
       </c>
       <c r="B20" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1275,7 +1278,7 @@
         <v>45</v>
       </c>
       <c r="B21" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>37</v>
@@ -1286,7 +1289,7 @@
         <v>45</v>
       </c>
       <c r="B22" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>7</v>
@@ -1297,7 +1300,7 @@
         <v>45</v>
       </c>
       <c r="B23" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>19</v>
@@ -1308,10 +1311,10 @@
         <v>45</v>
       </c>
       <c r="B24" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1319,7 +1322,7 @@
         <v>45</v>
       </c>
       <c r="B25" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>19</v>
@@ -1330,10 +1333,10 @@
         <v>45</v>
       </c>
       <c r="B26" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>78</v>
+        <v>178</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1341,10 +1344,10 @@
         <v>45</v>
       </c>
       <c r="B27" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>19</v>
+        <v>178</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1352,10 +1355,10 @@
         <v>45</v>
       </c>
       <c r="B28" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>81</v>
+        <v>178</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1363,10 +1366,10 @@
         <v>45</v>
       </c>
       <c r="B29" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>19</v>
+        <v>178</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1377,7 +1380,7 @@
         <v>38</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>83</v>
+        <v>181</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1385,10 +1388,10 @@
         <v>45</v>
       </c>
       <c r="B31" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>85</v>
+        <v>180</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1399,7 +1402,7 @@
         <v>40</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1410,7 +1413,7 @@
         <v>42</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1418,10 +1421,10 @@
         <v>45</v>
       </c>
       <c r="B34" t="s">
+        <v>148</v>
+      </c>
+      <c r="C34" s="1" t="s">
         <v>149</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1429,7 +1432,7 @@
         <v>45</v>
       </c>
       <c r="B35" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>7</v>
@@ -1440,7 +1443,7 @@
         <v>45</v>
       </c>
       <c r="B36" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>51</v>
@@ -1451,10 +1454,10 @@
         <v>45</v>
       </c>
       <c r="B37" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1465,7 +1468,7 @@
         <v>16</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1473,10 +1476,10 @@
         <v>45</v>
       </c>
       <c r="B39" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1484,7 +1487,7 @@
     </row>
     <row r="41" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B41" t="s">
         <v>13</v>
@@ -1495,10 +1498,10 @@
     </row>
     <row r="42" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
+        <v>92</v>
+      </c>
+      <c r="B42" t="s">
         <v>93</v>
-      </c>
-      <c r="B42" t="s">
-        <v>94</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>48</v>
@@ -1506,7 +1509,7 @@
     </row>
     <row r="43" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B43" t="s">
         <v>49</v>
@@ -1517,7 +1520,7 @@
     </row>
     <row r="44" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B44" t="s">
         <v>50</v>
@@ -1528,10 +1531,10 @@
     </row>
     <row r="45" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B45" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>19</v>
@@ -1539,18 +1542,18 @@
     </row>
     <row r="46" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B46" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="47" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B47" t="s">
         <v>53</v>
@@ -1561,10 +1564,10 @@
     </row>
     <row r="48" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B48" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>19</v>
@@ -1572,10 +1575,10 @@
     </row>
     <row r="49" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B49" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>19</v>
@@ -1583,10 +1586,10 @@
     </row>
     <row r="50" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B50" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>7</v>
@@ -1594,10 +1597,10 @@
     </row>
     <row r="51" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B51" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>8</v>
@@ -1605,29 +1608,29 @@
     </row>
     <row r="52" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B52" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B53" t="s">
+        <v>98</v>
+      </c>
+      <c r="C53" s="1" t="s">
         <v>99</v>
-      </c>
-      <c r="C53" s="1" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B54" t="s">
         <v>18</v>
@@ -1638,7 +1641,7 @@
     </row>
     <row r="55" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B55" t="s">
         <v>20</v>
@@ -1649,10 +1652,10 @@
     </row>
     <row r="56" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B56" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>19</v>
@@ -1660,7 +1663,7 @@
     </row>
     <row r="57" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B57" t="s">
         <v>23</v>
@@ -1671,32 +1674,32 @@
     </row>
     <row r="58" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B58" t="s">
         <v>24</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="59" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B59" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="60" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B60" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>19</v>
@@ -1704,65 +1707,65 @@
     </row>
     <row r="61" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B61" t="s">
+        <v>63</v>
+      </c>
+      <c r="C61" s="1" t="s">
         <v>64</v>
-      </c>
-      <c r="C61" s="1" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="62" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B62" t="s">
         <v>30</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="63" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B63" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="64" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B64" t="s">
         <v>32</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="65" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B65" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="66" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B66" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C66" s="1" t="s">
         <v>37</v>
@@ -1770,10 +1773,10 @@
     </row>
     <row r="67" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B67" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C67" s="1" t="s">
         <v>7</v>
@@ -1781,10 +1784,10 @@
     </row>
     <row r="68" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>19</v>
@@ -1792,21 +1795,21 @@
     </row>
     <row r="69" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B69" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="70" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B70" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C70" s="1" t="s">
         <v>19</v>
@@ -1814,109 +1817,109 @@
     </row>
     <row r="71" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B71" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>78</v>
+        <v>178</v>
       </c>
     </row>
     <row r="72" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B72" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>19</v>
+        <v>178</v>
       </c>
     </row>
     <row r="73" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B73" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>81</v>
+        <v>178</v>
       </c>
     </row>
     <row r="74" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B74" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>19</v>
+        <v>178</v>
       </c>
     </row>
     <row r="75" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B75" t="s">
         <v>38</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>83</v>
+        <v>181</v>
       </c>
     </row>
     <row r="76" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B76" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="77" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B77" t="s">
         <v>40</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="78" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B78" t="s">
         <v>42</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="79" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B79" t="s">
+        <v>148</v>
+      </c>
+      <c r="C79" s="1" t="s">
         <v>149</v>
-      </c>
-      <c r="C79" s="1" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="80" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B80" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C80" s="1" t="s">
         <v>7</v>
@@ -1924,10 +1927,10 @@
     </row>
     <row r="81" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B81" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C81" s="1" t="s">
         <v>51</v>
@@ -1935,18 +1938,18 @@
     </row>
     <row r="82" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B82" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="83" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B83" t="s">
         <v>16</v>
@@ -1957,13 +1960,13 @@
     </row>
     <row r="84" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B84" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>89</v>
+        <v>178</v>
       </c>
     </row>
     <row r="85" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1971,54 +1974,54 @@
     </row>
     <row r="86" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B86" t="s">
         <v>13</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="87" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B87" t="s">
+        <v>105</v>
+      </c>
+      <c r="C87" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="C87" s="1" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="88" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B88" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="89" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B89" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>54</v>
+        <v>7</v>
       </c>
     </row>
     <row r="90" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B90" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C90" s="1" t="s">
         <v>8</v>
@@ -2026,29 +2029,29 @@
     </row>
     <row r="91" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B91" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="92" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B92" t="s">
+        <v>56</v>
+      </c>
+      <c r="C92" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="C92" s="1" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="93" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B93" t="s">
         <v>53</v>
@@ -2059,10 +2062,10 @@
     </row>
     <row r="94" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B94" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C94" s="1" t="s">
         <v>19</v>
@@ -2070,21 +2073,21 @@
     </row>
     <row r="95" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B95" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="96" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B96" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C96" s="1" t="s">
         <v>19</v>
@@ -2092,10 +2095,10 @@
     </row>
     <row r="97" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B97" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C97" s="1" t="s">
         <v>19</v>
@@ -2103,10 +2106,10 @@
     </row>
     <row r="98" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B98" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C98" s="3">
         <v>2</v>
@@ -2114,76 +2117,76 @@
     </row>
     <row r="99" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B99" t="s">
+        <v>110</v>
+      </c>
+      <c r="C99" s="1" t="s">
         <v>111</v>
-      </c>
-      <c r="C99" s="1" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="100" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B100" t="s">
+        <v>112</v>
+      </c>
+      <c r="C100" s="1" t="s">
         <v>113</v>
-      </c>
-      <c r="C100" s="1" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="101" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B101" t="s">
+        <v>114</v>
+      </c>
+      <c r="C101" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="C101" s="1" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="102" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B102" t="s">
+        <v>116</v>
+      </c>
+      <c r="C102" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="C102" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="103" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B103" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="104" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B104" t="s">
+        <v>56</v>
+      </c>
+      <c r="C104" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="C104" s="1" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="105" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B105" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C105" s="1" t="s">
         <v>7</v>
@@ -2191,10 +2194,10 @@
     </row>
     <row r="106" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B106" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C106" s="1" t="s">
         <v>19</v>
@@ -2202,32 +2205,32 @@
     </row>
     <row r="107" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B107" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="108" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B108" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="109" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B109" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C109" s="1" t="s">
         <v>19</v>
@@ -2235,76 +2238,76 @@
     </row>
     <row r="110" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B110" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="111" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B111" t="s">
+        <v>63</v>
+      </c>
+      <c r="C111" s="1" t="s">
         <v>64</v>
-      </c>
-      <c r="C111" s="1" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="112" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B112" t="s">
         <v>30</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="113" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B113" t="s">
+        <v>66</v>
+      </c>
+      <c r="C113" s="1" t="s">
         <v>67</v>
-      </c>
-      <c r="C113" s="1" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="114" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B114" t="s">
         <v>32</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="115" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B115" t="s">
+        <v>69</v>
+      </c>
+      <c r="C115" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="C115" s="1" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="116" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B116" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C116" s="1" t="s">
         <v>37</v>
@@ -2312,10 +2315,10 @@
     </row>
     <row r="117" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B117" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C117" s="1" t="s">
         <v>7</v>
@@ -2323,10 +2326,10 @@
     </row>
     <row r="118" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B118" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C118" s="1" t="s">
         <v>19</v>
@@ -2334,43 +2337,43 @@
     </row>
     <row r="119" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B119" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C119" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="120" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B120" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="121" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B121" t="s">
+        <v>76</v>
+      </c>
+      <c r="C121" s="1" t="s">
         <v>77</v>
-      </c>
-      <c r="C121" s="1" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="122" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B122" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C122" s="1" t="s">
         <v>19</v>
@@ -2378,68 +2381,68 @@
     </row>
     <row r="123" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B123" t="s">
+        <v>79</v>
+      </c>
+      <c r="C123" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="C123" s="1" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="124" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B124" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="125" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B125" t="s">
         <v>38</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="126" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B126" t="s">
+        <v>83</v>
+      </c>
+      <c r="C126" s="1" t="s">
         <v>84</v>
-      </c>
-      <c r="C126" s="1" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="127" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B127" t="s">
         <v>40</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="128" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B128" t="s">
         <v>42</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -2478,7 +2481,7 @@
     </row>
     <row r="3" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B3" t="s">
         <v>15</v>
@@ -2513,15 +2516,15 @@
         <v>24</v>
       </c>
       <c r="B7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2529,7 +2532,7 @@
         <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2558,10 +2561,10 @@
     </row>
     <row r="13" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>154</v>
+      </c>
+      <c r="B13" t="s">
         <v>155</v>
-      </c>
-      <c r="B13" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2574,26 +2577,26 @@
     </row>
     <row r="15" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B15" t="s">
-        <v>158</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B16" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B17" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2606,10 +2609,10 @@
     </row>
     <row r="19" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B19" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2617,7 +2620,7 @@
         <v>34</v>
       </c>
       <c r="B20" t="s">
-        <v>164</v>
+        <v>179</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2630,7 +2633,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="B22" t="s">
         <v>37</v>
@@ -2711,7 +2714,7 @@
     </row>
     <row r="4" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B4" t="s">
         <v>5</v>
@@ -2719,7 +2722,7 @@
     </row>
     <row r="5" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="B5" t="s">
         <v>6</v>
@@ -2727,7 +2730,7 @@
     </row>
     <row r="6" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B6" t="s">
         <v>7</v>
@@ -2735,7 +2738,7 @@
     </row>
     <row r="7" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B7" t="s">
         <v>8</v>
@@ -2743,7 +2746,7 @@
     </row>
     <row r="8" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B8" t="s">
         <v>9</v>
@@ -2751,23 +2754,23 @@
     </row>
     <row r="9" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B9" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="B10" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B11" t="s">
         <v>10</v>
@@ -2775,7 +2778,7 @@
     </row>
     <row r="12" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="B12" t="s">
         <v>8</v>
@@ -2783,7 +2786,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="B13" t="s">
         <v>11</v>
@@ -2791,15 +2794,15 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="B14" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B15" t="s">
         <v>12</v>
@@ -2807,7 +2810,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B16" t="s">
         <v>19</v>
@@ -2815,7 +2818,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B17" t="s">
         <v>19</v>
@@ -2823,7 +2826,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="B18" t="s">
         <v>19</v>
@@ -2831,7 +2834,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="B19" t="s">
         <v>19</v>
@@ -2861,7 +2864,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>19</v>
@@ -2869,7 +2872,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>7</v>
@@ -2877,23 +2880,23 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>140</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>19</v>
@@ -2901,15 +2904,15 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>19</v>
@@ -2917,15 +2920,15 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>7</v>
@@ -2933,23 +2936,23 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>132</v>
+      </c>
+      <c r="B11" t="s">
         <v>133</v>
-      </c>
-      <c r="B11" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>134</v>
+      </c>
+      <c r="B12" t="s">
         <v>135</v>
-      </c>
-      <c r="B12" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B13" t="s">
         <v>19</v>
@@ -2957,7 +2960,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B14" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
feat: schedule flow 100% pass rate - both variants
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Hari.Prasad/jobbot/dazn-tests/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D74F6815-8762-6143-9D97-3044B8672F8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{813C3524-B172-B14E-AF63-375B40EB825D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17280" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Landing page" sheetId="1" r:id="rId1"/>
@@ -313,9 +313,6 @@
     <t>Upsell Highlight text</t>
   </si>
   <si>
-    <t>{{PPV_NAME}} &amp; {{SECONDARY_PPV}}.</t>
-  </si>
-  <si>
     <t>HDR and Dolby 5.1 surround sound on select events.</t>
   </si>
   <si>
@@ -605,6 +602,9 @@
   </si>
   <si>
     <t>Pay-per-views included at no extra cost. Minimum of 12 events per year including {{PPV_NAME}}.</t>
+  </si>
+  <si>
+    <t>Choose how to buy|Choose your plan</t>
   </si>
 </sst>
 </file>
@@ -1004,7 +1004,7 @@
     </row>
     <row r="2" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B2" t="s">
         <v>19</v>
@@ -1020,7 +1020,7 @@
     </row>
     <row r="4" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B4" t="s">
         <v>60</v>
@@ -1028,7 +1028,7 @@
     </row>
     <row r="5" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B5" t="s">
         <v>19</v>
@@ -1071,7 +1071,7 @@
         <v>13</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>46</v>
+        <v>181</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1148,7 +1148,7 @@
         <v>55</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1190,7 +1190,7 @@
         <v>45</v>
       </c>
       <c r="B13" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>60</v>
@@ -1245,7 +1245,7 @@
         <v>45</v>
       </c>
       <c r="B18" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>67</v>
@@ -1267,7 +1267,7 @@
         <v>45</v>
       </c>
       <c r="B20" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>70</v>
@@ -1336,7 +1336,7 @@
         <v>76</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1347,7 +1347,7 @@
         <v>78</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1358,7 +1358,7 @@
         <v>79</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1369,7 +1369,7 @@
         <v>81</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1380,7 +1380,7 @@
         <v>38</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1388,10 +1388,10 @@
         <v>45</v>
       </c>
       <c r="B31" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1402,7 +1402,7 @@
         <v>40</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1413,7 +1413,7 @@
         <v>42</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1421,10 +1421,10 @@
         <v>45</v>
       </c>
       <c r="B34" t="s">
+        <v>147</v>
+      </c>
+      <c r="C34" s="1" t="s">
         <v>148</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1432,7 +1432,7 @@
         <v>45</v>
       </c>
       <c r="B35" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>7</v>
@@ -1443,7 +1443,7 @@
         <v>45</v>
       </c>
       <c r="B36" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>51</v>
@@ -1454,7 +1454,7 @@
         <v>45</v>
       </c>
       <c r="B37" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>65</v>
@@ -1468,7 +1468,7 @@
         <v>16</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1476,10 +1476,10 @@
         <v>45</v>
       </c>
       <c r="B39" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1487,7 +1487,7 @@
     </row>
     <row r="41" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B41" t="s">
         <v>13</v>
@@ -1498,10 +1498,10 @@
     </row>
     <row r="42" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
+        <v>91</v>
+      </c>
+      <c r="B42" t="s">
         <v>92</v>
-      </c>
-      <c r="B42" t="s">
-        <v>93</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>48</v>
@@ -1509,7 +1509,7 @@
     </row>
     <row r="43" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B43" t="s">
         <v>49</v>
@@ -1520,7 +1520,7 @@
     </row>
     <row r="44" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B44" t="s">
         <v>50</v>
@@ -1531,10 +1531,10 @@
     </row>
     <row r="45" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B45" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>19</v>
@@ -1542,10 +1542,10 @@
     </row>
     <row r="46" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B46" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>60</v>
@@ -1553,7 +1553,7 @@
     </row>
     <row r="47" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B47" t="s">
         <v>53</v>
@@ -1564,10 +1564,10 @@
     </row>
     <row r="48" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B48" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>19</v>
@@ -1575,10 +1575,10 @@
     </row>
     <row r="49" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B49" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>19</v>
@@ -1586,7 +1586,7 @@
     </row>
     <row r="50" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B50" t="s">
         <v>58</v>
@@ -1597,7 +1597,7 @@
     </row>
     <row r="51" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B51" t="s">
         <v>54</v>
@@ -1608,29 +1608,29 @@
     </row>
     <row r="52" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B52" t="s">
         <v>55</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B53" t="s">
+        <v>97</v>
+      </c>
+      <c r="C53" s="1" t="s">
         <v>98</v>
-      </c>
-      <c r="C53" s="1" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B54" t="s">
         <v>18</v>
@@ -1641,7 +1641,7 @@
     </row>
     <row r="55" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B55" t="s">
         <v>20</v>
@@ -1652,10 +1652,10 @@
     </row>
     <row r="56" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B56" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>19</v>
@@ -1663,7 +1663,7 @@
     </row>
     <row r="57" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B57" t="s">
         <v>23</v>
@@ -1674,29 +1674,29 @@
     </row>
     <row r="58" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B58" t="s">
         <v>24</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="59" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B59" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="60" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B60" t="s">
         <v>62</v>
@@ -1707,7 +1707,7 @@
     </row>
     <row r="61" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B61" t="s">
         <v>63</v>
@@ -1718,7 +1718,7 @@
     </row>
     <row r="62" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B62" t="s">
         <v>30</v>
@@ -1729,10 +1729,10 @@
     </row>
     <row r="63" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B63" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C63" s="1" t="s">
         <v>67</v>
@@ -1740,7 +1740,7 @@
     </row>
     <row r="64" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B64" t="s">
         <v>32</v>
@@ -1751,10 +1751,10 @@
     </row>
     <row r="65" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B65" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C65" s="1" t="s">
         <v>70</v>
@@ -1762,7 +1762,7 @@
     </row>
     <row r="66" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B66" t="s">
         <v>71</v>
@@ -1773,7 +1773,7 @@
     </row>
     <row r="67" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B67" t="s">
         <v>72</v>
@@ -1784,7 +1784,7 @@
     </row>
     <row r="68" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B68" t="s">
         <v>73</v>
@@ -1795,7 +1795,7 @@
     </row>
     <row r="69" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B69" t="s">
         <v>74</v>
@@ -1806,7 +1806,7 @@
     </row>
     <row r="70" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B70" t="s">
         <v>75</v>
@@ -1817,109 +1817,109 @@
     </row>
     <row r="71" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B71" t="s">
         <v>76</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="72" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B72" t="s">
         <v>78</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="73" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B73" t="s">
         <v>79</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="74" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B74" t="s">
         <v>81</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="75" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B75" t="s">
         <v>38</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="76" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B76" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>84</v>
+        <v>179</v>
       </c>
     </row>
     <row r="77" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B77" t="s">
         <v>40</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="78" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B78" t="s">
         <v>42</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="79" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B79" t="s">
+        <v>147</v>
+      </c>
+      <c r="C79" s="1" t="s">
         <v>148</v>
-      </c>
-      <c r="C79" s="1" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="80" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B80" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C80" s="1" t="s">
         <v>7</v>
@@ -1927,10 +1927,10 @@
     </row>
     <row r="81" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B81" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C81" s="1" t="s">
         <v>51</v>
@@ -1938,10 +1938,10 @@
     </row>
     <row r="82" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B82" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C82" s="1" t="s">
         <v>65</v>
@@ -1949,7 +1949,7 @@
     </row>
     <row r="83" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B83" t="s">
         <v>16</v>
@@ -1960,13 +1960,13 @@
     </row>
     <row r="84" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B84" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="85" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1974,32 +1974,32 @@
     </row>
     <row r="86" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B86" t="s">
         <v>13</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="87" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B87" t="s">
+        <v>104</v>
+      </c>
+      <c r="C87" s="1" t="s">
         <v>105</v>
-      </c>
-      <c r="C87" s="1" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="88" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B88" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C88" s="1" t="s">
         <v>65</v>
@@ -2007,10 +2007,10 @@
     </row>
     <row r="89" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B89" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C89" s="1" t="s">
         <v>7</v>
@@ -2018,7 +2018,7 @@
     </row>
     <row r="90" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B90" t="s">
         <v>54</v>
@@ -2029,18 +2029,18 @@
     </row>
     <row r="91" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B91" t="s">
         <v>55</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="92" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B92" t="s">
         <v>56</v>
@@ -2051,7 +2051,7 @@
     </row>
     <row r="93" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B93" t="s">
         <v>53</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="94" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B94" t="s">
         <v>59</v>
@@ -2073,10 +2073,10 @@
     </row>
     <row r="95" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B95" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C95" s="1" t="s">
         <v>60</v>
@@ -2084,7 +2084,7 @@
     </row>
     <row r="96" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B96" t="s">
         <v>61</v>
@@ -2095,10 +2095,10 @@
     </row>
     <row r="97" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B97" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C97" s="1" t="s">
         <v>19</v>
@@ -2106,10 +2106,10 @@
     </row>
     <row r="98" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B98" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C98" s="3">
         <v>2</v>
@@ -2117,62 +2117,62 @@
     </row>
     <row r="99" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B99" t="s">
+        <v>109</v>
+      </c>
+      <c r="C99" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="C99" s="1" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="100" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B100" t="s">
+        <v>111</v>
+      </c>
+      <c r="C100" s="1" t="s">
         <v>112</v>
-      </c>
-      <c r="C100" s="1" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="101" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B101" t="s">
+        <v>113</v>
+      </c>
+      <c r="C101" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="C101" s="1" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="102" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B102" t="s">
+        <v>115</v>
+      </c>
+      <c r="C102" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="C102" s="1" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="103" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B103" t="s">
         <v>55</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="104" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B104" t="s">
         <v>56</v>
@@ -2183,10 +2183,10 @@
     </row>
     <row r="105" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B105" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C105" s="1" t="s">
         <v>7</v>
@@ -2194,10 +2194,10 @@
     </row>
     <row r="106" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B106" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C106" s="1" t="s">
         <v>19</v>
@@ -2205,10 +2205,10 @@
     </row>
     <row r="107" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B107" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C107" s="1" t="s">
         <v>60</v>
@@ -2216,10 +2216,10 @@
     </row>
     <row r="108" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B108" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C108" s="1" t="s">
         <v>77</v>
@@ -2227,10 +2227,10 @@
     </row>
     <row r="109" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B109" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C109" s="1" t="s">
         <v>19</v>
@@ -2238,10 +2238,10 @@
     </row>
     <row r="110" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B110" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C110" s="1" t="s">
         <v>80</v>
@@ -2249,7 +2249,7 @@
     </row>
     <row r="111" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B111" t="s">
         <v>63</v>
@@ -2260,7 +2260,7 @@
     </row>
     <row r="112" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B112" t="s">
         <v>30</v>
@@ -2271,7 +2271,7 @@
     </row>
     <row r="113" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B113" t="s">
         <v>66</v>
@@ -2282,7 +2282,7 @@
     </row>
     <row r="114" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B114" t="s">
         <v>32</v>
@@ -2293,7 +2293,7 @@
     </row>
     <row r="115" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B115" t="s">
         <v>69</v>
@@ -2304,7 +2304,7 @@
     </row>
     <row r="116" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B116" t="s">
         <v>71</v>
@@ -2315,7 +2315,7 @@
     </row>
     <row r="117" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B117" t="s">
         <v>72</v>
@@ -2326,7 +2326,7 @@
     </row>
     <row r="118" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B118" t="s">
         <v>73</v>
@@ -2337,7 +2337,7 @@
     </row>
     <row r="119" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B119" t="s">
         <v>74</v>
@@ -2348,18 +2348,18 @@
     </row>
     <row r="120" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B120" t="s">
         <v>75</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="121" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B121" t="s">
         <v>76</v>
@@ -2370,7 +2370,7 @@
     </row>
     <row r="122" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B122" t="s">
         <v>78</v>
@@ -2381,7 +2381,7 @@
     </row>
     <row r="123" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B123" t="s">
         <v>79</v>
@@ -2392,18 +2392,18 @@
     </row>
     <row r="124" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B124" t="s">
         <v>81</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="125" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B125" t="s">
         <v>38</v>
@@ -2414,35 +2414,35 @@
     </row>
     <row r="126" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B126" t="s">
         <v>83</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>84</v>
+        <v>179</v>
       </c>
     </row>
     <row r="127" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B127" t="s">
         <v>40</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="128" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B128" t="s">
         <v>42</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -2459,8 +2459,8 @@
   <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="144.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="153.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2481,7 +2481,7 @@
     </row>
     <row r="3" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B3" t="s">
         <v>15</v>
@@ -2516,15 +2516,15 @@
         <v>24</v>
       </c>
       <c r="B7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2532,7 +2532,7 @@
         <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2561,10 +2561,10 @@
     </row>
     <row r="13" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>153</v>
+      </c>
+      <c r="B13" t="s">
         <v>154</v>
-      </c>
-      <c r="B13" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2577,7 +2577,7 @@
     </row>
     <row r="15" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B15" t="s">
         <v>31</v>
@@ -2585,18 +2585,18 @@
     </row>
     <row r="16" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>156</v>
+      </c>
+      <c r="B16" t="s">
         <v>157</v>
-      </c>
-      <c r="B16" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B17" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2609,10 +2609,10 @@
     </row>
     <row r="19" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
+        <v>159</v>
+      </c>
+      <c r="B19" t="s">
         <v>160</v>
-      </c>
-      <c r="B19" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2620,7 +2620,7 @@
         <v>34</v>
       </c>
       <c r="B20" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2633,7 +2633,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B22" t="s">
         <v>37</v>
@@ -2684,7 +2684,7 @@
   <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="78.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2722,7 +2722,7 @@
     </row>
     <row r="5" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B5" t="s">
         <v>6</v>
@@ -2746,7 +2746,7 @@
     </row>
     <row r="8" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B8" t="s">
         <v>9</v>
@@ -2754,23 +2754,23 @@
     </row>
     <row r="9" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B9" t="s">
-        <v>155</v>
+        <v>177</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>165</v>
+      </c>
+      <c r="B10" t="s">
         <v>166</v>
-      </c>
-      <c r="B10" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B11" t="s">
         <v>10</v>
@@ -2778,7 +2778,7 @@
     </row>
     <row r="12" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B12" t="s">
         <v>8</v>
@@ -2786,7 +2786,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B13" t="s">
         <v>11</v>
@@ -2794,15 +2794,15 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>170</v>
+      </c>
+      <c r="B14" t="s">
         <v>171</v>
-      </c>
-      <c r="B14" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B15" t="s">
         <v>12</v>
@@ -2810,7 +2810,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B16" t="s">
         <v>19</v>
@@ -2818,7 +2818,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B17" t="s">
         <v>19</v>
@@ -2826,7 +2826,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B18" t="s">
         <v>19</v>
@@ -2834,7 +2834,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B19" t="s">
         <v>19</v>
@@ -2842,6 +2842,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -2864,7 +2865,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>19</v>
@@ -2880,7 +2881,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>60</v>
@@ -2888,15 +2889,15 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>139</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>19</v>
@@ -2904,15 +2905,15 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>19</v>
@@ -2920,7 +2921,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>60</v>
@@ -2928,7 +2929,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>7</v>
@@ -2936,23 +2937,23 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>131</v>
+      </c>
+      <c r="B11" t="s">
         <v>132</v>
-      </c>
-      <c r="B11" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>133</v>
+      </c>
+      <c r="B12" t="s">
         <v>134</v>
-      </c>
-      <c r="B12" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B13" t="s">
         <v>19</v>
@@ -2960,7 +2961,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B14" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
100% working new user PPV purchase journey from Schedule and Landing page
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Hari.Prasad/jobbot/dazn-tests/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{813C3524-B172-B14E-AF63-375B40EB825D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{012E86D4-8191-CD41-9D8F-CA0490A4AB84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17280" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17440" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Landing page" sheetId="1" r:id="rId1"/>
     <sheet name="PPV page" sheetId="2" r:id="rId2"/>
     <sheet name="Dazn Plan page" sheetId="3" r:id="rId3"/>
-    <sheet name="Monthly Payment page" sheetId="4" r:id="rId4"/>
+    <sheet name="Payment page" sheetId="4" r:id="rId4"/>
     <sheet name="Schedule page" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -36,30 +36,8 @@
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="796" uniqueCount="237">
   <si>
     <t>Field</t>
   </si>
@@ -76,9 +54,6 @@
     <t>Your payment is encrypted and you can change how you pay at any time.</t>
   </si>
   <si>
-    <t>{{DAZN_TIER}}</t>
-  </si>
-  <si>
     <t>Change</t>
   </si>
   <si>
@@ -307,9 +282,6 @@
     <t>PPV2 Included tag</t>
   </si>
   <si>
-    <t>Pay-per-views included at no extra cost. Minimum of 12 events per year including {{PPV_NAME}} &amp; {{SECONDARY_PPV}}.</t>
-  </si>
-  <si>
     <t>Upsell Highlight text</t>
   </si>
   <si>
@@ -595,9 +567,6 @@
     <t>N/A</t>
   </si>
   <si>
-    <t>Then ₹{{ANNUAL_PRICE}} /month for {{ANNUAL_MONTHS}} months.</t>
-  </si>
-  <si>
     <t>{{PPV_NAME}}.</t>
   </si>
   <si>
@@ -605,6 +574,180 @@
   </si>
   <si>
     <t>Choose how to buy|Choose your plan</t>
+  </si>
+  <si>
+    <t>Ultimate</t>
+  </si>
+  <si>
+    <t>Annual Pay Monthly Option</t>
+  </si>
+  <si>
+    <t>Annual Pay Monthly Title</t>
+  </si>
+  <si>
+    <t>Annual - Pay Monthly</t>
+  </si>
+  <si>
+    <t>Annual Pay Monthly Price</t>
+  </si>
+  <si>
+    <t>{{ANNUAL_PAY_MONTHLY_PRICE}}</t>
+  </si>
+  <si>
+    <t>Annual Pay Monthly Price Length</t>
+  </si>
+  <si>
+    <t>Annual Pay Monthly Contract Text</t>
+  </si>
+  <si>
+    <t>12 month contract</t>
+  </si>
+  <si>
+    <t>Annual Pay Monthly Selected</t>
+  </si>
+  <si>
+    <t>Annual Pay Upfront Option</t>
+  </si>
+  <si>
+    <t>Annual Pay Upfront Title</t>
+  </si>
+  <si>
+    <t>Annual - Pay Upfront</t>
+  </si>
+  <si>
+    <t>Annual Pay Upfront Save Badge</t>
+  </si>
+  <si>
+    <t>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</t>
+  </si>
+  <si>
+    <t>Annual Pay Upfront Price</t>
+  </si>
+  <si>
+    <t>{{ANNUAL_UPFRONT_PRICE}}</t>
+  </si>
+  <si>
+    <t>Annual Pay Upfront Price Length</t>
+  </si>
+  <si>
+    <t>/year</t>
+  </si>
+  <si>
+    <t>Annual Pay Upfront Description</t>
+  </si>
+  <si>
+    <t>Annual contract. Auto renews. Pay for a year upfront to get the best value deal.</t>
+  </si>
+  <si>
+    <t>Annual Pay Upfront Selected</t>
+  </si>
+  <si>
+    <t>Continue with DAZN Ultimate</t>
+  </si>
+  <si>
+    <t>Included Section Title</t>
+  </si>
+  <si>
+    <t>Included in Ultimate</t>
+  </si>
+  <si>
+    <t>Included Section Highlight</t>
+  </si>
+  <si>
+    <t>Ultimate Feature 1</t>
+  </si>
+  <si>
+    <t>Ultimate Feature 1 Highlight</t>
+  </si>
+  <si>
+    <t>Ultimate Feature 2</t>
+  </si>
+  <si>
+    <t>Highlights from LALIGA, Bundesliga and Saudi Pro League.</t>
+  </si>
+  <si>
+    <t>Ultimate Feature 3</t>
+  </si>
+  <si>
+    <t>Tier</t>
+  </si>
+  <si>
+    <t>Standard</t>
+  </si>
+  <si>
+    <t>Then {{CURRENCY}}{{ANNUAL_PRICE}} /month for {{ANNUAL_MONTHS}} months.</t>
+  </si>
+  <si>
+    <t>Included Section Highlight Color</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>Rate Plan</t>
+  </si>
+  <si>
+    <t>Common</t>
+  </si>
+  <si>
+    <t>All</t>
+  </si>
+  <si>
+    <t>DAZN Standard</t>
+  </si>
+  <si>
+    <t>Annual Pay Monthly</t>
+  </si>
+  <si>
+    <t>Choose how to pay</t>
+  </si>
+  <si>
+    <t>Annual - pay over time - First Month Free</t>
+  </si>
+  <si>
+    <t>Rate Plan Original Price</t>
+  </si>
+  <si>
+    <t>{{CURRENCY}}{{ANNUAL_PRICE}}</t>
+  </si>
+  <si>
+    <t>Rate Plan Discounted Price</t>
+  </si>
+  <si>
+    <t>Your Annual (pay over time) total plan yearly amount is {{CURRENCY}}{{ANNUAL_TOTAL}} (1 months at {{CURRENCY}}0/month, then {{ANNUAL_MONTHS}} months at {{CURRENCY}}{{ANNUAL_PRICE}}) and will renew automatically on {{RENEWAL_DATE}} at the existing price at the moment of the renewal. You can cancel this auto-renewal in My Account.</t>
+  </si>
+  <si>
+    <t>Rate Plan Price</t>
+  </si>
+  <si>
+    <t>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</t>
+  </si>
+  <si>
+    <t>Next Payment Label</t>
+  </si>
+  <si>
+    <t>Next payment on {{NEXT_PAYMENT_DATE}}</t>
+  </si>
+  <si>
+    <t>Your Monthly Saver plan will renew automatically on {{RENEWAL_DATE}}. Cancel this auto-renewal in My Account.</t>
+  </si>
+  <si>
+    <t>Annual Pay Upfront</t>
+  </si>
+  <si>
+    <t>{{ANNUAL_UPFRONT_PRICE}}/year</t>
+  </si>
+  <si>
+    <t>Next Annual payment on {{NEXT_PAYMENT_DATE}}</t>
+  </si>
+  <si>
+    <t>You can cancel the renewal to this subscription in My Account. You will still have full access to DAZN until the end of your annual cycle.</t>
+  </si>
+  <si>
+    <t>Don't Miss Live on DAZN Section</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pay-per-views included at no extra cost. Minimum of 12 events per year including {{SECONDARY_PPV}} &amp; {{PPV_NAME}} </t>
   </si>
 </sst>
 </file>
@@ -671,7 +814,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -682,6 +825,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -987,11 +1133,11 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="92.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1004,38 +1150,47 @@
     </row>
     <row r="2" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>124</v>
+        <v>235</v>
       </c>
       <c r="B2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>122</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>125</v>
+        <v>57</v>
       </c>
       <c r="B4" t="s">
-        <v>60</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>124</v>
+      </c>
+      <c r="B6" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -1054,7 +1209,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -1065,421 +1220,420 @@
     </row>
     <row r="2" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B10" t="s">
+        <v>55</v>
+      </c>
+      <c r="C10" s="6" t="s">
         <v>56</v>
-      </c>
-      <c r="C10" s="1" t="e" cm="1">
-        <f t="array" ref="C10">+DAZN Standard</f>
-        <v>#NAME?</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B12" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B13" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B16" t="s">
+        <v>62</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>63</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B17" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B18" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B19" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B20" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B21" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B22" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B23" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B24" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B25" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B26" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B27" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B28" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B29" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B30" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B31" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B32" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B33" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B34" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B35" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B36" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B37" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B38" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B39" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1487,486 +1641,486 @@
     </row>
     <row r="41" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B41" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B42" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B43" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B44" t="s">
+        <v>49</v>
+      </c>
+      <c r="C44" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B45" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B46" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="47" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B47" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="48" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B48" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B49" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B50" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B51" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B52" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B53" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B54" t="s">
+        <v>17</v>
+      </c>
+      <c r="C54" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="C54" s="1" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B55" t="s">
+        <v>19</v>
+      </c>
+      <c r="C55" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="C55" s="1" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B56" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="57" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B57" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="58" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B58" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="59" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B59" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="60" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B60" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="61" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B61" t="s">
+        <v>62</v>
+      </c>
+      <c r="C61" s="1" t="s">
         <v>63</v>
-      </c>
-      <c r="C61" s="1" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="62" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B62" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="63" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B63" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="64" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B64" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="65" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B65" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="66" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B66" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="67" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B67" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="68" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B68" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="69" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B69" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="70" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B70" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="71" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B71" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="72" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B72" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="73" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B73" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="74" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B74" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="75" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B75" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
     </row>
     <row r="76" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B76" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
     </row>
     <row r="77" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B77" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="78" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B78" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="79" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B79" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="80" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B80" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="81" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B81" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="82" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B82" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="83" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B83" t="s">
+        <v>15</v>
+      </c>
+      <c r="C83" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="C83" s="1" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="84" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B84" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="85" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1974,142 +2128,142 @@
     </row>
     <row r="86" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B86" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="87" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
+        <v>100</v>
+      </c>
+      <c r="B87" t="s">
         <v>102</v>
       </c>
-      <c r="B87" t="s">
-        <v>104</v>
-      </c>
       <c r="C87" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="88" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B88" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="89" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B89" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="90" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B90" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="91" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B91" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="92" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B92" t="s">
+        <v>55</v>
+      </c>
+      <c r="C92" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="C92" s="1" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="93" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B93" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="94" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B94" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="95" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B95" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="96" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B96" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="97" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B97" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="98" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B98" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C98" s="3">
         <v>2</v>
@@ -2117,332 +2271,332 @@
     </row>
     <row r="99" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B99" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="100" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B100" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="101" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B101" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="102" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B102" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="103" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B103" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="104" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B104" t="s">
+        <v>55</v>
+      </c>
+      <c r="C104" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="C104" s="1" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="105" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B105" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="106" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B106" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="107" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B107" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="108" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B108" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="109" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B109" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="110" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B110" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="111" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B111" t="s">
+        <v>62</v>
+      </c>
+      <c r="C111" s="1" t="s">
         <v>63</v>
-      </c>
-      <c r="C111" s="1" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="112" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B112" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="113" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B113" t="s">
+        <v>65</v>
+      </c>
+      <c r="C113" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="C113" s="1" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="114" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B114" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="115" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B115" t="s">
+        <v>68</v>
+      </c>
+      <c r="C115" s="1" t="s">
         <v>69</v>
-      </c>
-      <c r="C115" s="1" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="116" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B116" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C116" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="117" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B117" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="118" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B118" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="119" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B119" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C119" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="120" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B120" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="121" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B121" t="s">
+        <v>75</v>
+      </c>
+      <c r="C121" s="1" t="s">
         <v>76</v>
-      </c>
-      <c r="C121" s="1" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="122" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B122" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C122" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="123" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B123" t="s">
+        <v>78</v>
+      </c>
+      <c r="C123" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="C123" s="1" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="124" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B124" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="125" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B125" t="s">
-        <v>38</v>
-      </c>
-      <c r="C125" s="1" t="s">
-        <v>82</v>
+        <v>37</v>
+      </c>
+      <c r="C125" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="126" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B126" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
     </row>
     <row r="127" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B127" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="128" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B128" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -2456,223 +2610,556 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="153.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="153.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>210</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>211</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
         <v>13</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="3" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>211</v>
+      </c>
+      <c r="B3" t="s">
+        <v>149</v>
+      </c>
+      <c r="C3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>151</v>
-      </c>
-      <c r="B3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
         <v>18</v>
       </c>
-      <c r="B4" t="s">
+    </row>
+    <row r="5" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>211</v>
+      </c>
+      <c r="B5" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="C5" t="s">
         <v>20</v>
       </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="6" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>211</v>
+      </c>
+      <c r="B6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>211</v>
+      </c>
+      <c r="B7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>211</v>
+      </c>
+      <c r="B8" t="s">
+        <v>150</v>
+      </c>
+      <c r="C8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>211</v>
+      </c>
+      <c r="B9" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B6" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>152</v>
-      </c>
-      <c r="B8" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C9" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>26</v>
+        <v>211</v>
       </c>
       <c r="B10" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>211</v>
+      </c>
+      <c r="B11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>211</v>
+      </c>
+      <c r="B12" t="s">
         <v>27</v>
       </c>
-      <c r="B11" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+      <c r="C12" t="s">
         <v>28</v>
       </c>
-      <c r="B12" t="s">
+    </row>
+    <row r="13" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>211</v>
+      </c>
+      <c r="B13" t="s">
+        <v>151</v>
+      </c>
+      <c r="C13" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>211</v>
+      </c>
+      <c r="B14" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
+      <c r="C14" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>211</v>
+      </c>
+      <c r="B15" t="s">
         <v>153</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C15" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>211</v>
+      </c>
+      <c r="B16" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>30</v>
-      </c>
-      <c r="B14" t="s">
+      <c r="C16" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>211</v>
+      </c>
+      <c r="B17" t="s">
+        <v>156</v>
+      </c>
+      <c r="C17" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>211</v>
+      </c>
+      <c r="B18" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>155</v>
-      </c>
-      <c r="B15" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>156</v>
-      </c>
-      <c r="B16" t="s">
+      <c r="C18" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>211</v>
+      </c>
+      <c r="B19" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+      <c r="C19" t="s">
         <v>158</v>
       </c>
-      <c r="B17" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>32</v>
-      </c>
-      <c r="B18" t="s">
+    </row>
+    <row r="20" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>211</v>
+      </c>
+      <c r="B20" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
+      <c r="C20" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>211</v>
+      </c>
+      <c r="B21" t="s">
+        <v>34</v>
+      </c>
+      <c r="C21" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>211</v>
+      </c>
+      <c r="B22" t="s">
         <v>159</v>
       </c>
-      <c r="B19" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>34</v>
-      </c>
-      <c r="B20" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+      <c r="C22" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>211</v>
+      </c>
+      <c r="B23" t="s">
+        <v>37</v>
+      </c>
+      <c r="C23" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>211</v>
+      </c>
+      <c r="B24" t="s">
+        <v>39</v>
+      </c>
+      <c r="C24" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>211</v>
+      </c>
+      <c r="B25" t="s">
+        <v>41</v>
+      </c>
+      <c r="C25" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>211</v>
+      </c>
+      <c r="B26" t="s">
+        <v>15</v>
+      </c>
+      <c r="C26" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>210</v>
+      </c>
+      <c r="B29" t="s">
+        <v>0</v>
+      </c>
+      <c r="C29" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>179</v>
+      </c>
+      <c r="B30" t="s">
+        <v>12</v>
+      </c>
+      <c r="C30" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>179</v>
+      </c>
+      <c r="B31" t="s">
+        <v>180</v>
+      </c>
+      <c r="C31" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>179</v>
+      </c>
+      <c r="B32" t="s">
+        <v>181</v>
+      </c>
+      <c r="C32" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>179</v>
+      </c>
+      <c r="B33" t="s">
+        <v>183</v>
+      </c>
+      <c r="C33" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>179</v>
+      </c>
+      <c r="B34" t="s">
+        <v>185</v>
+      </c>
+      <c r="C34" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>179</v>
+      </c>
+      <c r="B35" t="s">
+        <v>186</v>
+      </c>
+      <c r="C35" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>179</v>
+      </c>
+      <c r="B36" t="s">
+        <v>188</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>179</v>
+      </c>
+      <c r="B37" t="s">
+        <v>189</v>
+      </c>
+      <c r="C37" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>179</v>
+      </c>
+      <c r="B38" t="s">
+        <v>190</v>
+      </c>
+      <c r="C38" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>179</v>
+      </c>
+      <c r="B39" t="s">
+        <v>192</v>
+      </c>
+      <c r="C39" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>179</v>
+      </c>
+      <c r="B40" t="s">
+        <v>194</v>
+      </c>
+      <c r="C40" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>179</v>
+      </c>
+      <c r="B41" t="s">
+        <v>196</v>
+      </c>
+      <c r="C41" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>179</v>
+      </c>
+      <c r="B42" t="s">
+        <v>198</v>
+      </c>
+      <c r="C42" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>179</v>
+      </c>
+      <c r="B43" t="s">
+        <v>200</v>
+      </c>
+      <c r="C43" t="s">
         <v>35</v>
       </c>
-      <c r="B21" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>161</v>
-      </c>
-      <c r="B22" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>38</v>
-      </c>
-      <c r="B23" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
-        <v>40</v>
-      </c>
-      <c r="B24" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
-        <v>42</v>
-      </c>
-      <c r="B25" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
-        <v>16</v>
-      </c>
-      <c r="B26" t="s">
-        <v>17</v>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>179</v>
+      </c>
+      <c r="B44" t="s">
+        <v>15</v>
+      </c>
+      <c r="C44" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>179</v>
+      </c>
+      <c r="B45" t="s">
+        <v>202</v>
+      </c>
+      <c r="C45" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>179</v>
+      </c>
+      <c r="B46" t="s">
+        <v>204</v>
+      </c>
+      <c r="C46" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>179</v>
+      </c>
+      <c r="B47" t="s">
+        <v>213</v>
+      </c>
+      <c r="C47" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>179</v>
+      </c>
+      <c r="B48" t="s">
+        <v>205</v>
+      </c>
+      <c r="C48" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>179</v>
+      </c>
+      <c r="B49" t="s">
+        <v>206</v>
+      </c>
+      <c r="C49" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>179</v>
+      </c>
+      <c r="B50" t="s">
+        <v>207</v>
+      </c>
+      <c r="C50" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>179</v>
+      </c>
+      <c r="B51" t="s">
+        <v>209</v>
+      </c>
+      <c r="C51" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -2681,163 +3168,825 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="78.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="255.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>210</v>
+      </c>
+      <c r="B1" t="s">
+        <v>215</v>
+      </c>
+      <c r="C1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>216</v>
       </c>
       <c r="B2" t="s">
+        <v>217</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>216</v>
+      </c>
+      <c r="B3" t="s">
+        <v>217</v>
+      </c>
+      <c r="C3" t="s">
+        <v>160</v>
+      </c>
+      <c r="D3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>216</v>
+      </c>
+      <c r="B4" t="s">
+        <v>217</v>
+      </c>
+      <c r="C4" t="s">
+        <v>172</v>
+      </c>
+      <c r="D4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>216</v>
+      </c>
+      <c r="B5" t="s">
+        <v>217</v>
+      </c>
+      <c r="C5" t="s">
+        <v>173</v>
+      </c>
+      <c r="D5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>216</v>
+      </c>
+      <c r="B6" t="s">
+        <v>217</v>
+      </c>
+      <c r="C6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>210</v>
+      </c>
+      <c r="B8" t="s">
+        <v>215</v>
+      </c>
+      <c r="C8" t="s">
+        <v>0</v>
+      </c>
+      <c r="D8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>211</v>
+      </c>
+      <c r="B9" t="s">
+        <v>214</v>
+      </c>
+      <c r="C9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B10" t="s">
+        <v>214</v>
+      </c>
+      <c r="C10" t="s">
+        <v>55</v>
+      </c>
+      <c r="D10" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>211</v>
+      </c>
+      <c r="B11" t="s">
+        <v>214</v>
+      </c>
+      <c r="C11" t="s">
+        <v>57</v>
+      </c>
+      <c r="D11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>211</v>
+      </c>
+      <c r="B12" t="s">
+        <v>214</v>
+      </c>
+      <c r="C12" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>211</v>
+      </c>
+      <c r="B13" t="s">
+        <v>214</v>
+      </c>
+      <c r="C13" t="s">
+        <v>161</v>
+      </c>
+      <c r="D13" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>211</v>
+      </c>
+      <c r="B14" t="s">
+        <v>214</v>
+      </c>
+      <c r="C14" t="s">
         <v>162</v>
       </c>
-      <c r="B5" t="s">
+      <c r="D14" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>211</v>
+      </c>
+      <c r="B15" t="s">
+        <v>214</v>
+      </c>
+      <c r="C15" t="s">
+        <v>163</v>
+      </c>
+      <c r="D15" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>211</v>
+      </c>
+      <c r="B16" t="s">
+        <v>214</v>
+      </c>
+      <c r="C16" t="s">
+        <v>165</v>
+      </c>
+      <c r="D16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>211</v>
+      </c>
+      <c r="B17" t="s">
+        <v>214</v>
+      </c>
+      <c r="C17" t="s">
+        <v>166</v>
+      </c>
+      <c r="D17" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>211</v>
+      </c>
+      <c r="B18" t="s">
+        <v>214</v>
+      </c>
+      <c r="C18" t="s">
+        <v>167</v>
+      </c>
+      <c r="D18" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>211</v>
+      </c>
+      <c r="B19" t="s">
+        <v>214</v>
+      </c>
+      <c r="C19" t="s">
+        <v>168</v>
+      </c>
+      <c r="D19" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>211</v>
+      </c>
+      <c r="B20" t="s">
+        <v>214</v>
+      </c>
+      <c r="C20" t="s">
+        <v>170</v>
+      </c>
+      <c r="D20" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>211</v>
+      </c>
+      <c r="B21" t="s">
+        <v>214</v>
+      </c>
+      <c r="C21" t="s">
+        <v>171</v>
+      </c>
+      <c r="D21" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>210</v>
+      </c>
+      <c r="B23" t="s">
+        <v>215</v>
+      </c>
+      <c r="C23" t="s">
+        <v>0</v>
+      </c>
+      <c r="D23" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>211</v>
+      </c>
+      <c r="B24" t="s">
+        <v>219</v>
+      </c>
+      <c r="C24" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>211</v>
+      </c>
+      <c r="B25" t="s">
+        <v>219</v>
+      </c>
+      <c r="C25" t="s">
+        <v>55</v>
+      </c>
+      <c r="D25" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>211</v>
+      </c>
+      <c r="B26" t="s">
+        <v>219</v>
+      </c>
+      <c r="C26" t="s">
+        <v>57</v>
+      </c>
+      <c r="D26" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>58</v>
-      </c>
-      <c r="B6" t="s">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>211</v>
+      </c>
+      <c r="B27" t="s">
+        <v>219</v>
+      </c>
+      <c r="C27" t="s">
+        <v>53</v>
+      </c>
+      <c r="D27" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>54</v>
-      </c>
-      <c r="B7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>163</v>
-      </c>
-      <c r="B8" t="s">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>211</v>
+      </c>
+      <c r="B28" t="s">
+        <v>219</v>
+      </c>
+      <c r="C28" t="s">
+        <v>215</v>
+      </c>
+      <c r="D28" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>211</v>
+      </c>
+      <c r="B29" t="s">
+        <v>219</v>
+      </c>
+      <c r="C29" t="s">
+        <v>222</v>
+      </c>
+      <c r="D29" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>211</v>
+      </c>
+      <c r="B30" t="s">
+        <v>219</v>
+      </c>
+      <c r="C30" t="s">
+        <v>224</v>
+      </c>
+      <c r="D30" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>211</v>
+      </c>
+      <c r="B31" t="s">
+        <v>219</v>
+      </c>
+      <c r="C31" t="s">
+        <v>165</v>
+      </c>
+      <c r="D31" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>211</v>
+      </c>
+      <c r="B32" t="s">
+        <v>219</v>
+      </c>
+      <c r="C32" t="s">
+        <v>166</v>
+      </c>
+      <c r="D32" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>211</v>
+      </c>
+      <c r="B33" t="s">
+        <v>219</v>
+      </c>
+      <c r="C33" t="s">
+        <v>167</v>
+      </c>
+      <c r="D33" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>211</v>
+      </c>
+      <c r="B34" t="s">
+        <v>219</v>
+      </c>
+      <c r="C34" t="s">
+        <v>168</v>
+      </c>
+      <c r="D34" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>211</v>
+      </c>
+      <c r="B35" t="s">
+        <v>219</v>
+      </c>
+      <c r="C35" t="s">
+        <v>170</v>
+      </c>
+      <c r="D35" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>211</v>
+      </c>
+      <c r="B36" t="s">
+        <v>219</v>
+      </c>
+      <c r="C36" t="s">
+        <v>171</v>
+      </c>
+      <c r="D36" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>179</v>
+      </c>
+      <c r="B38" t="s">
+        <v>219</v>
+      </c>
+      <c r="C38" t="s">
+        <v>12</v>
+      </c>
+      <c r="D38" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>179</v>
+      </c>
+      <c r="B39" t="s">
+        <v>219</v>
+      </c>
+      <c r="C39" t="s">
+        <v>55</v>
+      </c>
+      <c r="D39" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>179</v>
+      </c>
+      <c r="B40" t="s">
+        <v>219</v>
+      </c>
+      <c r="C40" t="s">
+        <v>57</v>
+      </c>
+      <c r="D40" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>179</v>
+      </c>
+      <c r="B41" t="s">
+        <v>219</v>
+      </c>
+      <c r="C41" t="s">
+        <v>53</v>
+      </c>
+      <c r="D41" t="s">
         <v>164</v>
       </c>
-      <c r="B9" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>179</v>
+      </c>
+      <c r="B42" t="s">
+        <v>219</v>
+      </c>
+      <c r="C42" t="s">
+        <v>215</v>
+      </c>
+      <c r="D42" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>179</v>
+      </c>
+      <c r="B43" t="s">
+        <v>219</v>
+      </c>
+      <c r="C43" t="s">
+        <v>226</v>
+      </c>
+      <c r="D43" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>179</v>
+      </c>
+      <c r="B44" t="s">
+        <v>219</v>
+      </c>
+      <c r="C44" t="s">
         <v>165</v>
       </c>
-      <c r="B10" t="s">
+      <c r="D44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>179</v>
+      </c>
+      <c r="B45" t="s">
+        <v>219</v>
+      </c>
+      <c r="C45" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>167</v>
-      </c>
-      <c r="B11" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+      <c r="D45" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>179</v>
+      </c>
+      <c r="B46" t="s">
+        <v>219</v>
+      </c>
+      <c r="C46" t="s">
+        <v>228</v>
+      </c>
+      <c r="D46" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>179</v>
+      </c>
+      <c r="B47" t="s">
+        <v>219</v>
+      </c>
+      <c r="C47" t="s">
         <v>168</v>
       </c>
-      <c r="B12" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>169</v>
-      </c>
-      <c r="B13" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
+      <c r="D47" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>179</v>
+      </c>
+      <c r="B48" t="s">
+        <v>219</v>
+      </c>
+      <c r="C48" t="s">
         <v>170</v>
       </c>
-      <c r="B14" t="s">
+      <c r="D48" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>179</v>
+      </c>
+      <c r="B49" t="s">
+        <v>219</v>
+      </c>
+      <c r="C49" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>172</v>
-      </c>
-      <c r="B15" t="s">
+      <c r="D49" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>179</v>
+      </c>
+      <c r="B51" t="s">
+        <v>231</v>
+      </c>
+      <c r="C51" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>173</v>
-      </c>
-      <c r="B16" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>174</v>
-      </c>
-      <c r="B17" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>175</v>
-      </c>
-      <c r="B18" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>176</v>
-      </c>
-      <c r="B19" t="s">
-        <v>19</v>
+      <c r="D51" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>179</v>
+      </c>
+      <c r="B52" t="s">
+        <v>231</v>
+      </c>
+      <c r="C52" t="s">
+        <v>55</v>
+      </c>
+      <c r="D52" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>179</v>
+      </c>
+      <c r="B53" t="s">
+        <v>231</v>
+      </c>
+      <c r="C53" t="s">
+        <v>57</v>
+      </c>
+      <c r="D53" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>179</v>
+      </c>
+      <c r="B54" t="s">
+        <v>231</v>
+      </c>
+      <c r="C54" t="s">
+        <v>53</v>
+      </c>
+      <c r="D54" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>179</v>
+      </c>
+      <c r="B55" t="s">
+        <v>231</v>
+      </c>
+      <c r="C55" t="s">
+        <v>215</v>
+      </c>
+      <c r="D55" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>179</v>
+      </c>
+      <c r="B56" t="s">
+        <v>231</v>
+      </c>
+      <c r="C56" t="s">
+        <v>226</v>
+      </c>
+      <c r="D56" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>179</v>
+      </c>
+      <c r="B57" t="s">
+        <v>231</v>
+      </c>
+      <c r="C57" t="s">
+        <v>165</v>
+      </c>
+      <c r="D57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>179</v>
+      </c>
+      <c r="B58" t="s">
+        <v>231</v>
+      </c>
+      <c r="C58" t="s">
+        <v>166</v>
+      </c>
+      <c r="D58" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>179</v>
+      </c>
+      <c r="B59" t="s">
+        <v>231</v>
+      </c>
+      <c r="C59" t="s">
+        <v>228</v>
+      </c>
+      <c r="D59" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>179</v>
+      </c>
+      <c r="B60" t="s">
+        <v>231</v>
+      </c>
+      <c r="C60" t="s">
+        <v>168</v>
+      </c>
+      <c r="D60" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>179</v>
+      </c>
+      <c r="B61" t="s">
+        <v>231</v>
+      </c>
+      <c r="C61" t="s">
+        <v>170</v>
+      </c>
+      <c r="D61" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>179</v>
+      </c>
+      <c r="B62" t="s">
+        <v>231</v>
+      </c>
+      <c r="C62" t="s">
+        <v>171</v>
+      </c>
+      <c r="D62" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -2865,106 +4014,106 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B11" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B12" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Merge Gopi's source/main: pages cleanup, utils updates, cookie banner fix, surfacing points, DaznPlan config
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -15,8 +15,7 @@
     <sheet name="Upgrade Confirmation page" sheetId="10" r:id="rId10"/>
     <sheet name="Phone Number page" sheetId="11" r:id="rId11"/>
     <sheet name="OTP page" sheetId="12" r:id="rId12"/>
-    <sheet name="Home of Boxing" sheetId="13" r:id="rId13"/>
-    <sheet name="Home page" sheetId="14" r:id="rId14"/>
+    <sheet name="Home page" sheetId="13" r:id="rId13"/>
   </sheets>
 </workbook>
 </file>
@@ -425,7 +424,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Don&amp;apos;t Miss Live on DAZN Section</v>
+        <v>Don't Miss Live on DAZN Section</v>
       </c>
       <c r="B2" t="str">
         <v>Yes</v>
@@ -472,7 +471,7 @@
         <v>Buy Now Button</v>
       </c>
       <c r="B6" t="str">
-        <v>Buy now</v>
+        <v>Yes</v>
       </c>
       <c r="C6" t="str">
         <v>landing</v>
@@ -732,7 +731,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:C22"/>
   </ignoredErrors>
@@ -792,7 +790,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
   </ignoredErrors>
@@ -816,7 +813,7 @@
         <v>Page Title</v>
       </c>
       <c r="B2" t="str">
-        <v>Verify your phone</v>
+        <v>Enter the code below to continue</v>
       </c>
     </row>
     <row r="3">
@@ -852,7 +849,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
   </ignoredErrors>
@@ -861,7 +857,12 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C6"/>
+  <cols>
+    <col min="1" max="1" width="21.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -876,21 +877,21 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>home-boxing-banner</v>
+        <v>home-biggest-fights</v>
       </c>
       <c r="B2" t="str">
-        <v>Best of Boxing Section</v>
+        <v>The Biggest Fights Heading</v>
       </c>
       <c r="C2" t="str">
-        <v>Present</v>
+        <v>The Biggest Fights</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>home-boxing-banner</v>
+        <v>home-biggest-fights</v>
       </c>
       <c r="B3" t="str">
-        <v>Banner - Event Title</v>
+        <v>PPV Name</v>
       </c>
       <c r="C3" t="str">
         <v>{{PPV_NAME}}</v>
@@ -898,10 +899,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>home-boxing-banner</v>
+        <v>home-biggest-fights</v>
       </c>
       <c r="B4" t="str">
-        <v>Banner - Event Date</v>
+        <v>PPV Date and Time Text</v>
       </c>
       <c r="C4" t="str">
         <v>{{PPV_DATE}}</v>
@@ -909,268 +910,36 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>home-boxing-banner</v>
+        <v>home-biggest-fights</v>
       </c>
       <c r="B5" t="str">
-        <v>Banner - Event Description</v>
+        <v>PPV Image Present</v>
       </c>
       <c r="C5" t="str">
-        <v>{{PPV_DESCRIPTION}}</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>home-boxing-banner</v>
+        <v>home-biggest-fights</v>
       </c>
       <c r="B6" t="str">
-        <v>Banner - Buy Now CTA</v>
+        <v>Buy Now CTA</v>
       </c>
       <c r="C6" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>home-boxing-banner</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Banner - Fight Card CTA</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>home-boxing-tile</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Best of Boxing Section</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Present</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>home-boxing-tile</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Popup - Event Title</v>
-      </c>
-      <c r="C9" t="str">
-        <v>{{PPV_NAME}}</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>home-boxing-tile</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Popup - Event Date</v>
-      </c>
-      <c r="C10" t="str">
-        <v>{{PPV_DATE}}</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>home-boxing-tile</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Popup - Promoter</v>
-      </c>
-      <c r="C11" t="str">
-        <v>{{PPV_PROMOTER}}</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>home-boxing-tile</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Popup - Buy Now CTA</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>home-boxing-tile</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Popup - Event Description</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>home-boxing-tile</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Popup - Close Button</v>
-      </c>
-      <c r="C14" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C14"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Flow</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Field</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Expected</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>home-page-banner</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Banner - Event Title</v>
-      </c>
-      <c r="C2" t="str">
-        <v>{{PPV_NAME}}</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>home-page-banner</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Banner - Event Date</v>
-      </c>
-      <c r="C3" t="str">
-        <v>{{PPV_DATE}}</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>home-page-banner</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Banner - Event Description</v>
-      </c>
-      <c r="C4" t="str">
-        <v>{{PPV_DESCRIPTION}}</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>home-page-banner</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Banner - Buy Now CTA</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>home-page-banner</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Banner - Fight Card CTA</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>home-page-dont-miss</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Popup - Event Title</v>
-      </c>
-      <c r="C7" t="str">
-        <v>{{PPV_NAME}}</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>home-page-dont-miss</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Popup - Event Date</v>
-      </c>
-      <c r="C8" t="str">
-        <v>{{PPV_DATE}}</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>home-page-dont-miss</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Popup - Promoter</v>
-      </c>
-      <c r="C9" t="str">
-        <v>{{PPV_PROMOTER}}</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>home-page-dont-miss</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Popup - Buy Now CTA</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>home-page-dont-miss</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Popup - Event Description</v>
-      </c>
-      <c r="C11" t="str">
-        <v>{{PPV_DESCRIPTION}}</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>home-page-dont-miss</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Popup - Close Button</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Visible</v>
+        <v>Buy now</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C55"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1210,7 +979,7 @@
         <v>Event Subtitle</v>
       </c>
       <c r="B4" t="str">
-        <v>{{BOXING_BANNER_SUBTITLE}}</v>
+        <v>Main Event  AO Arena, Manchester  11:30 pm.</v>
       </c>
       <c r="C4" t="str">
         <v>boxing</v>
@@ -1273,76 +1042,76 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Bundle Section Present</v>
+        <v>Upcoming Big Fights Heading</v>
       </c>
       <c r="B10" t="str">
-        <v>Yes</v>
+        <v>Upcoming Big Fights</v>
       </c>
       <c r="C10" t="str">
-        <v>boxing-bundle</v>
+        <v>boxing-upcoming</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Bundle Section Title</v>
+        <v>PPV Name</v>
       </c>
       <c r="B11" t="str">
-        <v>{{BUNDLE_SECTION_TITLE}}</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="C11" t="str">
-        <v>boxing-bundle</v>
+        <v>boxing-upcoming</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Bundle Section Subtitle</v>
+        <v>PPV Date and Time Text</v>
       </c>
       <c r="B12" t="str">
-        <v>{{BUNDLE_SECTION_SUBTITLE}}</v>
+        <v>{{PPV_DATE}}</v>
       </c>
       <c r="C12" t="str">
-        <v>boxing-bundle</v>
+        <v>boxing-upcoming</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Bundle Title</v>
+        <v>PPV Description Text</v>
       </c>
       <c r="B13" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>{{PPV_LOCATION}}</v>
       </c>
       <c r="C13" t="str">
-        <v>boxing-bundle</v>
+        <v>boxing-upcoming</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Bundle Description</v>
+        <v>PPV Image Present</v>
       </c>
       <c r="B14" t="str">
-        <v>{{BUNDLE_DESCRIPTION}}</v>
+        <v>Yes</v>
       </c>
       <c r="C14" t="str">
-        <v>boxing-bundle</v>
+        <v>boxing-upcoming</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Bundle Price</v>
+        <v>Buy Now CTA</v>
       </c>
       <c r="B15" t="str">
-        <v>{{BUNDLE_PRICE}}</v>
+        <v>Buy now</v>
       </c>
       <c r="C15" t="str">
-        <v>boxing-bundle</v>
+        <v>boxing-upcoming</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Bundle Original Price</v>
+        <v>Bundle Section Present</v>
       </c>
       <c r="B16" t="str">
-        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
+        <v>Yes</v>
       </c>
       <c r="C16" t="str">
         <v>boxing-bundle</v>
@@ -1350,10 +1119,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Bundle Save Badge</v>
+        <v>Bundle Section Title</v>
       </c>
       <c r="B17" t="str">
-        <v>{{BUNDLE_SAVE_BADGE}}</v>
+        <v>{{BUNDLE_SECTION_TITLE}}</v>
       </c>
       <c r="C17" t="str">
         <v>boxing-bundle</v>
@@ -1361,10 +1130,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Bundle Fight Count</v>
+        <v>Bundle Section Subtitle</v>
       </c>
       <c r="B18" t="str">
-        <v>{{BUNDLE_FIGHT_COUNT}}</v>
+        <v>{{BUNDLE_SECTION_SUBTITLE}}</v>
       </c>
       <c r="C18" t="str">
         <v>boxing-bundle</v>
@@ -1372,10 +1141,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Bundle PPV 1 Name</v>
+        <v>Bundle Title</v>
       </c>
       <c r="B19" t="str">
-        <v>{{BUNDLE_PPV1_NAME}}</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="C19" t="str">
         <v>boxing-bundle</v>
@@ -1383,10 +1152,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Bundle PPV 1 Date</v>
+        <v>Bundle Description</v>
       </c>
       <c r="B20" t="str">
-        <v>{{BUNDLE_PPV1_LANDING_DATE}}</v>
+        <v>{{BUNDLE_DESCRIPTION}}</v>
       </c>
       <c r="C20" t="str">
         <v>boxing-bundle</v>
@@ -1394,10 +1163,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Bundle PPV 1 Image</v>
+        <v>Bundle Price</v>
       </c>
       <c r="B21" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_PRICE}}</v>
       </c>
       <c r="C21" t="str">
         <v>boxing-bundle</v>
@@ -1405,10 +1174,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Bundle PPV 2 Name</v>
+        <v>Bundle Original Price</v>
       </c>
       <c r="B22" t="str">
-        <v>{{BUNDLE_PPV2_NAME}}</v>
+        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
       </c>
       <c r="C22" t="str">
         <v>boxing-bundle</v>
@@ -1416,10 +1185,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Bundle PPV 2 Date</v>
+        <v>Bundle Save Badge</v>
       </c>
       <c r="B23" t="str">
-        <v>{{BUNDLE_PPV2_LANDING_DATE}}</v>
+        <v>{{BUNDLE_SAVE_BADGE}}</v>
       </c>
       <c r="C23" t="str">
         <v>boxing-bundle</v>
@@ -1427,10 +1196,10 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Bundle PPV 2 Image</v>
+        <v>Bundle Fight Count</v>
       </c>
       <c r="B24" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_FIGHT_COUNT}}</v>
       </c>
       <c r="C24" t="str">
         <v>boxing-bundle</v>
@@ -1438,10 +1207,10 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Get Started CTA</v>
+        <v>Bundle PPV 1 Name</v>
       </c>
       <c r="B25" t="str">
-        <v>Get Started</v>
+        <v>{{BUNDLE_PPV1_NAME}}</v>
       </c>
       <c r="C25" t="str">
         <v>boxing-bundle</v>
@@ -1449,76 +1218,76 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Page Title</v>
+        <v>Bundle PPV 1 Date</v>
       </c>
       <c r="B26" t="str">
-        <v>Choose the right plan for you.</v>
+        <v>{{BUNDLE_PPV1_LANDING_DATE}}</v>
       </c>
       <c r="C26" t="str">
-        <v>boxing-bundle-ppv</v>
+        <v>boxing-bundle</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Header Sub Text</v>
+        <v>Bundle PPV 1 Image</v>
       </c>
       <c r="B27" t="str">
-        <v>To watch your pay-per-view, you&amp;apos;ll need a DAZN plan.</v>
+        <v>Yes</v>
       </c>
       <c r="C27" t="str">
-        <v>boxing-bundle-ppv</v>
+        <v>boxing-bundle</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Bundle Card Title</v>
+        <v>Bundle PPV 2 Name</v>
       </c>
       <c r="B28" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>{{BUNDLE_PPV2_NAME}}</v>
       </c>
       <c r="C28" t="str">
-        <v>boxing-bundle-ppv</v>
+        <v>boxing-bundle</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Bundle Card Description</v>
+        <v>Bundle PPV 2 Date</v>
       </c>
       <c r="B29" t="str">
-        <v>{{BUNDLE_PPV_CARD_DESCRIPTION}}</v>
+        <v>{{BUNDLE_PPV2_LANDING_DATE}}</v>
       </c>
       <c r="C29" t="str">
-        <v>boxing-bundle-ppv</v>
+        <v>boxing-bundle</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Bundle Card Selected</v>
+        <v>Bundle PPV 2 Image</v>
       </c>
       <c r="B30" t="str">
         <v>Yes</v>
       </c>
       <c r="C30" t="str">
-        <v>boxing-bundle-ppv</v>
+        <v>boxing-bundle</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Bundle Card Price</v>
+        <v>Get Started CTA</v>
       </c>
       <c r="B31" t="str">
-        <v>{{BUNDLE_PRICE}}</v>
+        <v>Get Started</v>
       </c>
       <c r="C31" t="str">
-        <v>boxing-bundle-ppv</v>
+        <v>boxing-bundle</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Bundle Card Original Price</v>
+        <v>Page Title</v>
       </c>
       <c r="B32" t="str">
-        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
+        <v>Choose the right plan for you.</v>
       </c>
       <c r="C32" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1526,10 +1295,10 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Bundle Card Save Badge</v>
+        <v>Header Sub Text</v>
       </c>
       <c r="B33" t="str">
-        <v>{{BUNDLE_SAVE_BADGE}}</v>
+        <v>To watch your pay-per-view, you'll need a DAZN plan.</v>
       </c>
       <c r="C33" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1537,10 +1306,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Bundle PPV 1 Full Name</v>
+        <v>Bundle Card Title</v>
       </c>
       <c r="B34" t="str">
-        <v>{{BUNDLE_PPV1_FULL_NAME}}</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="C34" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1548,10 +1317,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Bundle PPV 1 PPV Date</v>
+        <v>Bundle Card Description</v>
       </c>
       <c r="B35" t="str">
-        <v>{{BUNDLE_PPV1_DATE}}</v>
+        <v>{{BUNDLE_PPV_CARD_DESCRIPTION}}</v>
       </c>
       <c r="C35" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1559,7 +1328,7 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Bundle PPV 1 PPV Image</v>
+        <v>Bundle Card Selected</v>
       </c>
       <c r="B36" t="str">
         <v>Yes</v>
@@ -1570,10 +1339,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Bundle PPV 2 Full Name</v>
+        <v>Bundle Card Price</v>
       </c>
       <c r="B37" t="str">
-        <v>{{BUNDLE_PPV2_FULL_NAME}}</v>
+        <v>{{BUNDLE_PRICE}}</v>
       </c>
       <c r="C37" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1581,10 +1350,10 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Bundle PPV 2 PPV Date</v>
+        <v>Bundle Card Original Price</v>
       </c>
       <c r="B38" t="str">
-        <v>{{BUNDLE_PPV2_DATE}}</v>
+        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
       </c>
       <c r="C38" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1592,10 +1361,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Bundle PPV 2 PPV Image</v>
+        <v>Bundle Card Save Badge</v>
       </c>
       <c r="B39" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_SAVE_BADGE}}</v>
       </c>
       <c r="C39" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1603,10 +1372,10 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Upsell Section Present</v>
+        <v>Bundle PPV 1 Full Name</v>
       </c>
       <c r="B40" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_PPV1_FULL_NAME}}</v>
       </c>
       <c r="C40" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1614,10 +1383,10 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Upsell Badge</v>
+        <v>Bundle PPV 1 PPV Date</v>
       </c>
       <c r="B41" t="str">
-        <v>The Ultimate Fan Package</v>
+        <v>{{BUNDLE_PPV1_DATE}}</v>
       </c>
       <c r="C41" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1625,10 +1394,10 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Upsell Plan Name</v>
+        <v>Bundle PPV 1 PPV Image</v>
       </c>
       <c r="B42" t="str">
-        <v>DAZN Ultimate</v>
+        <v>Yes</v>
       </c>
       <c r="C42" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1636,10 +1405,10 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Upsell Price</v>
+        <v>Bundle PPV 2 Full Name</v>
       </c>
       <c r="B43" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
+        <v>{{BUNDLE_PPV2_FULL_NAME}}</v>
       </c>
       <c r="C43" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1647,10 +1416,10 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Upsell Contract Text</v>
+        <v>Bundle PPV 2 PPV Date</v>
       </c>
       <c r="B44" t="str">
-        <v>Annual contract. Auto renews.</v>
+        <v>{{BUNDLE_PPV2_DATE}}</v>
       </c>
       <c r="C44" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1658,10 +1427,10 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Fights Included Text</v>
+        <v>Bundle PPV 2 PPV Image</v>
       </c>
       <c r="B45" t="str">
-        <v>All these fights included and more.</v>
+        <v>Yes</v>
       </c>
       <c r="C45" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1669,10 +1438,10 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Upsell Feature 1</v>
+        <v>Upsell Section Present</v>
       </c>
       <c r="B46" t="str">
-        <v>Minimum 12 pay-per-views a year included at no extra cost.</v>
+        <v>Yes</v>
       </c>
       <c r="C46" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1680,10 +1449,10 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Upsell Feature 2</v>
+        <v>Upsell Badge</v>
       </c>
       <c r="B47" t="str">
-        <v>185+ fights a year from the world&amp;apos;s best promoters.</v>
+        <v>The Ultimate Fan Package</v>
       </c>
       <c r="C47" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1691,10 +1460,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Upsell Feature 3</v>
+        <v>Upsell Plan Name</v>
       </c>
       <c r="B48" t="str">
-        <v>HDR and Dolby 5.1 surround sound on select events</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="C48" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1702,18 +1471,84 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>CTA Button</v>
+        <v>Upsell Price</v>
       </c>
       <c r="B49" t="str">
-        <v>Continue with DAZN Ultimate</v>
+        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
       </c>
       <c r="C49" t="str">
         <v>boxing-bundle-ppv</v>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Upsell Contract Text</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Annual contract. Auto renews.</v>
+      </c>
+      <c r="C50" t="str">
+        <v>boxing-bundle-ppv</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>Fights Included Text</v>
+      </c>
+      <c r="B51" t="str">
+        <v>All these fights included and more.</v>
+      </c>
+      <c r="C51" t="str">
+        <v>boxing-bundle-ppv</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Upsell Feature 1</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Minimum 12 pay-per-views a year included at no extra cost.</v>
+      </c>
+      <c r="C52" t="str">
+        <v>boxing-bundle-ppv</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Upsell Feature 2</v>
+      </c>
+      <c r="B53" t="str">
+        <v>185+ fights a year from the world's best promoters.</v>
+      </c>
+      <c r="C53" t="str">
+        <v>boxing-bundle-ppv</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>Upsell Feature 3</v>
+      </c>
+      <c r="B54" t="str">
+        <v>HDR and Dolby 5.1 surround sound on select events</v>
+      </c>
+      <c r="C54" t="str">
+        <v>boxing-bundle-ppv</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>CTA Button</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Continue with DAZN Ultimate</v>
+      </c>
+      <c r="C55" t="str">
+        <v>boxing-bundle-ppv</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C49"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C55"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1746,6 +1581,9 @@
       <c r="C2" t="str">
         <v>Choose the right plan for you.</v>
       </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -1755,7 +1593,10 @@
         <v>Header Sub Text</v>
       </c>
       <c r="C3" t="str">
-        <v>To watch your pay-per-view, you&amp;apos;ll need a DAZN plan.</v>
+        <v>To watch your pay-per-view, you'll need a DAZN plan.</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -1768,6 +1609,9 @@
       <c r="C4" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -1779,6 +1623,9 @@
       <c r="C5" t="str">
         <v>N/A</v>
       </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -1790,6 +1637,9 @@
       <c r="C6" t="str">
         <v>Yes</v>
       </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -1801,6 +1651,9 @@
       <c r="C7" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -1812,6 +1665,9 @@
       <c r="C8" t="str">
         <v>{{PPV_PRICE}}</v>
       </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -1823,6 +1679,9 @@
       <c r="C9" t="str">
         <v>{{CURRENCY}}</v>
       </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -1848,6 +1707,9 @@
       <c r="C11" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -1859,6 +1721,9 @@
       <c r="C12" t="str">
         <v>Yes</v>
       </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -1870,6 +1735,9 @@
       <c r="C13" t="str">
         <v>{{PPV_DATE}}</v>
       </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -1881,6 +1749,9 @@
       <c r="C14" t="str">
         <v>Yes</v>
       </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -1892,6 +1763,9 @@
       <c r="C15" t="str">
         <v>PPV: {{PPV_NAME}}</v>
       </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -1903,6 +1777,9 @@
       <c r="C16" t="str">
         <v>{{PPV_CARD_DESCRIPTION}}</v>
       </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -1914,6 +1791,9 @@
       <c r="C17" t="str">
         <v>Yes</v>
       </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -1925,6 +1805,9 @@
       <c r="C18" t="str">
         <v>The Ultimate Fan Package</v>
       </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -1936,6 +1819,9 @@
       <c r="C19" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -1947,6 +1833,9 @@
       <c r="C20" t="str">
         <v>N/A</v>
       </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -1958,6 +1847,9 @@
       <c r="C21" t="str">
         <v>{{UPSELL_PRICE}}</v>
       </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -1969,6 +1861,9 @@
       <c r="C22" t="str">
         <v>/month</v>
       </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -1980,6 +1875,9 @@
       <c r="C23" t="str">
         <v>N/A</v>
       </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -1991,6 +1889,9 @@
       <c r="C24" t="str">
         <v>{{UPSELL_OFFER_TEXT}}</v>
       </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -2002,6 +1903,9 @@
       <c r="C25" t="str">
         <v>{{UPSELL_SECTION_HEADING}}</v>
       </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -2013,6 +1917,9 @@
       <c r="C26" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -2024,6 +1931,9 @@
       <c r="C27" t="str">
         <v>Yes</v>
       </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -2035,6 +1945,9 @@
       <c r="C28" t="str">
         <v>{{PPV_DATE}}</v>
       </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -2046,6 +1959,9 @@
       <c r="C29" t="str">
         <v>N/A</v>
       </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -2057,6 +1973,9 @@
       <c r="C30" t="str">
         <v>N/A</v>
       </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -2068,6 +1987,9 @@
       <c r="C31" t="str">
         <v>N/A</v>
       </c>
+      <c r="D31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -2079,6 +2001,9 @@
       <c r="C32" t="str">
         <v>N/A</v>
       </c>
+      <c r="D32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -2090,6 +2015,9 @@
       <c r="C33" t="str">
         <v>N/A</v>
       </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -2101,6 +2029,9 @@
       <c r="C34" t="str">
         <v>{{UPSELL_FEATURE_1}}</v>
       </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -2112,6 +2043,9 @@
       <c r="C35" t="str">
         <v>N/A</v>
       </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -2123,6 +2057,9 @@
       <c r="C36" t="str">
         <v>{{UPSELL_FEATURE_2}}</v>
       </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -2134,6 +2071,9 @@
       <c r="C37" t="str">
         <v>{{UPSELL_FEATURE_3}}</v>
       </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -2145,6 +2085,9 @@
       <c r="C38" t="str">
         <v>N/A</v>
       </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -2156,6 +2099,9 @@
       <c r="C39" t="str">
         <v>N/A</v>
       </c>
+      <c r="D39" t="str">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -2167,6 +2113,9 @@
       <c r="C40" t="str">
         <v>N/A</v>
       </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -2178,6 +2127,9 @@
       <c r="C41" t="str">
         <v>N/A</v>
       </c>
+      <c r="D41" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -2189,6 +2141,9 @@
       <c r="C42" t="str">
         <v>{{PPV_CTA_TEXT}}</v>
       </c>
+      <c r="D42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -2214,6 +2169,9 @@
       <c r="C44" t="str">
         <v>Choose your plan</v>
       </c>
+      <c r="D44" t="str">
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -2225,6 +2183,9 @@
       <c r="C45" t="str">
         <v>Buy {{PPV_NAME}} with DAZN Standard or get it included in DAZN Ultimate.</v>
       </c>
+      <c r="D45" t="str">
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -2236,6 +2197,9 @@
       <c r="C46" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="D46" t="str">
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -2247,6 +2211,9 @@
       <c r="C47" t="str">
         <v>get it included in DAZN Ultimate.</v>
       </c>
+      <c r="D47" t="str">
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -2258,6 +2225,9 @@
       <c r="C48" t="str">
         <v>Yes</v>
       </c>
+      <c r="D48" t="str">
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -2269,6 +2239,9 @@
       <c r="C49" t="str">
         <v>{{PPV_DATE}}</v>
       </c>
+      <c r="D49" t="str">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -2280,6 +2253,9 @@
       <c r="C50" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="D50" t="str">
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -2291,6 +2267,9 @@
       <c r="C51" t="str">
         <v>Yes</v>
       </c>
+      <c r="D51" t="str">
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -2302,6 +2281,9 @@
       <c r="C52" t="str">
         <v>Yes</v>
       </c>
+      <c r="D52" t="str">
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -2313,6 +2295,9 @@
       <c r="C53" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="D53" t="str">
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -2324,6 +2309,9 @@
       <c r="C54" t="str">
         <v>{{PPV_PRICE}}</v>
       </c>
+      <c r="D54" t="str">
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -2335,6 +2323,9 @@
       <c r="C55" t="str">
         <v>{{CURRENCY}}</v>
       </c>
+      <c r="D55" t="str">
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -2346,6 +2337,9 @@
       <c r="C56" t="str">
         <v>Choose your subscription</v>
       </c>
+      <c r="D56" t="str">
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -2357,6 +2351,9 @@
       <c r="C57" t="str">
         <v>Yes</v>
       </c>
+      <c r="D57" t="str">
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -2368,6 +2365,9 @@
       <c r="C58" t="str">
         <v>7-day free trial of DAZN Standard</v>
       </c>
+      <c r="D58" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -2379,6 +2379,9 @@
       <c r="C59" t="str">
         <v>Yes</v>
       </c>
+      <c r="D59" t="str">
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -2390,6 +2393,9 @@
       <c r="C60" t="str">
         <v>Yes</v>
       </c>
+      <c r="D60" t="str">
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -2401,6 +2407,9 @@
       <c r="C61" t="str">
         <v>7-days free access to DAZN Standard.</v>
       </c>
+      <c r="D61" t="str">
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -2412,6 +2421,9 @@
       <c r="C62" t="str">
         <v>Cancel anytime during the trial and only pay for the fight. After the trial you move onto a Monthly Flex plan for {{CURRENCY}}{{MONTHLY_PRICE}}/month. You will not lose access to the pay-per-view[s].</v>
       </c>
+      <c r="D62" t="str">
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -2423,6 +2435,9 @@
       <c r="C63" t="str">
         <v>Yes</v>
       </c>
+      <c r="D63" t="str">
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -2434,6 +2449,9 @@
       <c r="C64" t="str">
         <v>Pay-per-views included</v>
       </c>
+      <c r="D64" t="str">
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -2445,6 +2463,9 @@
       <c r="C65" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="D65" t="str">
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -2456,6 +2477,9 @@
       <c r="C66" t="str">
         <v>From</v>
       </c>
+      <c r="D66" t="str">
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -2467,6 +2491,9 @@
       <c r="C67" t="str">
         <v>{{UPSELL_PRICE}}</v>
       </c>
+      <c r="D67" t="str">
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -2478,6 +2505,9 @@
       <c r="C68" t="str">
         <v>/ month</v>
       </c>
+      <c r="D68" t="str">
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -2489,6 +2519,9 @@
       <c r="C69" t="str">
         <v>Annual contract. Auto renews.</v>
       </c>
+      <c r="D69" t="str">
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -2500,6 +2533,9 @@
       <c r="C70" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="D70" t="str">
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -2511,6 +2547,9 @@
       <c r="C71" t="str">
         <v>Yes</v>
       </c>
+      <c r="D71" t="str">
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -2522,6 +2561,9 @@
       <c r="C72" t="str">
         <v>{{PPV_DATE}}</v>
       </c>
+      <c r="D72" t="str">
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -2533,6 +2575,9 @@
       <c r="C73" t="str">
         <v>Yes</v>
       </c>
+      <c r="D73" t="str">
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -2544,6 +2589,9 @@
       <c r="C74" t="str">
         <v>N/A</v>
       </c>
+      <c r="D74" t="str">
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -2555,6 +2603,9 @@
       <c r="C75" t="str">
         <v>N/A</v>
       </c>
+      <c r="D75" t="str">
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -2566,6 +2617,9 @@
       <c r="C76" t="str">
         <v>N/A</v>
       </c>
+      <c r="D76" t="str">
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -2577,6 +2631,9 @@
       <c r="C77" t="str">
         <v>N/A</v>
       </c>
+      <c r="D77" t="str">
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -2588,6 +2645,9 @@
       <c r="C78" t="str">
         <v>Pay-per-views included at no extra cost. Minimum of 12 events per year including {{PPV_NAME}}.</v>
       </c>
+      <c r="D78" t="str">
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -2599,6 +2659,9 @@
       <c r="C79" t="str">
         <v>{{PPV_NAME}}.</v>
       </c>
+      <c r="D79" t="str">
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -2610,6 +2673,9 @@
       <c r="C80" t="str">
         <v>HDR and Dolby 5.1 surround sound on select events.</v>
       </c>
+      <c r="D80" t="str">
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -2621,6 +2687,9 @@
       <c r="C81" t="str">
         <v>185+ fights a year from the best promoters</v>
       </c>
+      <c r="D81" t="str">
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -2632,6 +2701,9 @@
       <c r="C82" t="str">
         <v>Whats included</v>
       </c>
+      <c r="D82" t="str">
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -2643,6 +2715,9 @@
       <c r="C83" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="D83" t="str">
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -2654,6 +2729,9 @@
       <c r="C84" t="str">
         <v>get it included in DAZN Ultimate.</v>
       </c>
+      <c r="D84" t="str">
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -2665,6 +2743,9 @@
       <c r="C85" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="D85" t="str">
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -2676,6 +2757,9 @@
       <c r="C86" t="str">
         <v>Continue with PPV + 7-day free trial</v>
       </c>
+      <c r="D86" t="str">
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -2686,6 +2770,9 @@
       </c>
       <c r="C87" t="str">
         <v>N/A</v>
+      </c>
+      <c r="D87" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -2697,7 +2784,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:D37"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2709,6 +2796,9 @@
       <c r="C1" t="str">
         <v>Expected</v>
       </c>
+      <c r="D1" t="str">
+        <v>Flow</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -2720,6 +2810,9 @@
       <c r="C2" t="str">
         <v>{{PLAN_PAGE_TITLE}}</v>
       </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -2731,6 +2824,9 @@
       <c r="C3" t="str">
         <v>Yes</v>
       </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -2742,6 +2838,9 @@
       <c r="C4" t="str">
         <v>Flex – Pay Monthly</v>
       </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -2753,6 +2852,9 @@
       <c r="C5" t="str">
         <v>{{FLEX_BADGE}}</v>
       </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -2764,6 +2866,9 @@
       <c r="C6" t="str">
         <v>{{FLEX_DESCRIPTION}}</v>
       </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -2775,6 +2880,9 @@
       <c r="C7" t="str">
         <v>Yes</v>
       </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -2786,6 +2894,9 @@
       <c r="C8" t="str">
         <v>{{FLEX_TODAY_TEXT}}</v>
       </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -2797,6 +2908,9 @@
       <c r="C9" t="str">
         <v>{{FLEX_FUTURE_TEXT}}</v>
       </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -2808,6 +2922,9 @@
       <c r="C10" t="str">
         <v>Yes</v>
       </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -2819,6 +2936,9 @@
       <c r="C11" t="str">
         <v>{{ANNUAL_SAVINGS_BADGE}}</v>
       </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -2830,6 +2950,9 @@
       <c r="C12" t="str">
         <v>Annual - Pay Monthly</v>
       </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -2841,6 +2964,9 @@
       <c r="C13" t="str">
         <v>1 MONTH FREE</v>
       </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -2852,6 +2978,9 @@
       <c r="C14" t="str">
         <v>then {{CURRENCY}}{{ANNUAL_PRICE}}/month for {{ANNUAL_MONTHS}} months</v>
       </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -2863,6 +2992,9 @@
       <c r="C15" t="str">
         <v>Annual contract. Auto renews.</v>
       </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -2872,7 +3004,10 @@
         <v>Annual Feature 1</v>
       </c>
       <c r="C16" t="str">
-        <v>185+ fights a year from the world&amp;apos;s best promoters.</v>
+        <v>185+ fights a year from the world's best promoters.</v>
+      </c>
+      <c r="D16" t="str">
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -2885,6 +3020,9 @@
       <c r="C17" t="str">
         <v>Additional cost for pay-per-view events.</v>
       </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -2896,6 +3034,9 @@
       <c r="C18" t="str">
         <v>Full HD video resolution.</v>
       </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -2907,6 +3048,9 @@
       <c r="C19" t="str">
         <v>No</v>
       </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -2918,6 +3062,9 @@
       <c r="C20" t="str">
         <v>{{PLAN_CTA_BUTTON}}</v>
       </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -2929,6 +3076,9 @@
       <c r="C21" t="str">
         <v>{{PLAN_PAGE_TITLE}}</v>
       </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -2940,6 +3090,9 @@
       <c r="C22" t="str">
         <v>Yes</v>
       </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -2951,6 +3104,9 @@
       <c r="C23" t="str">
         <v>Annual - Pay Monthly</v>
       </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -2962,6 +3118,9 @@
       <c r="C24" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
       </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -2973,6 +3132,9 @@
       <c r="C25" t="str">
         <v>/ month</v>
       </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -2984,6 +3146,9 @@
       <c r="C26" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_CONTRACT_TEXT}}</v>
       </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -2995,6 +3160,9 @@
       <c r="C27" t="str">
         <v>Yes</v>
       </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -3006,6 +3174,9 @@
       <c r="C28" t="str">
         <v>Yes</v>
       </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -3017,6 +3188,9 @@
       <c r="C29" t="str">
         <v>Annual - Pay Upfront</v>
       </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -3028,6 +3202,9 @@
       <c r="C30" t="str">
         <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
       </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -3039,6 +3216,9 @@
       <c r="C31" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE_DISPLAY}}</v>
       </c>
+      <c r="D31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -3050,6 +3230,9 @@
       <c r="C32" t="str">
         <v>/year</v>
       </c>
+      <c r="D32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -3061,6 +3244,9 @@
       <c r="C33" t="str">
         <v>No</v>
       </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -3072,6 +3258,9 @@
       <c r="C34" t="str">
         <v>Minimum 12 pay-per-views a year included at no extra cost.</v>
       </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -3081,7 +3270,10 @@
         <v>Ultimate Feature 2</v>
       </c>
       <c r="C35" t="str">
-        <v>185+ fights a year from the world&amp;apos;s best promoters.</v>
+        <v>185+ fights a year from the world's best promoters.</v>
+      </c>
+      <c r="D35" t="str">
+        <v/>
       </c>
     </row>
     <row r="36">
@@ -3094,6 +3286,9 @@
       <c r="C36" t="str">
         <v>HDR and Dolby 5.1 surround sound on select events.</v>
       </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -3105,17 +3300,20 @@
       <c r="C37" t="str">
         <v>{{PLAN_CTA_BUTTON}}</v>
       </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D37"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E98"/>
+  <dimension ref="A1:E96"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3145,7 +3343,10 @@
         <v>Header</v>
       </c>
       <c r="D2" t="str">
-        <v>Your payment is encrypted and you can change how you pay at any time.|81% OFF for your first month|20% OFF for 12 months|First month free</v>
+        <v>Your payment is encrypted and you can change how you pay at any time.</v>
+      </c>
+      <c r="E2" t="str">
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -3161,6 +3362,9 @@
       <c r="D3" t="str">
         <v>Change</v>
       </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -3175,6 +3379,9 @@
       <c r="D4" t="str">
         <v>Yes</v>
       </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -3189,6 +3396,9 @@
       <c r="D5" t="str">
         <v>Yes</v>
       </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -3203,6 +3413,9 @@
       <c r="D6" t="str">
         <v>Yes</v>
       </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -3268,6 +3481,9 @@
       <c r="D10" t="str">
         <v>Yes</v>
       </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -3316,6 +3532,9 @@
       <c r="D13" t="str">
         <v>DAZN Standard</v>
       </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -3330,6 +3549,9 @@
       <c r="D14" t="str">
         <v>{{PAYMENT_PLAN_NAME}}</v>
       </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -3344,6 +3566,9 @@
       <c r="D15" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -3358,6 +3583,9 @@
       <c r="D16" t="str">
         <v>{{PAYMENT_FREE_TEXT}}</v>
       </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -3372,6 +3600,9 @@
       <c r="D17" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -3386,6 +3617,9 @@
       <c r="D18" t="str">
         <v>{{PPV_PRICE}}</v>
       </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -3400,6 +3634,9 @@
       <c r="D19" t="str">
         <v>Today you pay</v>
       </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -3414,6 +3651,9 @@
       <c r="D20" t="str">
         <v>{{PPV_PRICE}}</v>
       </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -3428,6 +3668,9 @@
       <c r="D21" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -3442,6 +3685,9 @@
       <c r="D22" t="str">
         <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -3456,6 +3702,9 @@
       <c r="D23" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -3470,6 +3719,9 @@
       <c r="D24" t="str">
         <v>DAZN Standard</v>
       </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -3484,6 +3736,9 @@
       <c r="D25" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -3498,6 +3753,9 @@
       <c r="D26" t="str">
         <v>{{PPV_PRICE}}</v>
       </c>
+      <c r="E26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -3512,6 +3770,9 @@
       <c r="D27" t="str">
         <v>{{RATE_PLAN_LABEL}}</v>
       </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -3526,6 +3787,9 @@
       <c r="D28" t="str">
         <v>{{CURRENCY}}{{ANNUAL_PRICE}}</v>
       </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -3540,6 +3804,9 @@
       <c r="D29" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -3554,6 +3821,9 @@
       <c r="D30" t="str">
         <v>Today you pay</v>
       </c>
+      <c r="E30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -3568,6 +3838,9 @@
       <c r="D31" t="str">
         <v>{{PPV_PRICE}}</v>
       </c>
+      <c r="E31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -3582,6 +3855,9 @@
       <c r="D32" t="str">
         <v>{{CANCELLATION_TEXT_ANNUAL}}</v>
       </c>
+      <c r="E32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -3596,6 +3872,9 @@
       <c r="D33" t="str">
         <v>Yes</v>
       </c>
+      <c r="E33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -3610,6 +3889,9 @@
       <c r="D34" t="str">
         <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
+      <c r="E34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -3624,6 +3906,9 @@
       <c r="D35" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -3638,6 +3923,9 @@
       <c r="D36" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -3652,6 +3940,9 @@
       <c r="D37" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -3666,6 +3957,9 @@
       <c r="D38" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -3678,7 +3972,10 @@
         <v>Rate Plan</v>
       </c>
       <c r="D39" t="str">
-        <v>{{PAYMENT_PLAN_LABEL}}</v>
+        <v>Annual - Pay Monthly</v>
+      </c>
+      <c r="E39" t="str">
+        <v/>
       </c>
     </row>
     <row r="40">
@@ -3694,6 +3991,9 @@
       <c r="D40" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
       </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -3708,6 +4008,9 @@
       <c r="D41" t="str">
         <v>Today you pay</v>
       </c>
+      <c r="E41" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -3722,6 +4025,9 @@
       <c r="D42" t="str">
         <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
+      <c r="E42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -3736,6 +4042,9 @@
       <c r="D43" t="str">
         <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
+      <c r="E43" t="str">
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -3750,6 +4059,9 @@
       <c r="D44" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
       </c>
+      <c r="E44" t="str">
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -3764,6 +4076,9 @@
       <c r="D45" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E45" t="str">
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -3778,6 +4093,9 @@
       <c r="D46" t="str">
         <v>Yes</v>
       </c>
+      <c r="E46" t="str">
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -3792,6 +4110,9 @@
       <c r="D47" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E47" t="str">
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -3806,6 +4127,9 @@
       <c r="D48" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="E48" t="str">
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -3820,6 +4144,9 @@
       <c r="D49" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="E49" t="str">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -3834,6 +4161,9 @@
       <c r="D50" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E50" t="str">
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -3848,6 +4178,9 @@
       <c r="D51" t="str">
         <v>Annual - Pay Upfront</v>
       </c>
+      <c r="E51" t="str">
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -3862,6 +4195,9 @@
       <c r="D52" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE}}/year</v>
       </c>
+      <c r="E52" t="str">
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -3876,6 +4212,9 @@
       <c r="D53" t="str">
         <v>Today you pay</v>
       </c>
+      <c r="E53" t="str">
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -3890,6 +4229,9 @@
       <c r="D54" t="str">
         <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
+      <c r="E54" t="str">
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -3904,6 +4246,9 @@
       <c r="D55" t="str">
         <v>Next Annual payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
+      <c r="E55" t="str">
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -3918,6 +4263,9 @@
       <c r="D56" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE}}</v>
       </c>
+      <c r="E56" t="str">
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -3932,6 +4280,9 @@
       <c r="D57" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E57" t="str">
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -3946,6 +4297,9 @@
       <c r="D58" t="str">
         <v>Yes</v>
       </c>
+      <c r="E58" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -3960,6 +4314,9 @@
       <c r="D59" t="str">
         <v>{{PAYMENT_PAGE_TITLE}}</v>
       </c>
+      <c r="E59" t="str">
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -3974,6 +4331,9 @@
       <c r="D60" t="str">
         <v>DAZN Standard</v>
       </c>
+      <c r="E60" t="str">
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -3988,6 +4348,9 @@
       <c r="D61" t="str">
         <v>{{BUNDLE_NAME}}</v>
       </c>
+      <c r="E61" t="str">
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -4002,6 +4365,9 @@
       <c r="D62" t="str">
         <v>{{BUNDLE_PRICE}}</v>
       </c>
+      <c r="E62" t="str">
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -4016,6 +4382,9 @@
       <c r="D63" t="str">
         <v>{{BUNDLE_TODAY_YOU_PAY_STANDARD}}</v>
       </c>
+      <c r="E63" t="str">
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -4030,6 +4399,9 @@
       <c r="D64" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E64" t="str">
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -4044,6 +4416,9 @@
       <c r="D65" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E65" t="str">
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -4058,6 +4433,9 @@
       <c r="D66" t="str">
         <v>DAZN Standard</v>
       </c>
+      <c r="E66" t="str">
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -4072,6 +4450,9 @@
       <c r="D67" t="str">
         <v>Annual - Pay Monthly</v>
       </c>
+      <c r="E67" t="str">
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -4086,6 +4467,9 @@
       <c r="D68" t="str">
         <v>First month free</v>
       </c>
+      <c r="E68" t="str">
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -4100,6 +4484,9 @@
       <c r="D69" t="str">
         <v>{{BUNDLE_NAME}}</v>
       </c>
+      <c r="E69" t="str">
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -4114,6 +4501,9 @@
       <c r="D70" t="str">
         <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
       </c>
+      <c r="E70" t="str">
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -4128,6 +4518,9 @@
       <c r="D71" t="str">
         <v>{{BUNDLE_PRICE}}</v>
       </c>
+      <c r="E71" t="str">
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -4142,6 +4535,9 @@
       <c r="D72" t="str">
         <v>{{BUNDLE_DISCOUNT}}</v>
       </c>
+      <c r="E72" t="str">
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -4156,6 +4552,9 @@
       <c r="D73" t="str">
         <v>{{BUNDLE_TODAY_YOU_PAY_STANDARD}}</v>
       </c>
+      <c r="E73" t="str">
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -4170,6 +4569,9 @@
       <c r="D74" t="str">
         <v>{{CANCELLATION_TEXT_ANNUAL}}</v>
       </c>
+      <c r="E74" t="str">
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -4184,6 +4586,9 @@
       <c r="D75" t="str">
         <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
+      <c r="E75" t="str">
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -4198,6 +4603,9 @@
       <c r="D76" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E76" t="str">
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -4212,6 +4620,9 @@
       <c r="D77" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="E77" t="str">
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -4224,7 +4635,10 @@
         <v>Rate Plan</v>
       </c>
       <c r="D78" t="str">
-        <v>{{PAYMENT_PLAN_LABEL}}</v>
+        <v>Annual - Pay Monthly</v>
+      </c>
+      <c r="E78" t="str">
+        <v/>
       </c>
     </row>
     <row r="79">
@@ -4240,6 +4654,9 @@
       <c r="D79" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
       </c>
+      <c r="E79" t="str">
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -4254,6 +4671,9 @@
       <c r="D80" t="str">
         <v>{{BUNDLE_NAME}}</v>
       </c>
+      <c r="E80" t="str">
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -4268,6 +4688,9 @@
       <c r="D81" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E81" t="str">
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -4282,6 +4705,9 @@
       <c r="D82" t="str">
         <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
+      <c r="E82" t="str">
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -4296,6 +4722,9 @@
       <c r="D83" t="str">
         <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
+      <c r="E83" t="str">
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -4310,6 +4739,9 @@
       <c r="D84" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
       </c>
+      <c r="E84" t="str">
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -4324,6 +4756,9 @@
       <c r="D85" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E85" t="str">
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -4338,6 +4773,9 @@
       <c r="D86" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E86" t="str">
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -4352,6 +4790,9 @@
       <c r="D87" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="E87" t="str">
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -4366,6 +4807,9 @@
       <c r="D88" t="str">
         <v>Annual - Pay Upfront</v>
       </c>
+      <c r="E88" t="str">
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
@@ -4380,6 +4824,9 @@
       <c r="D89" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE}}/year</v>
       </c>
+      <c r="E89" t="str">
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -4394,6 +4841,9 @@
       <c r="D90" t="str">
         <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
       </c>
+      <c r="E90" t="str">
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -4408,6 +4858,9 @@
       <c r="D91" t="str">
         <v>{{BUNDLE_NAME}}</v>
       </c>
+      <c r="E91" t="str">
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -4422,6 +4875,9 @@
       <c r="D92" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E92" t="str">
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
@@ -4436,6 +4892,9 @@
       <c r="D93" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE}}</v>
       </c>
+      <c r="E93" t="str">
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
@@ -4450,6 +4909,9 @@
       <c r="D94" t="str">
         <v>Next Annual payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
+      <c r="E94" t="str">
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
@@ -4464,6 +4926,9 @@
       <c r="D95" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE}}</v>
       </c>
+      <c r="E95" t="str">
+        <v/>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
@@ -4478,39 +4943,13 @@
       <c r="D96" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="str">
-        <v>Ultimate</v>
-      </c>
-      <c r="B97" t="str">
-        <v>Annual Pay Monthly</v>
-      </c>
-      <c r="C97" t="str">
-        <v>Discount Badge</v>
-      </c>
-      <c r="D97" t="str">
-        <v>{{DISCOUNT_BADGE}}</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="str">
-        <v>Ultimate</v>
-      </c>
-      <c r="B98" t="str">
-        <v>Annual Pay Monthly Bundle</v>
-      </c>
-      <c r="C98" t="str">
-        <v>Discount Badge</v>
-      </c>
-      <c r="D98" t="str">
-        <v>{{DISCOUNT_BADGE}}</v>
+      <c r="E96" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E98"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E96"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4632,7 +5071,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B14"/>
   </ignoredErrors>
@@ -4708,7 +5146,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B8"/>
   </ignoredErrors>
@@ -4904,7 +5341,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B23"/>
   </ignoredErrors>
@@ -5044,7 +5480,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B16"/>
   </ignoredErrors>

</xml_diff>

<commit_message>
Fixed Excel missing sheets
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -15,6 +15,13 @@
     <sheet name="Upgrade Confirmation page" sheetId="10" r:id="rId10"/>
     <sheet name="Phone Number page" sheetId="11" r:id="rId11"/>
     <sheet name="OTP page" sheetId="12" r:id="rId12"/>
+    <sheet name="Home of Boxing" sheetId="13" r:id="rId13"/>
+    <sheet name="Home page" sheetId="14" r:id="rId14"/>
+    <sheet name="Standalone PPV page" sheetId="15" r:id="rId15"/>
+    <sheet name="Upsell First Success page" sheetId="16" r:id="rId16"/>
+    <sheet name="Upsell Second Success page" sheetId="17" r:id="rId17"/>
+    <sheet name="Upsell Payment page" sheetId="18" r:id="rId18"/>
+    <sheet name="Search page" sheetId="19" r:id="rId19"/>
   </sheets>
 </workbook>
 </file>
@@ -409,6 +416,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C6"/>
+  <cols>
+    <col min="1" max="1" width="33.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="9.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -470,7 +482,7 @@
         <v>Buy Now Button</v>
       </c>
       <c r="B6" t="str">
-        <v>Yes</v>
+        <v>Buy now</v>
       </c>
       <c r="C6" t="str">
         <v>landing</v>
@@ -486,6 +498,11 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C22"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="50.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -739,6 +756,10 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B6"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="64.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -798,6 +819,10 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B6"/>
+  <cols>
+    <col min="1" max="1" width="19.83203125" customWidth="1"/>
+    <col min="2" max="2" width="34.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -812,7 +837,7 @@
         <v>Page Title</v>
       </c>
       <c r="B2" t="str">
-        <v>Enter the code below to continue</v>
+        <v>Verify your phone</v>
       </c>
     </row>
     <row r="3">
@@ -854,9 +879,332 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C14"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="90.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Flow</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Field</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Expected</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>home-boxing-banner</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Best of Boxing Section</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Present</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>home-boxing-banner</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Banner - Event Title</v>
+      </c>
+      <c r="C3" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>home-boxing-banner</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Banner - Event Date</v>
+      </c>
+      <c r="C4" t="str">
+        <v>{{PPV_DATE}}</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>home-boxing-banner</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Banner - Event Description</v>
+      </c>
+      <c r="C5" t="str">
+        <v>{{PPV_DESCRIPTION}}</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>home-boxing-banner</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Banner - Buy Now CTA</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>home-boxing-banner</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Banner - Fight Card CTA</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>home-boxing-tile</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Best of Boxing Section</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Present</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>home-boxing-tile</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Popup - Event Title</v>
+      </c>
+      <c r="C9" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>home-boxing-tile</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Popup - Event Date</v>
+      </c>
+      <c r="C10" t="str">
+        <v>{{PPV_DATE}}</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>home-boxing-tile</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Popup - Promoter</v>
+      </c>
+      <c r="C11" t="str">
+        <v>{{PPV_PROMOTER}}</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>home-boxing-tile</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Popup - Buy Now CTA</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>home-boxing-tile</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Popup - Event Description</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>home-boxing-tile</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Popup - Close Button</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C14"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C12"/>
+  <cols>
+    <col min="1" max="1" width="21.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="21.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Flow</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Field</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Expected</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>home-page-banner</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Banner - Event Title</v>
+      </c>
+      <c r="C2" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>home-page-banner</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Banner - Event Date</v>
+      </c>
+      <c r="C3" t="str">
+        <v>{{PPV_DATE}}</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>home-page-banner</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Banner - Event Description</v>
+      </c>
+      <c r="C4" t="str">
+        <v>{{PPV_DESCRIPTION}}</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>home-page-banner</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Banner - Buy Now CTA</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>home-page-banner</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Banner - Fight Card CTA</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Popup - Event Title</v>
+      </c>
+      <c r="C7" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Popup - Event Date</v>
+      </c>
+      <c r="C8" t="str">
+        <v>{{PPV_DATE}}</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Popup - Promoter</v>
+      </c>
+      <c r="C9" t="str">
+        <v>{{PPV_PROMOTER}}</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Popup - Buy Now CTA</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Popup - Event Description</v>
+      </c>
+      <c r="C11" t="str">
+        <v>{{PPV_DESCRIPTION}}</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Popup - Close Button</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C12"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C31"/>
+  <cols>
+    <col min="1" max="1" width="33.83203125" customWidth="1"/>
+    <col min="2" max="2" width="124.83203125" customWidth="1"/>
+    <col min="3" max="3" width="11.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -866,6 +1214,663 @@
         <v>Expected</v>
       </c>
       <c r="C1" t="str">
+        <v>State</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Page Title</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Choose a plan that's right for you</v>
+      </c>
+      <c r="C2" t="str">
+        <v>checked</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Page Heading</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Buy {{PPV_NAME}} with a 7-day free trial</v>
+      </c>
+      <c r="C3" t="str">
+        <v>checked</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>PPV Image Present</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="C4" t="str">
+        <v>checked</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>PPV Date Badge</v>
+      </c>
+      <c r="B5" t="str">
+        <v>{{PPV_DATE}}</v>
+      </c>
+      <c r="C5" t="str">
+        <v>checked</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>PPV Name</v>
+      </c>
+      <c r="B6" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+      <c r="C6" t="str">
+        <v>checked</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>PPV Price</v>
+      </c>
+      <c r="B7" t="str">
+        <v>{{CURRENCY}}{{PPV_PRICE_RAW}}</v>
+      </c>
+      <c r="C7" t="str">
+        <v>checked</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>PPV Checkbox State</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Checked</v>
+      </c>
+      <c r="C8" t="str">
+        <v>checked</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Section Label</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Choose your subscription</v>
+      </c>
+      <c r="C9" t="str">
+        <v>checked</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Flex Title</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Flex – Pay Monthly</v>
+      </c>
+      <c r="C10" t="str">
+        <v>checked</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Flex Badge</v>
+      </c>
+      <c r="B11" t="str">
+        <v>7 DAY FREE TRIAL</v>
+      </c>
+      <c r="C11" t="str">
+        <v>checked</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Flex Description</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Only pay for the fight. Cancel anytime before the end of the trial.</v>
+      </c>
+      <c r="C12" t="str">
+        <v>checked</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Flex Today Text</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Only pay for the fight and start your 7-day free trial of DAZN Standard</v>
+      </c>
+      <c r="C13" t="str">
+        <v>checked</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Flex Future Date</v>
+      </c>
+      <c r="B14" t="str">
+        <v>In 7 days • {{FLEX_FUTURE_DATE_SHORT}}</v>
+      </c>
+      <c r="C14" t="str">
+        <v>checked</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Flex Future Text</v>
+      </c>
+      <c r="B15" t="str">
+        <v>You will start your DAZN Standard plan at {{CURRENCY}}{{MONTHLY_PRICE}}/month. Cancel anytime before the end of the trial.</v>
+      </c>
+      <c r="C15" t="str">
+        <v>checked</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Annual Title</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Annual - Pay Monthly</v>
+      </c>
+      <c r="C16" t="str">
+        <v>checked</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Annual Badge</v>
+      </c>
+      <c r="B17" t="str">
+        <v>SAVE {{CURRENCY}}{{ANNUAL_SAVINGS}} A YEAR</v>
+      </c>
+      <c r="C17" t="str">
+        <v>checked</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Annual Description</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Annual contract. Auto renews.</v>
+      </c>
+      <c r="C18" t="str">
+        <v>checked</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Annual Price</v>
+      </c>
+      <c r="B19" t="str">
+        <v>{{CURRENCY}}{{ANNUAL_PRICE}}/month for 12 months</v>
+      </c>
+      <c r="C19" t="str">
+        <v>checked</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>CTA Button (Flex selected)</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Continue with 7-day free trial</v>
+      </c>
+      <c r="C20" t="str">
+        <v>checked</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>CTA Button (APM selected)</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Continue</v>
+      </c>
+      <c r="C21" t="str">
+        <v>checked</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Plans Visible Count (checked)</v>
+      </c>
+      <c r="B22" t="str">
+        <v>2</v>
+      </c>
+      <c r="C22" t="str">
+        <v>checked</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Plans Visible Count (unchecked)</v>
+      </c>
+      <c r="B23" t="str">
+        <v>3</v>
+      </c>
+      <c r="C23" t="str">
+        <v>unchecked</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Flex Title (unchecked)</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Flex – Pay Monthly</v>
+      </c>
+      <c r="C24" t="str">
+        <v>unchecked</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Flex Description (unchecked)</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Billed monthly. Cancel anytime.</v>
+      </c>
+      <c r="C25" t="str">
+        <v>unchecked</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Flex Price (unchecked)</v>
+      </c>
+      <c r="B26" t="str">
+        <v>{{CURRENCY}}{{MONTHLY_PRICE}}/month</v>
+      </c>
+      <c r="C26" t="str">
+        <v>unchecked</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>APM Title (unchecked)</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Annual - Pay Monthly</v>
+      </c>
+      <c r="C27" t="str">
+        <v>unchecked</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>APU Title (unchecked)</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Annual - Pay Upfront</v>
+      </c>
+      <c r="C28" t="str">
+        <v>unchecked</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>APU Description (unchecked)</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Annual contract. Auto renews.</v>
+      </c>
+      <c r="C29" t="str">
+        <v>unchecked</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>APU Price (unchecked)</v>
+      </c>
+      <c r="B30" t="str">
+        <v>{{CURRENCY}}{{ANNUAL_UPFRONT_PRICE}}/year</v>
+      </c>
+      <c r="C30" t="str">
+        <v>unchecked</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>APU Save Badge (unchecked)</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
+      </c>
+      <c r="C31" t="str">
+        <v>unchecked</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C31"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B7"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="21.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Field</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Expected</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Payment Success Text</v>
+      </c>
+      <c r="B2" t="str">
+        <v>{{SUCCESS_HEADING}}</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Upsell Heading</v>
+      </c>
+      <c r="B3" t="str">
+        <v>{{UPSELL_HEADING}}</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Upsell Image Present</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Upsell Date Badge</v>
+      </c>
+      <c r="B5" t="str">
+        <v>{{UPSELL_DATE}}</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Upsell Buy CTA</v>
+      </c>
+      <c r="B6" t="str">
+        <v>{{UPSELL_BUY_CTA}}</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>No Thanks Link</v>
+      </c>
+      <c r="B7" t="str">
+        <v>No thanks</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B7"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Field</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Expected</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Payment Success Text</v>
+      </c>
+      <c r="B2" t="str">
+        <v>{{SECOND_SUCCESS_HEADING}}</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Bet Offer Title</v>
+      </c>
+      <c r="B3" t="str">
+        <v>{{BET_OFFER_TITLE}}</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Bet Heading</v>
+      </c>
+      <c r="B4" t="str">
+        <v>{{BET_HEADING}}</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Bet Image Present</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Activate Betting CTA</v>
+      </c>
+      <c r="B6" t="str">
+        <v>{{BET_CTA}}</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Maybe Later Link</v>
+      </c>
+      <c r="B7" t="str">
+        <v>{{BET_DISMISS}}</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B11"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Field</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Expected</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Page Title</v>
+      </c>
+      <c r="B2" t="str">
+        <v>{{FURY_PAYMENT_TITLE}}</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>PPV Image Present</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Date Badge</v>
+      </c>
+      <c r="B4" t="str">
+        <v>{{FURY_PAYMENT_DATE}}</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>PPV Price</v>
+      </c>
+      <c r="B5" t="str">
+        <v>{{FURY_PAYMENT_PRICE}}</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Payment Type</v>
+      </c>
+      <c r="B6" t="str">
+        <v>{{FURY_PAYMENT_TYPE}}</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Today you pay</v>
+      </c>
+      <c r="B7" t="str">
+        <v>{{FURY_PAYMENT_TODAY}}</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Payment Instruction</v>
+      </c>
+      <c r="B8" t="str">
+        <v>{{FURY_PAYMENT_TEXT}}</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Saved Card</v>
+      </c>
+      <c r="B9" t="str">
+        <v>{{FURY_SAVED_CARD}}</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>More Payment Methods</v>
+      </c>
+      <c r="B10" t="str">
+        <v>More payment methods</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Redeem Promo Code</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Redeem promo code</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B11"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B5"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Field</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Expected</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>PPV Tile Present</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>PPV Name</v>
+      </c>
+      <c r="B3" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>PPV Date</v>
+      </c>
+      <c r="B4" t="str">
+        <v>{{PPV_DATE}}</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Buy Now Button</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B5"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C55"/>
+  <cols>
+    <col min="1" max="1" width="29.83203125" customWidth="1"/>
+    <col min="2" max="2" width="60.83203125" customWidth="1"/>
+    <col min="3" max="3" width="19.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Field</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Expected</v>
+      </c>
+      <c r="C1" t="str">
         <v>Flow</v>
       </c>
     </row>
@@ -896,7 +1901,7 @@
         <v>Event Subtitle</v>
       </c>
       <c r="B4" t="str">
-        <v>Main Event  AO Arena, Manchester  11:30 pm.</v>
+        <v>{{BOXING_BANNER_SUBTITLE}}</v>
       </c>
       <c r="C4" t="str">
         <v>boxing</v>
@@ -1472,7 +2477,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D87"/>
+  <dimension ref="A1:D102"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="37.83203125" customWidth="1"/>
+    <col min="3" max="3" width="201.83203125" customWidth="1"/>
+    <col min="4" max="4" width="9.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1678,7 +2689,7 @@
         <v>PPV Card Title</v>
       </c>
       <c r="C15" t="str">
-        <v>PPV: {{PPV_NAME}}</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="D15" t="str">
         <v/>
@@ -1787,10 +2798,10 @@
         <v>variant1</v>
       </c>
       <c r="B23" t="str">
-        <v>Upsell Billing Text</v>
+        <v>Upsell Crossed Price</v>
       </c>
       <c r="C23" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_CONTRACT_TEXT}}</v>
+        <v>{{UPSELL_CROSSED_PRICE}}</v>
       </c>
       <c r="D23" t="str">
         <v/>
@@ -1801,10 +2812,10 @@
         <v>variant1</v>
       </c>
       <c r="B24" t="str">
-        <v>Upsell Offer Text</v>
+        <v>Upsell Contract Text</v>
       </c>
       <c r="C24" t="str">
-        <v>{{UPSELL_OFFER_TEXT}}</v>
+        <v>Annual contract. Auto renews.</v>
       </c>
       <c r="D24" t="str">
         <v/>
@@ -1815,10 +2826,10 @@
         <v>variant1</v>
       </c>
       <c r="B25" t="str">
-        <v>Upsell Section Heading</v>
+        <v>Upsell Billing Text</v>
       </c>
       <c r="C25" t="str">
-        <v>{{UPSELL_SECTION_HEADING}}</v>
+        <v>{{ANNUAL_PAY_MONTHLY_CONTRACT_TEXT}}</v>
       </c>
       <c r="D25" t="str">
         <v/>
@@ -1829,10 +2840,10 @@
         <v>variant1</v>
       </c>
       <c r="B26" t="str">
-        <v>Included PPV1 Name</v>
+        <v>Upsell Offer Text</v>
       </c>
       <c r="C26" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>{{UPSELL_OFFER_TEXT}}</v>
       </c>
       <c r="D26" t="str">
         <v/>
@@ -1843,10 +2854,10 @@
         <v>variant1</v>
       </c>
       <c r="B27" t="str">
-        <v>PPV1 Image Present on ultimate tier</v>
+        <v>Upsell Section Heading</v>
       </c>
       <c r="C27" t="str">
-        <v>Yes</v>
+        <v>{{UPSELL_SECTION_HEADING}}</v>
       </c>
       <c r="D27" t="str">
         <v/>
@@ -1857,10 +2868,10 @@
         <v>variant1</v>
       </c>
       <c r="B28" t="str">
-        <v>PPV1 Date Text on ultimate tier</v>
+        <v>Included PPV1 Name</v>
       </c>
       <c r="C28" t="str">
-        <v>{{PPV_DATE}}</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="D28" t="str">
         <v/>
@@ -1871,10 +2882,10 @@
         <v>variant1</v>
       </c>
       <c r="B29" t="str">
-        <v>PPV1 Included tag</v>
+        <v>PPV1 Image Present on ultimate tier</v>
       </c>
       <c r="C29" t="str">
-        <v>N/A</v>
+        <v>Yes</v>
       </c>
       <c r="D29" t="str">
         <v/>
@@ -1885,10 +2896,10 @@
         <v>variant1</v>
       </c>
       <c r="B30" t="str">
-        <v>Included PPV2 Name</v>
+        <v>PPV1 Date Text on ultimate tier</v>
       </c>
       <c r="C30" t="str">
-        <v>N/A</v>
+        <v>{{PPV_DATE}}</v>
       </c>
       <c r="D30" t="str">
         <v/>
@@ -1899,7 +2910,7 @@
         <v>variant1</v>
       </c>
       <c r="B31" t="str">
-        <v>PPV2 Image Present on ultimate tier</v>
+        <v>PPV1 Included tag</v>
       </c>
       <c r="C31" t="str">
         <v>N/A</v>
@@ -1913,7 +2924,7 @@
         <v>variant1</v>
       </c>
       <c r="B32" t="str">
-        <v>PPV2 Date Text on ultimate tier</v>
+        <v>Included PPV2 Name</v>
       </c>
       <c r="C32" t="str">
         <v>N/A</v>
@@ -1927,7 +2938,7 @@
         <v>variant1</v>
       </c>
       <c r="B33" t="str">
-        <v>PPV2 Included tag</v>
+        <v>PPV2 Image Present on ultimate tier</v>
       </c>
       <c r="C33" t="str">
         <v>N/A</v>
@@ -1941,10 +2952,10 @@
         <v>variant1</v>
       </c>
       <c r="B34" t="str">
-        <v>Upsell Feature 1</v>
+        <v>PPV2 Date Text on ultimate tier</v>
       </c>
       <c r="C34" t="str">
-        <v>{{UPSELL_FEATURE_1}}</v>
+        <v>N/A</v>
       </c>
       <c r="D34" t="str">
         <v/>
@@ -1955,7 +2966,7 @@
         <v>variant1</v>
       </c>
       <c r="B35" t="str">
-        <v>Upsell Highlight Text</v>
+        <v>PPV2 Included tag</v>
       </c>
       <c r="C35" t="str">
         <v>N/A</v>
@@ -1969,10 +2980,10 @@
         <v>variant1</v>
       </c>
       <c r="B36" t="str">
-        <v>Upsell Feature 2</v>
+        <v>Upsell Feature 1</v>
       </c>
       <c r="C36" t="str">
-        <v>{{UPSELL_FEATURE_2}}</v>
+        <v>{{UPSELL_FEATURE_1}}</v>
       </c>
       <c r="D36" t="str">
         <v/>
@@ -1983,10 +2994,10 @@
         <v>variant1</v>
       </c>
       <c r="B37" t="str">
-        <v>Upsell Feature 3</v>
+        <v>Upsell Highlight Text</v>
       </c>
       <c r="C37" t="str">
-        <v>{{UPSELL_FEATURE_3}}</v>
+        <v>N/A</v>
       </c>
       <c r="D37" t="str">
         <v/>
@@ -1997,10 +3008,10 @@
         <v>variant1</v>
       </c>
       <c r="B38" t="str">
-        <v>Whats Included CTA</v>
+        <v>Upsell Feature 2</v>
       </c>
       <c r="C38" t="str">
-        <v>N/A</v>
+        <v>{{UPSELL_FEATURE_2}}</v>
       </c>
       <c r="D38" t="str">
         <v/>
@@ -2011,10 +3022,10 @@
         <v>variant1</v>
       </c>
       <c r="B39" t="str">
-        <v>Gold Highlight 1</v>
+        <v>Upsell Feature 3</v>
       </c>
       <c r="C39" t="str">
-        <v>N/A</v>
+        <v>{{UPSELL_FEATURE_3}}</v>
       </c>
       <c r="D39" t="str">
         <v/>
@@ -2025,7 +3036,7 @@
         <v>variant1</v>
       </c>
       <c r="B40" t="str">
-        <v>Gold Highlight 2</v>
+        <v>Whats Included CTA</v>
       </c>
       <c r="C40" t="str">
         <v>N/A</v>
@@ -2039,7 +3050,7 @@
         <v>variant1</v>
       </c>
       <c r="B41" t="str">
-        <v>Gold Highlight 3</v>
+        <v>Gold Highlight 1</v>
       </c>
       <c r="C41" t="str">
         <v>N/A</v>
@@ -2053,10 +3064,10 @@
         <v>variant1</v>
       </c>
       <c r="B42" t="str">
-        <v>CTA Button</v>
+        <v>Gold Highlight 2</v>
       </c>
       <c r="C42" t="str">
-        <v>{{PPV_CTA_TEXT}}</v>
+        <v>N/A</v>
       </c>
       <c r="D42" t="str">
         <v/>
@@ -2067,206 +3078,206 @@
         <v>variant1</v>
       </c>
       <c r="B43" t="str">
-        <v>CTA Without PPV</v>
+        <v>Gold Highlight 3</v>
       </c>
       <c r="C43" t="str">
-        <v>Subscribe without a pay-per-view</v>
+        <v>N/A</v>
       </c>
       <c r="D43" t="str">
-        <v>newuser</v>
+        <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>variant2</v>
+        <v>variant1</v>
       </c>
       <c r="B44" t="str">
-        <v>Page Title</v>
+        <v>Bundle Name</v>
       </c>
       <c r="C44" t="str">
-        <v>Choose your plan</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="D44" t="str">
-        <v/>
+        <v>bundle</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>variant2</v>
+        <v>variant1</v>
       </c>
       <c r="B45" t="str">
-        <v>Header Full Copy</v>
+        <v>Bundle Description</v>
       </c>
       <c r="C45" t="str">
-        <v>Buy {{PPV_NAME}} with DAZN Standard or get it included in DAZN Ultimate.</v>
+        <v>{{BUNDLE_DESCRIPTION}}</v>
       </c>
       <c r="D45" t="str">
-        <v/>
+        <v>bundle</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>variant2</v>
+        <v>variant1</v>
       </c>
       <c r="B46" t="str">
-        <v>Header Highlight Text1</v>
+        <v>Bundle Monthly Price</v>
       </c>
       <c r="C46" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>{{BUNDLE_MONTHLY_PRICE}}</v>
       </c>
       <c r="D46" t="str">
-        <v/>
+        <v>bundle</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>variant2</v>
+        <v>variant1</v>
       </c>
       <c r="B47" t="str">
-        <v>Header Highlight Text2</v>
+        <v>Bundle Price</v>
       </c>
       <c r="C47" t="str">
-        <v>get it included in DAZN Ultimate.</v>
+        <v>{{BUNDLE_PRICE}}</v>
       </c>
       <c r="D47" t="str">
-        <v/>
+        <v>bundle</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>variant2</v>
+        <v>variant1</v>
       </c>
       <c r="B48" t="str">
-        <v>PPV Image</v>
+        <v>Bundle Original Price</v>
       </c>
       <c r="C48" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
       </c>
       <c r="D48" t="str">
-        <v/>
+        <v>bundle</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>variant2</v>
+        <v>variant1</v>
       </c>
       <c r="B49" t="str">
-        <v>Event Date and Time</v>
+        <v>Bundle Fight Count</v>
       </c>
       <c r="C49" t="str">
-        <v>{{PPV_DATE}}</v>
+        <v>{{BUNDLE_FIGHT_COUNT}}</v>
       </c>
       <c r="D49" t="str">
-        <v/>
+        <v>bundle</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>variant2</v>
+        <v>variant1</v>
       </c>
       <c r="B50" t="str">
-        <v>Event Name</v>
+        <v>Bundle Save Badge</v>
       </c>
       <c r="C50" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>{{BUNDLE_SAVE_BADGE}}</v>
       </c>
       <c r="D50" t="str">
-        <v/>
+        <v>bundle</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>variant2</v>
+        <v>variant1</v>
       </c>
       <c r="B51" t="str">
-        <v>PPV Checkbox Present</v>
+        <v>Bundle PPV 1 Full Name</v>
       </c>
       <c r="C51" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_PPV1_FULL_NAME}}</v>
       </c>
       <c r="D51" t="str">
-        <v/>
+        <v>bundle</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>variant2</v>
+        <v>variant1</v>
       </c>
       <c r="B52" t="str">
-        <v>PPV Selected</v>
+        <v>Bundle PPV 1 Date</v>
       </c>
       <c r="C52" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_PPV1_DATE}}</v>
       </c>
       <c r="D52" t="str">
-        <v/>
+        <v>bundle</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>variant2</v>
+        <v>variant1</v>
       </c>
       <c r="B53" t="str">
-        <v>PPV Name</v>
+        <v>Bundle PPV 1 Image</v>
       </c>
       <c r="C53" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>Yes</v>
       </c>
       <c r="D53" t="str">
-        <v/>
+        <v>bundle</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>variant2</v>
+        <v>variant1</v>
       </c>
       <c r="B54" t="str">
-        <v>PPV Price</v>
+        <v>Bundle PPV 2 Full Name</v>
       </c>
       <c r="C54" t="str">
-        <v>{{PPV_PRICE}}</v>
+        <v>{{BUNDLE_PPV2_FULL_NAME}}</v>
       </c>
       <c r="D54" t="str">
-        <v/>
+        <v>bundle</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>variant2</v>
+        <v>variant1</v>
       </c>
       <c r="B55" t="str">
-        <v>Currency</v>
+        <v>Bundle PPV 2 Date</v>
       </c>
       <c r="C55" t="str">
-        <v>{{CURRENCY}}</v>
+        <v>{{BUNDLE_PPV2_DATE}}</v>
       </c>
       <c r="D55" t="str">
-        <v/>
+        <v>bundle</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>variant2</v>
+        <v>variant1</v>
       </c>
       <c r="B56" t="str">
-        <v>Subscription Section Title</v>
+        <v>Bundle PPV 2 Image</v>
       </c>
       <c r="C56" t="str">
-        <v>Choose your subscription</v>
+        <v>Yes</v>
       </c>
       <c r="D56" t="str">
-        <v/>
+        <v>bundle</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>variant2</v>
+        <v>variant1</v>
       </c>
       <c r="B57" t="str">
-        <v>Trial Card Present</v>
+        <v>CTA Button</v>
       </c>
       <c r="C57" t="str">
-        <v>Yes</v>
+        <v>{{PPV_CTA_TEXT}}</v>
       </c>
       <c r="D57" t="str">
         <v/>
@@ -2274,16 +3285,16 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>variant2</v>
+        <v>variant1</v>
       </c>
       <c r="B58" t="str">
-        <v>Trial Title</v>
+        <v>CTA Without PPV</v>
       </c>
       <c r="C58" t="str">
-        <v>7-day free trial of DAZN Standard</v>
+        <v>Subscribe without a pay-per-view</v>
       </c>
       <c r="D58" t="str">
-        <v/>
+        <v>newuser</v>
       </c>
     </row>
     <row r="59">
@@ -2291,10 +3302,10 @@
         <v>variant2</v>
       </c>
       <c r="B59" t="str">
-        <v>Trial Radio Present</v>
+        <v>Page Title</v>
       </c>
       <c r="C59" t="str">
-        <v>Yes</v>
+        <v>Choose your plan</v>
       </c>
       <c r="D59" t="str">
         <v/>
@@ -2305,10 +3316,10 @@
         <v>variant2</v>
       </c>
       <c r="B60" t="str">
-        <v>Trial Selected</v>
+        <v>Header Full Copy</v>
       </c>
       <c r="C60" t="str">
-        <v>Yes</v>
+        <v>Buy {{PPV_NAME}} with DAZN Standard or get it included in DAZN Ultimate.</v>
       </c>
       <c r="D60" t="str">
         <v/>
@@ -2319,10 +3330,10 @@
         <v>variant2</v>
       </c>
       <c r="B61" t="str">
-        <v>Trial Feature 1</v>
+        <v>Header Highlight Text1</v>
       </c>
       <c r="C61" t="str">
-        <v>7-days free access to DAZN Standard.</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="D61" t="str">
         <v/>
@@ -2333,10 +3344,10 @@
         <v>variant2</v>
       </c>
       <c r="B62" t="str">
-        <v>Trial Feature 2</v>
+        <v>Header Highlight Text2</v>
       </c>
       <c r="C62" t="str">
-        <v>Cancel anytime during the trial and only pay for the fight. After the trial you move onto a Monthly Flex plan for {{CURRENCY}}{{MONTHLY_PRICE}}/month. You will not lose access to the pay-per-view[s].</v>
+        <v>get it included in DAZN Ultimate.</v>
       </c>
       <c r="D62" t="str">
         <v/>
@@ -2347,7 +3358,7 @@
         <v>variant2</v>
       </c>
       <c r="B63" t="str">
-        <v>Upsell Section Present</v>
+        <v>PPV Image</v>
       </c>
       <c r="C63" t="str">
         <v>Yes</v>
@@ -2361,10 +3372,10 @@
         <v>variant2</v>
       </c>
       <c r="B64" t="str">
-        <v>Upsell Label</v>
+        <v>Event Date and Time</v>
       </c>
       <c r="C64" t="str">
-        <v>Pay-per-views included</v>
+        <v>{{PPV_DATE}}</v>
       </c>
       <c r="D64" t="str">
         <v/>
@@ -2375,10 +3386,10 @@
         <v>variant2</v>
       </c>
       <c r="B65" t="str">
-        <v>Upsell Plan Name</v>
+        <v>Event Name</v>
       </c>
       <c r="C65" t="str">
-        <v>DAZN Ultimate</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="D65" t="str">
         <v/>
@@ -2389,10 +3400,10 @@
         <v>variant2</v>
       </c>
       <c r="B66" t="str">
-        <v>Upsell Price Text</v>
+        <v>PPV Checkbox Present</v>
       </c>
       <c r="C66" t="str">
-        <v>From</v>
+        <v>Yes</v>
       </c>
       <c r="D66" t="str">
         <v/>
@@ -2403,10 +3414,10 @@
         <v>variant2</v>
       </c>
       <c r="B67" t="str">
-        <v>Upsell Price</v>
+        <v>PPV Selected</v>
       </c>
       <c r="C67" t="str">
-        <v>{{UPSELL_PRICE}}</v>
+        <v>Yes</v>
       </c>
       <c r="D67" t="str">
         <v/>
@@ -2417,10 +3428,10 @@
         <v>variant2</v>
       </c>
       <c r="B68" t="str">
-        <v>Upsell Price Length</v>
+        <v>PPV Name</v>
       </c>
       <c r="C68" t="str">
-        <v>/ month</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="D68" t="str">
         <v/>
@@ -2431,10 +3442,10 @@
         <v>variant2</v>
       </c>
       <c r="B69" t="str">
-        <v>Upsell Billing Text</v>
+        <v>PPV Price</v>
       </c>
       <c r="C69" t="str">
-        <v>Annual contract. Auto renews.</v>
+        <v>{{PPV_PRICE}}</v>
       </c>
       <c r="D69" t="str">
         <v/>
@@ -2445,10 +3456,10 @@
         <v>variant2</v>
       </c>
       <c r="B70" t="str">
-        <v>Included PPV1 Name</v>
+        <v>Currency</v>
       </c>
       <c r="C70" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>{{CURRENCY}}</v>
       </c>
       <c r="D70" t="str">
         <v/>
@@ -2459,10 +3470,10 @@
         <v>variant2</v>
       </c>
       <c r="B71" t="str">
-        <v>PPV1 Image Present on ultimate tier</v>
+        <v>Subscription Section Title</v>
       </c>
       <c r="C71" t="str">
-        <v>Yes</v>
+        <v>Choose your subscription</v>
       </c>
       <c r="D71" t="str">
         <v/>
@@ -2473,10 +3484,10 @@
         <v>variant2</v>
       </c>
       <c r="B72" t="str">
-        <v>PPV1 Date Text on ultimate tier</v>
+        <v>Trial Card Present</v>
       </c>
       <c r="C72" t="str">
-        <v>{{PPV_DATE}}</v>
+        <v>Yes</v>
       </c>
       <c r="D72" t="str">
         <v/>
@@ -2487,10 +3498,10 @@
         <v>variant2</v>
       </c>
       <c r="B73" t="str">
-        <v>PPV1 Included tag</v>
+        <v>Trial Title</v>
       </c>
       <c r="C73" t="str">
-        <v>Yes</v>
+        <v>7-day free trial of DAZN Standard</v>
       </c>
       <c r="D73" t="str">
         <v/>
@@ -2501,10 +3512,10 @@
         <v>variant2</v>
       </c>
       <c r="B74" t="str">
-        <v>Included PPV2 Name</v>
+        <v>Trial Radio Present</v>
       </c>
       <c r="C74" t="str">
-        <v>N/A</v>
+        <v>Yes</v>
       </c>
       <c r="D74" t="str">
         <v/>
@@ -2515,10 +3526,10 @@
         <v>variant2</v>
       </c>
       <c r="B75" t="str">
-        <v>PPV2 Image Present on ultimate tier</v>
+        <v>Trial Selected</v>
       </c>
       <c r="C75" t="str">
-        <v>N/A</v>
+        <v>Yes</v>
       </c>
       <c r="D75" t="str">
         <v/>
@@ -2529,10 +3540,10 @@
         <v>variant2</v>
       </c>
       <c r="B76" t="str">
-        <v>PPV2 Date Text on ultimate tier</v>
+        <v>Trial Feature 1</v>
       </c>
       <c r="C76" t="str">
-        <v>N/A</v>
+        <v>7-days free access to DAZN Standard.</v>
       </c>
       <c r="D76" t="str">
         <v/>
@@ -2543,10 +3554,10 @@
         <v>variant2</v>
       </c>
       <c r="B77" t="str">
-        <v>PPV2 Included tag</v>
+        <v>Trial Feature 2</v>
       </c>
       <c r="C77" t="str">
-        <v>N/A</v>
+        <v>Cancel anytime during the trial and only pay for the fight. After the trial you move onto a Monthly Flex plan for {{CURRENCY}}{{MONTHLY_PRICE}}/month. You will not lose access to the pay-per-view[s].</v>
       </c>
       <c r="D77" t="str">
         <v/>
@@ -2557,10 +3568,10 @@
         <v>variant2</v>
       </c>
       <c r="B78" t="str">
-        <v>Upsell Feature 1</v>
+        <v>Upsell Section Present</v>
       </c>
       <c r="C78" t="str">
-        <v>Pay-per-views included at no extra cost. Minimum of 12 events per year including {{PPV_NAME}}.</v>
+        <v>Yes</v>
       </c>
       <c r="D78" t="str">
         <v/>
@@ -2571,10 +3582,10 @@
         <v>variant2</v>
       </c>
       <c r="B79" t="str">
-        <v>Upsell Highlight Text</v>
+        <v>Upsell Label</v>
       </c>
       <c r="C79" t="str">
-        <v>{{PPV_NAME}}.</v>
+        <v>Pay-per-views included</v>
       </c>
       <c r="D79" t="str">
         <v/>
@@ -2585,10 +3596,10 @@
         <v>variant2</v>
       </c>
       <c r="B80" t="str">
-        <v>Upsell Feature 2</v>
+        <v>Upsell Plan Name</v>
       </c>
       <c r="C80" t="str">
-        <v>HDR and Dolby 5.1 surround sound on select events.</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="D80" t="str">
         <v/>
@@ -2599,10 +3610,10 @@
         <v>variant2</v>
       </c>
       <c r="B81" t="str">
-        <v>Upsell Feature 3</v>
+        <v>Upsell Price Text</v>
       </c>
       <c r="C81" t="str">
-        <v>185+ fights a year from the best promoters</v>
+        <v>From</v>
       </c>
       <c r="D81" t="str">
         <v/>
@@ -2613,10 +3624,10 @@
         <v>variant2</v>
       </c>
       <c r="B82" t="str">
-        <v>Whats Included CTA</v>
+        <v>Upsell Price</v>
       </c>
       <c r="C82" t="str">
-        <v>Whats included</v>
+        <v>{{UPSELL_PRICE}}</v>
       </c>
       <c r="D82" t="str">
         <v/>
@@ -2627,10 +3638,10 @@
         <v>variant2</v>
       </c>
       <c r="B83" t="str">
-        <v>Gold Highlight 1</v>
+        <v>Upsell Price Length</v>
       </c>
       <c r="C83" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>/ month</v>
       </c>
       <c r="D83" t="str">
         <v/>
@@ -2641,10 +3652,10 @@
         <v>variant2</v>
       </c>
       <c r="B84" t="str">
-        <v>Gold Highlight 2</v>
+        <v>Upsell Billing Text</v>
       </c>
       <c r="C84" t="str">
-        <v>get it included in DAZN Ultimate.</v>
+        <v>Annual contract. Auto renews.</v>
       </c>
       <c r="D84" t="str">
         <v/>
@@ -2655,10 +3666,10 @@
         <v>variant2</v>
       </c>
       <c r="B85" t="str">
-        <v>Gold Highlight 3</v>
+        <v>Included PPV1 Name</v>
       </c>
       <c r="C85" t="str">
-        <v>DAZN Ultimate</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="D85" t="str">
         <v/>
@@ -2669,10 +3680,10 @@
         <v>variant2</v>
       </c>
       <c r="B86" t="str">
-        <v>CTA Button</v>
+        <v>PPV1 Image Present on ultimate tier</v>
       </c>
       <c r="C86" t="str">
-        <v>Continue with PPV + 7-day free trial</v>
+        <v>Yes</v>
       </c>
       <c r="D86" t="str">
         <v/>
@@ -2683,18 +3694,228 @@
         <v>variant2</v>
       </c>
       <c r="B87" t="str">
+        <v>PPV1 Date Text on ultimate tier</v>
+      </c>
+      <c r="C87" t="str">
+        <v>{{PPV_DATE}}</v>
+      </c>
+      <c r="D87" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>variant2</v>
+      </c>
+      <c r="B88" t="str">
+        <v>PPV1 Included tag</v>
+      </c>
+      <c r="C88" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="D88" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>variant2</v>
+      </c>
+      <c r="B89" t="str">
+        <v>Included PPV2 Name</v>
+      </c>
+      <c r="C89" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="D89" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>variant2</v>
+      </c>
+      <c r="B90" t="str">
+        <v>PPV2 Image Present on ultimate tier</v>
+      </c>
+      <c r="C90" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="D90" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>variant2</v>
+      </c>
+      <c r="B91" t="str">
+        <v>PPV2 Date Text on ultimate tier</v>
+      </c>
+      <c r="C91" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="D91" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>variant2</v>
+      </c>
+      <c r="B92" t="str">
+        <v>PPV2 Included tag</v>
+      </c>
+      <c r="C92" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="D92" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>variant2</v>
+      </c>
+      <c r="B93" t="str">
+        <v>Upsell Feature 1</v>
+      </c>
+      <c r="C93" t="str">
+        <v>Pay-per-views included at no extra cost. Minimum of 12 events per year including {{PPV_NAME}}.</v>
+      </c>
+      <c r="D93" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>variant2</v>
+      </c>
+      <c r="B94" t="str">
+        <v>Upsell Highlight Text</v>
+      </c>
+      <c r="C94" t="str">
+        <v>{{PPV_NAME}}.</v>
+      </c>
+      <c r="D94" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>variant2</v>
+      </c>
+      <c r="B95" t="str">
+        <v>Upsell Feature 2</v>
+      </c>
+      <c r="C95" t="str">
+        <v>HDR and Dolby 5.1 surround sound on select events.</v>
+      </c>
+      <c r="D95" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>variant2</v>
+      </c>
+      <c r="B96" t="str">
+        <v>Upsell Feature 3</v>
+      </c>
+      <c r="C96" t="str">
+        <v>185+ fights a year from the best promoters</v>
+      </c>
+      <c r="D96" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>variant2</v>
+      </c>
+      <c r="B97" t="str">
+        <v>Whats Included CTA</v>
+      </c>
+      <c r="C97" t="str">
+        <v>Whats included</v>
+      </c>
+      <c r="D97" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>variant2</v>
+      </c>
+      <c r="B98" t="str">
+        <v>Gold Highlight 1</v>
+      </c>
+      <c r="C98" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+      <c r="D98" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>variant2</v>
+      </c>
+      <c r="B99" t="str">
+        <v>Gold Highlight 2</v>
+      </c>
+      <c r="C99" t="str">
+        <v>get it included in DAZN Ultimate.</v>
+      </c>
+      <c r="D99" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>variant2</v>
+      </c>
+      <c r="B100" t="str">
+        <v>Gold Highlight 3</v>
+      </c>
+      <c r="C100" t="str">
+        <v>DAZN Ultimate</v>
+      </c>
+      <c r="D100" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>variant2</v>
+      </c>
+      <c r="B101" t="str">
+        <v>CTA Button</v>
+      </c>
+      <c r="C101" t="str">
+        <v>Continue with PPV + 7-day free trial</v>
+      </c>
+      <c r="D101" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>variant2</v>
+      </c>
+      <c r="B102" t="str">
         <v>CTA Without PPV</v>
       </c>
-      <c r="C87" t="str">
+      <c r="C102" t="str">
         <v>N/A</v>
       </c>
-      <c r="D87" t="str">
+      <c r="D102" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D87"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D102"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2702,6 +3923,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D37"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="34.83203125" customWidth="1"/>
+    <col min="3" max="3" width="70.83203125" customWidth="1"/>
+    <col min="4" max="4" width="6.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3230,7 +4457,14 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F100"/>
+  <dimension ref="A1:E98"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="27.83203125" customWidth="1"/>
+    <col min="3" max="3" width="28.83203125" customWidth="1"/>
+    <col min="4" max="4" width="160.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3248,9 +4482,6 @@
       <c r="E1" t="str">
         <v>Flow</v>
       </c>
-      <c r="F1" t="str">
-        <v>Type</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -3591,9 +4822,6 @@
       <c r="E21" t="str">
         <v/>
       </c>
-      <c r="F21" t="str">
-        <v>contains</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -3781,9 +5009,6 @@
       <c r="E32" t="str">
         <v/>
       </c>
-      <c r="F32" t="str">
-        <v>contains</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -4005,9 +5230,6 @@
       <c r="E45" t="str">
         <v/>
       </c>
-      <c r="F45" t="str">
-        <v>contains</v>
-      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -4031,13 +5253,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B47" t="str">
-        <v>Annual Pay Upfront</v>
+        <v>Annual Pay Monthly</v>
       </c>
       <c r="C47" t="str">
-        <v>Page Title</v>
+        <v>Discount Badge</v>
       </c>
       <c r="D47" t="str">
-        <v>Choose how to pay</v>
+        <v>{{DISCOUNT_BADGE}}</v>
       </c>
       <c r="E47" t="str">
         <v/>
@@ -4051,10 +5273,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C48" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D48" t="str">
-        <v>DAZN Ultimate</v>
+        <v>Choose how to pay</v>
       </c>
       <c r="E48" t="str">
         <v/>
@@ -4068,10 +5290,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C49" t="str">
-        <v>PPV Name</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D49" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="E49" t="str">
         <v/>
@@ -4085,10 +5307,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C50" t="str">
-        <v>PPV Price</v>
+        <v>PPV Name</v>
       </c>
       <c r="D50" t="str">
-        <v>{{CURRENCY}}0</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="E50" t="str">
         <v/>
@@ -4102,10 +5324,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C51" t="str">
-        <v>Rate Plan</v>
+        <v>PPV Price</v>
       </c>
       <c r="D51" t="str">
-        <v>Annual - Pay Upfront</v>
+        <v>{{CURRENCY}}0</v>
       </c>
       <c r="E51" t="str">
         <v/>
@@ -4119,10 +5341,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C52" t="str">
-        <v>Rate Plan Price</v>
+        <v>Rate Plan</v>
       </c>
       <c r="D52" t="str">
-        <v>{{ANNUAL_UPFRONT_PRICE}}/year</v>
+        <v>Annual - Pay Upfront</v>
       </c>
       <c r="E52" t="str">
         <v/>
@@ -4136,10 +5358,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C53" t="str">
-        <v>Today You Pay Text</v>
+        <v>Rate Plan Price</v>
       </c>
       <c r="D53" t="str">
-        <v>Today you pay</v>
+        <v>{{ANNUAL_UPFRONT_PRICE}}/year</v>
       </c>
       <c r="E53" t="str">
         <v/>
@@ -4153,10 +5375,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C54" t="str">
-        <v>Today You Pay Price</v>
+        <v>Today You Pay Text</v>
       </c>
       <c r="D54" t="str">
-        <v>{{TODAY_YOU_PAY_PRICE}}</v>
+        <v>Today you pay</v>
       </c>
       <c r="E54" t="str">
         <v/>
@@ -4170,10 +5392,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C55" t="str">
-        <v>Next Payment Label</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D55" t="str">
-        <v>Next Annual payment on {{NEXT_PAYMENT_DATE}}</v>
+        <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
       <c r="E55" t="str">
         <v/>
@@ -4187,10 +5409,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C56" t="str">
-        <v>Next Payment Price</v>
+        <v>Next Payment Label</v>
       </c>
       <c r="D56" t="str">
-        <v>{{ANNUAL_UPFRONT_PRICE}}</v>
+        <v>Next Annual payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
       <c r="E56" t="str">
         <v/>
@@ -4204,16 +5426,13 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C57" t="str">
-        <v>Cancellation Text</v>
+        <v>Next Payment Price</v>
       </c>
       <c r="D57" t="str">
-        <v>{{CANCELLATION_TEXT}}</v>
+        <v>{{ANNUAL_UPFRONT_PRICE}}</v>
       </c>
       <c r="E57" t="str">
         <v/>
-      </c>
-      <c r="F57" t="str">
-        <v>contains</v>
       </c>
     </row>
     <row r="58">
@@ -4224,10 +5443,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C58" t="str">
-        <v>Redeem Promo Code CTA</v>
+        <v>Cancellation Text</v>
       </c>
       <c r="D58" t="str">
-        <v>Yes</v>
+        <v>{{CANCELLATION_TEXT}}</v>
       </c>
       <c r="E58" t="str">
         <v/>
@@ -4235,16 +5454,16 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Standard</v>
+        <v>Ultimate</v>
       </c>
       <c r="B59" t="str">
-        <v>Monthly Bundle</v>
+        <v>Annual Pay Upfront</v>
       </c>
       <c r="C59" t="str">
-        <v>Page Title</v>
+        <v>Redeem Promo Code CTA</v>
       </c>
       <c r="D59" t="str">
-        <v>{{PAYMENT_PAGE_TITLE}}</v>
+        <v>Yes</v>
       </c>
       <c r="E59" t="str">
         <v/>
@@ -4258,10 +5477,10 @@
         <v>Monthly Bundle</v>
       </c>
       <c r="C60" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D60" t="str">
-        <v>DAZN Standard</v>
+        <v>{{PAYMENT_PAGE_TITLE}}</v>
       </c>
       <c r="E60" t="str">
         <v/>
@@ -4275,10 +5494,10 @@
         <v>Monthly Bundle</v>
       </c>
       <c r="C61" t="str">
-        <v>Bundle Name</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D61" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>DAZN Standard</v>
       </c>
       <c r="E61" t="str">
         <v/>
@@ -4292,10 +5511,10 @@
         <v>Monthly Bundle</v>
       </c>
       <c r="C62" t="str">
-        <v>Bundle Price</v>
+        <v>Bundle Name</v>
       </c>
       <c r="D62" t="str">
-        <v>{{BUNDLE_PRICE}}</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="E62" t="str">
         <v/>
@@ -4309,10 +5528,10 @@
         <v>Monthly Bundle</v>
       </c>
       <c r="C63" t="str">
-        <v>Today You Pay Price</v>
+        <v>Bundle Price</v>
       </c>
       <c r="D63" t="str">
-        <v>{{BUNDLE_TODAY_YOU_PAY_STANDARD}}</v>
+        <v>{{BUNDLE_PRICE}}</v>
       </c>
       <c r="E63" t="str">
         <v/>
@@ -4326,16 +5545,13 @@
         <v>Monthly Bundle</v>
       </c>
       <c r="C64" t="str">
-        <v>Cancellation Text</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D64" t="str">
-        <v>{{CANCELLATION_TEXT}}</v>
+        <v>{{BUNDLE_TODAY_YOU_PAY_STANDARD}}</v>
       </c>
       <c r="E64" t="str">
         <v/>
-      </c>
-      <c r="F64" t="str">
-        <v>contains</v>
       </c>
     </row>
     <row r="65">
@@ -4343,13 +5559,13 @@
         <v>Standard</v>
       </c>
       <c r="B65" t="str">
-        <v>Annual Pay Monthly Bundle</v>
+        <v>Monthly Bundle</v>
       </c>
       <c r="C65" t="str">
-        <v>Page Title</v>
+        <v>Cancellation Text</v>
       </c>
       <c r="D65" t="str">
-        <v>Choose how to pay</v>
+        <v>{{CANCELLATION_TEXT}}</v>
       </c>
       <c r="E65" t="str">
         <v/>
@@ -4363,10 +5579,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C66" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D66" t="str">
-        <v>DAZN Standard</v>
+        <v>Choose how to pay</v>
       </c>
       <c r="E66" t="str">
         <v/>
@@ -4380,10 +5596,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C67" t="str">
-        <v>Rate Plan</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D67" t="str">
-        <v>Annual - Pay Monthly</v>
+        <v>DAZN Standard</v>
       </c>
       <c r="E67" t="str">
         <v/>
@@ -4397,10 +5613,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C68" t="str">
-        <v>First Month Free Text</v>
+        <v>Rate Plan</v>
       </c>
       <c r="D68" t="str">
-        <v>First month free</v>
+        <v>Annual - Pay Monthly</v>
       </c>
       <c r="E68" t="str">
         <v/>
@@ -4414,10 +5630,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C69" t="str">
-        <v>Bundle Name</v>
+        <v>First Month Free Text</v>
       </c>
       <c r="D69" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>First month free</v>
       </c>
       <c r="E69" t="str">
         <v/>
@@ -4431,10 +5647,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C70" t="str">
-        <v>Bundle Original Price</v>
+        <v>Bundle Name</v>
       </c>
       <c r="D70" t="str">
-        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="E70" t="str">
         <v/>
@@ -4448,10 +5664,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C71" t="str">
-        <v>Bundle Price</v>
+        <v>Bundle Original Price</v>
       </c>
       <c r="D71" t="str">
-        <v>{{BUNDLE_PRICE}}</v>
+        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
       </c>
       <c r="E71" t="str">
         <v/>
@@ -4465,10 +5681,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C72" t="str">
-        <v>Bundle Discount</v>
+        <v>Bundle Price</v>
       </c>
       <c r="D72" t="str">
-        <v>{{BUNDLE_DISCOUNT}}</v>
+        <v>{{BUNDLE_PRICE}}</v>
       </c>
       <c r="E72" t="str">
         <v/>
@@ -4482,10 +5698,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C73" t="str">
-        <v>Today You Pay Price</v>
+        <v>Bundle Discount</v>
       </c>
       <c r="D73" t="str">
-        <v>{{BUNDLE_TODAY_YOU_PAY_STANDARD}}</v>
+        <v>{{BUNDLE_DISCOUNT}}</v>
       </c>
       <c r="E73" t="str">
         <v/>
@@ -4499,16 +5715,13 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C74" t="str">
-        <v>Cancellation Text</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D74" t="str">
-        <v>{{CANCELLATION_TEXT_ANNUAL}}</v>
+        <v>{{BUNDLE_TODAY_YOU_PAY_STANDARD}}</v>
       </c>
       <c r="E74" t="str">
         <v/>
-      </c>
-      <c r="F74" t="str">
-        <v>contains</v>
       </c>
     </row>
     <row r="75">
@@ -4519,10 +5732,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C75" t="str">
-        <v>Ultimate Upsell Text</v>
+        <v>Cancellation Text</v>
       </c>
       <c r="D75" t="str">
-        <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
+        <v>{{CANCELLATION_TEXT_ANNUAL}}</v>
       </c>
       <c r="E75" t="str">
         <v/>
@@ -4530,16 +5743,16 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Ultimate</v>
+        <v>Standard</v>
       </c>
       <c r="B76" t="str">
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C76" t="str">
-        <v>Page Title</v>
+        <v>Ultimate Upsell Text</v>
       </c>
       <c r="D76" t="str">
-        <v>Choose how to pay</v>
+        <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
       <c r="E76" t="str">
         <v/>
@@ -4553,10 +5766,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C77" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D77" t="str">
-        <v>DAZN Ultimate</v>
+        <v>Choose how to pay</v>
       </c>
       <c r="E77" t="str">
         <v/>
@@ -4570,10 +5783,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C78" t="str">
-        <v>Rate Plan</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D78" t="str">
-        <v>Annual - Pay Monthly</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="E78" t="str">
         <v/>
@@ -4587,10 +5800,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C79" t="str">
-        <v>Rate Plan Price</v>
+        <v>Rate Plan</v>
       </c>
       <c r="D79" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
+        <v>Annual - Pay Monthly</v>
       </c>
       <c r="E79" t="str">
         <v/>
@@ -4604,10 +5817,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C80" t="str">
-        <v>Bundle Name</v>
+        <v>Rate Plan Price</v>
       </c>
       <c r="D80" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
       </c>
       <c r="E80" t="str">
         <v/>
@@ -4621,10 +5834,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C81" t="str">
-        <v>Bundle Price</v>
+        <v>Bundle Name</v>
       </c>
       <c r="D81" t="str">
-        <v>{{CURRENCY}}0</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="E81" t="str">
         <v/>
@@ -4638,10 +5851,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C82" t="str">
-        <v>Today You Pay Price</v>
+        <v>Bundle Price</v>
       </c>
       <c r="D82" t="str">
-        <v>{{TODAY_YOU_PAY_PRICE}}</v>
+        <v>{{CURRENCY}}0</v>
       </c>
       <c r="E82" t="str">
         <v/>
@@ -4655,10 +5868,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C83" t="str">
-        <v>Next Payment Label</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D83" t="str">
-        <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
+        <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
       <c r="E83" t="str">
         <v/>
@@ -4672,10 +5885,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C84" t="str">
-        <v>Next Payment Price</v>
+        <v>Next Payment Label</v>
       </c>
       <c r="D84" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
+        <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
       <c r="E84" t="str">
         <v/>
@@ -4689,16 +5902,13 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C85" t="str">
-        <v>Cancellation Text</v>
+        <v>Next Payment Price</v>
       </c>
       <c r="D85" t="str">
-        <v>{{CANCELLATION_TEXT}}</v>
+        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
       </c>
       <c r="E85" t="str">
         <v/>
-      </c>
-      <c r="F85" t="str">
-        <v>contains</v>
       </c>
     </row>
     <row r="86">
@@ -4706,13 +5916,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B86" t="str">
-        <v>Annual Pay Upfront Bundle</v>
+        <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C86" t="str">
-        <v>Page Title</v>
+        <v>Cancellation Text</v>
       </c>
       <c r="D86" t="str">
-        <v>Choose how to pay</v>
+        <v>{{CANCELLATION_TEXT}}</v>
       </c>
       <c r="E86" t="str">
         <v/>
@@ -4723,13 +5933,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B87" t="str">
-        <v>Annual Pay Upfront Bundle</v>
+        <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C87" t="str">
-        <v>DAZN Tier</v>
+        <v>Discount Badge</v>
       </c>
       <c r="D87" t="str">
-        <v>DAZN Ultimate</v>
+        <v>{{DISCOUNT_BADGE}}</v>
       </c>
       <c r="E87" t="str">
         <v/>
@@ -4743,10 +5953,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C88" t="str">
-        <v>Rate Plan</v>
+        <v>Page Title</v>
       </c>
       <c r="D88" t="str">
-        <v>Annual - Pay Upfront</v>
+        <v>Choose how to pay</v>
       </c>
       <c r="E88" t="str">
         <v/>
@@ -4760,10 +5970,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C89" t="str">
-        <v>Rate Plan Price</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D89" t="str">
-        <v>{{ANNUAL_UPFRONT_PRICE}}/year</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="E89" t="str">
         <v/>
@@ -4777,10 +5987,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C90" t="str">
-        <v>Save Badge</v>
+        <v>Rate Plan</v>
       </c>
       <c r="D90" t="str">
-        <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
+        <v>Annual - Pay Upfront</v>
       </c>
       <c r="E90" t="str">
         <v/>
@@ -4794,10 +6004,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C91" t="str">
-        <v>Bundle Name</v>
+        <v>Rate Plan Price</v>
       </c>
       <c r="D91" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>{{ANNUAL_UPFRONT_PRICE}}/year</v>
       </c>
       <c r="E91" t="str">
         <v/>
@@ -4811,10 +6021,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C92" t="str">
-        <v>Bundle Price</v>
+        <v>Save Badge</v>
       </c>
       <c r="D92" t="str">
-        <v>{{CURRENCY}}0</v>
+        <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
       </c>
       <c r="E92" t="str">
         <v/>
@@ -4828,10 +6038,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C93" t="str">
-        <v>Today You Pay Price</v>
+        <v>Bundle Name</v>
       </c>
       <c r="D93" t="str">
-        <v>{{ANNUAL_UPFRONT_PRICE}}</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="E93" t="str">
         <v/>
@@ -4845,10 +6055,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C94" t="str">
-        <v>Next Payment Label</v>
+        <v>Bundle Price</v>
       </c>
       <c r="D94" t="str">
-        <v>Next Annual payment on {{NEXT_PAYMENT_DATE}}</v>
+        <v>{{CURRENCY}}0</v>
       </c>
       <c r="E94" t="str">
         <v/>
@@ -4862,7 +6072,7 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C95" t="str">
-        <v>Next Payment Price</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D95" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE}}</v>
@@ -4879,90 +6089,63 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C96" t="str">
-        <v>Cancellation Text</v>
+        <v>Next Payment Label</v>
       </c>
       <c r="D96" t="str">
-        <v>{{CANCELLATION_TEXT}}</v>
+        <v>Next Annual payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
       <c r="E96" t="str">
         <v/>
-      </c>
-      <c r="F96" t="str">
-        <v>contains</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>standard</v>
+        <v>Ultimate</v>
       </c>
       <c r="B97" t="str">
-        <v>monthly</v>
+        <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C97" t="str">
-        <v>Ultimate Upsell Banner Present</v>
+        <v>Next Payment Price</v>
       </c>
       <c r="D97" t="str">
-        <v>Yes</v>
+        <v>{{ANNUAL_UPFRONT_PRICE}}</v>
+      </c>
+      <c r="E97" t="str">
+        <v/>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>standard</v>
+        <v>Ultimate</v>
       </c>
       <c r="B98" t="str">
-        <v>monthly</v>
+        <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C98" t="str">
-        <v>Ultimate Upsell Price</v>
+        <v>Cancellation Text</v>
       </c>
       <c r="D98" t="str">
-        <v>{{ULTIMATE_ANNUAL_PAY_MONTHLY_PRICE}}</v>
-      </c>
-      <c r="F98" t="str">
-        <v>contains</v>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="str">
-        <v>standard</v>
-      </c>
-      <c r="B99" t="str">
-        <v>annual pay monthly</v>
-      </c>
-      <c r="C99" t="str">
-        <v>Ultimate Upsell Banner Present</v>
-      </c>
-      <c r="D99" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="str">
-        <v>standard</v>
-      </c>
-      <c r="B100" t="str">
-        <v>annual pay monthly</v>
-      </c>
-      <c r="C100" t="str">
-        <v>Ultimate Upsell Price</v>
-      </c>
-      <c r="D100" t="str">
-        <v>{{ULTIMATE_ANNUAL_PAY_MONTHLY_PRICE}}</v>
-      </c>
-      <c r="F100" t="str">
-        <v>contains</v>
+        <v>{{CANCELLATION_TEXT}}</v>
+      </c>
+      <c r="E98" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F100"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E98"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
+  <cols>
+    <col min="1" max="1" width="27.83203125" customWidth="1"/>
+    <col min="2" max="2" width="21.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5062,7 +6245,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Popup Buy Now CTA</v>
+        <v>Popup Buy Now CTA Present</v>
       </c>
       <c r="B13" t="str">
         <v>Yes</v>
@@ -5070,15 +6253,23 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
+        <v>Popup Buy Now CTA Text</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Buy now</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
         <v>Popup Close Button</v>
       </c>
-      <c r="B14" t="str">
+      <c r="B15" t="str">
         <v>Yes</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B15"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5086,6 +6277,10 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B8"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="25.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5160,7 +6355,11 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:B23"/>
+  <cols>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="70.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5169,9 +6368,6 @@
       <c r="B1" t="str">
         <v>Expected</v>
       </c>
-      <c r="C1" t="str">
-        <v>Type</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -5196,9 +6392,6 @@
       <c r="B4" t="str">
         <v>Buy {{PPV_NAME}}, or get it included in a DAZN Ultimate subscription</v>
       </c>
-      <c r="C4" t="str">
-        <v>contains</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -5311,9 +6504,6 @@
       <c r="B18" t="str">
         <v>{{UPSELL_FEATURE_1}}</v>
       </c>
-      <c r="C18" t="str">
-        <v>contains</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -5330,9 +6520,6 @@
       <c r="B20" t="str">
         <v>{{UPSELL_FEATURE_2}}</v>
       </c>
-      <c r="C20" t="str">
-        <v>contains</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -5341,9 +6528,6 @@
       <c r="B21" t="str">
         <v>{{UPSELL_FEATURE_3}}</v>
       </c>
-      <c r="C21" t="str">
-        <v>contains</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -5360,13 +6544,10 @@
       <c r="B23" t="str">
         <v>{{PPV_CTA_TEXT}}</v>
       </c>
-      <c r="C23" t="str">
-        <v>contains</v>
-      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B23"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5374,6 +6555,10 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B16"/>
+  <cols>
+    <col min="1" max="1" width="29.83203125" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>

<commit_message>
imported glory page and reports
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -415,7 +415,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -549,9 +549,20 @@
         <v>landing-page-banner</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>PPV Image Present</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="C13" t="str">
+        <v>landing</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C13"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -929,7 +940,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1085,16 +1096,38 @@
         <v>Visible</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>home-boxing-banner</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Banner Image Present</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>home-boxing-tile</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Popup Image Present</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C16"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C26"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1338,9 +1371,53 @@
         <v>Visible</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>home-page-banner</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Banner Image Present</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Popup Image Present</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>home-biggest-fights</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Popup Image Present</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>home-page-dazntile</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Banner Image Present</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C26"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1932,7 +2009,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1974,9 +2051,17 @@
         <v>Yes</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>PPV Image Present</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6312,7 +6397,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6434,9 +6519,17 @@
         <v>Yes</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>PPV Image Present</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B16"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fixed switch from landing
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -2620,7 +2620,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D102"/>
+  <dimension ref="A1:D94"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="37.83203125" customWidth="1"/>
@@ -2675,10 +2675,10 @@
         <v>variant1</v>
       </c>
       <c r="B4" t="str">
-        <v>Header Highlight Text1</v>
+        <v>Header Highlight Text2</v>
       </c>
       <c r="C4" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>N/A</v>
       </c>
       <c r="D4" t="str">
         <v/>
@@ -2689,10 +2689,10 @@
         <v>variant1</v>
       </c>
       <c r="B5" t="str">
-        <v>Header Highlight Text2</v>
+        <v>Event Name</v>
       </c>
       <c r="C5" t="str">
-        <v>N/A</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="D5" t="str">
         <v/>
@@ -2703,10 +2703,10 @@
         <v>variant1</v>
       </c>
       <c r="B6" t="str">
-        <v>Hero Image</v>
+        <v>PPV Per Fight Text</v>
       </c>
       <c r="C6" t="str">
-        <v>Yes</v>
+        <v>/fight</v>
       </c>
       <c r="D6" t="str">
         <v/>
@@ -2717,10 +2717,10 @@
         <v>variant1</v>
       </c>
       <c r="B7" t="str">
-        <v>Event Name</v>
+        <v>PPV Price</v>
       </c>
       <c r="C7" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>{{PPV_PRICE}}</v>
       </c>
       <c r="D7" t="str">
         <v/>
@@ -2731,10 +2731,10 @@
         <v>variant1</v>
       </c>
       <c r="B8" t="str">
-        <v>PPV Price</v>
+        <v>Currency</v>
       </c>
       <c r="C8" t="str">
-        <v>{{PPV_PRICE}}</v>
+        <v>{{CURRENCY}}</v>
       </c>
       <c r="D8" t="str">
         <v/>
@@ -2745,13 +2745,13 @@
         <v>variant1</v>
       </c>
       <c r="B9" t="str">
-        <v>Currency</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="C9" t="str">
-        <v>{{CURRENCY}}</v>
+        <v>+DAZN Standard</v>
       </c>
       <c r="D9" t="str">
-        <v/>
+        <v>newuser</v>
       </c>
     </row>
     <row r="10">
@@ -2759,13 +2759,13 @@
         <v>variant1</v>
       </c>
       <c r="B10" t="str">
-        <v>DAZN Tier</v>
+        <v>PPV Name</v>
       </c>
       <c r="C10" t="str">
-        <v>+DAZN Standard</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="D10" t="str">
-        <v>newuser</v>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -2773,10 +2773,10 @@
         <v>variant1</v>
       </c>
       <c r="B11" t="str">
-        <v>PPV Name</v>
+        <v>PPV Image Present</v>
       </c>
       <c r="C11" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>Yes</v>
       </c>
       <c r="D11" t="str">
         <v/>
@@ -2787,10 +2787,10 @@
         <v>variant1</v>
       </c>
       <c r="B12" t="str">
-        <v>PPV Image Present</v>
+        <v>PPV Date and Time Text</v>
       </c>
       <c r="C12" t="str">
-        <v>Yes</v>
+        <v>{{PPV_DATE}}</v>
       </c>
       <c r="D12" t="str">
         <v/>
@@ -2801,10 +2801,10 @@
         <v>variant1</v>
       </c>
       <c r="B13" t="str">
-        <v>PPV Date and Time Text</v>
+        <v>Radio Selected</v>
       </c>
       <c r="C13" t="str">
-        <v>{{PPV_DATE}}</v>
+        <v>Yes</v>
       </c>
       <c r="D13" t="str">
         <v/>
@@ -2815,10 +2815,10 @@
         <v>variant1</v>
       </c>
       <c r="B14" t="str">
-        <v>Radio Selected</v>
+        <v>PPV Card Title</v>
       </c>
       <c r="C14" t="str">
-        <v>Yes</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="D14" t="str">
         <v/>
@@ -2829,10 +2829,10 @@
         <v>variant1</v>
       </c>
       <c r="B15" t="str">
-        <v>PPV Card Title</v>
+        <v>PPV Card Description</v>
       </c>
       <c r="C15" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>{{PPV_CARD_DESCRIPTION}}</v>
       </c>
       <c r="D15" t="str">
         <v/>
@@ -2843,10 +2843,10 @@
         <v>variant1</v>
       </c>
       <c r="B16" t="str">
-        <v>PPV Card Description</v>
+        <v>Upsell Section Present</v>
       </c>
       <c r="C16" t="str">
-        <v>{{PPV_CARD_DESCRIPTION}}</v>
+        <v>Yes</v>
       </c>
       <c r="D16" t="str">
         <v/>
@@ -2857,10 +2857,10 @@
         <v>variant1</v>
       </c>
       <c r="B17" t="str">
-        <v>Upsell Section Present</v>
+        <v>Upsell Badge</v>
       </c>
       <c r="C17" t="str">
-        <v>Yes</v>
+        <v>The Ultimate Fan Package</v>
       </c>
       <c r="D17" t="str">
         <v/>
@@ -2871,10 +2871,10 @@
         <v>variant1</v>
       </c>
       <c r="B18" t="str">
-        <v>Upsell Badge</v>
+        <v>Upsell Plan Name</v>
       </c>
       <c r="C18" t="str">
-        <v>The Ultimate Fan Package</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="D18" t="str">
         <v/>
@@ -2885,10 +2885,10 @@
         <v>variant1</v>
       </c>
       <c r="B19" t="str">
-        <v>Upsell Plan Name</v>
+        <v>Upsell Price Text</v>
       </c>
       <c r="C19" t="str">
-        <v>DAZN Ultimate</v>
+        <v>N/A</v>
       </c>
       <c r="D19" t="str">
         <v/>
@@ -2899,10 +2899,10 @@
         <v>variant1</v>
       </c>
       <c r="B20" t="str">
-        <v>Upsell Price Text</v>
+        <v>Upsell Price</v>
       </c>
       <c r="C20" t="str">
-        <v>N/A</v>
+        <v>{{UPSELL_PRICE}}</v>
       </c>
       <c r="D20" t="str">
         <v/>
@@ -2913,10 +2913,10 @@
         <v>variant1</v>
       </c>
       <c r="B21" t="str">
-        <v>Upsell Price</v>
+        <v>Upsell Price Length</v>
       </c>
       <c r="C21" t="str">
-        <v>{{UPSELL_PRICE}}</v>
+        <v>{{UPSELL_PRICE_LENGTH}}</v>
       </c>
       <c r="D21" t="str">
         <v/>
@@ -2927,10 +2927,10 @@
         <v>variant1</v>
       </c>
       <c r="B22" t="str">
-        <v>Upsell Price Length</v>
+        <v>Upsell Crossed Price</v>
       </c>
       <c r="C22" t="str">
-        <v>{{UPSELL_PRICE_LENGTH}}</v>
+        <v>{{UPSELL_CROSSED_PRICE}}</v>
       </c>
       <c r="D22" t="str">
         <v/>
@@ -2941,10 +2941,10 @@
         <v>variant1</v>
       </c>
       <c r="B23" t="str">
-        <v>Upsell Crossed Price</v>
+        <v>Upsell Billing Text</v>
       </c>
       <c r="C23" t="str">
-        <v>{{UPSELL_CROSSED_PRICE}}</v>
+        <v>{{ANNUAL_PAY_MONTHLY_CONTRACT_TEXT}}</v>
       </c>
       <c r="D23" t="str">
         <v/>
@@ -2955,13 +2955,13 @@
         <v>variant1</v>
       </c>
       <c r="B24" t="str">
-        <v>Upsell Contract Text</v>
+        <v>Upsell Offer Text</v>
       </c>
       <c r="C24" t="str">
-        <v>Annual contract. Auto renews.</v>
+        <v>{{UPSELL_OFFER_TEXT}}</v>
       </c>
       <c r="D24" t="str">
-        <v/>
+        <v>offer</v>
       </c>
     </row>
     <row r="25">
@@ -2969,10 +2969,10 @@
         <v>variant1</v>
       </c>
       <c r="B25" t="str">
-        <v>Upsell Billing Text</v>
+        <v>Upsell Section Heading</v>
       </c>
       <c r="C25" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_CONTRACT_TEXT}}</v>
+        <v>{{UPSELL_SECTION_HEADING}}</v>
       </c>
       <c r="D25" t="str">
         <v/>
@@ -2983,13 +2983,13 @@
         <v>variant1</v>
       </c>
       <c r="B26" t="str">
-        <v>Upsell Offer Text</v>
+        <v>PPV1 Included tag</v>
       </c>
       <c r="C26" t="str">
-        <v>{{UPSELL_OFFER_TEXT}}</v>
+        <v>N/A</v>
       </c>
       <c r="D26" t="str">
-        <v>offer</v>
+        <v/>
       </c>
     </row>
     <row r="27">
@@ -2997,10 +2997,10 @@
         <v>variant1</v>
       </c>
       <c r="B27" t="str">
-        <v>Upsell Section Heading</v>
+        <v>Included PPV2 Name</v>
       </c>
       <c r="C27" t="str">
-        <v>{{UPSELL_SECTION_HEADING}}</v>
+        <v>N/A</v>
       </c>
       <c r="D27" t="str">
         <v/>
@@ -3011,10 +3011,10 @@
         <v>variant1</v>
       </c>
       <c r="B28" t="str">
-        <v>Included PPV1 Name</v>
+        <v>PPV2 Image Present on ultimate tier</v>
       </c>
       <c r="C28" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>N/A</v>
       </c>
       <c r="D28" t="str">
         <v/>
@@ -3025,10 +3025,10 @@
         <v>variant1</v>
       </c>
       <c r="B29" t="str">
-        <v>PPV1 Image Present on ultimate tier</v>
+        <v>PPV2 Date Text on ultimate tier</v>
       </c>
       <c r="C29" t="str">
-        <v>Yes</v>
+        <v>N/A</v>
       </c>
       <c r="D29" t="str">
         <v/>
@@ -3039,10 +3039,10 @@
         <v>variant1</v>
       </c>
       <c r="B30" t="str">
-        <v>PPV1 Upsell Tile Date</v>
+        <v>PPV2 Included tag</v>
       </c>
       <c r="C30" t="str">
-        <v>{{PPV1_UPSELL_TILE_DATE}}</v>
+        <v>N/A</v>
       </c>
       <c r="D30" t="str">
         <v/>
@@ -3053,10 +3053,10 @@
         <v>variant1</v>
       </c>
       <c r="B31" t="str">
-        <v>PPV1 Included tag</v>
+        <v>Upsell Feature 1</v>
       </c>
       <c r="C31" t="str">
-        <v>N/A</v>
+        <v>{{UPSELL_FEATURE_1}}</v>
       </c>
       <c r="D31" t="str">
         <v/>
@@ -3067,7 +3067,7 @@
         <v>variant1</v>
       </c>
       <c r="B32" t="str">
-        <v>Included PPV2 Name</v>
+        <v>Upsell Highlight Text</v>
       </c>
       <c r="C32" t="str">
         <v>N/A</v>
@@ -3081,10 +3081,10 @@
         <v>variant1</v>
       </c>
       <c r="B33" t="str">
-        <v>PPV2 Image Present on ultimate tier</v>
+        <v>Upsell Feature 2</v>
       </c>
       <c r="C33" t="str">
-        <v>N/A</v>
+        <v>{{UPSELL_FEATURE_2}}</v>
       </c>
       <c r="D33" t="str">
         <v/>
@@ -3095,10 +3095,10 @@
         <v>variant1</v>
       </c>
       <c r="B34" t="str">
-        <v>PPV2 Date Text on ultimate tier</v>
+        <v>Upsell Feature 3</v>
       </c>
       <c r="C34" t="str">
-        <v>N/A</v>
+        <v>{{UPSELL_FEATURE_3}}</v>
       </c>
       <c r="D34" t="str">
         <v/>
@@ -3109,7 +3109,7 @@
         <v>variant1</v>
       </c>
       <c r="B35" t="str">
-        <v>PPV2 Included tag</v>
+        <v>Whats Included CTA</v>
       </c>
       <c r="C35" t="str">
         <v>N/A</v>
@@ -3123,10 +3123,10 @@
         <v>variant1</v>
       </c>
       <c r="B36" t="str">
-        <v>Upsell Feature 1</v>
+        <v>Gold Highlight 1</v>
       </c>
       <c r="C36" t="str">
-        <v>{{UPSELL_FEATURE_1}}</v>
+        <v>N/A</v>
       </c>
       <c r="D36" t="str">
         <v/>
@@ -3137,7 +3137,7 @@
         <v>variant1</v>
       </c>
       <c r="B37" t="str">
-        <v>Upsell Highlight Text</v>
+        <v>Gold Highlight 2</v>
       </c>
       <c r="C37" t="str">
         <v>N/A</v>
@@ -3151,10 +3151,10 @@
         <v>variant1</v>
       </c>
       <c r="B38" t="str">
-        <v>Upsell Feature 2</v>
+        <v>Gold Highlight 3</v>
       </c>
       <c r="C38" t="str">
-        <v>{{UPSELL_FEATURE_2}}</v>
+        <v>N/A</v>
       </c>
       <c r="D38" t="str">
         <v/>
@@ -3165,13 +3165,13 @@
         <v>variant1</v>
       </c>
       <c r="B39" t="str">
-        <v>Upsell Feature 3</v>
+        <v>Bundle Name</v>
       </c>
       <c r="C39" t="str">
-        <v>{{UPSELL_FEATURE_3}}</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="D39" t="str">
-        <v/>
+        <v>bundle</v>
       </c>
     </row>
     <row r="40">
@@ -3179,13 +3179,13 @@
         <v>variant1</v>
       </c>
       <c r="B40" t="str">
-        <v>Whats Included CTA</v>
+        <v>Bundle Description</v>
       </c>
       <c r="C40" t="str">
-        <v>N/A</v>
+        <v>{{BUNDLE_DESCRIPTION}}</v>
       </c>
       <c r="D40" t="str">
-        <v/>
+        <v>bundle</v>
       </c>
     </row>
     <row r="41">
@@ -3193,13 +3193,13 @@
         <v>variant1</v>
       </c>
       <c r="B41" t="str">
-        <v>Gold Highlight 1</v>
+        <v>Bundle Monthly Price</v>
       </c>
       <c r="C41" t="str">
-        <v>N/A</v>
+        <v>{{BUNDLE_MONTHLY_PRICE}}</v>
       </c>
       <c r="D41" t="str">
-        <v/>
+        <v>bundle</v>
       </c>
     </row>
     <row r="42">
@@ -3207,13 +3207,13 @@
         <v>variant1</v>
       </c>
       <c r="B42" t="str">
-        <v>Gold Highlight 2</v>
+        <v>Bundle Price</v>
       </c>
       <c r="C42" t="str">
-        <v>N/A</v>
+        <v>{{BUNDLE_PRICE}}</v>
       </c>
       <c r="D42" t="str">
-        <v/>
+        <v>bundle</v>
       </c>
     </row>
     <row r="43">
@@ -3221,13 +3221,13 @@
         <v>variant1</v>
       </c>
       <c r="B43" t="str">
-        <v>Gold Highlight 3</v>
+        <v>Bundle Original Price</v>
       </c>
       <c r="C43" t="str">
-        <v>N/A</v>
+        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
       </c>
       <c r="D43" t="str">
-        <v/>
+        <v>bundle</v>
       </c>
     </row>
     <row r="44">
@@ -3235,10 +3235,10 @@
         <v>variant1</v>
       </c>
       <c r="B44" t="str">
-        <v>Bundle Name</v>
+        <v>Bundle Fight Count</v>
       </c>
       <c r="C44" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>{{BUNDLE_FIGHT_COUNT}}</v>
       </c>
       <c r="D44" t="str">
         <v>bundle</v>
@@ -3249,10 +3249,10 @@
         <v>variant1</v>
       </c>
       <c r="B45" t="str">
-        <v>Bundle Description</v>
+        <v>Bundle Save Badge</v>
       </c>
       <c r="C45" t="str">
-        <v>{{BUNDLE_DESCRIPTION}}</v>
+        <v>{{BUNDLE_SAVE_BADGE}}</v>
       </c>
       <c r="D45" t="str">
         <v>bundle</v>
@@ -3263,10 +3263,10 @@
         <v>variant1</v>
       </c>
       <c r="B46" t="str">
-        <v>Bundle Monthly Price</v>
+        <v>Bundle PPV 1 Full Name</v>
       </c>
       <c r="C46" t="str">
-        <v>{{BUNDLE_MONTHLY_PRICE}}</v>
+        <v>{{BUNDLE_PPV1_FULL_NAME}}</v>
       </c>
       <c r="D46" t="str">
         <v>bundle</v>
@@ -3277,10 +3277,10 @@
         <v>variant1</v>
       </c>
       <c r="B47" t="str">
-        <v>Bundle Price</v>
+        <v>Bundle PPV 1 Date</v>
       </c>
       <c r="C47" t="str">
-        <v>{{BUNDLE_PRICE}}</v>
+        <v>{{BUNDLE_PPV1_DATE}}</v>
       </c>
       <c r="D47" t="str">
         <v>bundle</v>
@@ -3291,10 +3291,10 @@
         <v>variant1</v>
       </c>
       <c r="B48" t="str">
-        <v>Bundle Original Price</v>
+        <v>Bundle PPV 1 Image</v>
       </c>
       <c r="C48" t="str">
-        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
+        <v>Yes</v>
       </c>
       <c r="D48" t="str">
         <v>bundle</v>
@@ -3305,10 +3305,10 @@
         <v>variant1</v>
       </c>
       <c r="B49" t="str">
-        <v>Bundle Fight Count</v>
+        <v>Bundle PPV 2 Full Name</v>
       </c>
       <c r="C49" t="str">
-        <v>{{BUNDLE_FIGHT_COUNT}}</v>
+        <v>{{BUNDLE_PPV2_FULL_NAME}}</v>
       </c>
       <c r="D49" t="str">
         <v>bundle</v>
@@ -3319,10 +3319,10 @@
         <v>variant1</v>
       </c>
       <c r="B50" t="str">
-        <v>Bundle Save Badge</v>
+        <v>Bundle PPV 2 Date</v>
       </c>
       <c r="C50" t="str">
-        <v>{{BUNDLE_SAVE_BADGE}}</v>
+        <v>{{BUNDLE_PPV2_DATE}}</v>
       </c>
       <c r="D50" t="str">
         <v>bundle</v>
@@ -3333,10 +3333,10 @@
         <v>variant1</v>
       </c>
       <c r="B51" t="str">
-        <v>Bundle PPV 1 Full Name</v>
+        <v>Bundle PPV 2 Image</v>
       </c>
       <c r="C51" t="str">
-        <v>{{BUNDLE_PPV1_FULL_NAME}}</v>
+        <v>Yes</v>
       </c>
       <c r="D51" t="str">
         <v>bundle</v>
@@ -3347,13 +3347,13 @@
         <v>variant1</v>
       </c>
       <c r="B52" t="str">
-        <v>Bundle PPV 1 Date</v>
+        <v>CTA Button</v>
       </c>
       <c r="C52" t="str">
-        <v>{{BUNDLE_PPV1_DATE}}</v>
+        <v>{{PPV_CTA_TEXT}}</v>
       </c>
       <c r="D52" t="str">
-        <v>bundle</v>
+        <v/>
       </c>
     </row>
     <row r="53">
@@ -3361,66 +3361,66 @@
         <v>variant1</v>
       </c>
       <c r="B53" t="str">
-        <v>Bundle PPV 1 Image</v>
+        <v>CTA Without PPV</v>
       </c>
       <c r="C53" t="str">
-        <v>Yes</v>
+        <v>Subscribe without a pay-per-view</v>
       </c>
       <c r="D53" t="str">
-        <v>bundle</v>
+        <v>newuser</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>variant1</v>
+        <v>variant2</v>
       </c>
       <c r="B54" t="str">
-        <v>Bundle PPV 2 Full Name</v>
+        <v>Page Title</v>
       </c>
       <c r="C54" t="str">
-        <v>{{BUNDLE_PPV2_FULL_NAME}}</v>
+        <v>Choose your plan</v>
       </c>
       <c r="D54" t="str">
-        <v>bundle</v>
+        <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>variant1</v>
+        <v>variant2</v>
       </c>
       <c r="B55" t="str">
-        <v>Bundle PPV 2 Date</v>
+        <v>Header Full Copy</v>
       </c>
       <c r="C55" t="str">
-        <v>{{BUNDLE_PPV2_DATE}}</v>
+        <v>Buy {{PPV_NAME}} with DAZN Standard or get it included in DAZN Ultimate.</v>
       </c>
       <c r="D55" t="str">
-        <v>bundle</v>
+        <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>variant1</v>
+        <v>variant2</v>
       </c>
       <c r="B56" t="str">
-        <v>Bundle PPV 2 Image</v>
+        <v>Header Highlight Text2</v>
       </c>
       <c r="C56" t="str">
-        <v>Yes</v>
+        <v>get it included in DAZN Ultimate.</v>
       </c>
       <c r="D56" t="str">
-        <v>bundle</v>
+        <v/>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>variant1</v>
+        <v>variant2</v>
       </c>
       <c r="B57" t="str">
-        <v>CTA Button</v>
+        <v>PPV Image</v>
       </c>
       <c r="C57" t="str">
-        <v>{{PPV_CTA_TEXT}}</v>
+        <v>Yes</v>
       </c>
       <c r="D57" t="str">
         <v/>
@@ -3428,16 +3428,16 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>variant1</v>
+        <v>variant2</v>
       </c>
       <c r="B58" t="str">
-        <v>CTA Without PPV</v>
+        <v>Event Date and Time</v>
       </c>
       <c r="C58" t="str">
-        <v>Subscribe without a pay-per-view</v>
+        <v>{{PPV_DATE}}</v>
       </c>
       <c r="D58" t="str">
-        <v>newuser</v>
+        <v/>
       </c>
     </row>
     <row r="59">
@@ -3445,10 +3445,10 @@
         <v>variant2</v>
       </c>
       <c r="B59" t="str">
-        <v>Page Title</v>
+        <v>Event Name</v>
       </c>
       <c r="C59" t="str">
-        <v>Choose your plan</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="D59" t="str">
         <v/>
@@ -3459,10 +3459,10 @@
         <v>variant2</v>
       </c>
       <c r="B60" t="str">
-        <v>Header Full Copy</v>
+        <v>PPV Checkbox Present</v>
       </c>
       <c r="C60" t="str">
-        <v>Buy {{PPV_NAME}} with DAZN Standard or get it included in DAZN Ultimate.</v>
+        <v>Yes</v>
       </c>
       <c r="D60" t="str">
         <v/>
@@ -3473,10 +3473,10 @@
         <v>variant2</v>
       </c>
       <c r="B61" t="str">
-        <v>Header Highlight Text1</v>
+        <v>PPV Selected</v>
       </c>
       <c r="C61" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>Yes</v>
       </c>
       <c r="D61" t="str">
         <v/>
@@ -3487,10 +3487,10 @@
         <v>variant2</v>
       </c>
       <c r="B62" t="str">
-        <v>Header Highlight Text2</v>
+        <v>PPV Name</v>
       </c>
       <c r="C62" t="str">
-        <v>get it included in DAZN Ultimate.</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="D62" t="str">
         <v/>
@@ -3501,10 +3501,10 @@
         <v>variant2</v>
       </c>
       <c r="B63" t="str">
-        <v>PPV Image</v>
+        <v>PPV Per Fight Text</v>
       </c>
       <c r="C63" t="str">
-        <v>Yes</v>
+        <v>/fight</v>
       </c>
       <c r="D63" t="str">
         <v/>
@@ -3515,10 +3515,10 @@
         <v>variant2</v>
       </c>
       <c r="B64" t="str">
-        <v>Event Date and Time</v>
+        <v>PPV Price</v>
       </c>
       <c r="C64" t="str">
-        <v>{{PPV_DATE}}</v>
+        <v>{{PPV_PRICE}}</v>
       </c>
       <c r="D64" t="str">
         <v/>
@@ -3529,10 +3529,10 @@
         <v>variant2</v>
       </c>
       <c r="B65" t="str">
-        <v>Event Name</v>
+        <v>Currency</v>
       </c>
       <c r="C65" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>{{CURRENCY}}</v>
       </c>
       <c r="D65" t="str">
         <v/>
@@ -3543,10 +3543,10 @@
         <v>variant2</v>
       </c>
       <c r="B66" t="str">
-        <v>PPV Checkbox Present</v>
+        <v>Subscription Section Title</v>
       </c>
       <c r="C66" t="str">
-        <v>Yes</v>
+        <v>Choose your subscription</v>
       </c>
       <c r="D66" t="str">
         <v/>
@@ -3557,7 +3557,7 @@
         <v>variant2</v>
       </c>
       <c r="B67" t="str">
-        <v>PPV Selected</v>
+        <v>Trial Card Present</v>
       </c>
       <c r="C67" t="str">
         <v>Yes</v>
@@ -3571,10 +3571,10 @@
         <v>variant2</v>
       </c>
       <c r="B68" t="str">
-        <v>PPV Name</v>
+        <v>Trial Title</v>
       </c>
       <c r="C68" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>7-day free trial of DAZN Standard</v>
       </c>
       <c r="D68" t="str">
         <v/>
@@ -3585,10 +3585,10 @@
         <v>variant2</v>
       </c>
       <c r="B69" t="str">
-        <v>PPV Price</v>
+        <v>Trial Radio Present</v>
       </c>
       <c r="C69" t="str">
-        <v>{{PPV_PRICE}}</v>
+        <v>Yes</v>
       </c>
       <c r="D69" t="str">
         <v/>
@@ -3599,10 +3599,10 @@
         <v>variant2</v>
       </c>
       <c r="B70" t="str">
-        <v>Currency</v>
+        <v>Trial Selected</v>
       </c>
       <c r="C70" t="str">
-        <v>{{CURRENCY}}</v>
+        <v>Yes</v>
       </c>
       <c r="D70" t="str">
         <v/>
@@ -3613,10 +3613,10 @@
         <v>variant2</v>
       </c>
       <c r="B71" t="str">
-        <v>Subscription Section Title</v>
+        <v>Trial Feature 1</v>
       </c>
       <c r="C71" t="str">
-        <v>Choose your subscription</v>
+        <v>7-days free access to DAZN Standard.</v>
       </c>
       <c r="D71" t="str">
         <v/>
@@ -3627,10 +3627,10 @@
         <v>variant2</v>
       </c>
       <c r="B72" t="str">
-        <v>Trial Card Present</v>
+        <v>Trial Feature 2</v>
       </c>
       <c r="C72" t="str">
-        <v>Yes</v>
+        <v>Cancel anytime during the trial and only pay for the fight. After the trial you move onto a Monthly Flex plan for {{CURRENCY}}{{MONTHLY_PRICE}}/month. You will not lose access to the pay-per-view[s].</v>
       </c>
       <c r="D72" t="str">
         <v/>
@@ -3641,10 +3641,10 @@
         <v>variant2</v>
       </c>
       <c r="B73" t="str">
-        <v>Trial Title</v>
+        <v>Upsell Section Present</v>
       </c>
       <c r="C73" t="str">
-        <v>7-day free trial of DAZN Standard</v>
+        <v>Yes</v>
       </c>
       <c r="D73" t="str">
         <v/>
@@ -3655,10 +3655,10 @@
         <v>variant2</v>
       </c>
       <c r="B74" t="str">
-        <v>Trial Radio Present</v>
+        <v>Upsell Label</v>
       </c>
       <c r="C74" t="str">
-        <v>Yes</v>
+        <v>Pay-per-views included</v>
       </c>
       <c r="D74" t="str">
         <v/>
@@ -3669,10 +3669,10 @@
         <v>variant2</v>
       </c>
       <c r="B75" t="str">
-        <v>Trial Selected</v>
+        <v>Upsell Plan Name</v>
       </c>
       <c r="C75" t="str">
-        <v>Yes</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="D75" t="str">
         <v/>
@@ -3683,10 +3683,10 @@
         <v>variant2</v>
       </c>
       <c r="B76" t="str">
-        <v>Trial Feature 1</v>
+        <v>Upsell Price Text</v>
       </c>
       <c r="C76" t="str">
-        <v>7-days free access to DAZN Standard.</v>
+        <v>From</v>
       </c>
       <c r="D76" t="str">
         <v/>
@@ -3697,10 +3697,10 @@
         <v>variant2</v>
       </c>
       <c r="B77" t="str">
-        <v>Trial Feature 2</v>
+        <v>Upsell Price</v>
       </c>
       <c r="C77" t="str">
-        <v>Cancel anytime during the trial and only pay for the fight. After the trial you move onto a Monthly Flex plan for {{CURRENCY}}{{MONTHLY_PRICE}}/month. You will not lose access to the pay-per-view[s].</v>
+        <v>{{UPSELL_PRICE}}</v>
       </c>
       <c r="D77" t="str">
         <v/>
@@ -3711,10 +3711,10 @@
         <v>variant2</v>
       </c>
       <c r="B78" t="str">
-        <v>Upsell Section Present</v>
+        <v>Upsell Price Length</v>
       </c>
       <c r="C78" t="str">
-        <v>Yes</v>
+        <v>{{UPSELL_PRICE_LENGTH}}</v>
       </c>
       <c r="D78" t="str">
         <v/>
@@ -3725,10 +3725,10 @@
         <v>variant2</v>
       </c>
       <c r="B79" t="str">
-        <v>Upsell Label</v>
+        <v>Upsell Billing Text</v>
       </c>
       <c r="C79" t="str">
-        <v>Pay-per-views included</v>
+        <v>Annual contract. Auto renews.</v>
       </c>
       <c r="D79" t="str">
         <v/>
@@ -3739,10 +3739,10 @@
         <v>variant2</v>
       </c>
       <c r="B80" t="str">
-        <v>Upsell Plan Name</v>
+        <v>PPV1 Included tag</v>
       </c>
       <c r="C80" t="str">
-        <v>DAZN Ultimate</v>
+        <v>Yes</v>
       </c>
       <c r="D80" t="str">
         <v/>
@@ -3753,10 +3753,10 @@
         <v>variant2</v>
       </c>
       <c r="B81" t="str">
-        <v>Upsell Price Text</v>
+        <v>Included PPV2 Name</v>
       </c>
       <c r="C81" t="str">
-        <v>From</v>
+        <v>N/A</v>
       </c>
       <c r="D81" t="str">
         <v/>
@@ -3767,10 +3767,10 @@
         <v>variant2</v>
       </c>
       <c r="B82" t="str">
-        <v>Upsell Price</v>
+        <v>PPV2 Image Present on ultimate tier</v>
       </c>
       <c r="C82" t="str">
-        <v>{{UPSELL_PRICE}}</v>
+        <v>N/A</v>
       </c>
       <c r="D82" t="str">
         <v/>
@@ -3781,10 +3781,10 @@
         <v>variant2</v>
       </c>
       <c r="B83" t="str">
-        <v>Upsell Price Length</v>
+        <v>PPV2 Date Text on ultimate tier</v>
       </c>
       <c r="C83" t="str">
-        <v>{{UPSELL_PRICE_LENGTH}}</v>
+        <v>N/A</v>
       </c>
       <c r="D83" t="str">
         <v/>
@@ -3795,10 +3795,10 @@
         <v>variant2</v>
       </c>
       <c r="B84" t="str">
-        <v>Upsell Billing Text</v>
+        <v>PPV2 Included tag</v>
       </c>
       <c r="C84" t="str">
-        <v>Annual contract. Auto renews.</v>
+        <v>N/A</v>
       </c>
       <c r="D84" t="str">
         <v/>
@@ -3809,10 +3809,10 @@
         <v>variant2</v>
       </c>
       <c r="B85" t="str">
-        <v>Included PPV1 Name</v>
+        <v>Upsell Feature 1</v>
       </c>
       <c r="C85" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>Pay-per-views included at no extra cost. Minimum of 12 events per year including {{PPV_NAME}}.</v>
       </c>
       <c r="D85" t="str">
         <v/>
@@ -3823,10 +3823,10 @@
         <v>variant2</v>
       </c>
       <c r="B86" t="str">
-        <v>PPV1 Image Present on ultimate tier</v>
+        <v>Upsell Highlight Text</v>
       </c>
       <c r="C86" t="str">
-        <v>Yes</v>
+        <v>{{PPV_NAME}}.</v>
       </c>
       <c r="D86" t="str">
         <v/>
@@ -3837,10 +3837,10 @@
         <v>variant2</v>
       </c>
       <c r="B87" t="str">
-        <v>PPV1 Upsell Tile Date</v>
+        <v>Upsell Feature 2</v>
       </c>
       <c r="C87" t="str">
-        <v>{{PPV1_UPSELL_TILE_DATE}}</v>
+        <v>HDR and Dolby 5.1 surround sound on select events.</v>
       </c>
       <c r="D87" t="str">
         <v/>
@@ -3851,10 +3851,10 @@
         <v>variant2</v>
       </c>
       <c r="B88" t="str">
-        <v>PPV1 Included tag</v>
+        <v>Upsell Feature 3</v>
       </c>
       <c r="C88" t="str">
-        <v>Yes</v>
+        <v>185+ fights a year from the best promoters</v>
       </c>
       <c r="D88" t="str">
         <v/>
@@ -3865,10 +3865,10 @@
         <v>variant2</v>
       </c>
       <c r="B89" t="str">
-        <v>Included PPV2 Name</v>
+        <v>Whats Included CTA</v>
       </c>
       <c r="C89" t="str">
-        <v>N/A</v>
+        <v>Whats included</v>
       </c>
       <c r="D89" t="str">
         <v/>
@@ -3879,10 +3879,10 @@
         <v>variant2</v>
       </c>
       <c r="B90" t="str">
-        <v>PPV2 Image Present on ultimate tier</v>
+        <v>Gold Highlight 1</v>
       </c>
       <c r="C90" t="str">
-        <v>N/A</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="D90" t="str">
         <v/>
@@ -3893,10 +3893,10 @@
         <v>variant2</v>
       </c>
       <c r="B91" t="str">
-        <v>PPV2 Date Text on ultimate tier</v>
+        <v>Gold Highlight 2</v>
       </c>
       <c r="C91" t="str">
-        <v>N/A</v>
+        <v>get it included in DAZN Ultimate.</v>
       </c>
       <c r="D91" t="str">
         <v/>
@@ -3907,10 +3907,10 @@
         <v>variant2</v>
       </c>
       <c r="B92" t="str">
-        <v>PPV2 Included tag</v>
+        <v>Gold Highlight 3</v>
       </c>
       <c r="C92" t="str">
-        <v>N/A</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="D92" t="str">
         <v/>
@@ -3921,10 +3921,10 @@
         <v>variant2</v>
       </c>
       <c r="B93" t="str">
-        <v>Upsell Feature 1</v>
+        <v>CTA Button</v>
       </c>
       <c r="C93" t="str">
-        <v>Pay-per-views included at no extra cost. Minimum of 12 events per year including {{PPV_NAME}}.</v>
+        <v>Continue with PPV + 7-day free trial</v>
       </c>
       <c r="D93" t="str">
         <v/>
@@ -3935,130 +3935,18 @@
         <v>variant2</v>
       </c>
       <c r="B94" t="str">
-        <v>Upsell Highlight Text</v>
+        <v>CTA Without PPV</v>
       </c>
       <c r="C94" t="str">
-        <v>{{PPV_NAME}}.</v>
+        <v>N/A</v>
       </c>
       <c r="D94" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="str">
-        <v>variant2</v>
-      </c>
-      <c r="B95" t="str">
-        <v>Upsell Feature 2</v>
-      </c>
-      <c r="C95" t="str">
-        <v>HDR and Dolby 5.1 surround sound on select events.</v>
-      </c>
-      <c r="D95" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="str">
-        <v>variant2</v>
-      </c>
-      <c r="B96" t="str">
-        <v>Upsell Feature 3</v>
-      </c>
-      <c r="C96" t="str">
-        <v>185+ fights a year from the best promoters</v>
-      </c>
-      <c r="D96" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="str">
-        <v>variant2</v>
-      </c>
-      <c r="B97" t="str">
-        <v>Whats Included CTA</v>
-      </c>
-      <c r="C97" t="str">
-        <v>Whats included</v>
-      </c>
-      <c r="D97" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="str">
-        <v>variant2</v>
-      </c>
-      <c r="B98" t="str">
-        <v>Gold Highlight 1</v>
-      </c>
-      <c r="C98" t="str">
-        <v>{{PPV_NAME}}</v>
-      </c>
-      <c r="D98" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="str">
-        <v>variant2</v>
-      </c>
-      <c r="B99" t="str">
-        <v>Gold Highlight 2</v>
-      </c>
-      <c r="C99" t="str">
-        <v>get it included in DAZN Ultimate.</v>
-      </c>
-      <c r="D99" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="str">
-        <v>variant2</v>
-      </c>
-      <c r="B100" t="str">
-        <v>Gold Highlight 3</v>
-      </c>
-      <c r="C100" t="str">
-        <v>DAZN Ultimate</v>
-      </c>
-      <c r="D100" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="str">
-        <v>variant2</v>
-      </c>
-      <c r="B101" t="str">
-        <v>CTA Button</v>
-      </c>
-      <c r="C101" t="str">
-        <v>Continue with PPV + 7-day free trial</v>
-      </c>
-      <c r="D101" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="str">
-        <v>variant2</v>
-      </c>
-      <c r="B102" t="str">
-        <v>CTA Without PPV</v>
-      </c>
-      <c r="C102" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="D102" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D102"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D94"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4600,7 +4488,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E102"/>
+  <dimension ref="A1:E103"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="27.83203125" customWidth="1"/>
@@ -4634,10 +4522,10 @@
         <v>All</v>
       </c>
       <c r="C2" t="str">
-        <v>Header</v>
+        <v>Payment Method Heading</v>
       </c>
       <c r="D2" t="str">
-        <v>Your payment is encrypted and you can change how you pay at any time.</v>
+        <v>Payment method</v>
       </c>
       <c r="E2" t="str">
         <v/>
@@ -4651,10 +4539,10 @@
         <v>All</v>
       </c>
       <c r="C3" t="str">
-        <v>Plan Change CTA</v>
+        <v>Purchase Summary Heading</v>
       </c>
       <c r="D3" t="str">
-        <v>Change</v>
+        <v>Purchase summary</v>
       </c>
       <c r="E3" t="str">
         <v/>
@@ -4668,10 +4556,10 @@
         <v>All</v>
       </c>
       <c r="C4" t="str">
-        <v>Credit &amp; Debit Card Option</v>
+        <v>Plan Change CTA</v>
       </c>
       <c r="D4" t="str">
-        <v>Yes</v>
+        <v>Change</v>
       </c>
       <c r="E4" t="str">
         <v/>
@@ -4685,7 +4573,7 @@
         <v>All</v>
       </c>
       <c r="C5" t="str">
-        <v>PayPal Option</v>
+        <v>Credit &amp; Debit Card Option</v>
       </c>
       <c r="D5" t="str">
         <v>Yes</v>
@@ -4702,7 +4590,7 @@
         <v>All</v>
       </c>
       <c r="C6" t="str">
-        <v>Google Pay Option</v>
+        <v>PayPal Option</v>
       </c>
       <c r="D6" t="str">
         <v>Yes</v>
@@ -4719,13 +4607,13 @@
         <v>All</v>
       </c>
       <c r="C7" t="str">
-        <v>Saved Card Present</v>
+        <v>Google Pay Option</v>
       </c>
       <c r="D7" t="str">
         <v>Yes</v>
       </c>
       <c r="E7" t="str">
-        <v>myaccount</v>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -4736,13 +4624,13 @@
         <v>All</v>
       </c>
       <c r="C8" t="str">
-        <v>Signed In As Text</v>
+        <v>Saved Card Present</v>
       </c>
       <c r="D8" t="str">
-        <v>Signed in as {{FIRST_NAME}} {{LAST_NAME}}</v>
+        <v>Yes</v>
       </c>
       <c r="E8" t="str">
-        <v>returning</v>
+        <v>myaccount</v>
       </c>
     </row>
     <row r="9">
@@ -4753,10 +4641,10 @@
         <v>All</v>
       </c>
       <c r="C9" t="str">
-        <v>Log Out Present</v>
+        <v>Signed In As Text</v>
       </c>
       <c r="D9" t="str">
-        <v>Yes</v>
+        <v>Signed in as {{FIRST_NAME}} {{LAST_NAME}}</v>
       </c>
       <c r="E9" t="str">
         <v>returning</v>
@@ -4770,30 +4658,30 @@
         <v>All</v>
       </c>
       <c r="C10" t="str">
-        <v>Redeem Promo Code CTA</v>
+        <v>Log Out Present</v>
       </c>
       <c r="D10" t="str">
         <v>Yes</v>
       </c>
       <c r="E10" t="str">
-        <v/>
+        <v>returning</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Standard</v>
+        <v>Common</v>
       </c>
       <c r="B11" t="str">
-        <v>Monthly</v>
+        <v>All</v>
       </c>
       <c r="C11" t="str">
-        <v>Page Title</v>
+        <v>Redeem Promo Code CTA</v>
       </c>
       <c r="D11" t="str">
-        <v>{{PAYMENT_PAGE_TITLE}}</v>
+        <v>Yes</v>
       </c>
       <c r="E11" t="str">
-        <v>newuser</v>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -4810,7 +4698,7 @@
         <v>{{PAYMENT_PAGE_TITLE}}</v>
       </c>
       <c r="E12" t="str">
-        <v>myaccount</v>
+        <v>newuser</v>
       </c>
     </row>
     <row r="13">
@@ -4821,13 +4709,13 @@
         <v>Monthly</v>
       </c>
       <c r="C13" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D13" t="str">
-        <v>DAZN Standard</v>
+        <v>{{PAYMENT_PAGE_TITLE}}</v>
       </c>
       <c r="E13" t="str">
-        <v/>
+        <v>myaccount</v>
       </c>
     </row>
     <row r="14">
@@ -4838,10 +4726,10 @@
         <v>Monthly</v>
       </c>
       <c r="C14" t="str">
-        <v>Plan Name</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D14" t="str">
-        <v>{{PAYMENT_PLAN_NAME}}</v>
+        <v>DAZN Standard</v>
       </c>
       <c r="E14" t="str">
         <v/>
@@ -4855,10 +4743,10 @@
         <v>Monthly</v>
       </c>
       <c r="C15" t="str">
-        <v>Plan Subtitle</v>
+        <v>Plan Name</v>
       </c>
       <c r="D15" t="str">
-        <v>{{PAYMENT_FLEX_CANCEL_NOTICE}}</v>
+        <v>{{PAYMENT_PLAN_NAME}}</v>
       </c>
       <c r="E15" t="str">
         <v/>
@@ -4872,10 +4760,10 @@
         <v>Monthly</v>
       </c>
       <c r="C16" t="str">
-        <v>First Month Free Price</v>
+        <v>Plan Subtitle</v>
       </c>
       <c r="D16" t="str">
-        <v>{{CURRENCY}}0</v>
+        <v>{{PAYMENT_FLEX_CANCEL_NOTICE}}</v>
       </c>
       <c r="E16" t="str">
         <v/>
@@ -4889,10 +4777,10 @@
         <v>Monthly</v>
       </c>
       <c r="C17" t="str">
-        <v>First Month Free Text</v>
+        <v>First Month Free Price</v>
       </c>
       <c r="D17" t="str">
-        <v>{{PAYMENT_FREE_TEXT}}</v>
+        <v>{{CURRENCY}}0</v>
       </c>
       <c r="E17" t="str">
         <v/>
@@ -4906,10 +4794,10 @@
         <v>Monthly</v>
       </c>
       <c r="C18" t="str">
-        <v>PPV Name</v>
+        <v>First Month Free Text</v>
       </c>
       <c r="D18" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>{{PAYMENT_FREE_TEXT}}</v>
       </c>
       <c r="E18" t="str">
         <v/>
@@ -4923,10 +4811,10 @@
         <v>Monthly</v>
       </c>
       <c r="C19" t="str">
-        <v>PPV Price</v>
+        <v>PPV Name</v>
       </c>
       <c r="D19" t="str">
-        <v>{{PPV_PRICE}}</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="E19" t="str">
         <v/>
@@ -4940,10 +4828,10 @@
         <v>Monthly</v>
       </c>
       <c r="C20" t="str">
-        <v>Today You Pay Text</v>
+        <v>PPV Price</v>
       </c>
       <c r="D20" t="str">
-        <v>Today you pay</v>
+        <v>{{PPV_PRICE}}</v>
       </c>
       <c r="E20" t="str">
         <v/>
@@ -4957,10 +4845,10 @@
         <v>Monthly</v>
       </c>
       <c r="C21" t="str">
-        <v>Today You Pay Price</v>
+        <v>Today You Pay Text</v>
       </c>
       <c r="D21" t="str">
-        <v>{{PPV_PRICE}}</v>
+        <v>Today you pay</v>
       </c>
       <c r="E21" t="str">
         <v/>
@@ -4974,10 +4862,10 @@
         <v>Monthly</v>
       </c>
       <c r="C22" t="str">
-        <v>Cancellation Text</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D22" t="str">
-        <v>{{CANCELLATION_TEXT}}</v>
+        <v>{{PPV_PRICE}}</v>
       </c>
       <c r="E22" t="str">
         <v/>
@@ -4991,10 +4879,10 @@
         <v>Monthly</v>
       </c>
       <c r="C23" t="str">
-        <v>Legal Text</v>
+        <v>Cancellation Text</v>
       </c>
       <c r="D23" t="str">
-        <v>{{PAYMENT_FLEX_LEGAL_TEXT}}</v>
+        <v>{{CANCELLATION_TEXT}}</v>
       </c>
       <c r="E23" t="str">
         <v/>
@@ -5008,10 +4896,10 @@
         <v>Monthly</v>
       </c>
       <c r="C24" t="str">
-        <v>Ultimate Upsell Text</v>
+        <v>Legal Text</v>
       </c>
       <c r="D24" t="str">
-        <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
+        <v>{{PAYMENT_FLEX_LEGAL_TEXT}}</v>
       </c>
       <c r="E24" t="str">
         <v/>
@@ -5022,13 +4910,13 @@
         <v>Standard</v>
       </c>
       <c r="B25" t="str">
-        <v>Annual Pay Monthly</v>
+        <v>Monthly</v>
       </c>
       <c r="C25" t="str">
-        <v>Page Title</v>
+        <v>Ultimate Upsell Text</v>
       </c>
       <c r="D25" t="str">
-        <v>Choose how to pay</v>
+        <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
       <c r="E25" t="str">
         <v/>
@@ -5042,10 +4930,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C26" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D26" t="str">
-        <v>DAZN Standard</v>
+        <v>Choose how to pay</v>
       </c>
       <c r="E26" t="str">
         <v/>
@@ -5059,10 +4947,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C27" t="str">
-        <v>PPV Name</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D27" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>DAZN Standard</v>
       </c>
       <c r="E27" t="str">
         <v/>
@@ -5076,10 +4964,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C28" t="str">
-        <v>PPV Price</v>
+        <v>PPV Name</v>
       </c>
       <c r="D28" t="str">
-        <v>{{PPV_PRICE}}</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="E28" t="str">
         <v/>
@@ -5093,10 +4981,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C29" t="str">
-        <v>Rate Plan</v>
+        <v>PPV Price</v>
       </c>
       <c r="D29" t="str">
-        <v>{{RATE_PLAN_LABEL}}</v>
+        <v>{{PPV_PRICE}}</v>
       </c>
       <c r="E29" t="str">
         <v/>
@@ -5110,10 +4998,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C30" t="str">
-        <v>Rate Plan Original Price</v>
+        <v>Rate Plan</v>
       </c>
       <c r="D30" t="str">
-        <v>{{CURRENCY}}{{ANNUAL_PRICE}}</v>
+        <v>{{RATE_PLAN_LABEL}}</v>
       </c>
       <c r="E30" t="str">
         <v/>
@@ -5127,10 +5015,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C31" t="str">
-        <v>Rate Plan Discounted Price</v>
+        <v>Rate Plan Original Price</v>
       </c>
       <c r="D31" t="str">
-        <v>{{CURRENCY}}0</v>
+        <v>{{CURRENCY}}{{ANNUAL_PRICE}}</v>
       </c>
       <c r="E31" t="str">
         <v/>
@@ -5144,10 +5032,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C32" t="str">
-        <v>Today You Pay Text</v>
+        <v>Rate Plan Discounted Price</v>
       </c>
       <c r="D32" t="str">
-        <v>Today you pay</v>
+        <v>{{CURRENCY}}0</v>
       </c>
       <c r="E32" t="str">
         <v/>
@@ -5161,10 +5049,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C33" t="str">
-        <v>Today You Pay Price</v>
+        <v>Today You Pay Text</v>
       </c>
       <c r="D33" t="str">
-        <v>{{PPV_PRICE}}</v>
+        <v>Today you pay</v>
       </c>
       <c r="E33" t="str">
         <v/>
@@ -5178,10 +5066,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C34" t="str">
-        <v>Cancellation Text</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D34" t="str">
-        <v>{{CANCELLATION_TEXT_ANNUAL}}</v>
+        <v>{{PPV_PRICE}}</v>
       </c>
       <c r="E34" t="str">
         <v/>
@@ -5195,10 +5083,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C35" t="str">
-        <v>Redeem Promo Code CTA</v>
+        <v>Cancellation Text</v>
       </c>
       <c r="D35" t="str">
-        <v>Yes</v>
+        <v>{{CANCELLATION_TEXT_ANNUAL}}</v>
       </c>
       <c r="E35" t="str">
         <v/>
@@ -5212,10 +5100,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C36" t="str">
-        <v>Ultimate Upsell Text</v>
+        <v>Redeem Promo Code CTA</v>
       </c>
       <c r="D36" t="str">
-        <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
+        <v>Yes</v>
       </c>
       <c r="E36" t="str">
         <v/>
@@ -5223,16 +5111,16 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Ultimate</v>
+        <v>Standard</v>
       </c>
       <c r="B37" t="str">
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C37" t="str">
-        <v>Page Title</v>
+        <v>Ultimate Upsell Text</v>
       </c>
       <c r="D37" t="str">
-        <v>Choose how to pay</v>
+        <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
       <c r="E37" t="str">
         <v/>
@@ -5246,10 +5134,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C38" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D38" t="str">
-        <v>DAZN Ultimate</v>
+        <v>Choose how to pay</v>
       </c>
       <c r="E38" t="str">
         <v/>
@@ -5263,10 +5151,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C39" t="str">
-        <v>PPV Name</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D39" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="E39" t="str">
         <v/>
@@ -5280,10 +5168,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C40" t="str">
-        <v>PPV Price</v>
+        <v>PPV Name</v>
       </c>
       <c r="D40" t="str">
-        <v>{{CURRENCY}}0</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="E40" t="str">
         <v/>
@@ -5297,10 +5185,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C41" t="str">
-        <v>Rate Plan</v>
+        <v>PPV Price</v>
       </c>
       <c r="D41" t="str">
-        <v>Annual - Pay Monthly</v>
+        <v>{{CURRENCY}}0</v>
       </c>
       <c r="E41" t="str">
         <v/>
@@ -5314,10 +5202,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C42" t="str">
-        <v>Rate Plan Price</v>
+        <v>Rate Plan</v>
       </c>
       <c r="D42" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
+        <v>Annual - Pay Monthly</v>
       </c>
       <c r="E42" t="str">
         <v/>
@@ -5331,10 +5219,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C43" t="str">
-        <v>Plan Subtitle</v>
+        <v>Rate Plan Price</v>
       </c>
       <c r="D43" t="str">
-        <v>Billed monthly. 12-month contract.</v>
+        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
       </c>
       <c r="E43" t="str">
         <v/>
@@ -5348,10 +5236,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C44" t="str">
-        <v>Today You Pay Text</v>
+        <v>Plan Subtitle</v>
       </c>
       <c r="D44" t="str">
-        <v>Today you pay</v>
+        <v>Billed monthly. 12-month contract.</v>
       </c>
       <c r="E44" t="str">
         <v/>
@@ -5365,10 +5253,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C45" t="str">
-        <v>Today You Pay Price</v>
+        <v>Today You Pay Text</v>
       </c>
       <c r="D45" t="str">
-        <v>{{TODAY_YOU_PAY_PRICE}}</v>
+        <v>Today you pay</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -5382,10 +5270,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C46" t="str">
-        <v>Next Payment Label</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D46" t="str">
-        <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
+        <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
       <c r="E46" t="str">
         <v/>
@@ -5399,10 +5287,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C47" t="str">
-        <v>Next Payment Price</v>
+        <v>Next Payment Label</v>
       </c>
       <c r="D47" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
+        <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
       <c r="E47" t="str">
         <v/>
@@ -5416,10 +5304,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C48" t="str">
-        <v>Cancellation Text</v>
+        <v>Next Payment Price</v>
       </c>
       <c r="D48" t="str">
-        <v>{{CANCELLATION_TEXT}}</v>
+        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
       </c>
       <c r="E48" t="str">
         <v/>
@@ -5433,10 +5321,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C49" t="str">
-        <v>Redeem Promo Code CTA</v>
+        <v>Cancellation Text</v>
       </c>
       <c r="D49" t="str">
-        <v>Yes</v>
+        <v>{{CANCELLATION_TEXT}}</v>
       </c>
       <c r="E49" t="str">
         <v/>
@@ -5450,10 +5338,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C50" t="str">
-        <v>Discount Badge</v>
+        <v>Redeem Promo Code CTA</v>
       </c>
       <c r="D50" t="str">
-        <v>{{DISCOUNT_BADGE}}</v>
+        <v>Yes</v>
       </c>
       <c r="E50" t="str">
         <v/>
@@ -5464,13 +5352,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B51" t="str">
-        <v>Annual Pay Upfront</v>
+        <v>Annual Pay Monthly</v>
       </c>
       <c r="C51" t="str">
-        <v>Page Title</v>
+        <v>Discount Badge</v>
       </c>
       <c r="D51" t="str">
-        <v>Choose how to pay</v>
+        <v>{{DISCOUNT_BADGE}}</v>
       </c>
       <c r="E51" t="str">
         <v/>
@@ -5484,10 +5372,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C52" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D52" t="str">
-        <v>DAZN Ultimate</v>
+        <v>Choose how to pay</v>
       </c>
       <c r="E52" t="str">
         <v/>
@@ -5501,10 +5389,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C53" t="str">
-        <v>PPV Name</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D53" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="E53" t="str">
         <v/>
@@ -5518,10 +5406,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C54" t="str">
-        <v>PPV Price</v>
+        <v>PPV Name</v>
       </c>
       <c r="D54" t="str">
-        <v>{{CURRENCY}}0</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="E54" t="str">
         <v/>
@@ -5535,10 +5423,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C55" t="str">
-        <v>Rate Plan</v>
+        <v>PPV Price</v>
       </c>
       <c r="D55" t="str">
-        <v>Annual - Pay Upfront</v>
+        <v>{{CURRENCY}}0</v>
       </c>
       <c r="E55" t="str">
         <v/>
@@ -5552,10 +5440,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C56" t="str">
-        <v>Rate Plan Price</v>
+        <v>Rate Plan</v>
       </c>
       <c r="D56" t="str">
-        <v>{{ANNUAL_UPFRONT_PRICE}}/year</v>
+        <v>Annual - Pay Upfront</v>
       </c>
       <c r="E56" t="str">
         <v/>
@@ -5569,10 +5457,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C57" t="str">
-        <v>Plan Subtitle</v>
+        <v>Rate Plan Price</v>
       </c>
       <c r="D57" t="str">
-        <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}. Pay for the full year up front|Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
+        <v>{{ANNUAL_UPFRONT_PRICE}}/year</v>
       </c>
       <c r="E57" t="str">
         <v/>
@@ -5586,10 +5474,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C58" t="str">
-        <v>Today You Pay Text</v>
+        <v>Plan Subtitle</v>
       </c>
       <c r="D58" t="str">
-        <v>Today you pay</v>
+        <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}. Pay for the full year up front|Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
       </c>
       <c r="E58" t="str">
         <v/>
@@ -5603,10 +5491,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C59" t="str">
-        <v>Today You Pay Price</v>
+        <v>Today You Pay Text</v>
       </c>
       <c r="D59" t="str">
-        <v>{{TODAY_YOU_PAY_PRICE}}</v>
+        <v>Today you pay</v>
       </c>
       <c r="E59" t="str">
         <v/>
@@ -5620,10 +5508,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C60" t="str">
-        <v>Next Payment Label</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D60" t="str">
-        <v>Next Annual payment on {{NEXT_PAYMENT_DATE}}</v>
+        <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
       <c r="E60" t="str">
         <v/>
@@ -5637,10 +5525,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C61" t="str">
-        <v>Next Payment Price</v>
+        <v>Next Payment Label</v>
       </c>
       <c r="D61" t="str">
-        <v>{{ANNUAL_UPFRONT_PRICE}}</v>
+        <v>Next Annual payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
       <c r="E61" t="str">
         <v/>
@@ -5654,10 +5542,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C62" t="str">
-        <v>Cancellation Text</v>
+        <v>Next Payment Price</v>
       </c>
       <c r="D62" t="str">
-        <v>{{CANCELLATION_TEXT}}</v>
+        <v>{{ANNUAL_UPFRONT_PRICE}}</v>
       </c>
       <c r="E62" t="str">
         <v/>
@@ -5671,10 +5559,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C63" t="str">
-        <v>Redeem Promo Code CTA</v>
+        <v>Cancellation Text</v>
       </c>
       <c r="D63" t="str">
-        <v>Yes</v>
+        <v>{{CANCELLATION_TEXT}}</v>
       </c>
       <c r="E63" t="str">
         <v/>
@@ -5682,16 +5570,16 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Standard</v>
+        <v>Ultimate</v>
       </c>
       <c r="B64" t="str">
-        <v>Monthly Bundle</v>
+        <v>Annual Pay Upfront</v>
       </c>
       <c r="C64" t="str">
-        <v>Page Title</v>
+        <v>Redeem Promo Code CTA</v>
       </c>
       <c r="D64" t="str">
-        <v>{{PAYMENT_PAGE_TITLE}}</v>
+        <v>Yes</v>
       </c>
       <c r="E64" t="str">
         <v/>
@@ -5705,10 +5593,10 @@
         <v>Monthly Bundle</v>
       </c>
       <c r="C65" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D65" t="str">
-        <v>DAZN Standard</v>
+        <v>{{PAYMENT_PAGE_TITLE}}</v>
       </c>
       <c r="E65" t="str">
         <v/>
@@ -5722,10 +5610,10 @@
         <v>Monthly Bundle</v>
       </c>
       <c r="C66" t="str">
-        <v>Bundle Name</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D66" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>DAZN Standard</v>
       </c>
       <c r="E66" t="str">
         <v/>
@@ -5739,10 +5627,10 @@
         <v>Monthly Bundle</v>
       </c>
       <c r="C67" t="str">
-        <v>Bundle Price</v>
+        <v>Bundle Name</v>
       </c>
       <c r="D67" t="str">
-        <v>{{BUNDLE_PRICE}}</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="E67" t="str">
         <v/>
@@ -5756,10 +5644,10 @@
         <v>Monthly Bundle</v>
       </c>
       <c r="C68" t="str">
-        <v>Today You Pay Price</v>
+        <v>Bundle Price</v>
       </c>
       <c r="D68" t="str">
-        <v>{{BUNDLE_TODAY_YOU_PAY_STANDARD}}</v>
+        <v>{{BUNDLE_PRICE}}</v>
       </c>
       <c r="E68" t="str">
         <v/>
@@ -5773,10 +5661,10 @@
         <v>Monthly Bundle</v>
       </c>
       <c r="C69" t="str">
-        <v>Cancellation Text</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D69" t="str">
-        <v>{{CANCELLATION_TEXT}}</v>
+        <v>{{BUNDLE_TODAY_YOU_PAY_STANDARD}}</v>
       </c>
       <c r="E69" t="str">
         <v/>
@@ -5787,13 +5675,13 @@
         <v>Standard</v>
       </c>
       <c r="B70" t="str">
-        <v>Annual Pay Monthly Bundle</v>
+        <v>Monthly Bundle</v>
       </c>
       <c r="C70" t="str">
-        <v>Page Title</v>
+        <v>Cancellation Text</v>
       </c>
       <c r="D70" t="str">
-        <v>Choose how to pay</v>
+        <v>{{CANCELLATION_TEXT}}</v>
       </c>
       <c r="E70" t="str">
         <v/>
@@ -5807,10 +5695,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C71" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D71" t="str">
-        <v>DAZN Standard</v>
+        <v>Choose how to pay</v>
       </c>
       <c r="E71" t="str">
         <v/>
@@ -5824,10 +5712,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C72" t="str">
-        <v>Rate Plan</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D72" t="str">
-        <v>Annual - Pay Monthly</v>
+        <v>DAZN Standard</v>
       </c>
       <c r="E72" t="str">
         <v/>
@@ -5841,10 +5729,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C73" t="str">
-        <v>First Month Free Text</v>
+        <v>Rate Plan</v>
       </c>
       <c r="D73" t="str">
-        <v>First month free</v>
+        <v>Annual - Pay Monthly</v>
       </c>
       <c r="E73" t="str">
         <v/>
@@ -5858,10 +5746,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C74" t="str">
-        <v>Bundle Name</v>
+        <v>First Month Free Text</v>
       </c>
       <c r="D74" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>First month free</v>
       </c>
       <c r="E74" t="str">
         <v/>
@@ -5875,10 +5763,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C75" t="str">
-        <v>Bundle Original Price</v>
+        <v>Bundle Name</v>
       </c>
       <c r="D75" t="str">
-        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="E75" t="str">
         <v/>
@@ -5892,10 +5780,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C76" t="str">
-        <v>Bundle Price</v>
+        <v>Bundle Original Price</v>
       </c>
       <c r="D76" t="str">
-        <v>{{BUNDLE_PRICE}}</v>
+        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
       </c>
       <c r="E76" t="str">
         <v/>
@@ -5909,10 +5797,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C77" t="str">
-        <v>Bundle Discount</v>
+        <v>Bundle Price</v>
       </c>
       <c r="D77" t="str">
-        <v>{{BUNDLE_DISCOUNT}}</v>
+        <v>{{BUNDLE_PRICE}}</v>
       </c>
       <c r="E77" t="str">
         <v/>
@@ -5926,10 +5814,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C78" t="str">
-        <v>Today You Pay Price</v>
+        <v>Bundle Discount</v>
       </c>
       <c r="D78" t="str">
-        <v>{{BUNDLE_TODAY_YOU_PAY_STANDARD}}</v>
+        <v>{{BUNDLE_DISCOUNT}}</v>
       </c>
       <c r="E78" t="str">
         <v/>
@@ -5943,10 +5831,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C79" t="str">
-        <v>Cancellation Text</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D79" t="str">
-        <v>{{CANCELLATION_TEXT_ANNUAL}}</v>
+        <v>{{BUNDLE_TODAY_YOU_PAY_STANDARD}}</v>
       </c>
       <c r="E79" t="str">
         <v/>
@@ -5960,10 +5848,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C80" t="str">
-        <v>Ultimate Upsell Text</v>
+        <v>Cancellation Text</v>
       </c>
       <c r="D80" t="str">
-        <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
+        <v>{{CANCELLATION_TEXT_ANNUAL}}</v>
       </c>
       <c r="E80" t="str">
         <v/>
@@ -5971,16 +5859,16 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>Ultimate</v>
+        <v>Standard</v>
       </c>
       <c r="B81" t="str">
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C81" t="str">
-        <v>Page Title</v>
+        <v>Ultimate Upsell Text</v>
       </c>
       <c r="D81" t="str">
-        <v>Choose how to pay</v>
+        <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
       <c r="E81" t="str">
         <v/>
@@ -5994,10 +5882,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C82" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D82" t="str">
-        <v>DAZN Ultimate</v>
+        <v>Choose how to pay</v>
       </c>
       <c r="E82" t="str">
         <v/>
@@ -6011,10 +5899,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C83" t="str">
-        <v>Rate Plan</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D83" t="str">
-        <v>Annual - Pay Monthly</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="E83" t="str">
         <v/>
@@ -6028,10 +5916,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C84" t="str">
-        <v>Rate Plan Price</v>
+        <v>Rate Plan</v>
       </c>
       <c r="D84" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
+        <v>Annual - Pay Monthly</v>
       </c>
       <c r="E84" t="str">
         <v/>
@@ -6045,10 +5933,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C85" t="str">
-        <v>Bundle Name</v>
+        <v>Rate Plan Price</v>
       </c>
       <c r="D85" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
       </c>
       <c r="E85" t="str">
         <v/>
@@ -6062,10 +5950,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C86" t="str">
-        <v>Bundle Price</v>
+        <v>Bundle Name</v>
       </c>
       <c r="D86" t="str">
-        <v>{{CURRENCY}}0</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="E86" t="str">
         <v/>
@@ -6079,10 +5967,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C87" t="str">
-        <v>Today You Pay Price</v>
+        <v>Bundle Price</v>
       </c>
       <c r="D87" t="str">
-        <v>{{TODAY_YOU_PAY_PRICE}}</v>
+        <v>{{CURRENCY}}0</v>
       </c>
       <c r="E87" t="str">
         <v/>
@@ -6096,10 +5984,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C88" t="str">
-        <v>Next Payment Label</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D88" t="str">
-        <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
+        <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
       <c r="E88" t="str">
         <v/>
@@ -6113,10 +6001,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C89" t="str">
-        <v>Next Payment Price</v>
+        <v>Next Payment Label</v>
       </c>
       <c r="D89" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
+        <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
       <c r="E89" t="str">
         <v/>
@@ -6130,10 +6018,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C90" t="str">
-        <v>Cancellation Text</v>
+        <v>Next Payment Price</v>
       </c>
       <c r="D90" t="str">
-        <v>{{CANCELLATION_TEXT}}</v>
+        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
       </c>
       <c r="E90" t="str">
         <v/>
@@ -6147,10 +6035,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C91" t="str">
-        <v>Discount Badge</v>
+        <v>Cancellation Text</v>
       </c>
       <c r="D91" t="str">
-        <v>{{DISCOUNT_BADGE}}</v>
+        <v>{{CANCELLATION_TEXT}}</v>
       </c>
       <c r="E91" t="str">
         <v/>
@@ -6161,13 +6049,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B92" t="str">
-        <v>Annual Pay Upfront Bundle</v>
+        <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C92" t="str">
-        <v>Page Title</v>
+        <v>Discount Badge</v>
       </c>
       <c r="D92" t="str">
-        <v>Choose how to pay</v>
+        <v>{{DISCOUNT_BADGE}}</v>
       </c>
       <c r="E92" t="str">
         <v/>
@@ -6181,10 +6069,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C93" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D93" t="str">
-        <v>DAZN Ultimate</v>
+        <v>Choose how to pay</v>
       </c>
       <c r="E93" t="str">
         <v/>
@@ -6198,10 +6086,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C94" t="str">
-        <v>Rate Plan</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D94" t="str">
-        <v>Annual - Pay Upfront</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="E94" t="str">
         <v/>
@@ -6215,10 +6103,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C95" t="str">
-        <v>Rate Plan Price</v>
+        <v>Rate Plan</v>
       </c>
       <c r="D95" t="str">
-        <v>{{ANNUAL_UPFRONT_PRICE}}/year</v>
+        <v>Annual - Pay Upfront</v>
       </c>
       <c r="E95" t="str">
         <v/>
@@ -6232,10 +6120,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C96" t="str">
-        <v>Save Badge</v>
+        <v>Rate Plan Price</v>
       </c>
       <c r="D96" t="str">
-        <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
+        <v>{{ANNUAL_UPFRONT_PRICE}}/year</v>
       </c>
       <c r="E96" t="str">
         <v/>
@@ -6249,10 +6137,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C97" t="str">
-        <v>Bundle Name</v>
+        <v>Save Badge</v>
       </c>
       <c r="D97" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
       </c>
       <c r="E97" t="str">
         <v/>
@@ -6266,10 +6154,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C98" t="str">
-        <v>Bundle Price</v>
+        <v>Bundle Name</v>
       </c>
       <c r="D98" t="str">
-        <v>{{CURRENCY}}0</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="E98" t="str">
         <v/>
@@ -6283,10 +6171,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C99" t="str">
-        <v>Today You Pay Price</v>
+        <v>Bundle Price</v>
       </c>
       <c r="D99" t="str">
-        <v>{{ANNUAL_UPFRONT_PRICE}}</v>
+        <v>{{CURRENCY}}0</v>
       </c>
       <c r="E99" t="str">
         <v/>
@@ -6300,10 +6188,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C100" t="str">
-        <v>Next Payment Label</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D100" t="str">
-        <v>Next Annual payment on {{NEXT_PAYMENT_DATE}}</v>
+        <v>{{ANNUAL_UPFRONT_PRICE}}</v>
       </c>
       <c r="E100" t="str">
         <v/>
@@ -6317,10 +6205,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C101" t="str">
-        <v>Next Payment Price</v>
+        <v>Next Payment Label</v>
       </c>
       <c r="D101" t="str">
-        <v>{{ANNUAL_UPFRONT_PRICE}}</v>
+        <v>Next Annual payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
       <c r="E101" t="str">
         <v/>
@@ -6334,18 +6222,35 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C102" t="str">
+        <v>Next Payment Price</v>
+      </c>
+      <c r="D102" t="str">
+        <v>{{ANNUAL_UPFRONT_PRICE}}</v>
+      </c>
+      <c r="E102" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>Ultimate</v>
+      </c>
+      <c r="B103" t="str">
+        <v>Annual Pay Upfront Bundle</v>
+      </c>
+      <c r="C103" t="str">
         <v>Cancellation Text</v>
       </c>
-      <c r="D102" t="str">
+      <c r="D103" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
-      <c r="E102" t="str">
+      <c r="E103" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E102"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E103"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: add myaccount subscription status flow and popup dismissal fixes
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -515,7 +515,7 @@
         <v>Banner - Event Description</v>
       </c>
       <c r="B9" t="str">
-        <v>{{PPV_DESCRIPTION}}</v>
+        <v>{{BANNER_DESCRIPTION}}</v>
       </c>
       <c r="C9" t="str">
         <v>landing-page-banner</v>
@@ -1006,7 +1006,7 @@
         <v>Banner - Event Description</v>
       </c>
       <c r="C5" t="str">
-        <v>{{PPV_DESCRIPTION}}</v>
+        <v>{{BANNER_DESCRIPTION}}</v>
       </c>
     </row>
     <row r="6">
@@ -1165,7 +1165,7 @@
         <v>Banner - Event Description</v>
       </c>
       <c r="C4" t="str">
-        <v>{{PPV_DESCRIPTION}}</v>
+        <v>{{BANNER_DESCRIPTION}}</v>
       </c>
     </row>
     <row r="5">
@@ -2121,7 +2121,7 @@
         <v>PPV Name</v>
       </c>
       <c r="B11" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>{{PPV_DISPLAY_NAME}}</v>
       </c>
       <c r="C11" t="str">
         <v>boxing-upcoming</v>
@@ -2692,7 +2692,7 @@
         <v>Event Name</v>
       </c>
       <c r="C5" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>{{PPV_DISPLAY_NAME}}</v>
       </c>
       <c r="D5" t="str">
         <v/>
@@ -2818,7 +2818,7 @@
         <v>PPV Card Title</v>
       </c>
       <c r="C14" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>{{PPV_DISPLAY_NAME}}</v>
       </c>
       <c r="D14" t="str">
         <v/>
@@ -3448,7 +3448,7 @@
         <v>Event Name</v>
       </c>
       <c r="C59" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>{{PPV_DISPLAY_NAME}}</v>
       </c>
       <c r="D59" t="str">
         <v/>
@@ -3490,7 +3490,7 @@
         <v>PPV Name</v>
       </c>
       <c r="C62" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>{{PPV_DISPLAY_NAME}}</v>
       </c>
       <c r="D62" t="str">
         <v/>
@@ -4305,7 +4305,7 @@
         <v>Annual Pay Monthly Price Length</v>
       </c>
       <c r="C25" t="str">
-        <v>/ month</v>
+        <v>/month</v>
       </c>
       <c r="D25" t="str">
         <v/>

</xml_diff>

<commit_message>
fix: home-page-dont-miss carousel navigation + chevron scope fixes
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -22,6 +22,7 @@
     <sheet name="Upsell Second Success page" sheetId="17" r:id="rId17"/>
     <sheet name="Upsell Payment page" sheetId="18" r:id="rId18"/>
     <sheet name="Search page" sheetId="19" r:id="rId19"/>
+    <sheet name="Paywall" sheetId="20" r:id="rId20"/>
   </sheets>
 </workbook>
 </file>
@@ -947,11 +948,11 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C21"/>
   <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
-    <col min="3" max="3" width="90.83203125" customWidth="1"/>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="32.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1036,7 +1037,7 @@
         <v>home-boxing-tile</v>
       </c>
       <c r="B8" t="str">
-        <v>Best of Boxing Section</v>
+        <v>Home of Boxing Section Present</v>
       </c>
       <c r="C8" t="str">
         <v>Present</v>
@@ -1047,10 +1048,10 @@
         <v>home-boxing-tile</v>
       </c>
       <c r="B9" t="str">
-        <v>Popup - Event Title</v>
+        <v>Selected Boxing Tile</v>
       </c>
       <c r="C9" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="10">
@@ -1058,10 +1059,10 @@
         <v>home-boxing-tile</v>
       </c>
       <c r="B10" t="str">
-        <v>Popup - Event Date</v>
+        <v>Event Title</v>
       </c>
       <c r="C10" t="str">
-        <v>{{PPV_DATE}}</v>
+        <v>{{PPV_NAME}}</v>
       </c>
     </row>
     <row r="11">
@@ -1069,10 +1070,10 @@
         <v>home-boxing-tile</v>
       </c>
       <c r="B11" t="str">
-        <v>Popup - Promoter</v>
+        <v>Event Date</v>
       </c>
       <c r="C11" t="str">
-        <v>{{PPV_PROMOTER}}</v>
+        <v>{{PPV_DATE}}</v>
       </c>
     </row>
     <row r="12">
@@ -1080,10 +1081,10 @@
         <v>home-boxing-tile</v>
       </c>
       <c r="B12" t="str">
-        <v>Popup - Buy Now CTA</v>
+        <v>Promoter</v>
       </c>
       <c r="C12" t="str">
-        <v>Visible</v>
+        <v>{{PPV_PROMOTER}}</v>
       </c>
     </row>
     <row r="13">
@@ -1091,10 +1092,10 @@
         <v>home-boxing-tile</v>
       </c>
       <c r="B13" t="str">
-        <v>Popup - Event Description</v>
+        <v>PPV Badge</v>
       </c>
       <c r="C13" t="str">
-        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="14">
@@ -1102,26 +1103,103 @@
         <v>home-boxing-tile</v>
       </c>
       <c r="B14" t="str">
-        <v>Popup - Close Button</v>
+        <v>Lock Icon</v>
       </c>
       <c r="C14" t="str">
-        <v>Visible</v>
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>home-kickboxing-tile</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Home of Boxing Section Present</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Present</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>home-kickboxing-tile</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Selected Boxing Tile</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>home-kickboxing-tile</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Event Title</v>
+      </c>
+      <c r="C17" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>home-kickboxing-tile</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Event Date</v>
+      </c>
+      <c r="C18" t="str">
+        <v>{{PPV_DATE}}</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>home-kickboxing-tile</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Promoter</v>
+      </c>
+      <c r="C19" t="str">
+        <v>{{PPV_PROMOTER}}</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>home-kickboxing-tile</v>
+      </c>
+      <c r="B20" t="str">
+        <v>PPV Badge</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>home-kickboxing-tile</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Lock Icon</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Yes</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C21"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C22"/>
   <cols>
     <col min="1" max="1" width="21.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
-    <col min="3" max="3" width="90.83203125" customWidth="1"/>
+    <col min="2" max="2" width="32.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1195,10 +1273,10 @@
         <v>home-page-dont-miss</v>
       </c>
       <c r="B7" t="str">
-        <v>Popup - Event Title</v>
+        <v>Don't Miss Section Present</v>
       </c>
       <c r="C7" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>Present</v>
       </c>
     </row>
     <row r="8">
@@ -1206,10 +1284,10 @@
         <v>home-page-dont-miss</v>
       </c>
       <c r="B8" t="str">
-        <v>Popup - Event Date</v>
+        <v>Don't Miss Tile Present</v>
       </c>
       <c r="C8" t="str">
-        <v>{{PPV_DATE}}</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="9">
@@ -1217,10 +1295,10 @@
         <v>home-page-dont-miss</v>
       </c>
       <c r="B9" t="str">
-        <v>Popup - Promoter</v>
+        <v>Don't Miss Event Title</v>
       </c>
       <c r="C9" t="str">
-        <v>{{PPV_PROMOTER}}</v>
+        <v>{{PPV_NAME}}</v>
       </c>
     </row>
     <row r="10">
@@ -1228,10 +1306,10 @@
         <v>home-page-dont-miss</v>
       </c>
       <c r="B10" t="str">
-        <v>Popup - Buy Now CTA</v>
+        <v>Don't Miss Event Date</v>
       </c>
       <c r="C10" t="str">
-        <v>Visible</v>
+        <v>{{PPV_DATE}}</v>
       </c>
     </row>
     <row r="11">
@@ -1239,10 +1317,10 @@
         <v>home-page-dont-miss</v>
       </c>
       <c r="B11" t="str">
-        <v>Popup - Event Description</v>
+        <v>Don't Miss Promoter</v>
       </c>
       <c r="C11" t="str">
-        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
+        <v>{{PPV_PROMOTER}}</v>
       </c>
     </row>
     <row r="12">
@@ -1250,32 +1328,32 @@
         <v>home-page-dont-miss</v>
       </c>
       <c r="B12" t="str">
-        <v>Popup - Close Button</v>
+        <v>PPV Badge Present</v>
       </c>
       <c r="C12" t="str">
-        <v>Visible</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>home-biggest-fights</v>
+        <v>home-page-dont-miss</v>
       </c>
       <c r="B13" t="str">
-        <v>Biggest Fights Section</v>
+        <v>Locked Badge Present</v>
       </c>
       <c r="C13" t="str">
-        <v>The Biggest Fights|Saturday Fight Night|Fight Night|Upcoming Big Fights|Big Fights</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>home-biggest-fights</v>
+        <v>home-page-dont-miss</v>
       </c>
       <c r="B14" t="str">
-        <v>Popup - Event Title</v>
+        <v>Reminder Icon Present</v>
       </c>
       <c r="C14" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="15">
@@ -1283,10 +1361,10 @@
         <v>home-biggest-fights</v>
       </c>
       <c r="B15" t="str">
-        <v>Popup - Event Date</v>
+        <v>Biggest Fights Section Present</v>
       </c>
       <c r="C15" t="str">
-        <v>{{PPV_DATE}}</v>
+        <v>Present</v>
       </c>
     </row>
     <row r="16">
@@ -1294,10 +1372,10 @@
         <v>home-biggest-fights</v>
       </c>
       <c r="B16" t="str">
-        <v>Popup - Promoter</v>
+        <v>Biggest Fights Tile Present</v>
       </c>
       <c r="C16" t="str">
-        <v>{{PPV_PROMOTER}}</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="17">
@@ -1305,10 +1383,10 @@
         <v>home-biggest-fights</v>
       </c>
       <c r="B17" t="str">
-        <v>Popup - Buy Now CTA</v>
+        <v>Event Title</v>
       </c>
       <c r="C17" t="str">
-        <v>Visible</v>
+        <v>{{PPV_NAME}}</v>
       </c>
     </row>
     <row r="18">
@@ -1316,10 +1394,10 @@
         <v>home-biggest-fights</v>
       </c>
       <c r="B18" t="str">
-        <v>Popup - Event Description</v>
+        <v>Event Date</v>
       </c>
       <c r="C18" t="str">
-        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
+        <v>{{PPV_DATE}}</v>
       </c>
     </row>
     <row r="19">
@@ -1327,15 +1405,48 @@
         <v>home-biggest-fights</v>
       </c>
       <c r="B19" t="str">
-        <v>Popup - Close Button</v>
+        <v>Promoter</v>
       </c>
       <c r="C19" t="str">
-        <v>Visible</v>
+        <v>{{PPV_PROMOTER}}</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>home-biggest-fights</v>
+      </c>
+      <c r="B20" t="str">
+        <v>PPV Badge</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>home-biggest-fights</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Lock Icon</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>home-biggest-fights</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Reminder Icon</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Yes</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C22"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1944,7 +2055,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B4"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -1982,24 +2093,16 @@
         <v>{{PPV_DATE}}</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Buy Now Button</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C54"/>
   <cols>
     <col min="1" max="1" width="29.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
@@ -2052,10 +2155,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Saturday Badge</v>
+        <v>Or Separator</v>
       </c>
       <c r="B5" t="str">
-        <v>SATURDAY</v>
+        <v>or</v>
       </c>
       <c r="C5" t="str">
         <v>boxing</v>
@@ -2063,10 +2166,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Or Separator</v>
+        <v>Buy Fight CTA</v>
       </c>
       <c r="B6" t="str">
-        <v>or</v>
+        <v>Buy this fight for {{PPV_PRICE}}</v>
       </c>
       <c r="C6" t="str">
         <v>boxing</v>
@@ -2074,10 +2177,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Buy Fight CTA</v>
+        <v>Get Included CTA</v>
       </c>
       <c r="B7" t="str">
-        <v>Buy this fight for {{PPV_PRICE}}</v>
+        <v>Get included in DAZN Ultimate</v>
       </c>
       <c r="C7" t="str">
         <v>boxing</v>
@@ -2085,10 +2188,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Get Included CTA</v>
+        <v>Best Value Badge</v>
       </c>
       <c r="B8" t="str">
-        <v>Get included in DAZN Ultimate</v>
+        <v>Best value for boxing fans</v>
       </c>
       <c r="C8" t="str">
         <v>boxing</v>
@@ -2096,21 +2199,21 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Best Value Badge</v>
+        <v>Upcoming Big Fights Heading</v>
       </c>
       <c r="B9" t="str">
-        <v>Best value for boxing fans</v>
+        <v>Upcoming Big Fights</v>
       </c>
       <c r="C9" t="str">
-        <v>boxing</v>
+        <v>boxing-upcoming</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Upcoming Big Fights Heading</v>
+        <v>PPV Name</v>
       </c>
       <c r="B10" t="str">
-        <v>Upcoming Big Fights</v>
+        <v>{{PPV_DISPLAY_NAME}}</v>
       </c>
       <c r="C10" t="str">
         <v>boxing-upcoming</v>
@@ -2118,10 +2221,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>PPV Name</v>
+        <v>PPV Date and Time Text</v>
       </c>
       <c r="B11" t="str">
-        <v>{{PPV_DISPLAY_NAME}}</v>
+        <v>{{PPV_DATE}}</v>
       </c>
       <c r="C11" t="str">
         <v>boxing-upcoming</v>
@@ -2129,10 +2232,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>PPV Date and Time Text</v>
+        <v>PPV Description Text</v>
       </c>
       <c r="B12" t="str">
-        <v>{{PPV_DATE}}</v>
+        <v>{{PPV_LOCATION}}</v>
       </c>
       <c r="C12" t="str">
         <v>boxing-upcoming</v>
@@ -2140,10 +2243,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>PPV Description Text</v>
+        <v>PPV Image Present</v>
       </c>
       <c r="B13" t="str">
-        <v>{{PPV_LOCATION}}</v>
+        <v>Yes</v>
       </c>
       <c r="C13" t="str">
         <v>boxing-upcoming</v>
@@ -2151,10 +2254,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>PPV Image Present</v>
+        <v>Buy Now CTA</v>
       </c>
       <c r="B14" t="str">
-        <v>Yes</v>
+        <v>Buy now</v>
       </c>
       <c r="C14" t="str">
         <v>boxing-upcoming</v>
@@ -2162,21 +2265,21 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Buy Now CTA</v>
+        <v>Bundle Section Present</v>
       </c>
       <c r="B15" t="str">
-        <v>Buy now</v>
+        <v>Yes</v>
       </c>
       <c r="C15" t="str">
-        <v>boxing-upcoming</v>
+        <v>boxing-bundle</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Bundle Section Present</v>
+        <v>Bundle Section Title</v>
       </c>
       <c r="B16" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_SECTION_TITLE}}</v>
       </c>
       <c r="C16" t="str">
         <v>boxing-bundle</v>
@@ -2184,10 +2287,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Bundle Section Title</v>
+        <v>Bundle Section Subtitle</v>
       </c>
       <c r="B17" t="str">
-        <v>{{BUNDLE_SECTION_TITLE}}</v>
+        <v>{{BUNDLE_SECTION_SUBTITLE}}</v>
       </c>
       <c r="C17" t="str">
         <v>boxing-bundle</v>
@@ -2195,10 +2298,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Bundle Section Subtitle</v>
+        <v>Bundle Title</v>
       </c>
       <c r="B18" t="str">
-        <v>{{BUNDLE_SECTION_SUBTITLE}}</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="C18" t="str">
         <v>boxing-bundle</v>
@@ -2206,10 +2309,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Bundle Title</v>
+        <v>Bundle Description</v>
       </c>
       <c r="B19" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>{{BUNDLE_DESCRIPTION}}</v>
       </c>
       <c r="C19" t="str">
         <v>boxing-bundle</v>
@@ -2217,10 +2320,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Bundle Description</v>
+        <v>Bundle Price</v>
       </c>
       <c r="B20" t="str">
-        <v>{{BUNDLE_DESCRIPTION}}</v>
+        <v>{{BUNDLE_PRICE}}</v>
       </c>
       <c r="C20" t="str">
         <v>boxing-bundle</v>
@@ -2228,10 +2331,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Bundle Price</v>
+        <v>Bundle Original Price</v>
       </c>
       <c r="B21" t="str">
-        <v>{{BUNDLE_PRICE}}</v>
+        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
       </c>
       <c r="C21" t="str">
         <v>boxing-bundle</v>
@@ -2239,10 +2342,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Bundle Original Price</v>
+        <v>Bundle Save Badge</v>
       </c>
       <c r="B22" t="str">
-        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
+        <v>{{BUNDLE_SAVE_BADGE}}</v>
       </c>
       <c r="C22" t="str">
         <v>boxing-bundle</v>
@@ -2250,10 +2353,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Bundle Save Badge</v>
+        <v>Bundle Fight Count</v>
       </c>
       <c r="B23" t="str">
-        <v>{{BUNDLE_SAVE_BADGE}}</v>
+        <v>{{BUNDLE_FIGHT_COUNT}}</v>
       </c>
       <c r="C23" t="str">
         <v>boxing-bundle</v>
@@ -2261,10 +2364,10 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Bundle Fight Count</v>
+        <v>Bundle PPV 1 Name</v>
       </c>
       <c r="B24" t="str">
-        <v>{{BUNDLE_FIGHT_COUNT}}</v>
+        <v>{{BUNDLE_PPV1_NAME}}</v>
       </c>
       <c r="C24" t="str">
         <v>boxing-bundle</v>
@@ -2272,10 +2375,10 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Bundle PPV 1 Name</v>
+        <v>Bundle PPV 1 Date</v>
       </c>
       <c r="B25" t="str">
-        <v>{{BUNDLE_PPV1_NAME}}</v>
+        <v>{{BUNDLE_PPV1_LANDING_DATE}}</v>
       </c>
       <c r="C25" t="str">
         <v>boxing-bundle</v>
@@ -2283,10 +2386,10 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Bundle PPV 1 Date</v>
+        <v>Bundle PPV 1 Image</v>
       </c>
       <c r="B26" t="str">
-        <v>{{BUNDLE_PPV1_LANDING_DATE}}</v>
+        <v>Yes</v>
       </c>
       <c r="C26" t="str">
         <v>boxing-bundle</v>
@@ -2294,10 +2397,10 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Bundle PPV 1 Image</v>
+        <v>Bundle PPV 2 Name</v>
       </c>
       <c r="B27" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_PPV2_NAME}}</v>
       </c>
       <c r="C27" t="str">
         <v>boxing-bundle</v>
@@ -2305,10 +2408,10 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Bundle PPV 2 Name</v>
+        <v>Bundle PPV 2 Date</v>
       </c>
       <c r="B28" t="str">
-        <v>{{BUNDLE_PPV2_NAME}}</v>
+        <v>{{BUNDLE_PPV2_LANDING_DATE}}</v>
       </c>
       <c r="C28" t="str">
         <v>boxing-bundle</v>
@@ -2316,10 +2419,10 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Bundle PPV 2 Date</v>
+        <v>Bundle PPV 2 Image</v>
       </c>
       <c r="B29" t="str">
-        <v>{{BUNDLE_PPV2_LANDING_DATE}}</v>
+        <v>Yes</v>
       </c>
       <c r="C29" t="str">
         <v>boxing-bundle</v>
@@ -2327,10 +2430,10 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Bundle PPV 2 Image</v>
+        <v>Get Started CTA</v>
       </c>
       <c r="B30" t="str">
-        <v>Yes</v>
+        <v>Get Started</v>
       </c>
       <c r="C30" t="str">
         <v>boxing-bundle</v>
@@ -2338,21 +2441,21 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Get Started CTA</v>
+        <v>Page Title</v>
       </c>
       <c r="B31" t="str">
-        <v>Get Started</v>
+        <v>Choose the right plan for you.</v>
       </c>
       <c r="C31" t="str">
-        <v>boxing-bundle</v>
+        <v>boxing-bundle-ppv</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Page Title</v>
+        <v>Header Sub Text</v>
       </c>
       <c r="B32" t="str">
-        <v>Choose the right plan for you.</v>
+        <v>To watch your pay-per-view, you'll need a DAZN plan.</v>
       </c>
       <c r="C32" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2360,10 +2463,10 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Header Sub Text</v>
+        <v>Bundle Card Title</v>
       </c>
       <c r="B33" t="str">
-        <v>To watch your pay-per-view, you'll need a DAZN plan.</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="C33" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2371,10 +2474,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Bundle Card Title</v>
+        <v>Bundle Card Description</v>
       </c>
       <c r="B34" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>{{BUNDLE_PPV_CARD_DESCRIPTION}}</v>
       </c>
       <c r="C34" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2382,10 +2485,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Bundle Card Description</v>
+        <v>Bundle Card Selected</v>
       </c>
       <c r="B35" t="str">
-        <v>{{BUNDLE_PPV_CARD_DESCRIPTION}}</v>
+        <v>Yes</v>
       </c>
       <c r="C35" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2393,10 +2496,10 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Bundle Card Selected</v>
+        <v>Bundle Card Price</v>
       </c>
       <c r="B36" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_PRICE}}</v>
       </c>
       <c r="C36" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2404,10 +2507,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Bundle Card Price</v>
+        <v>Bundle Card Original Price</v>
       </c>
       <c r="B37" t="str">
-        <v>{{BUNDLE_PRICE}}</v>
+        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
       </c>
       <c r="C37" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2415,10 +2518,10 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Bundle Card Original Price</v>
+        <v>Bundle Card Save Badge</v>
       </c>
       <c r="B38" t="str">
-        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
+        <v>{{BUNDLE_SAVE_BADGE}}</v>
       </c>
       <c r="C38" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2426,10 +2529,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Bundle Card Save Badge</v>
+        <v>Bundle PPV 1 Full Name</v>
       </c>
       <c r="B39" t="str">
-        <v>{{BUNDLE_SAVE_BADGE}}</v>
+        <v>{{BUNDLE_PPV1_FULL_NAME}}</v>
       </c>
       <c r="C39" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2437,10 +2540,10 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Bundle PPV 1 Full Name</v>
+        <v>Bundle PPV 1 PPV Date</v>
       </c>
       <c r="B40" t="str">
-        <v>{{BUNDLE_PPV1_FULL_NAME}}</v>
+        <v>{{BUNDLE_PPV1_DATE}}</v>
       </c>
       <c r="C40" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2448,10 +2551,10 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Bundle PPV 1 PPV Date</v>
+        <v>Bundle PPV 1 PPV Image</v>
       </c>
       <c r="B41" t="str">
-        <v>{{BUNDLE_PPV1_DATE}}</v>
+        <v>Yes</v>
       </c>
       <c r="C41" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2459,10 +2562,10 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Bundle PPV 1 PPV Image</v>
+        <v>Bundle PPV 2 Full Name</v>
       </c>
       <c r="B42" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_PPV2_FULL_NAME}}</v>
       </c>
       <c r="C42" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2470,10 +2573,10 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Bundle PPV 2 Full Name</v>
+        <v>Bundle PPV 2 PPV Date</v>
       </c>
       <c r="B43" t="str">
-        <v>{{BUNDLE_PPV2_FULL_NAME}}</v>
+        <v>{{BUNDLE_PPV2_DATE}}</v>
       </c>
       <c r="C43" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2481,10 +2584,10 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Bundle PPV 2 PPV Date</v>
+        <v>Bundle PPV 2 PPV Image</v>
       </c>
       <c r="B44" t="str">
-        <v>{{BUNDLE_PPV2_DATE}}</v>
+        <v>Yes</v>
       </c>
       <c r="C44" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2492,7 +2595,7 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Bundle PPV 2 PPV Image</v>
+        <v>Upsell Section Present</v>
       </c>
       <c r="B45" t="str">
         <v>Yes</v>
@@ -2503,10 +2606,10 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Upsell Section Present</v>
+        <v>Upsell Badge</v>
       </c>
       <c r="B46" t="str">
-        <v>Yes</v>
+        <v>The Ultimate Fan Package</v>
       </c>
       <c r="C46" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2514,10 +2617,10 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Upsell Badge</v>
+        <v>Upsell Plan Name</v>
       </c>
       <c r="B47" t="str">
-        <v>The Ultimate Fan Package</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="C47" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2525,10 +2628,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Upsell Plan Name</v>
+        <v>Upsell Price</v>
       </c>
       <c r="B48" t="str">
-        <v>DAZN Ultimate</v>
+        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
       </c>
       <c r="C48" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2536,10 +2639,10 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Upsell Price</v>
+        <v>Upsell Contract Text</v>
       </c>
       <c r="B49" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
+        <v>Annual contract. Auto renews.</v>
       </c>
       <c r="C49" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2547,10 +2650,10 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Upsell Contract Text</v>
+        <v>Fights Included Text</v>
       </c>
       <c r="B50" t="str">
-        <v>Annual contract. Auto renews.</v>
+        <v>All these fights included and more.</v>
       </c>
       <c r="C50" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2558,10 +2661,10 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Fights Included Text</v>
+        <v>Upsell Feature 1</v>
       </c>
       <c r="B51" t="str">
-        <v>All these fights included and more.</v>
+        <v>Minimum 12 pay-per-views a year included at no extra cost.</v>
       </c>
       <c r="C51" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2569,10 +2672,10 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Upsell Feature 1</v>
+        <v>Upsell Feature 2</v>
       </c>
       <c r="B52" t="str">
-        <v>Minimum 12 pay-per-views a year included at no extra cost.</v>
+        <v>185+ fights a year from the world's best promoters.</v>
       </c>
       <c r="C52" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2580,10 +2683,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Upsell Feature 2</v>
+        <v>Upsell Feature 3</v>
       </c>
       <c r="B53" t="str">
-        <v>185+ fights a year from the world's best promoters.</v>
+        <v>HDR and Dolby 5.1 surround sound on select events</v>
       </c>
       <c r="C53" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2591,29 +2694,89 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Upsell Feature 3</v>
+        <v>CTA Button</v>
       </c>
       <c r="B54" t="str">
-        <v>HDR and Dolby 5.1 surround sound on select events</v>
+        <v>Continue with DAZN Ultimate</v>
       </c>
       <c r="C54" t="str">
         <v>boxing-bundle-ppv</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" t="str">
-        <v>CTA Button</v>
-      </c>
-      <c r="B55" t="str">
-        <v>Continue with DAZN Ultimate</v>
-      </c>
-      <c r="C55" t="str">
-        <v>boxing-bundle-ppv</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C55"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C54"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B7"/>
+  <cols>
+    <col min="1" max="1" width="29.83203125" customWidth="1"/>
+    <col min="2" max="2" width="90.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Field</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Expected</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Paywall - Event Title</v>
+      </c>
+      <c r="B2" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Paywall - Event Date</v>
+      </c>
+      <c r="B3" t="str">
+        <v>{{PPV_DATE}}</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Paywall - Promoter</v>
+      </c>
+      <c r="B4" t="str">
+        <v>{{PPV_PROMOTER}}</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Paywall - Buy Now CTA</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Paywall - Event Description</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Paywall - Close Button</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4488,7 +4651,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E103"/>
+  <dimension ref="A1:E104"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="27.83203125" customWidth="1"/>
@@ -4686,19 +4849,19 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Standard</v>
+        <v>Common</v>
       </c>
       <c r="B12" t="str">
-        <v>Monthly</v>
+        <v>All</v>
       </c>
       <c r="C12" t="str">
-        <v>Page Title</v>
+        <v>Excluding Tax Text</v>
       </c>
       <c r="D12" t="str">
-        <v>{{PAYMENT_PAGE_TITLE}}</v>
+        <v>N/A</v>
       </c>
       <c r="E12" t="str">
-        <v>newuser</v>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -4715,7 +4878,7 @@
         <v>{{PAYMENT_PAGE_TITLE}}</v>
       </c>
       <c r="E13" t="str">
-        <v>myaccount</v>
+        <v>newuser</v>
       </c>
     </row>
     <row r="14">
@@ -4726,13 +4889,13 @@
         <v>Monthly</v>
       </c>
       <c r="C14" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D14" t="str">
-        <v>DAZN Standard</v>
+        <v>{{PAYMENT_PAGE_TITLE}}</v>
       </c>
       <c r="E14" t="str">
-        <v/>
+        <v>myaccount</v>
       </c>
     </row>
     <row r="15">
@@ -4743,10 +4906,10 @@
         <v>Monthly</v>
       </c>
       <c r="C15" t="str">
-        <v>Plan Name</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D15" t="str">
-        <v>{{PAYMENT_PLAN_NAME}}</v>
+        <v>DAZN Standard</v>
       </c>
       <c r="E15" t="str">
         <v/>
@@ -4760,10 +4923,10 @@
         <v>Monthly</v>
       </c>
       <c r="C16" t="str">
-        <v>Plan Subtitle</v>
+        <v>Plan Name</v>
       </c>
       <c r="D16" t="str">
-        <v>{{PAYMENT_FLEX_CANCEL_NOTICE}}</v>
+        <v>{{PAYMENT_PLAN_NAME}}</v>
       </c>
       <c r="E16" t="str">
         <v/>
@@ -4777,10 +4940,10 @@
         <v>Monthly</v>
       </c>
       <c r="C17" t="str">
-        <v>First Month Free Price</v>
+        <v>Plan Subtitle</v>
       </c>
       <c r="D17" t="str">
-        <v>{{CURRENCY}}0</v>
+        <v>{{PAYMENT_FLEX_CANCEL_NOTICE}}</v>
       </c>
       <c r="E17" t="str">
         <v/>
@@ -4794,10 +4957,10 @@
         <v>Monthly</v>
       </c>
       <c r="C18" t="str">
-        <v>First Month Free Text</v>
+        <v>First Month Free Price</v>
       </c>
       <c r="D18" t="str">
-        <v>{{PAYMENT_FREE_TEXT}}</v>
+        <v>{{CURRENCY}}0</v>
       </c>
       <c r="E18" t="str">
         <v/>
@@ -4811,10 +4974,10 @@
         <v>Monthly</v>
       </c>
       <c r="C19" t="str">
-        <v>PPV Name</v>
+        <v>First Month Free Text</v>
       </c>
       <c r="D19" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>{{PAYMENT_FREE_TEXT}}</v>
       </c>
       <c r="E19" t="str">
         <v/>
@@ -4828,10 +4991,10 @@
         <v>Monthly</v>
       </c>
       <c r="C20" t="str">
-        <v>PPV Price</v>
+        <v>PPV Name</v>
       </c>
       <c r="D20" t="str">
-        <v>{{PPV_PRICE}}</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="E20" t="str">
         <v/>
@@ -4845,10 +5008,10 @@
         <v>Monthly</v>
       </c>
       <c r="C21" t="str">
-        <v>Today You Pay Text</v>
+        <v>PPV Price</v>
       </c>
       <c r="D21" t="str">
-        <v>Today you pay</v>
+        <v>{{PPV_PRICE}}</v>
       </c>
       <c r="E21" t="str">
         <v/>
@@ -4862,10 +5025,10 @@
         <v>Monthly</v>
       </c>
       <c r="C22" t="str">
-        <v>Today You Pay Price</v>
+        <v>Today You Pay Text</v>
       </c>
       <c r="D22" t="str">
-        <v>{{PPV_PRICE}}</v>
+        <v>Today you pay</v>
       </c>
       <c r="E22" t="str">
         <v/>
@@ -4879,10 +5042,10 @@
         <v>Monthly</v>
       </c>
       <c r="C23" t="str">
-        <v>Cancellation Text</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D23" t="str">
-        <v>{{CANCELLATION_TEXT}}</v>
+        <v>{{PPV_PRICE}}</v>
       </c>
       <c r="E23" t="str">
         <v/>
@@ -4896,10 +5059,10 @@
         <v>Monthly</v>
       </c>
       <c r="C24" t="str">
-        <v>Legal Text</v>
+        <v>Cancellation Text</v>
       </c>
       <c r="D24" t="str">
-        <v>{{PAYMENT_FLEX_LEGAL_TEXT}}</v>
+        <v>{{CANCELLATION_TEXT}}</v>
       </c>
       <c r="E24" t="str">
         <v/>
@@ -4913,10 +5076,10 @@
         <v>Monthly</v>
       </c>
       <c r="C25" t="str">
-        <v>Ultimate Upsell Text</v>
+        <v>Legal Text</v>
       </c>
       <c r="D25" t="str">
-        <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
+        <v>{{PAYMENT_FLEX_LEGAL_TEXT}}</v>
       </c>
       <c r="E25" t="str">
         <v/>
@@ -4927,13 +5090,13 @@
         <v>Standard</v>
       </c>
       <c r="B26" t="str">
-        <v>Annual Pay Monthly</v>
+        <v>Monthly</v>
       </c>
       <c r="C26" t="str">
-        <v>Page Title</v>
+        <v>Ultimate Upsell Text</v>
       </c>
       <c r="D26" t="str">
-        <v>Choose how to pay</v>
+        <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
       <c r="E26" t="str">
         <v/>
@@ -4947,10 +5110,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C27" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D27" t="str">
-        <v>DAZN Standard</v>
+        <v>Choose how to pay</v>
       </c>
       <c r="E27" t="str">
         <v/>
@@ -4964,10 +5127,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C28" t="str">
-        <v>PPV Name</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D28" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>DAZN Standard</v>
       </c>
       <c r="E28" t="str">
         <v/>
@@ -4981,10 +5144,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C29" t="str">
-        <v>PPV Price</v>
+        <v>PPV Name</v>
       </c>
       <c r="D29" t="str">
-        <v>{{PPV_PRICE}}</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="E29" t="str">
         <v/>
@@ -4998,10 +5161,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C30" t="str">
-        <v>Rate Plan</v>
+        <v>PPV Price</v>
       </c>
       <c r="D30" t="str">
-        <v>{{RATE_PLAN_LABEL}}</v>
+        <v>{{PPV_PRICE}}</v>
       </c>
       <c r="E30" t="str">
         <v/>
@@ -5015,10 +5178,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C31" t="str">
-        <v>Rate Plan Original Price</v>
+        <v>Rate Plan</v>
       </c>
       <c r="D31" t="str">
-        <v>{{CURRENCY}}{{ANNUAL_PRICE}}</v>
+        <v>{{RATE_PLAN_LABEL}}</v>
       </c>
       <c r="E31" t="str">
         <v/>
@@ -5032,10 +5195,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C32" t="str">
-        <v>Rate Plan Discounted Price</v>
+        <v>Rate Plan Original Price</v>
       </c>
       <c r="D32" t="str">
-        <v>{{CURRENCY}}0</v>
+        <v>{{CURRENCY}}{{ANNUAL_PRICE}}</v>
       </c>
       <c r="E32" t="str">
         <v/>
@@ -5049,10 +5212,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C33" t="str">
-        <v>Today You Pay Text</v>
+        <v>Rate Plan Discounted Price</v>
       </c>
       <c r="D33" t="str">
-        <v>Today you pay</v>
+        <v>{{CURRENCY}}0</v>
       </c>
       <c r="E33" t="str">
         <v/>
@@ -5066,10 +5229,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C34" t="str">
-        <v>Today You Pay Price</v>
+        <v>Today You Pay Text</v>
       </c>
       <c r="D34" t="str">
-        <v>{{PPV_PRICE}}</v>
+        <v>Today you pay</v>
       </c>
       <c r="E34" t="str">
         <v/>
@@ -5083,10 +5246,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C35" t="str">
-        <v>Cancellation Text</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D35" t="str">
-        <v>{{CANCELLATION_TEXT_ANNUAL}}</v>
+        <v>{{PPV_PRICE}}</v>
       </c>
       <c r="E35" t="str">
         <v/>
@@ -5100,10 +5263,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C36" t="str">
-        <v>Redeem Promo Code CTA</v>
+        <v>Cancellation Text</v>
       </c>
       <c r="D36" t="str">
-        <v>Yes</v>
+        <v>{{CANCELLATION_TEXT_ANNUAL}}</v>
       </c>
       <c r="E36" t="str">
         <v/>
@@ -5117,10 +5280,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C37" t="str">
-        <v>Ultimate Upsell Text</v>
+        <v>Redeem Promo Code CTA</v>
       </c>
       <c r="D37" t="str">
-        <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
+        <v>Yes</v>
       </c>
       <c r="E37" t="str">
         <v/>
@@ -5128,16 +5291,16 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Ultimate</v>
+        <v>Standard</v>
       </c>
       <c r="B38" t="str">
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C38" t="str">
-        <v>Page Title</v>
+        <v>Ultimate Upsell Text</v>
       </c>
       <c r="D38" t="str">
-        <v>Choose how to pay</v>
+        <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
       <c r="E38" t="str">
         <v/>
@@ -5151,10 +5314,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C39" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D39" t="str">
-        <v>DAZN Ultimate</v>
+        <v>Choose how to pay</v>
       </c>
       <c r="E39" t="str">
         <v/>
@@ -5168,10 +5331,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C40" t="str">
-        <v>PPV Name</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D40" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="E40" t="str">
         <v/>
@@ -5185,10 +5348,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C41" t="str">
-        <v>PPV Price</v>
+        <v>PPV Name</v>
       </c>
       <c r="D41" t="str">
-        <v>{{CURRENCY}}0</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="E41" t="str">
         <v/>
@@ -5202,10 +5365,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C42" t="str">
-        <v>Rate Plan</v>
+        <v>PPV Price</v>
       </c>
       <c r="D42" t="str">
-        <v>Annual - Pay Monthly</v>
+        <v>{{CURRENCY}}0</v>
       </c>
       <c r="E42" t="str">
         <v/>
@@ -5219,10 +5382,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C43" t="str">
-        <v>Rate Plan Price</v>
+        <v>Rate Plan</v>
       </c>
       <c r="D43" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
+        <v>Annual - Pay Monthly</v>
       </c>
       <c r="E43" t="str">
         <v/>
@@ -5236,10 +5399,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C44" t="str">
-        <v>Plan Subtitle</v>
+        <v>Rate Plan Price</v>
       </c>
       <c r="D44" t="str">
-        <v>Billed monthly. 12-month contract.</v>
+        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
       </c>
       <c r="E44" t="str">
         <v/>
@@ -5253,10 +5416,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C45" t="str">
-        <v>Today You Pay Text</v>
+        <v>Plan Subtitle</v>
       </c>
       <c r="D45" t="str">
-        <v>Today you pay</v>
+        <v>Billed monthly. 12-month contract.</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -5270,10 +5433,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C46" t="str">
-        <v>Today You Pay Price</v>
+        <v>Today You Pay Text</v>
       </c>
       <c r="D46" t="str">
-        <v>{{TODAY_YOU_PAY_PRICE}}</v>
+        <v>Today you pay</v>
       </c>
       <c r="E46" t="str">
         <v/>
@@ -5287,10 +5450,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C47" t="str">
-        <v>Next Payment Label</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D47" t="str">
-        <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
+        <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
       <c r="E47" t="str">
         <v/>
@@ -5304,10 +5467,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C48" t="str">
-        <v>Next Payment Price</v>
+        <v>Next Payment Label</v>
       </c>
       <c r="D48" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
+        <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
       <c r="E48" t="str">
         <v/>
@@ -5321,10 +5484,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C49" t="str">
-        <v>Cancellation Text</v>
+        <v>Next Payment Price</v>
       </c>
       <c r="D49" t="str">
-        <v>{{CANCELLATION_TEXT}}</v>
+        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
       </c>
       <c r="E49" t="str">
         <v/>
@@ -5338,10 +5501,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C50" t="str">
-        <v>Redeem Promo Code CTA</v>
+        <v>Cancellation Text</v>
       </c>
       <c r="D50" t="str">
-        <v>Yes</v>
+        <v>{{CANCELLATION_TEXT}}</v>
       </c>
       <c r="E50" t="str">
         <v/>
@@ -5355,10 +5518,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C51" t="str">
-        <v>Discount Badge</v>
+        <v>Redeem Promo Code CTA</v>
       </c>
       <c r="D51" t="str">
-        <v>{{DISCOUNT_BADGE}}</v>
+        <v>Yes</v>
       </c>
       <c r="E51" t="str">
         <v/>
@@ -5369,13 +5532,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B52" t="str">
-        <v>Annual Pay Upfront</v>
+        <v>Annual Pay Monthly</v>
       </c>
       <c r="C52" t="str">
-        <v>Page Title</v>
+        <v>Discount Badge</v>
       </c>
       <c r="D52" t="str">
-        <v>Choose how to pay</v>
+        <v>{{DISCOUNT_BADGE}}</v>
       </c>
       <c r="E52" t="str">
         <v/>
@@ -5389,10 +5552,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C53" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D53" t="str">
-        <v>DAZN Ultimate</v>
+        <v>Choose how to pay</v>
       </c>
       <c r="E53" t="str">
         <v/>
@@ -5406,10 +5569,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C54" t="str">
-        <v>PPV Name</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D54" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="E54" t="str">
         <v/>
@@ -5423,10 +5586,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C55" t="str">
-        <v>PPV Price</v>
+        <v>PPV Name</v>
       </c>
       <c r="D55" t="str">
-        <v>{{CURRENCY}}0</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="E55" t="str">
         <v/>
@@ -5440,10 +5603,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C56" t="str">
-        <v>Rate Plan</v>
+        <v>PPV Price</v>
       </c>
       <c r="D56" t="str">
-        <v>Annual - Pay Upfront</v>
+        <v>{{CURRENCY}}0</v>
       </c>
       <c r="E56" t="str">
         <v/>
@@ -5457,10 +5620,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C57" t="str">
-        <v>Rate Plan Price</v>
+        <v>Rate Plan</v>
       </c>
       <c r="D57" t="str">
-        <v>{{ANNUAL_UPFRONT_PRICE}}/year</v>
+        <v>Annual - Pay Upfront</v>
       </c>
       <c r="E57" t="str">
         <v/>
@@ -5474,10 +5637,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C58" t="str">
-        <v>Plan Subtitle</v>
+        <v>Rate Plan Price</v>
       </c>
       <c r="D58" t="str">
-        <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}. Pay for the full year up front|Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
+        <v>{{ANNUAL_UPFRONT_PRICE}}/year</v>
       </c>
       <c r="E58" t="str">
         <v/>
@@ -5491,10 +5654,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C59" t="str">
-        <v>Today You Pay Text</v>
+        <v>Plan Subtitle</v>
       </c>
       <c r="D59" t="str">
-        <v>Today you pay</v>
+        <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}. Pay for the full year up front|Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
       </c>
       <c r="E59" t="str">
         <v/>
@@ -5508,10 +5671,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C60" t="str">
-        <v>Today You Pay Price</v>
+        <v>Today You Pay Text</v>
       </c>
       <c r="D60" t="str">
-        <v>{{TODAY_YOU_PAY_PRICE}}</v>
+        <v>Today you pay</v>
       </c>
       <c r="E60" t="str">
         <v/>
@@ -5525,10 +5688,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C61" t="str">
-        <v>Next Payment Label</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D61" t="str">
-        <v>Next Annual payment on {{NEXT_PAYMENT_DATE}}</v>
+        <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
       <c r="E61" t="str">
         <v/>
@@ -5542,10 +5705,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C62" t="str">
-        <v>Next Payment Price</v>
+        <v>Next Payment Label</v>
       </c>
       <c r="D62" t="str">
-        <v>{{ANNUAL_UPFRONT_PRICE}}</v>
+        <v>Next Annual payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
       <c r="E62" t="str">
         <v/>
@@ -5559,10 +5722,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C63" t="str">
-        <v>Cancellation Text</v>
+        <v>Next Payment Price</v>
       </c>
       <c r="D63" t="str">
-        <v>{{CANCELLATION_TEXT}}</v>
+        <v>{{ANNUAL_UPFRONT_PRICE}}</v>
       </c>
       <c r="E63" t="str">
         <v/>
@@ -5576,10 +5739,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C64" t="str">
-        <v>Redeem Promo Code CTA</v>
+        <v>Cancellation Text</v>
       </c>
       <c r="D64" t="str">
-        <v>Yes</v>
+        <v>{{CANCELLATION_TEXT}}</v>
       </c>
       <c r="E64" t="str">
         <v/>
@@ -5587,16 +5750,16 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Standard</v>
+        <v>Ultimate</v>
       </c>
       <c r="B65" t="str">
-        <v>Monthly Bundle</v>
+        <v>Annual Pay Upfront</v>
       </c>
       <c r="C65" t="str">
-        <v>Page Title</v>
+        <v>Redeem Promo Code CTA</v>
       </c>
       <c r="D65" t="str">
-        <v>{{PAYMENT_PAGE_TITLE}}</v>
+        <v>Yes</v>
       </c>
       <c r="E65" t="str">
         <v/>
@@ -5610,10 +5773,10 @@
         <v>Monthly Bundle</v>
       </c>
       <c r="C66" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D66" t="str">
-        <v>DAZN Standard</v>
+        <v>{{PAYMENT_PAGE_TITLE}}</v>
       </c>
       <c r="E66" t="str">
         <v/>
@@ -5627,10 +5790,10 @@
         <v>Monthly Bundle</v>
       </c>
       <c r="C67" t="str">
-        <v>Bundle Name</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D67" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>DAZN Standard</v>
       </c>
       <c r="E67" t="str">
         <v/>
@@ -5644,10 +5807,10 @@
         <v>Monthly Bundle</v>
       </c>
       <c r="C68" t="str">
-        <v>Bundle Price</v>
+        <v>Bundle Name</v>
       </c>
       <c r="D68" t="str">
-        <v>{{BUNDLE_PRICE}}</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="E68" t="str">
         <v/>
@@ -5661,10 +5824,10 @@
         <v>Monthly Bundle</v>
       </c>
       <c r="C69" t="str">
-        <v>Today You Pay Price</v>
+        <v>Bundle Price</v>
       </c>
       <c r="D69" t="str">
-        <v>{{BUNDLE_TODAY_YOU_PAY_STANDARD}}</v>
+        <v>{{BUNDLE_PRICE}}</v>
       </c>
       <c r="E69" t="str">
         <v/>
@@ -5678,10 +5841,10 @@
         <v>Monthly Bundle</v>
       </c>
       <c r="C70" t="str">
-        <v>Cancellation Text</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D70" t="str">
-        <v>{{CANCELLATION_TEXT}}</v>
+        <v>{{BUNDLE_TODAY_YOU_PAY_STANDARD}}</v>
       </c>
       <c r="E70" t="str">
         <v/>
@@ -5692,13 +5855,13 @@
         <v>Standard</v>
       </c>
       <c r="B71" t="str">
-        <v>Annual Pay Monthly Bundle</v>
+        <v>Monthly Bundle</v>
       </c>
       <c r="C71" t="str">
-        <v>Page Title</v>
+        <v>Cancellation Text</v>
       </c>
       <c r="D71" t="str">
-        <v>Choose how to pay</v>
+        <v>{{CANCELLATION_TEXT}}</v>
       </c>
       <c r="E71" t="str">
         <v/>
@@ -5712,10 +5875,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C72" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D72" t="str">
-        <v>DAZN Standard</v>
+        <v>Choose how to pay</v>
       </c>
       <c r="E72" t="str">
         <v/>
@@ -5729,10 +5892,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C73" t="str">
-        <v>Rate Plan</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D73" t="str">
-        <v>Annual - Pay Monthly</v>
+        <v>DAZN Standard</v>
       </c>
       <c r="E73" t="str">
         <v/>
@@ -5746,10 +5909,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C74" t="str">
-        <v>First Month Free Text</v>
+        <v>Rate Plan</v>
       </c>
       <c r="D74" t="str">
-        <v>First month free</v>
+        <v>Annual - Pay Monthly</v>
       </c>
       <c r="E74" t="str">
         <v/>
@@ -5763,10 +5926,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C75" t="str">
-        <v>Bundle Name</v>
+        <v>First Month Free Text</v>
       </c>
       <c r="D75" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>First month free</v>
       </c>
       <c r="E75" t="str">
         <v/>
@@ -5780,10 +5943,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C76" t="str">
-        <v>Bundle Original Price</v>
+        <v>Bundle Name</v>
       </c>
       <c r="D76" t="str">
-        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="E76" t="str">
         <v/>
@@ -5797,10 +5960,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C77" t="str">
-        <v>Bundle Price</v>
+        <v>Bundle Original Price</v>
       </c>
       <c r="D77" t="str">
-        <v>{{BUNDLE_PRICE}}</v>
+        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
       </c>
       <c r="E77" t="str">
         <v/>
@@ -5814,10 +5977,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C78" t="str">
-        <v>Bundle Discount</v>
+        <v>Bundle Price</v>
       </c>
       <c r="D78" t="str">
-        <v>{{BUNDLE_DISCOUNT}}</v>
+        <v>{{BUNDLE_PRICE}}</v>
       </c>
       <c r="E78" t="str">
         <v/>
@@ -5831,10 +5994,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C79" t="str">
-        <v>Today You Pay Price</v>
+        <v>Bundle Discount</v>
       </c>
       <c r="D79" t="str">
-        <v>{{BUNDLE_TODAY_YOU_PAY_STANDARD}}</v>
+        <v>{{BUNDLE_DISCOUNT}}</v>
       </c>
       <c r="E79" t="str">
         <v/>
@@ -5848,10 +6011,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C80" t="str">
-        <v>Cancellation Text</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D80" t="str">
-        <v>{{CANCELLATION_TEXT_ANNUAL}}</v>
+        <v>{{BUNDLE_TODAY_YOU_PAY_STANDARD}}</v>
       </c>
       <c r="E80" t="str">
         <v/>
@@ -5865,10 +6028,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C81" t="str">
-        <v>Ultimate Upsell Text</v>
+        <v>Cancellation Text</v>
       </c>
       <c r="D81" t="str">
-        <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
+        <v>{{CANCELLATION_TEXT_ANNUAL}}</v>
       </c>
       <c r="E81" t="str">
         <v/>
@@ -5876,16 +6039,16 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>Ultimate</v>
+        <v>Standard</v>
       </c>
       <c r="B82" t="str">
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C82" t="str">
-        <v>Page Title</v>
+        <v>Ultimate Upsell Text</v>
       </c>
       <c r="D82" t="str">
-        <v>Choose how to pay</v>
+        <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
       <c r="E82" t="str">
         <v/>
@@ -5899,10 +6062,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C83" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D83" t="str">
-        <v>DAZN Ultimate</v>
+        <v>Choose how to pay</v>
       </c>
       <c r="E83" t="str">
         <v/>
@@ -5916,10 +6079,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C84" t="str">
-        <v>Rate Plan</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D84" t="str">
-        <v>Annual - Pay Monthly</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="E84" t="str">
         <v/>
@@ -5933,10 +6096,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C85" t="str">
-        <v>Rate Plan Price</v>
+        <v>Rate Plan</v>
       </c>
       <c r="D85" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
+        <v>Annual - Pay Monthly</v>
       </c>
       <c r="E85" t="str">
         <v/>
@@ -5950,10 +6113,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C86" t="str">
-        <v>Bundle Name</v>
+        <v>Rate Plan Price</v>
       </c>
       <c r="D86" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
       </c>
       <c r="E86" t="str">
         <v/>
@@ -5967,10 +6130,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C87" t="str">
-        <v>Bundle Price</v>
+        <v>Bundle Name</v>
       </c>
       <c r="D87" t="str">
-        <v>{{CURRENCY}}0</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="E87" t="str">
         <v/>
@@ -5984,10 +6147,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C88" t="str">
-        <v>Today You Pay Price</v>
+        <v>Bundle Price</v>
       </c>
       <c r="D88" t="str">
-        <v>{{TODAY_YOU_PAY_PRICE}}</v>
+        <v>{{CURRENCY}}0</v>
       </c>
       <c r="E88" t="str">
         <v/>
@@ -6001,10 +6164,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C89" t="str">
-        <v>Next Payment Label</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D89" t="str">
-        <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
+        <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
       <c r="E89" t="str">
         <v/>
@@ -6018,10 +6181,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C90" t="str">
-        <v>Next Payment Price</v>
+        <v>Next Payment Label</v>
       </c>
       <c r="D90" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
+        <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
       <c r="E90" t="str">
         <v/>
@@ -6035,10 +6198,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C91" t="str">
-        <v>Cancellation Text</v>
+        <v>Next Payment Price</v>
       </c>
       <c r="D91" t="str">
-        <v>{{CANCELLATION_TEXT}}</v>
+        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
       </c>
       <c r="E91" t="str">
         <v/>
@@ -6052,10 +6215,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C92" t="str">
-        <v>Discount Badge</v>
+        <v>Cancellation Text</v>
       </c>
       <c r="D92" t="str">
-        <v>{{DISCOUNT_BADGE}}</v>
+        <v>{{CANCELLATION_TEXT}}</v>
       </c>
       <c r="E92" t="str">
         <v/>
@@ -6066,13 +6229,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B93" t="str">
-        <v>Annual Pay Upfront Bundle</v>
+        <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C93" t="str">
-        <v>Page Title</v>
+        <v>Discount Badge</v>
       </c>
       <c r="D93" t="str">
-        <v>Choose how to pay</v>
+        <v>{{DISCOUNT_BADGE}}</v>
       </c>
       <c r="E93" t="str">
         <v/>
@@ -6086,10 +6249,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C94" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D94" t="str">
-        <v>DAZN Ultimate</v>
+        <v>Choose how to pay</v>
       </c>
       <c r="E94" t="str">
         <v/>
@@ -6103,10 +6266,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C95" t="str">
-        <v>Rate Plan</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D95" t="str">
-        <v>Annual - Pay Upfront</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="E95" t="str">
         <v/>
@@ -6120,10 +6283,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C96" t="str">
-        <v>Rate Plan Price</v>
+        <v>Rate Plan</v>
       </c>
       <c r="D96" t="str">
-        <v>{{ANNUAL_UPFRONT_PRICE}}/year</v>
+        <v>Annual - Pay Upfront</v>
       </c>
       <c r="E96" t="str">
         <v/>
@@ -6137,10 +6300,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C97" t="str">
-        <v>Save Badge</v>
+        <v>Rate Plan Price</v>
       </c>
       <c r="D97" t="str">
-        <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
+        <v>{{ANNUAL_UPFRONT_PRICE}}/year</v>
       </c>
       <c r="E97" t="str">
         <v/>
@@ -6154,10 +6317,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C98" t="str">
-        <v>Bundle Name</v>
+        <v>Save Badge</v>
       </c>
       <c r="D98" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
       </c>
       <c r="E98" t="str">
         <v/>
@@ -6171,10 +6334,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C99" t="str">
-        <v>Bundle Price</v>
+        <v>Bundle Name</v>
       </c>
       <c r="D99" t="str">
-        <v>{{CURRENCY}}0</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="E99" t="str">
         <v/>
@@ -6188,10 +6351,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C100" t="str">
-        <v>Today You Pay Price</v>
+        <v>Bundle Price</v>
       </c>
       <c r="D100" t="str">
-        <v>{{ANNUAL_UPFRONT_PRICE}}</v>
+        <v>{{CURRENCY}}0</v>
       </c>
       <c r="E100" t="str">
         <v/>
@@ -6205,10 +6368,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C101" t="str">
-        <v>Next Payment Label</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D101" t="str">
-        <v>Next Annual payment on {{NEXT_PAYMENT_DATE}}</v>
+        <v>{{ANNUAL_UPFRONT_PRICE}}</v>
       </c>
       <c r="E101" t="str">
         <v/>
@@ -6222,10 +6385,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C102" t="str">
-        <v>Next Payment Price</v>
+        <v>Next Payment Label</v>
       </c>
       <c r="D102" t="str">
-        <v>{{ANNUAL_UPFRONT_PRICE}}</v>
+        <v>Next Annual payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
       <c r="E102" t="str">
         <v/>
@@ -6239,28 +6402,45 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C103" t="str">
+        <v>Next Payment Price</v>
+      </c>
+      <c r="D103" t="str">
+        <v>{{ANNUAL_UPFRONT_PRICE}}</v>
+      </c>
+      <c r="E103" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>Ultimate</v>
+      </c>
+      <c r="B104" t="str">
+        <v>Annual Pay Upfront Bundle</v>
+      </c>
+      <c r="C104" t="str">
         <v>Cancellation Text</v>
       </c>
-      <c r="D103" t="str">
+      <c r="D104" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
-      <c r="E103" t="str">
+      <c r="E104" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E103"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E104"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B7"/>
   <cols>
-    <col min="1" max="1" width="27.83203125" customWidth="1"/>
-    <col min="2" max="2" width="90.83203125" customWidth="1"/>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6319,73 +6499,9 @@
         <v>{{PPV_PROMOTER}}</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Popup Image Present</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Popup Date</v>
-      </c>
-      <c r="B9" t="str">
-        <v>{{PPV_DATE}}</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Popup PPV Name</v>
-      </c>
-      <c r="B10" t="str">
-        <v>{{PPV_NAME}}</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Popup Promoter</v>
-      </c>
-      <c r="B11" t="str">
-        <v>{{PPV_PROMOTER}}</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Popup Description</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Popup Buy Now CTA Present</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Popup Buy Now CTA Text</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Buy now</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>Popup Close Button</v>
-      </c>
-      <c r="B15" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: fix ultimate tier selection on contextual PPV page for active standard users
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -948,11 +948,11 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C13"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="25.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -996,7 +996,7 @@
         <v>Banner - Event Date</v>
       </c>
       <c r="C4" t="str">
-        <v>{{PPV_DATE}}</v>
+        <v>{{LANDING_BANNER_DATE}}</v>
       </c>
     </row>
     <row r="5">
@@ -1067,135 +1067,47 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>home-boxing-tile</v>
+        <v>home-kickboxing-tile</v>
       </c>
       <c r="B11" t="str">
-        <v>Event Date</v>
+        <v>Home of Boxing Section Present</v>
       </c>
       <c r="C11" t="str">
-        <v>{{PPV_DATE}}</v>
+        <v>Present</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>home-boxing-tile</v>
+        <v>home-kickboxing-tile</v>
       </c>
       <c r="B12" t="str">
-        <v>Promoter</v>
+        <v>Selected Boxing Tile</v>
       </c>
       <c r="C12" t="str">
-        <v>{{PPV_PROMOTER}}</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>home-boxing-tile</v>
+        <v>home-kickboxing-tile</v>
       </c>
       <c r="B13" t="str">
-        <v>PPV Badge</v>
+        <v>Event Title</v>
       </c>
       <c r="C13" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>home-boxing-tile</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Lock Icon</v>
-      </c>
-      <c r="C14" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>home-kickboxing-tile</v>
-      </c>
-      <c r="B15" t="str">
-        <v>Home of Boxing Section Present</v>
-      </c>
-      <c r="C15" t="str">
-        <v>Present</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>home-kickboxing-tile</v>
-      </c>
-      <c r="B16" t="str">
-        <v>Selected Boxing Tile</v>
-      </c>
-      <c r="C16" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>home-kickboxing-tile</v>
-      </c>
-      <c r="B17" t="str">
-        <v>Event Title</v>
-      </c>
-      <c r="C17" t="str">
         <v>{{PPV_NAME}}</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>home-kickboxing-tile</v>
-      </c>
-      <c r="B18" t="str">
-        <v>Event Date</v>
-      </c>
-      <c r="C18" t="str">
-        <v>{{PPV_DATE}}</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>home-kickboxing-tile</v>
-      </c>
-      <c r="B19" t="str">
-        <v>Promoter</v>
-      </c>
-      <c r="C19" t="str">
-        <v>{{PPV_PROMOTER}}</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>home-kickboxing-tile</v>
-      </c>
-      <c r="B20" t="str">
-        <v>PPV Badge</v>
-      </c>
-      <c r="C20" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>home-kickboxing-tile</v>
-      </c>
-      <c r="B21" t="str">
-        <v>Lock Icon</v>
-      </c>
-      <c r="C21" t="str">
-        <v>Yes</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C13"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C17"/>
   <cols>
     <col min="1" max="1" width="21.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -1295,65 +1207,65 @@
         <v>home-page-dont-miss</v>
       </c>
       <c r="B9" t="str">
-        <v>Don't Miss Event Title</v>
+        <v>Locked Badge Present</v>
       </c>
       <c r="C9" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>home-page-dont-miss</v>
+        <v>home-biggest-fights</v>
       </c>
       <c r="B10" t="str">
-        <v>Don't Miss Event Date</v>
+        <v>Biggest Fights Section Present</v>
       </c>
       <c r="C10" t="str">
-        <v>{{PPV_DATE}}</v>
+        <v>Present</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>home-page-dont-miss</v>
+        <v>home-biggest-fights</v>
       </c>
       <c r="B11" t="str">
-        <v>Don't Miss Promoter</v>
+        <v>Biggest Fights Tile Present</v>
       </c>
       <c r="C11" t="str">
-        <v>{{PPV_PROMOTER}}</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>home-page-dont-miss</v>
+        <v>home-biggest-fights</v>
       </c>
       <c r="B12" t="str">
-        <v>PPV Badge Present</v>
+        <v>Event Title</v>
       </c>
       <c r="C12" t="str">
-        <v>Yes</v>
+        <v>{{PPV_NAME}}</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>home-page-dont-miss</v>
+        <v>home-biggest-fights</v>
       </c>
       <c r="B13" t="str">
-        <v>Locked Badge Present</v>
+        <v>Event Date</v>
       </c>
       <c r="C13" t="str">
-        <v>Yes</v>
+        <v>{{PPV_DATE}}</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>home-page-dont-miss</v>
+        <v>home-biggest-fights</v>
       </c>
       <c r="B14" t="str">
-        <v>Reminder Icon Present</v>
+        <v>Promoter</v>
       </c>
       <c r="C14" t="str">
-        <v>Yes</v>
+        <v>{{PPV_PROMOTER}}</v>
       </c>
     </row>
     <row r="15">
@@ -1361,10 +1273,10 @@
         <v>home-biggest-fights</v>
       </c>
       <c r="B15" t="str">
-        <v>Biggest Fights Section Present</v>
+        <v>PPV Badge</v>
       </c>
       <c r="C15" t="str">
-        <v>Present</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="16">
@@ -1372,7 +1284,7 @@
         <v>home-biggest-fights</v>
       </c>
       <c r="B16" t="str">
-        <v>Biggest Fights Tile Present</v>
+        <v>Lock Icon</v>
       </c>
       <c r="C16" t="str">
         <v>Yes</v>
@@ -1383,70 +1295,15 @@
         <v>home-biggest-fights</v>
       </c>
       <c r="B17" t="str">
-        <v>Event Title</v>
+        <v>Reminder Icon</v>
       </c>
       <c r="C17" t="str">
-        <v>{{PPV_NAME}}</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>home-biggest-fights</v>
-      </c>
-      <c r="B18" t="str">
-        <v>Event Date</v>
-      </c>
-      <c r="C18" t="str">
-        <v>{{PPV_DATE}}</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>home-biggest-fights</v>
-      </c>
-      <c r="B19" t="str">
-        <v>Promoter</v>
-      </c>
-      <c r="C19" t="str">
-        <v>{{PPV_PROMOTER}}</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>home-biggest-fights</v>
-      </c>
-      <c r="B20" t="str">
-        <v>PPV Badge</v>
-      </c>
-      <c r="C20" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>home-biggest-fights</v>
-      </c>
-      <c r="B21" t="str">
-        <v>Lock Icon</v>
-      </c>
-      <c r="C21" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>home-biggest-fights</v>
-      </c>
-      <c r="B22" t="str">
-        <v>Reminder Icon</v>
-      </c>
-      <c r="C22" t="str">
         <v>Yes</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C17"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4116,7 +3973,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D38"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -4255,10 +4112,10 @@
         <v>Standard</v>
       </c>
       <c r="B10" t="str">
-        <v>Annual Card Present</v>
+        <v>Flex Future Date</v>
       </c>
       <c r="C10" t="str">
-        <v>Yes</v>
+        <v>{{FLEX_FUTURE_DATE}}</v>
       </c>
       <c r="D10" t="str">
         <v/>
@@ -4269,10 +4126,10 @@
         <v>Standard</v>
       </c>
       <c r="B11" t="str">
-        <v>Annual Savings Badge</v>
+        <v>Annual Card Present</v>
       </c>
       <c r="C11" t="str">
-        <v>{{ANNUAL_SAVINGS_BADGE}}</v>
+        <v>Yes</v>
       </c>
       <c r="D11" t="str">
         <v/>
@@ -4283,10 +4140,10 @@
         <v>Standard</v>
       </c>
       <c r="B12" t="str">
-        <v>Annual Title</v>
+        <v>Annual Savings Badge</v>
       </c>
       <c r="C12" t="str">
-        <v>Annual - Pay Monthly</v>
+        <v>{{ANNUAL_SAVINGS_BADGE}}</v>
       </c>
       <c r="D12" t="str">
         <v/>
@@ -4297,10 +4154,10 @@
         <v>Standard</v>
       </c>
       <c r="B13" t="str">
-        <v>Annual Badge</v>
+        <v>Annual Title</v>
       </c>
       <c r="C13" t="str">
-        <v>1 MONTH FREE</v>
+        <v>Annual - Pay Monthly</v>
       </c>
       <c r="D13" t="str">
         <v/>
@@ -4311,10 +4168,10 @@
         <v>Standard</v>
       </c>
       <c r="B14" t="str">
-        <v>Annual Price Text</v>
+        <v>Annual Badge</v>
       </c>
       <c r="C14" t="str">
-        <v>then {{CURRENCY}}{{ANNUAL_PRICE}}/month for {{ANNUAL_MONTHS}} months</v>
+        <v>1 MONTH FREE</v>
       </c>
       <c r="D14" t="str">
         <v/>
@@ -4325,10 +4182,10 @@
         <v>Standard</v>
       </c>
       <c r="B15" t="str">
-        <v>Annual Contract Text</v>
+        <v>Annual Price Text</v>
       </c>
       <c r="C15" t="str">
-        <v>Annual contract. Auto renews.</v>
+        <v>then {{CURRENCY}}{{ANNUAL_PRICE}}/month for {{ANNUAL_MONTHS}} months</v>
       </c>
       <c r="D15" t="str">
         <v/>
@@ -4339,10 +4196,10 @@
         <v>Standard</v>
       </c>
       <c r="B16" t="str">
-        <v>Annual Feature 1</v>
+        <v>Annual Contract Text</v>
       </c>
       <c r="C16" t="str">
-        <v>185+ fights a year from the world's best promoters.</v>
+        <v>Annual contract. Auto renews.</v>
       </c>
       <c r="D16" t="str">
         <v/>
@@ -4353,10 +4210,10 @@
         <v>Standard</v>
       </c>
       <c r="B17" t="str">
-        <v>Annual Feature 2</v>
+        <v>Annual Feature 1</v>
       </c>
       <c r="C17" t="str">
-        <v>Additional cost for pay-per-view events.</v>
+        <v>185+ fights a year from the world's best promoters.</v>
       </c>
       <c r="D17" t="str">
         <v/>
@@ -4367,10 +4224,10 @@
         <v>Standard</v>
       </c>
       <c r="B18" t="str">
-        <v>Annual Feature 3</v>
+        <v>Annual Feature 2</v>
       </c>
       <c r="C18" t="str">
-        <v>Full HD video resolution.</v>
+        <v>Additional cost for pay-per-view events.</v>
       </c>
       <c r="D18" t="str">
         <v/>
@@ -4381,10 +4238,10 @@
         <v>Standard</v>
       </c>
       <c r="B19" t="str">
-        <v>Annual Selected</v>
+        <v>Annual Feature 3</v>
       </c>
       <c r="C19" t="str">
-        <v>No</v>
+        <v>Full HD video resolution.</v>
       </c>
       <c r="D19" t="str">
         <v/>
@@ -4395,10 +4252,10 @@
         <v>Standard</v>
       </c>
       <c r="B20" t="str">
-        <v>CTA Button</v>
+        <v>Annual Selected</v>
       </c>
       <c r="C20" t="str">
-        <v>{{PLAN_CTA_BUTTON}}</v>
+        <v>No</v>
       </c>
       <c r="D20" t="str">
         <v/>
@@ -4406,13 +4263,13 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Ultimate</v>
+        <v>Standard</v>
       </c>
       <c r="B21" t="str">
-        <v>Page Title</v>
+        <v>CTA Button</v>
       </c>
       <c r="C21" t="str">
-        <v>{{PLAN_PAGE_TITLE}}</v>
+        <v>{{PLAN_CTA_BUTTON}}</v>
       </c>
       <c r="D21" t="str">
         <v/>
@@ -4423,10 +4280,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B22" t="str">
-        <v>Annual Pay Monthly Option</v>
+        <v>Page Title</v>
       </c>
       <c r="C22" t="str">
-        <v>Yes</v>
+        <v>{{PLAN_PAGE_TITLE}}</v>
       </c>
       <c r="D22" t="str">
         <v/>
@@ -4437,10 +4294,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B23" t="str">
-        <v>Annual Pay Monthly Title</v>
+        <v>Annual Pay Monthly Option</v>
       </c>
       <c r="C23" t="str">
-        <v>Annual - Pay Monthly</v>
+        <v>Yes</v>
       </c>
       <c r="D23" t="str">
         <v/>
@@ -4451,10 +4308,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B24" t="str">
-        <v>Annual Pay Monthly Price</v>
+        <v>Annual Pay Monthly Title</v>
       </c>
       <c r="C24" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
+        <v>Annual - Pay Monthly</v>
       </c>
       <c r="D24" t="str">
         <v/>
@@ -4465,10 +4322,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B25" t="str">
-        <v>Annual Pay Monthly Price Length</v>
+        <v>Annual Pay Monthly Price</v>
       </c>
       <c r="C25" t="str">
-        <v>/month</v>
+        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
       </c>
       <c r="D25" t="str">
         <v/>
@@ -4479,10 +4336,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B26" t="str">
-        <v>Annual Pay Monthly Contract Text</v>
+        <v>Annual Pay Monthly Price Length</v>
       </c>
       <c r="C26" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_CONTRACT_TEXT}}</v>
+        <v>/month</v>
       </c>
       <c r="D26" t="str">
         <v/>
@@ -4493,10 +4350,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B27" t="str">
-        <v>Annual Pay Monthly Selected</v>
+        <v>Annual Pay Monthly Contract Text</v>
       </c>
       <c r="C27" t="str">
-        <v>Yes</v>
+        <v>{{ANNUAL_PAY_MONTHLY_CONTRACT_TEXT}}</v>
       </c>
       <c r="D27" t="str">
         <v/>
@@ -4507,7 +4364,7 @@
         <v>Ultimate</v>
       </c>
       <c r="B28" t="str">
-        <v>Annual Pay Upfront Option</v>
+        <v>Annual Pay Monthly Selected</v>
       </c>
       <c r="C28" t="str">
         <v>Yes</v>
@@ -4521,10 +4378,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B29" t="str">
-        <v>Annual Pay Upfront Title</v>
+        <v>Annual Pay Upfront Option</v>
       </c>
       <c r="C29" t="str">
-        <v>Annual - Pay Upfront</v>
+        <v>Yes</v>
       </c>
       <c r="D29" t="str">
         <v/>
@@ -4535,10 +4392,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B30" t="str">
-        <v>Annual Pay Upfront Save Badge</v>
+        <v>Annual Pay Upfront Title</v>
       </c>
       <c r="C30" t="str">
-        <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
+        <v>Annual - Pay Upfront</v>
       </c>
       <c r="D30" t="str">
         <v/>
@@ -4549,10 +4406,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B31" t="str">
-        <v>Annual Pay Upfront Price</v>
+        <v>Annual Pay Upfront Save Badge</v>
       </c>
       <c r="C31" t="str">
-        <v>{{ANNUAL_UPFRONT_PRICE_DISPLAY}}</v>
+        <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
       </c>
       <c r="D31" t="str">
         <v/>
@@ -4563,10 +4420,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B32" t="str">
-        <v>Annual Pay Upfront Price Length</v>
+        <v>Annual Pay Upfront Price</v>
       </c>
       <c r="C32" t="str">
-        <v>/year</v>
+        <v>{{ANNUAL_UPFRONT_PRICE_DISPLAY}}</v>
       </c>
       <c r="D32" t="str">
         <v/>
@@ -4577,10 +4434,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B33" t="str">
-        <v>Annual Pay Upfront Selected</v>
+        <v>Annual Pay Upfront Price Length</v>
       </c>
       <c r="C33" t="str">
-        <v>No</v>
+        <v>/year</v>
       </c>
       <c r="D33" t="str">
         <v/>
@@ -4591,10 +4448,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B34" t="str">
-        <v>Ultimate Feature 1</v>
+        <v>Annual Pay Upfront Selected</v>
       </c>
       <c r="C34" t="str">
-        <v>{{ULTIMATE_FEATURE_1}}</v>
+        <v>No</v>
       </c>
       <c r="D34" t="str">
         <v/>
@@ -4605,10 +4462,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B35" t="str">
-        <v>Ultimate Feature 2</v>
+        <v>Ultimate Feature 1</v>
       </c>
       <c r="C35" t="str">
-        <v>{{ULTIMATE_FEATURE_2}}</v>
+        <v>{{ULTIMATE_FEATURE_1}}</v>
       </c>
       <c r="D35" t="str">
         <v/>
@@ -4619,10 +4476,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B36" t="str">
-        <v>Ultimate Feature 3</v>
+        <v>Ultimate Feature 2</v>
       </c>
       <c r="C36" t="str">
-        <v>{{ULTIMATE_FEATURE_3}}</v>
+        <v>{{ULTIMATE_FEATURE_2}}</v>
       </c>
       <c r="D36" t="str">
         <v/>
@@ -4633,18 +4490,32 @@
         <v>Ultimate</v>
       </c>
       <c r="B37" t="str">
+        <v>Ultimate Feature 3</v>
+      </c>
+      <c r="C37" t="str">
+        <v>{{ULTIMATE_FEATURE_3}}</v>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Ultimate</v>
+      </c>
+      <c r="B38" t="str">
         <v>CTA Button</v>
       </c>
-      <c r="C37" t="str">
+      <c r="C38" t="str">
         <v>{{PLAN_CTA_BUTTON}}</v>
       </c>
-      <c r="D37" t="str">
+      <c r="D38" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D38"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: add PPV Description Text validation on PPV Payment page — validates actual text against BANNER_DESCRIPTION
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -6665,7 +6665,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <cols>
     <col min="1" max="1" width="29.83203125" customWidth="1"/>
     <col min="2" max="2" width="79.83203125" customWidth="1"/>
@@ -6705,55 +6705,55 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>PPV Image Present</v>
+        <v>PPV Description Text</v>
       </c>
       <c r="B5" t="str">
-        <v>Yes</v>
+        <v>{{BANNER_DESCRIPTION}}</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>PPV Date and Time</v>
+        <v>PPV Image Present</v>
       </c>
       <c r="B6" t="str">
-        <v>{{PPV_DATE}}</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Order Summary PPV Name</v>
+        <v>PPV Date and Time</v>
       </c>
       <c r="B7" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>{{PPV_DATE}}</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Today You Pay Text</v>
+        <v>Order Summary PPV Name</v>
       </c>
       <c r="B8" t="str">
-        <v>Today you pay</v>
+        <v>{{PPV_NAME}}</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Today You Pay Price</v>
+        <v>Today You Pay Text</v>
       </c>
       <c r="B9" t="str">
-        <v>{{PPV_PRICE}}</v>
+        <v>Today you pay</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Payment Method Present</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="B10" t="str">
-        <v>Yes</v>
+        <v>{{PPV_PRICE}}</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Pay Now Button</v>
+        <v>Payment Method Present</v>
       </c>
       <c r="B11" t="str">
         <v>Yes</v>
@@ -6761,7 +6761,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Secure Checkout</v>
+        <v>Pay Now Button</v>
       </c>
       <c r="B12" t="str">
         <v>Yes</v>
@@ -6769,7 +6769,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>More Payment Methods</v>
+        <v>Secure Checkout</v>
       </c>
       <c r="B13" t="str">
         <v>Yes</v>
@@ -6777,7 +6777,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Legal Text Present</v>
+        <v>More Payment Methods</v>
       </c>
       <c r="B14" t="str">
         <v>Yes</v>
@@ -6785,7 +6785,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Terms Link Present</v>
+        <v>Legal Text Present</v>
       </c>
       <c r="B15" t="str">
         <v>Yes</v>
@@ -6793,7 +6793,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Privacy Policy Link Present</v>
+        <v>Terms Link Present</v>
       </c>
       <c r="B16" t="str">
         <v>Yes</v>
@@ -6801,23 +6801,31 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Payment Type</v>
+        <v>Privacy Policy Link Present</v>
       </c>
       <c r="B17" t="str">
-        <v>One time payment</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
+        <v>Payment Type</v>
+      </c>
+      <c r="B18" t="str">
+        <v>One time payment</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
         <v>Payment Instruction Text</v>
       </c>
-      <c r="B18" t="str">
+      <c r="B19" t="str">
         <v>In order to purchase this event, please choose from the payment options below</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B19"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: add home-boxing-upcoming flow to Home of Boxing sheet — stops wrong tile/banner validation
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -948,7 +948,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C15"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -1067,7 +1067,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>home-kickboxing-tile</v>
+        <v>home-boxing-upcoming</v>
       </c>
       <c r="B11" t="str">
         <v>Home of Boxing Section Present</v>
@@ -1078,13 +1078,13 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>home-kickboxing-tile</v>
+        <v>home-boxing-upcoming</v>
       </c>
       <c r="B12" t="str">
-        <v>Selected Boxing Tile</v>
+        <v>Event Title</v>
       </c>
       <c r="C12" t="str">
-        <v>Yes</v>
+        <v>{{PPV_NAME}}</v>
       </c>
     </row>
     <row r="13">
@@ -1092,15 +1092,37 @@
         <v>home-kickboxing-tile</v>
       </c>
       <c r="B13" t="str">
+        <v>Home of Boxing Section Present</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Present</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>home-kickboxing-tile</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Selected Boxing Tile</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>home-kickboxing-tile</v>
+      </c>
+      <c r="B15" t="str">
         <v>Event Title</v>
       </c>
-      <c r="C13" t="str">
+      <c r="C15" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C15"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: social auth, subscribe-without-PPV flow, validation fixes & config updates
- Add AuthenticationManager with Google/Apple/Facebook/FIFA login support
- Add 'subscribe-without-pay-per-view' surfacing point with noPpvClick flow
- Update aj_joshua_prenga event config (location, dates, formatting)
- Fix Next Payment skip region: IT → IE (Ireland)
- Remove Saturday Badge validation (field no longer used)
- Add Excluding Tax text support (US region)
- Add Terms & Conditions text validation for Upgrade Confirmation
- Add annual plan selection (APM/APU) dynamic resolution
- Fix flex future date regex for US date format
- Improve banner description extraction (3-strategy approach)
- Add dotenv import in playwright.config.ts
- Update prod credentials in userstatus.json
- Integrate social login mid-flow in both new-user and existing-user specs
- Fix PaymentPage next payment validation (early return for GB/IE)
- Add error handling for MyAccountPage mid-page scroll
- Update PPV_Input.xlsx
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -416,6 +416,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C12"/>
+  <cols>
+    <col min="1" max="1" width="33.83203125" customWidth="1"/>
+    <col min="2" max="2" width="27.83203125" customWidth="1"/>
+    <col min="3" max="3" width="21.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -430,7 +435,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Don&amp;apos;t Miss Live on DAZN Section</v>
+        <v>Don't Miss Live on DAZN Section</v>
       </c>
       <c r="B2" t="str">
         <v>Yes</v>
@@ -550,7 +555,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:C12"/>
   </ignoredErrors>
@@ -559,7 +563,12 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="27.83203125" customWidth="1"/>
+    <col min="3" max="3" width="318.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -599,10 +608,10 @@
         <v>common</v>
       </c>
       <c r="B4" t="str">
-        <v>Payment Method Present</v>
+        <v>Terms And Conditions Text</v>
       </c>
       <c r="C4" t="str">
-        <v>Yes</v>
+        <v>By changing the terms of your subscription, you confirm that you have read and agree to our Terms and Conditions of Use (including the instruction regarding your right of withdrawal). Your subscription auto-renews unless you cancel before the end of the minimum term by selecting 'Cancel Subscription' in My Account.</v>
       </c>
     </row>
     <row r="5">
@@ -610,10 +619,10 @@
         <v>common</v>
       </c>
       <c r="B5" t="str">
-        <v>Confirm Button</v>
+        <v>Payment Method Present</v>
       </c>
       <c r="C5" t="str">
-        <v>Confirm</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="6">
@@ -621,21 +630,21 @@
         <v>common</v>
       </c>
       <c r="B6" t="str">
-        <v>Terms Link Present</v>
+        <v>Confirm Button</v>
       </c>
       <c r="C6" t="str">
-        <v>Yes</v>
+        <v>Confirm</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>annual pay upfront</v>
+        <v>common</v>
       </c>
       <c r="B7" t="str">
-        <v>Legal Text Line 1</v>
+        <v>Terms Link Present</v>
       </c>
       <c r="C7" t="str">
-        <v>Your plan will be changed to DAZN Ultimate today {{TODAY_DATE}} and your contract will last 12 months.</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="8">
@@ -643,10 +652,10 @@
         <v>annual pay upfront</v>
       </c>
       <c r="B8" t="str">
-        <v>Legal Text Line 2</v>
+        <v>Legal Text Line 1</v>
       </c>
       <c r="C8" t="str">
-        <v>Today you will be charged {{CURRENCY}}{{ANNUAL_UPFRONT_PRICE}} minus the remainder of your last payment which was not used in full. From {{NEXT_PAYMENT_DATE}} you will be charged {{CURRENCY}}{{ANNUAL_UPFRONT_PRICE}}/year.</v>
+        <v>Your plan will be changed to DAZN Ultimate today {{TODAY_DATE}} and your contract will last 12 months.</v>
       </c>
     </row>
     <row r="9">
@@ -654,10 +663,10 @@
         <v>annual pay upfront</v>
       </c>
       <c r="B9" t="str">
-        <v>Rate Plan</v>
+        <v>Legal Text Line 2</v>
       </c>
       <c r="C9" t="str">
-        <v>Annual - Pay Upfront</v>
+        <v>Today you will be charged {{CURRENCY}}{{ANNUAL_UPFRONT_PRICE}} minus the remainder of your last payment which was not used in full. From {{NEXT_PAYMENT_DATE}} you will be charged {{CURRENCY}}{{ANNUAL_UPFRONT_PRICE}}/year.</v>
       </c>
     </row>
     <row r="10">
@@ -665,10 +674,10 @@
         <v>annual pay upfront</v>
       </c>
       <c r="B10" t="str">
-        <v>Rate Plan Price</v>
+        <v>Rate Plan</v>
       </c>
       <c r="C10" t="str">
-        <v>{{ANNUAL_UPFRONT_PRICE}}</v>
+        <v>Annual - Pay Upfront</v>
       </c>
     </row>
     <row r="11">
@@ -676,10 +685,10 @@
         <v>annual pay upfront</v>
       </c>
       <c r="B11" t="str">
-        <v>Rate Plan Period</v>
+        <v>Rate Plan Price</v>
       </c>
       <c r="C11" t="str">
-        <v>/year</v>
+        <v>{{ANNUAL_UPFRONT_PRICE}}</v>
       </c>
     </row>
     <row r="12">
@@ -687,10 +696,10 @@
         <v>annual pay upfront</v>
       </c>
       <c r="B12" t="str">
-        <v>Rate Plan Description</v>
+        <v>Rate Plan Period</v>
       </c>
       <c r="C12" t="str">
-        <v>Get the best value when you pay upfront.</v>
+        <v>/year</v>
       </c>
     </row>
     <row r="13">
@@ -698,10 +707,10 @@
         <v>annual pay upfront</v>
       </c>
       <c r="B13" t="str">
-        <v>Next Payment Label</v>
+        <v>Rate Plan Description</v>
       </c>
       <c r="C13" t="str">
-        <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
+        <v>Get the best value when you pay upfront.</v>
       </c>
     </row>
     <row r="14">
@@ -709,21 +718,21 @@
         <v>annual pay upfront</v>
       </c>
       <c r="B14" t="str">
-        <v>Next Payment Date</v>
+        <v>Next Payment Label</v>
       </c>
       <c r="C14" t="str">
-        <v>{{NEXT_PAYMENT_DATE}}</v>
+        <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>annual pay monthly</v>
+        <v>annual pay upfront</v>
       </c>
       <c r="B15" t="str">
-        <v>Legal Text Line 1</v>
+        <v>Next Payment Date</v>
       </c>
       <c r="C15" t="str">
-        <v>Your plan will be changed to DAZN Ultimate today {{TODAY_DATE}} and your contract will last 12 months.</v>
+        <v>{{NEXT_PAYMENT_DATE}}</v>
       </c>
     </row>
     <row r="16">
@@ -731,10 +740,10 @@
         <v>annual pay monthly</v>
       </c>
       <c r="B16" t="str">
-        <v>Legal Text Line 2</v>
+        <v>Legal Text Line 1</v>
       </c>
       <c r="C16" t="str">
-        <v>Today you will be charged {{CURRENCY}}{{ANNUAL_PAY_MONTHLY_PRICE}} minus the remainder of your last payment which was not used in full. From {{NEXT_PAYMENT_DATE}} you will be charged {{CURRENCY}}{{ANNUAL_PAY_MONTHLY_PRICE}} /month.</v>
+        <v>Your plan will be changed to DAZN Ultimate today {{TODAY_DATE}} and your contract will last 12 months.</v>
       </c>
     </row>
     <row r="17">
@@ -742,10 +751,10 @@
         <v>annual pay monthly</v>
       </c>
       <c r="B17" t="str">
-        <v>Rate Plan</v>
+        <v>Legal Text Line 2</v>
       </c>
       <c r="C17" t="str">
-        <v>Annual - Pay Monthly</v>
+        <v>Today you will be charged {{CURRENCY}}{{ANNUAL_PAY_MONTHLY_PRICE}} minus the remainder of your last payment which was not used in full. From {{NEXT_PAYMENT_DATE}} you will be charged {{CURRENCY}}{{ANNUAL_PAY_MONTHLY_PRICE}} /month.</v>
       </c>
     </row>
     <row r="18">
@@ -753,10 +762,10 @@
         <v>annual pay monthly</v>
       </c>
       <c r="B18" t="str">
-        <v>Rate Plan Price</v>
+        <v>Rate Plan</v>
       </c>
       <c r="C18" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
+        <v>Annual - Pay Monthly</v>
       </c>
     </row>
     <row r="19">
@@ -764,10 +773,10 @@
         <v>annual pay monthly</v>
       </c>
       <c r="B19" t="str">
-        <v>Rate Plan Period</v>
+        <v>Rate Plan Price</v>
       </c>
       <c r="C19" t="str">
-        <v>/ month</v>
+        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
       </c>
     </row>
     <row r="20">
@@ -775,10 +784,10 @@
         <v>annual pay monthly</v>
       </c>
       <c r="B20" t="str">
-        <v>Rate Plan Description</v>
+        <v>Rate Plan Period</v>
       </c>
       <c r="C20" t="str">
-        <v>Annual contract. Paid in 12 monthly instalments.</v>
+        <v>/ month</v>
       </c>
     </row>
     <row r="21">
@@ -786,10 +795,10 @@
         <v>annual pay monthly</v>
       </c>
       <c r="B21" t="str">
-        <v>Next Payment Label</v>
+        <v>Rate Plan Description</v>
       </c>
       <c r="C21" t="str">
-        <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
+        <v>Annual contract. Paid in 12 monthly instalments.</v>
       </c>
     </row>
     <row r="22">
@@ -797,16 +806,26 @@
         <v>annual pay monthly</v>
       </c>
       <c r="B22" t="str">
+        <v>Next Payment Label</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>annual pay monthly</v>
+      </c>
+      <c r="B23" t="str">
         <v>Next Payment Date</v>
       </c>
-      <c r="C22" t="str">
+      <c r="C23" t="str">
         <v>{{NEXT_PAYMENT_DATE}}</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C23"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -814,6 +833,10 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B6"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="64.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -864,7 +887,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
   </ignoredErrors>
@@ -874,6 +896,10 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B6"/>
+  <cols>
+    <col min="1" max="1" width="19.83203125" customWidth="1"/>
+    <col min="2" max="2" width="34.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -924,7 +950,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
   </ignoredErrors>
@@ -934,6 +959,11 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C14"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="90.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1090,7 +1120,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:C14"/>
   </ignoredErrors>
@@ -1100,6 +1129,11 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C19"/>
+  <cols>
+    <col min="1" max="1" width="21.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="90.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1241,7 +1275,7 @@
         <v>Biggest Fights Section</v>
       </c>
       <c r="C13" t="str">
-        <v>The Biggest Fights|Saturday Fight Night|Fight Night|Upcoming Big Fights|Big Fights|Full Fights</v>
+        <v>The Biggest Fights|Saturday Fight Night|Fight Night|Upcoming Big Fights|Big Fights</v>
       </c>
     </row>
     <row r="14">
@@ -1311,7 +1345,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:C19"/>
   </ignoredErrors>
@@ -1321,6 +1354,11 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C31"/>
+  <cols>
+    <col min="1" max="1" width="33.83203125" customWidth="1"/>
+    <col min="2" max="2" width="124.83203125" customWidth="1"/>
+    <col min="3" max="3" width="11.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1338,7 +1376,7 @@
         <v>Page Title</v>
       </c>
       <c r="B2" t="str">
-        <v>Choose a plan that&amp;apos;s right for you</v>
+        <v>Choose a plan that's right for you</v>
       </c>
       <c r="C2" t="str">
         <v>checked</v>
@@ -1664,7 +1702,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:C31"/>
   </ignoredErrors>
@@ -1674,6 +1711,10 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B7"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="21.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1732,7 +1773,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
   </ignoredErrors>
@@ -1742,6 +1782,10 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B7"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1800,7 +1844,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
   </ignoredErrors>
@@ -1810,6 +1853,10 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B11"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="27.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1900,7 +1947,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B11"/>
   </ignoredErrors>
@@ -1910,6 +1956,10 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B5"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1952,7 +2002,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B5"/>
   </ignoredErrors>
@@ -1961,7 +2010,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C54"/>
+  <cols>
+    <col min="1" max="1" width="29.83203125" customWidth="1"/>
+    <col min="2" max="2" width="60.83203125" customWidth="1"/>
+    <col min="3" max="3" width="19.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2009,10 +2063,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>PPV Date and Time Text</v>
+        <v>Or Separator</v>
       </c>
       <c r="B5" t="str">
-        <v>{{PPV_DATE}}</v>
+        <v>or</v>
       </c>
       <c r="C5" t="str">
         <v>boxing</v>
@@ -2020,10 +2074,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Or Separator</v>
+        <v>Buy Fight CTA</v>
       </c>
       <c r="B6" t="str">
-        <v>or</v>
+        <v>Buy this fight for {{PPV_PRICE}}</v>
       </c>
       <c r="C6" t="str">
         <v>boxing</v>
@@ -2031,10 +2085,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Buy Fight CTA</v>
+        <v>Get Included CTA</v>
       </c>
       <c r="B7" t="str">
-        <v>Buy this fight for {{PPV_PRICE}}</v>
+        <v>Get included in DAZN Ultimate</v>
       </c>
       <c r="C7" t="str">
         <v>boxing</v>
@@ -2042,10 +2096,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Get Included CTA</v>
+        <v>Best Value Badge</v>
       </c>
       <c r="B8" t="str">
-        <v>Get included in DAZN Ultimate</v>
+        <v>Best value for boxing fans</v>
       </c>
       <c r="C8" t="str">
         <v>boxing</v>
@@ -2053,21 +2107,21 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Best Value Badge</v>
+        <v>Upcoming Big Fights Heading</v>
       </c>
       <c r="B9" t="str">
-        <v>Best value for boxing fans</v>
+        <v>Upcoming Big Fights</v>
       </c>
       <c r="C9" t="str">
-        <v>boxing</v>
+        <v>boxing-upcoming</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Upcoming Big Fights Heading</v>
+        <v>PPV Name</v>
       </c>
       <c r="B10" t="str">
-        <v>Upcoming Big Fights</v>
+        <v>{{PPV_DISPLAY_NAME}}</v>
       </c>
       <c r="C10" t="str">
         <v>boxing-upcoming</v>
@@ -2075,10 +2129,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>PPV Name</v>
+        <v>PPV Date and Time Text</v>
       </c>
       <c r="B11" t="str">
-        <v>{{PPV_DISPLAY_NAME}}</v>
+        <v>{{PPV_DATE}}</v>
       </c>
       <c r="C11" t="str">
         <v>boxing-upcoming</v>
@@ -2086,10 +2140,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>PPV Date and Time Text</v>
+        <v>PPV Description Text</v>
       </c>
       <c r="B12" t="str">
-        <v>{{PPV_DATE}}</v>
+        <v>{{PPV_LOCATION}}</v>
       </c>
       <c r="C12" t="str">
         <v>boxing-upcoming</v>
@@ -2097,10 +2151,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>PPV Description Text</v>
+        <v>PPV Image Present</v>
       </c>
       <c r="B13" t="str">
-        <v>{{PPV_LOCATION}}</v>
+        <v>Yes</v>
       </c>
       <c r="C13" t="str">
         <v>boxing-upcoming</v>
@@ -2108,10 +2162,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>PPV Image Present</v>
+        <v>Buy Now CTA</v>
       </c>
       <c r="B14" t="str">
-        <v>Yes</v>
+        <v>Buy now</v>
       </c>
       <c r="C14" t="str">
         <v>boxing-upcoming</v>
@@ -2119,21 +2173,21 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Buy Now CTA</v>
+        <v>Bundle Section Present</v>
       </c>
       <c r="B15" t="str">
-        <v>Buy now</v>
+        <v>Yes</v>
       </c>
       <c r="C15" t="str">
-        <v>boxing-upcoming</v>
+        <v>boxing-bundle</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Bundle Section Present</v>
+        <v>Bundle Section Title</v>
       </c>
       <c r="B16" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_SECTION_TITLE}}</v>
       </c>
       <c r="C16" t="str">
         <v>boxing-bundle</v>
@@ -2141,10 +2195,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Bundle Section Title</v>
+        <v>Bundle Section Subtitle</v>
       </c>
       <c r="B17" t="str">
-        <v>{{BUNDLE_SECTION_TITLE}}</v>
+        <v>{{BUNDLE_SECTION_SUBTITLE}}</v>
       </c>
       <c r="C17" t="str">
         <v>boxing-bundle</v>
@@ -2152,10 +2206,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Bundle Section Subtitle</v>
+        <v>Bundle Title</v>
       </c>
       <c r="B18" t="str">
-        <v>{{BUNDLE_SECTION_SUBTITLE}}</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="C18" t="str">
         <v>boxing-bundle</v>
@@ -2163,10 +2217,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Bundle Title</v>
+        <v>Bundle Description</v>
       </c>
       <c r="B19" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>{{BUNDLE_DESCRIPTION}}</v>
       </c>
       <c r="C19" t="str">
         <v>boxing-bundle</v>
@@ -2174,10 +2228,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Bundle Description</v>
+        <v>Bundle Price</v>
       </c>
       <c r="B20" t="str">
-        <v>{{BUNDLE_DESCRIPTION}}</v>
+        <v>{{BUNDLE_PRICE}}</v>
       </c>
       <c r="C20" t="str">
         <v>boxing-bundle</v>
@@ -2185,10 +2239,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Bundle Price</v>
+        <v>Bundle Original Price</v>
       </c>
       <c r="B21" t="str">
-        <v>{{BUNDLE_PRICE}}</v>
+        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
       </c>
       <c r="C21" t="str">
         <v>boxing-bundle</v>
@@ -2196,10 +2250,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Bundle Original Price</v>
+        <v>Bundle Save Badge</v>
       </c>
       <c r="B22" t="str">
-        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
+        <v>{{BUNDLE_SAVE_BADGE}}</v>
       </c>
       <c r="C22" t="str">
         <v>boxing-bundle</v>
@@ -2207,10 +2261,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Bundle Save Badge</v>
+        <v>Bundle Fight Count</v>
       </c>
       <c r="B23" t="str">
-        <v>{{BUNDLE_SAVE_BADGE}}</v>
+        <v>{{BUNDLE_FIGHT_COUNT}}</v>
       </c>
       <c r="C23" t="str">
         <v>boxing-bundle</v>
@@ -2218,10 +2272,10 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Bundle Fight Count</v>
+        <v>Bundle PPV 1 Name</v>
       </c>
       <c r="B24" t="str">
-        <v>{{BUNDLE_FIGHT_COUNT}}</v>
+        <v>{{BUNDLE_PPV1_NAME}}</v>
       </c>
       <c r="C24" t="str">
         <v>boxing-bundle</v>
@@ -2229,10 +2283,10 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Bundle PPV 1 Name</v>
+        <v>Bundle PPV 1 Date</v>
       </c>
       <c r="B25" t="str">
-        <v>{{BUNDLE_PPV1_NAME}}</v>
+        <v>{{BUNDLE_PPV1_LANDING_DATE}}</v>
       </c>
       <c r="C25" t="str">
         <v>boxing-bundle</v>
@@ -2240,10 +2294,10 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Bundle PPV 1 Date</v>
+        <v>Bundle PPV 1 Image</v>
       </c>
       <c r="B26" t="str">
-        <v>{{BUNDLE_PPV1_LANDING_DATE}}</v>
+        <v>Yes</v>
       </c>
       <c r="C26" t="str">
         <v>boxing-bundle</v>
@@ -2251,10 +2305,10 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Bundle PPV 1 Image</v>
+        <v>Bundle PPV 2 Name</v>
       </c>
       <c r="B27" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_PPV2_NAME}}</v>
       </c>
       <c r="C27" t="str">
         <v>boxing-bundle</v>
@@ -2262,10 +2316,10 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Bundle PPV 2 Name</v>
+        <v>Bundle PPV 2 Date</v>
       </c>
       <c r="B28" t="str">
-        <v>{{BUNDLE_PPV2_NAME}}</v>
+        <v>{{BUNDLE_PPV2_LANDING_DATE}}</v>
       </c>
       <c r="C28" t="str">
         <v>boxing-bundle</v>
@@ -2273,10 +2327,10 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Bundle PPV 2 Date</v>
+        <v>Bundle PPV 2 Image</v>
       </c>
       <c r="B29" t="str">
-        <v>{{BUNDLE_PPV2_LANDING_DATE}}</v>
+        <v>Yes</v>
       </c>
       <c r="C29" t="str">
         <v>boxing-bundle</v>
@@ -2284,10 +2338,10 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Bundle PPV 2 Image</v>
+        <v>Get Started CTA</v>
       </c>
       <c r="B30" t="str">
-        <v>Yes</v>
+        <v>Get Started</v>
       </c>
       <c r="C30" t="str">
         <v>boxing-bundle</v>
@@ -2295,21 +2349,21 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Get Started CTA</v>
+        <v>Page Title</v>
       </c>
       <c r="B31" t="str">
-        <v>Get Started</v>
+        <v>Choose the right plan for you.</v>
       </c>
       <c r="C31" t="str">
-        <v>boxing-bundle</v>
+        <v>boxing-bundle-ppv</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Page Title</v>
+        <v>Header Sub Text</v>
       </c>
       <c r="B32" t="str">
-        <v>Choose the right plan for you.</v>
+        <v>To watch your pay-per-view, you'll need a DAZN plan.</v>
       </c>
       <c r="C32" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2317,10 +2371,10 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Header Sub Text</v>
+        <v>Bundle Card Title</v>
       </c>
       <c r="B33" t="str">
-        <v>To watch your pay-per-view, you&amp;apos;ll need a DAZN plan.</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="C33" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2328,10 +2382,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Bundle Card Title</v>
+        <v>Bundle Card Description</v>
       </c>
       <c r="B34" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>{{BUNDLE_PPV_CARD_DESCRIPTION}}</v>
       </c>
       <c r="C34" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2339,10 +2393,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Bundle Card Description</v>
+        <v>Bundle Card Selected</v>
       </c>
       <c r="B35" t="str">
-        <v>{{BUNDLE_PPV_CARD_DESCRIPTION}}</v>
+        <v>Yes</v>
       </c>
       <c r="C35" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2350,10 +2404,10 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Bundle Card Selected</v>
+        <v>Bundle Card Price</v>
       </c>
       <c r="B36" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_PRICE}}</v>
       </c>
       <c r="C36" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2361,10 +2415,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Bundle Card Price</v>
+        <v>Bundle Card Original Price</v>
       </c>
       <c r="B37" t="str">
-        <v>{{BUNDLE_PRICE}}</v>
+        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
       </c>
       <c r="C37" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2372,10 +2426,10 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Bundle Card Original Price</v>
+        <v>Bundle Card Save Badge</v>
       </c>
       <c r="B38" t="str">
-        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
+        <v>{{BUNDLE_SAVE_BADGE}}</v>
       </c>
       <c r="C38" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2383,10 +2437,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Bundle Card Save Badge</v>
+        <v>Bundle PPV 1 Full Name</v>
       </c>
       <c r="B39" t="str">
-        <v>{{BUNDLE_SAVE_BADGE}}</v>
+        <v>{{BUNDLE_PPV1_FULL_NAME}}</v>
       </c>
       <c r="C39" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2394,10 +2448,10 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Bundle PPV 1 Full Name</v>
+        <v>Bundle PPV 1 PPV Date</v>
       </c>
       <c r="B40" t="str">
-        <v>{{BUNDLE_PPV1_FULL_NAME}}</v>
+        <v>{{BUNDLE_PPV1_DATE}}</v>
       </c>
       <c r="C40" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2405,10 +2459,10 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Bundle PPV 1 PPV Date</v>
+        <v>Bundle PPV 1 PPV Image</v>
       </c>
       <c r="B41" t="str">
-        <v>{{BUNDLE_PPV1_DATE}}</v>
+        <v>Yes</v>
       </c>
       <c r="C41" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2416,10 +2470,10 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Bundle PPV 1 PPV Image</v>
+        <v>Bundle PPV 2 Full Name</v>
       </c>
       <c r="B42" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_PPV2_FULL_NAME}}</v>
       </c>
       <c r="C42" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2427,10 +2481,10 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Bundle PPV 2 Full Name</v>
+        <v>Bundle PPV 2 PPV Date</v>
       </c>
       <c r="B43" t="str">
-        <v>{{BUNDLE_PPV2_FULL_NAME}}</v>
+        <v>{{BUNDLE_PPV2_DATE}}</v>
       </c>
       <c r="C43" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2438,10 +2492,10 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Bundle PPV 2 PPV Date</v>
+        <v>Bundle PPV 2 PPV Image</v>
       </c>
       <c r="B44" t="str">
-        <v>{{BUNDLE_PPV2_DATE}}</v>
+        <v>Yes</v>
       </c>
       <c r="C44" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2449,7 +2503,7 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Bundle PPV 2 PPV Image</v>
+        <v>Upsell Section Present</v>
       </c>
       <c r="B45" t="str">
         <v>Yes</v>
@@ -2460,10 +2514,10 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Upsell Section Present</v>
+        <v>Upsell Badge</v>
       </c>
       <c r="B46" t="str">
-        <v>Yes</v>
+        <v>The Ultimate Fan Package</v>
       </c>
       <c r="C46" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2471,10 +2525,10 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Upsell Badge</v>
+        <v>Upsell Plan Name</v>
       </c>
       <c r="B47" t="str">
-        <v>The Ultimate Fan Package</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="C47" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2482,10 +2536,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Upsell Plan Name</v>
+        <v>Upsell Price</v>
       </c>
       <c r="B48" t="str">
-        <v>DAZN Ultimate</v>
+        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
       </c>
       <c r="C48" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2493,10 +2547,10 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Upsell Price</v>
+        <v>Upsell Contract Text</v>
       </c>
       <c r="B49" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
+        <v>Annual contract. Auto renews.</v>
       </c>
       <c r="C49" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2504,10 +2558,10 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Upsell Contract Text</v>
+        <v>Fights Included Text</v>
       </c>
       <c r="B50" t="str">
-        <v>Annual contract. Auto renews.</v>
+        <v>All these fights included and more.</v>
       </c>
       <c r="C50" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2515,10 +2569,10 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Fights Included Text</v>
+        <v>Upsell Feature 1</v>
       </c>
       <c r="B51" t="str">
-        <v>All these fights included and more.</v>
+        <v>Minimum 12 pay-per-views a year included at no extra cost.</v>
       </c>
       <c r="C51" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2526,10 +2580,10 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Upsell Feature 1</v>
+        <v>Upsell Feature 2</v>
       </c>
       <c r="B52" t="str">
-        <v>Minimum 12 pay-per-views a year included at no extra cost.</v>
+        <v>185+ fights a year from the world's best promoters.</v>
       </c>
       <c r="C52" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2537,10 +2591,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Upsell Feature 2</v>
+        <v>Upsell Feature 3</v>
       </c>
       <c r="B53" t="str">
-        <v>185+ fights a year from the world&amp;apos;s best promoters.</v>
+        <v>HDR and Dolby 5.1 surround sound on select events</v>
       </c>
       <c r="C53" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2548,30 +2602,18 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Upsell Feature 3</v>
+        <v>CTA Button</v>
       </c>
       <c r="B54" t="str">
-        <v>HDR and Dolby 5.1 surround sound on select events</v>
+        <v>Continue with DAZN Ultimate</v>
       </c>
       <c r="C54" t="str">
         <v>boxing-bundle-ppv</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" t="str">
-        <v>CTA Button</v>
-      </c>
-      <c r="B55" t="str">
-        <v>Continue with DAZN Ultimate</v>
-      </c>
-      <c r="C55" t="str">
-        <v>boxing-bundle-ppv</v>
-      </c>
-    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C55"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C54"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2579,6 +2621,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D94"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="37.83203125" customWidth="1"/>
+    <col min="3" max="3" width="201.83203125" customWidth="1"/>
+    <col min="4" max="4" width="9.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2604,6 +2652,9 @@
       <c r="C2" t="str">
         <v>Choose the right plan for you.</v>
       </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -2613,7 +2664,10 @@
         <v>Header Sub Text</v>
       </c>
       <c r="C3" t="str">
-        <v>To watch your pay-per-view, you&amp;apos;ll need a DAZN plan.</v>
+        <v>To watch your pay-per-view, you'll need a DAZN plan.</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -2626,6 +2680,9 @@
       <c r="C4" t="str">
         <v>N/A</v>
       </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -2637,6 +2694,9 @@
       <c r="C5" t="str">
         <v>{{PPV_DISPLAY_NAME}}</v>
       </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -2648,6 +2708,9 @@
       <c r="C6" t="str">
         <v>/fight</v>
       </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -2659,6 +2722,9 @@
       <c r="C7" t="str">
         <v>{{PPV_PRICE}}</v>
       </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -2670,6 +2736,9 @@
       <c r="C8" t="str">
         <v>{{CURRENCY}}</v>
       </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -2695,6 +2764,9 @@
       <c r="C10" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -2706,6 +2778,9 @@
       <c r="C11" t="str">
         <v>Yes</v>
       </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -2717,6 +2792,9 @@
       <c r="C12" t="str">
         <v>{{PPV_DATE}}</v>
       </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -2728,6 +2806,9 @@
       <c r="C13" t="str">
         <v>Yes</v>
       </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -2739,6 +2820,9 @@
       <c r="C14" t="str">
         <v>{{PPV_DISPLAY_NAME}}</v>
       </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -2750,6 +2834,9 @@
       <c r="C15" t="str">
         <v>{{PPV_CARD_DESCRIPTION}}</v>
       </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -2761,6 +2848,9 @@
       <c r="C16" t="str">
         <v>Yes</v>
       </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -2772,6 +2862,9 @@
       <c r="C17" t="str">
         <v>The Ultimate Fan Package</v>
       </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -2783,6 +2876,9 @@
       <c r="C18" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -2794,6 +2890,9 @@
       <c r="C19" t="str">
         <v>N/A</v>
       </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -2805,6 +2904,9 @@
       <c r="C20" t="str">
         <v>{{UPSELL_PRICE}}</v>
       </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -2816,6 +2918,9 @@
       <c r="C21" t="str">
         <v>{{UPSELL_PRICE_LENGTH}}</v>
       </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -2827,6 +2932,9 @@
       <c r="C22" t="str">
         <v>{{UPSELL_CROSSED_PRICE}}</v>
       </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -2838,6 +2946,9 @@
       <c r="C23" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_CONTRACT_TEXT}}</v>
       </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -2863,6 +2974,9 @@
       <c r="C25" t="str">
         <v>{{UPSELL_SECTION_HEADING}}</v>
       </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -2874,6 +2988,9 @@
       <c r="C26" t="str">
         <v>N/A</v>
       </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -2885,6 +3002,9 @@
       <c r="C27" t="str">
         <v>N/A</v>
       </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -2896,6 +3016,9 @@
       <c r="C28" t="str">
         <v>N/A</v>
       </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -2907,6 +3030,9 @@
       <c r="C29" t="str">
         <v>N/A</v>
       </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -2918,6 +3044,9 @@
       <c r="C30" t="str">
         <v>N/A</v>
       </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -2929,6 +3058,9 @@
       <c r="C31" t="str">
         <v>{{UPSELL_FEATURE_1}}</v>
       </c>
+      <c r="D31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -2940,6 +3072,9 @@
       <c r="C32" t="str">
         <v>N/A</v>
       </c>
+      <c r="D32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -2951,6 +3086,9 @@
       <c r="C33" t="str">
         <v>{{UPSELL_FEATURE_2}}</v>
       </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -2962,6 +3100,9 @@
       <c r="C34" t="str">
         <v>{{UPSELL_FEATURE_3}}</v>
       </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -2973,6 +3114,9 @@
       <c r="C35" t="str">
         <v>N/A</v>
       </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -2984,6 +3128,9 @@
       <c r="C36" t="str">
         <v>N/A</v>
       </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -2995,6 +3142,9 @@
       <c r="C37" t="str">
         <v>N/A</v>
       </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -3006,6 +3156,9 @@
       <c r="C38" t="str">
         <v>N/A</v>
       </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -3199,6 +3352,9 @@
       <c r="C52" t="str">
         <v>{{PPV_CTA_TEXT}}</v>
       </c>
+      <c r="D52" t="str">
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -3224,6 +3380,9 @@
       <c r="C54" t="str">
         <v>Choose your plan</v>
       </c>
+      <c r="D54" t="str">
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -3235,6 +3394,9 @@
       <c r="C55" t="str">
         <v>Buy {{PPV_NAME}} with DAZN Standard or get it included in DAZN Ultimate.</v>
       </c>
+      <c r="D55" t="str">
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -3246,6 +3408,9 @@
       <c r="C56" t="str">
         <v>get it included in DAZN Ultimate.</v>
       </c>
+      <c r="D56" t="str">
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -3257,6 +3422,9 @@
       <c r="C57" t="str">
         <v>Yes</v>
       </c>
+      <c r="D57" t="str">
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -3268,6 +3436,9 @@
       <c r="C58" t="str">
         <v>{{PPV_DATE}}</v>
       </c>
+      <c r="D58" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -3279,6 +3450,9 @@
       <c r="C59" t="str">
         <v>{{PPV_DISPLAY_NAME}}</v>
       </c>
+      <c r="D59" t="str">
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -3290,6 +3464,9 @@
       <c r="C60" t="str">
         <v>Yes</v>
       </c>
+      <c r="D60" t="str">
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -3301,6 +3478,9 @@
       <c r="C61" t="str">
         <v>Yes</v>
       </c>
+      <c r="D61" t="str">
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -3312,6 +3492,9 @@
       <c r="C62" t="str">
         <v>{{PPV_DISPLAY_NAME}}</v>
       </c>
+      <c r="D62" t="str">
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -3323,6 +3506,9 @@
       <c r="C63" t="str">
         <v>/fight</v>
       </c>
+      <c r="D63" t="str">
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -3334,6 +3520,9 @@
       <c r="C64" t="str">
         <v>{{PPV_PRICE}}</v>
       </c>
+      <c r="D64" t="str">
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -3345,6 +3534,9 @@
       <c r="C65" t="str">
         <v>{{CURRENCY}}</v>
       </c>
+      <c r="D65" t="str">
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -3356,6 +3548,9 @@
       <c r="C66" t="str">
         <v>Choose your subscription</v>
       </c>
+      <c r="D66" t="str">
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -3367,6 +3562,9 @@
       <c r="C67" t="str">
         <v>Yes</v>
       </c>
+      <c r="D67" t="str">
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -3378,6 +3576,9 @@
       <c r="C68" t="str">
         <v>7-day free trial of DAZN Standard</v>
       </c>
+      <c r="D68" t="str">
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -3389,6 +3590,9 @@
       <c r="C69" t="str">
         <v>Yes</v>
       </c>
+      <c r="D69" t="str">
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -3400,6 +3604,9 @@
       <c r="C70" t="str">
         <v>Yes</v>
       </c>
+      <c r="D70" t="str">
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -3411,6 +3618,9 @@
       <c r="C71" t="str">
         <v>7-days free access to DAZN Standard.</v>
       </c>
+      <c r="D71" t="str">
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -3422,6 +3632,9 @@
       <c r="C72" t="str">
         <v>Cancel anytime during the trial and only pay for the fight. After the trial you move onto a Monthly Flex plan for {{CURRENCY}}{{MONTHLY_PRICE}}/month. You will not lose access to the pay-per-view[s].</v>
       </c>
+      <c r="D72" t="str">
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -3433,6 +3646,9 @@
       <c r="C73" t="str">
         <v>Yes</v>
       </c>
+      <c r="D73" t="str">
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -3444,6 +3660,9 @@
       <c r="C74" t="str">
         <v>Pay-per-views included</v>
       </c>
+      <c r="D74" t="str">
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -3455,6 +3674,9 @@
       <c r="C75" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="D75" t="str">
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -3466,6 +3688,9 @@
       <c r="C76" t="str">
         <v>From</v>
       </c>
+      <c r="D76" t="str">
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -3477,6 +3702,9 @@
       <c r="C77" t="str">
         <v>{{UPSELL_PRICE}}</v>
       </c>
+      <c r="D77" t="str">
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -3488,6 +3716,9 @@
       <c r="C78" t="str">
         <v>{{UPSELL_PRICE_LENGTH}}</v>
       </c>
+      <c r="D78" t="str">
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -3499,6 +3730,9 @@
       <c r="C79" t="str">
         <v>Annual contract. Auto renews.</v>
       </c>
+      <c r="D79" t="str">
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -3510,6 +3744,9 @@
       <c r="C80" t="str">
         <v>Yes</v>
       </c>
+      <c r="D80" t="str">
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -3521,6 +3758,9 @@
       <c r="C81" t="str">
         <v>N/A</v>
       </c>
+      <c r="D81" t="str">
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -3532,6 +3772,9 @@
       <c r="C82" t="str">
         <v>N/A</v>
       </c>
+      <c r="D82" t="str">
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -3543,6 +3786,9 @@
       <c r="C83" t="str">
         <v>N/A</v>
       </c>
+      <c r="D83" t="str">
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -3554,6 +3800,9 @@
       <c r="C84" t="str">
         <v>N/A</v>
       </c>
+      <c r="D84" t="str">
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -3565,6 +3814,9 @@
       <c r="C85" t="str">
         <v>Pay-per-views included at no extra cost. Minimum of 12 events per year including {{PPV_NAME}}.</v>
       </c>
+      <c r="D85" t="str">
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -3576,6 +3828,9 @@
       <c r="C86" t="str">
         <v>{{PPV_NAME}}.</v>
       </c>
+      <c r="D86" t="str">
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -3587,6 +3842,9 @@
       <c r="C87" t="str">
         <v>HDR and Dolby 5.1 surround sound on select events.</v>
       </c>
+      <c r="D87" t="str">
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -3598,6 +3856,9 @@
       <c r="C88" t="str">
         <v>185+ fights a year from the best promoters</v>
       </c>
+      <c r="D88" t="str">
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
@@ -3609,6 +3870,9 @@
       <c r="C89" t="str">
         <v>Whats included</v>
       </c>
+      <c r="D89" t="str">
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -3620,6 +3884,9 @@
       <c r="C90" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="D90" t="str">
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -3631,6 +3898,9 @@
       <c r="C91" t="str">
         <v>get it included in DAZN Ultimate.</v>
       </c>
+      <c r="D91" t="str">
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -3642,6 +3912,9 @@
       <c r="C92" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="D92" t="str">
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
@@ -3653,6 +3926,9 @@
       <c r="C93" t="str">
         <v>Continue with PPV + 7-day free trial</v>
       </c>
+      <c r="D93" t="str">
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
@@ -3664,9 +3940,11 @@
       <c r="C94" t="str">
         <v>N/A</v>
       </c>
+      <c r="D94" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:D94"/>
   </ignoredErrors>
@@ -3676,6 +3954,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D37"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="34.83203125" customWidth="1"/>
+    <col min="3" max="3" width="70.83203125" customWidth="1"/>
+    <col min="4" max="4" width="6.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3701,6 +3985,9 @@
       <c r="C2" t="str">
         <v>{{PLAN_PAGE_TITLE}}</v>
       </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -3712,6 +3999,9 @@
       <c r="C3" t="str">
         <v>Yes</v>
       </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -3723,6 +4013,9 @@
       <c r="C4" t="str">
         <v>Flex – Pay Monthly</v>
       </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -3734,6 +4027,9 @@
       <c r="C5" t="str">
         <v>{{FLEX_BADGE}}</v>
       </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -3745,6 +4041,9 @@
       <c r="C6" t="str">
         <v>{{FLEX_DESCRIPTION}}</v>
       </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -3756,6 +4055,9 @@
       <c r="C7" t="str">
         <v>Yes</v>
       </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -3767,6 +4069,9 @@
       <c r="C8" t="str">
         <v>{{FLEX_TODAY_TEXT}}</v>
       </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -3778,6 +4083,9 @@
       <c r="C9" t="str">
         <v>{{FLEX_FUTURE_TEXT}}</v>
       </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -3789,6 +4097,9 @@
       <c r="C10" t="str">
         <v>Yes</v>
       </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -3800,6 +4111,9 @@
       <c r="C11" t="str">
         <v>{{ANNUAL_SAVINGS_BADGE}}</v>
       </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -3811,6 +4125,9 @@
       <c r="C12" t="str">
         <v>Annual - Pay Monthly</v>
       </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -3822,6 +4139,9 @@
       <c r="C13" t="str">
         <v>1 MONTH FREE</v>
       </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -3833,6 +4153,9 @@
       <c r="C14" t="str">
         <v>then {{CURRENCY}}{{ANNUAL_PRICE}}/month for {{ANNUAL_MONTHS}} months</v>
       </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -3844,6 +4167,9 @@
       <c r="C15" t="str">
         <v>Annual contract. Auto renews.</v>
       </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -3853,7 +4179,10 @@
         <v>Annual Feature 1</v>
       </c>
       <c r="C16" t="str">
-        <v>185+ fights a year from the world&amp;apos;s best promoters.</v>
+        <v>185+ fights a year from the world's best promoters.</v>
+      </c>
+      <c r="D16" t="str">
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -3866,6 +4195,9 @@
       <c r="C17" t="str">
         <v>Additional cost for pay-per-view events.</v>
       </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -3877,6 +4209,9 @@
       <c r="C18" t="str">
         <v>Full HD video resolution.</v>
       </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -3888,6 +4223,9 @@
       <c r="C19" t="str">
         <v>No</v>
       </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -3899,6 +4237,9 @@
       <c r="C20" t="str">
         <v>{{PLAN_CTA_BUTTON}}</v>
       </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -3910,6 +4251,9 @@
       <c r="C21" t="str">
         <v>{{PLAN_PAGE_TITLE}}</v>
       </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -3921,6 +4265,9 @@
       <c r="C22" t="str">
         <v>Yes</v>
       </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -3932,6 +4279,9 @@
       <c r="C23" t="str">
         <v>Annual - Pay Monthly</v>
       </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -3943,6 +4293,9 @@
       <c r="C24" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
       </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -3954,6 +4307,9 @@
       <c r="C25" t="str">
         <v>/month</v>
       </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -3965,6 +4321,9 @@
       <c r="C26" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_CONTRACT_TEXT}}</v>
       </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -3976,6 +4335,9 @@
       <c r="C27" t="str">
         <v>Yes</v>
       </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -3987,6 +4349,9 @@
       <c r="C28" t="str">
         <v>Yes</v>
       </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -3998,6 +4363,9 @@
       <c r="C29" t="str">
         <v>Annual - Pay Upfront</v>
       </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -4009,6 +4377,9 @@
       <c r="C30" t="str">
         <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
       </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -4020,6 +4391,9 @@
       <c r="C31" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE_DISPLAY}}</v>
       </c>
+      <c r="D31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -4031,6 +4405,9 @@
       <c r="C32" t="str">
         <v>/year</v>
       </c>
+      <c r="D32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -4042,6 +4419,9 @@
       <c r="C33" t="str">
         <v>No</v>
       </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -4053,6 +4433,9 @@
       <c r="C34" t="str">
         <v>{{ULTIMATE_FEATURE_1}}</v>
       </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -4064,6 +4447,9 @@
       <c r="C35" t="str">
         <v>{{ULTIMATE_FEATURE_2}}</v>
       </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -4075,6 +4461,9 @@
       <c r="C36" t="str">
         <v>{{ULTIMATE_FEATURE_3}}</v>
       </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -4086,9 +4475,11 @@
       <c r="C37" t="str">
         <v>{{PLAN_CTA_BUTTON}}</v>
       </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:D37"/>
   </ignoredErrors>
@@ -4098,6 +4489,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E103"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="27.83203125" customWidth="1"/>
+    <col min="3" max="3" width="28.83203125" customWidth="1"/>
+    <col min="4" max="4" width="160.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4129,6 +4527,9 @@
       <c r="D2" t="str">
         <v>Payment method</v>
       </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -4143,6 +4544,9 @@
       <c r="D3" t="str">
         <v>Purchase summary</v>
       </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -4157,6 +4561,9 @@
       <c r="D4" t="str">
         <v>Change</v>
       </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -4171,6 +4578,9 @@
       <c r="D5" t="str">
         <v>Yes</v>
       </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -4185,6 +4595,9 @@
       <c r="D6" t="str">
         <v>Yes</v>
       </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -4199,6 +4612,9 @@
       <c r="D7" t="str">
         <v>Yes</v>
       </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -4264,6 +4680,9 @@
       <c r="D11" t="str">
         <v>Yes</v>
       </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -4312,6 +4731,9 @@
       <c r="D14" t="str">
         <v>DAZN Standard</v>
       </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -4326,6 +4748,9 @@
       <c r="D15" t="str">
         <v>{{PAYMENT_PLAN_NAME}}</v>
       </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -4340,6 +4765,9 @@
       <c r="D16" t="str">
         <v>{{PAYMENT_FLEX_CANCEL_NOTICE}}</v>
       </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -4354,6 +4782,9 @@
       <c r="D17" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -4368,6 +4799,9 @@
       <c r="D18" t="str">
         <v>{{PAYMENT_FREE_TEXT}}</v>
       </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -4382,6 +4816,9 @@
       <c r="D19" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -4396,6 +4833,9 @@
       <c r="D20" t="str">
         <v>{{PPV_PRICE}}</v>
       </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -4410,6 +4850,9 @@
       <c r="D21" t="str">
         <v>Today you pay</v>
       </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -4424,6 +4867,9 @@
       <c r="D22" t="str">
         <v>{{PPV_PRICE}}</v>
       </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -4438,6 +4884,9 @@
       <c r="D23" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -4452,6 +4901,9 @@
       <c r="D24" t="str">
         <v>{{PAYMENT_FLEX_LEGAL_TEXT}}</v>
       </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -4466,6 +4918,9 @@
       <c r="D25" t="str">
         <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -4480,6 +4935,9 @@
       <c r="D26" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -4494,6 +4952,9 @@
       <c r="D27" t="str">
         <v>DAZN Standard</v>
       </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -4508,6 +4969,9 @@
       <c r="D28" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -4522,6 +4986,9 @@
       <c r="D29" t="str">
         <v>{{PPV_PRICE}}</v>
       </c>
+      <c r="E29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -4536,6 +5003,9 @@
       <c r="D30" t="str">
         <v>{{RATE_PLAN_LABEL}}</v>
       </c>
+      <c r="E30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -4550,6 +5020,9 @@
       <c r="D31" t="str">
         <v>{{CURRENCY}}{{ANNUAL_PRICE}}</v>
       </c>
+      <c r="E31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -4564,6 +5037,9 @@
       <c r="D32" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -4578,6 +5054,9 @@
       <c r="D33" t="str">
         <v>Today you pay</v>
       </c>
+      <c r="E33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -4592,6 +5071,9 @@
       <c r="D34" t="str">
         <v>{{PPV_PRICE}}</v>
       </c>
+      <c r="E34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -4606,6 +5088,9 @@
       <c r="D35" t="str">
         <v>{{CANCELLATION_TEXT_ANNUAL}}</v>
       </c>
+      <c r="E35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -4620,6 +5105,9 @@
       <c r="D36" t="str">
         <v>Yes</v>
       </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -4634,6 +5122,9 @@
       <c r="D37" t="str">
         <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -4648,6 +5139,9 @@
       <c r="D38" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -4662,6 +5156,9 @@
       <c r="D39" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="E39" t="str">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -4676,6 +5173,9 @@
       <c r="D40" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -4690,6 +5190,9 @@
       <c r="D41" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E41" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -4704,6 +5207,9 @@
       <c r="D42" t="str">
         <v>Annual - Pay Monthly</v>
       </c>
+      <c r="E42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -4718,6 +5224,9 @@
       <c r="D43" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
       </c>
+      <c r="E43" t="str">
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -4732,6 +5241,9 @@
       <c r="D44" t="str">
         <v>Billed monthly. 12-month contract.</v>
       </c>
+      <c r="E44" t="str">
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -4746,6 +5258,9 @@
       <c r="D45" t="str">
         <v>Today you pay</v>
       </c>
+      <c r="E45" t="str">
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -4760,6 +5275,9 @@
       <c r="D46" t="str">
         <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
+      <c r="E46" t="str">
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -4774,6 +5292,9 @@
       <c r="D47" t="str">
         <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
+      <c r="E47" t="str">
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -4788,6 +5309,9 @@
       <c r="D48" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
       </c>
+      <c r="E48" t="str">
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -4802,6 +5326,9 @@
       <c r="D49" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E49" t="str">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -4816,6 +5343,9 @@
       <c r="D50" t="str">
         <v>Yes</v>
       </c>
+      <c r="E50" t="str">
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -4830,6 +5360,9 @@
       <c r="D51" t="str">
         <v>{{DISCOUNT_BADGE}}</v>
       </c>
+      <c r="E51" t="str">
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -4844,6 +5377,9 @@
       <c r="D52" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E52" t="str">
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -4858,6 +5394,9 @@
       <c r="D53" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="E53" t="str">
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -4872,6 +5411,9 @@
       <c r="D54" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="E54" t="str">
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -4886,6 +5428,9 @@
       <c r="D55" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E55" t="str">
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -4900,6 +5445,9 @@
       <c r="D56" t="str">
         <v>Annual - Pay Upfront</v>
       </c>
+      <c r="E56" t="str">
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -4914,6 +5462,9 @@
       <c r="D57" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE}}/year</v>
       </c>
+      <c r="E57" t="str">
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -4928,6 +5479,9 @@
       <c r="D58" t="str">
         <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}. Pay for the full year up front|Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
       </c>
+      <c r="E58" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -4942,6 +5496,9 @@
       <c r="D59" t="str">
         <v>Today you pay</v>
       </c>
+      <c r="E59" t="str">
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -4956,6 +5513,9 @@
       <c r="D60" t="str">
         <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
+      <c r="E60" t="str">
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -4970,6 +5530,9 @@
       <c r="D61" t="str">
         <v>Next Annual payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
+      <c r="E61" t="str">
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -4984,6 +5547,9 @@
       <c r="D62" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE}}</v>
       </c>
+      <c r="E62" t="str">
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -4998,6 +5564,9 @@
       <c r="D63" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E63" t="str">
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -5012,6 +5581,9 @@
       <c r="D64" t="str">
         <v>Yes</v>
       </c>
+      <c r="E64" t="str">
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -5026,6 +5598,9 @@
       <c r="D65" t="str">
         <v>{{PAYMENT_PAGE_TITLE}}</v>
       </c>
+      <c r="E65" t="str">
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -5040,6 +5615,9 @@
       <c r="D66" t="str">
         <v>DAZN Standard</v>
       </c>
+      <c r="E66" t="str">
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -5054,6 +5632,9 @@
       <c r="D67" t="str">
         <v>{{BUNDLE_NAME}}</v>
       </c>
+      <c r="E67" t="str">
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -5068,6 +5649,9 @@
       <c r="D68" t="str">
         <v>{{BUNDLE_PRICE}}</v>
       </c>
+      <c r="E68" t="str">
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -5082,6 +5666,9 @@
       <c r="D69" t="str">
         <v>{{BUNDLE_TODAY_YOU_PAY_STANDARD}}</v>
       </c>
+      <c r="E69" t="str">
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -5096,6 +5683,9 @@
       <c r="D70" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E70" t="str">
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -5110,6 +5700,9 @@
       <c r="D71" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E71" t="str">
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -5124,6 +5717,9 @@
       <c r="D72" t="str">
         <v>DAZN Standard</v>
       </c>
+      <c r="E72" t="str">
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -5138,6 +5734,9 @@
       <c r="D73" t="str">
         <v>Annual - Pay Monthly</v>
       </c>
+      <c r="E73" t="str">
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -5152,6 +5751,9 @@
       <c r="D74" t="str">
         <v>First month free</v>
       </c>
+      <c r="E74" t="str">
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -5166,6 +5768,9 @@
       <c r="D75" t="str">
         <v>{{BUNDLE_NAME}}</v>
       </c>
+      <c r="E75" t="str">
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -5180,6 +5785,9 @@
       <c r="D76" t="str">
         <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
       </c>
+      <c r="E76" t="str">
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -5194,6 +5802,9 @@
       <c r="D77" t="str">
         <v>{{BUNDLE_PRICE}}</v>
       </c>
+      <c r="E77" t="str">
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -5208,6 +5819,9 @@
       <c r="D78" t="str">
         <v>{{BUNDLE_DISCOUNT}}</v>
       </c>
+      <c r="E78" t="str">
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -5222,6 +5836,9 @@
       <c r="D79" t="str">
         <v>{{BUNDLE_TODAY_YOU_PAY_STANDARD}}</v>
       </c>
+      <c r="E79" t="str">
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -5236,6 +5853,9 @@
       <c r="D80" t="str">
         <v>{{CANCELLATION_TEXT_ANNUAL}}</v>
       </c>
+      <c r="E80" t="str">
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -5250,6 +5870,9 @@
       <c r="D81" t="str">
         <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
+      <c r="E81" t="str">
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -5264,6 +5887,9 @@
       <c r="D82" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E82" t="str">
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -5278,6 +5904,9 @@
       <c r="D83" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="E83" t="str">
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -5292,6 +5921,9 @@
       <c r="D84" t="str">
         <v>Annual - Pay Monthly</v>
       </c>
+      <c r="E84" t="str">
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -5306,6 +5938,9 @@
       <c r="D85" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
       </c>
+      <c r="E85" t="str">
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -5320,6 +5955,9 @@
       <c r="D86" t="str">
         <v>{{BUNDLE_NAME}}</v>
       </c>
+      <c r="E86" t="str">
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -5334,6 +5972,9 @@
       <c r="D87" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E87" t="str">
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -5348,6 +5989,9 @@
       <c r="D88" t="str">
         <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
+      <c r="E88" t="str">
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
@@ -5362,6 +6006,9 @@
       <c r="D89" t="str">
         <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
+      <c r="E89" t="str">
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -5376,6 +6023,9 @@
       <c r="D90" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
       </c>
+      <c r="E90" t="str">
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -5390,6 +6040,9 @@
       <c r="D91" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E91" t="str">
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -5404,6 +6057,9 @@
       <c r="D92" t="str">
         <v>{{DISCOUNT_BADGE}}</v>
       </c>
+      <c r="E92" t="str">
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
@@ -5418,6 +6074,9 @@
       <c r="D93" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E93" t="str">
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
@@ -5432,6 +6091,9 @@
       <c r="D94" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="E94" t="str">
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
@@ -5446,6 +6108,9 @@
       <c r="D95" t="str">
         <v>Annual - Pay Upfront</v>
       </c>
+      <c r="E95" t="str">
+        <v/>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
@@ -5460,6 +6125,9 @@
       <c r="D96" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE}}/year</v>
       </c>
+      <c r="E96" t="str">
+        <v/>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
@@ -5474,6 +6142,9 @@
       <c r="D97" t="str">
         <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
       </c>
+      <c r="E97" t="str">
+        <v/>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
@@ -5488,6 +6159,9 @@
       <c r="D98" t="str">
         <v>{{BUNDLE_NAME}}</v>
       </c>
+      <c r="E98" t="str">
+        <v/>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
@@ -5502,6 +6176,9 @@
       <c r="D99" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E99" t="str">
+        <v/>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
@@ -5516,6 +6193,9 @@
       <c r="D100" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE}}</v>
       </c>
+      <c r="E100" t="str">
+        <v/>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
@@ -5530,6 +6210,9 @@
       <c r="D101" t="str">
         <v>Next Annual payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
+      <c r="E101" t="str">
+        <v/>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
@@ -5544,6 +6227,9 @@
       <c r="D102" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE}}</v>
       </c>
+      <c r="E102" t="str">
+        <v/>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
@@ -5558,9 +6244,11 @@
       <c r="D103" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E103" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:E103"/>
   </ignoredErrors>
@@ -5570,6 +6258,10 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B15"/>
+  <cols>
+    <col min="1" max="1" width="27.83203125" customWidth="1"/>
+    <col min="2" max="2" width="90.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5692,7 +6384,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B15"/>
   </ignoredErrors>
@@ -5702,6 +6393,10 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B9"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="25.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5776,7 +6471,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B9"/>
   </ignoredErrors>
@@ -5786,6 +6480,10 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B23"/>
+  <cols>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="70.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5972,7 +6670,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B23"/>
   </ignoredErrors>
@@ -5982,6 +6679,10 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B18"/>
+  <cols>
+    <col min="1" max="1" width="29.83203125" customWidth="1"/>
+    <col min="2" max="2" width="79.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6012,7 +6713,7 @@
         <v>PPV Description</v>
       </c>
       <c r="B4" t="str">
-        <v>{{BANNER_DESCRIPTION}}</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="5">
@@ -6128,7 +6829,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B18"/>
   </ignoredErrors>

</xml_diff>

<commit_message>
Update PPV automation flows
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -416,11 +416,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C12"/>
-  <cols>
-    <col min="1" max="1" width="33.83203125" customWidth="1"/>
-    <col min="2" max="2" width="27.83203125" customWidth="1"/>
-    <col min="3" max="3" width="21.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -564,11 +559,6 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C23"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="27.83203125" customWidth="1"/>
-    <col min="3" max="3" width="318.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -833,10 +823,6 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B6"/>
-  <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="64.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -896,10 +882,6 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B6"/>
-  <cols>
-    <col min="1" max="1" width="19.83203125" customWidth="1"/>
-    <col min="2" max="2" width="34.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -958,12 +940,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
-    <col min="3" max="3" width="90.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:C24"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1119,21 +1096,126 @@
         <v>Visible</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Best of Boxing Section</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Present</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B16" t="str">
+        <v>PPV Tile Present</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B17" t="str">
+        <v>PPV Date</v>
+      </c>
+      <c r="C17" t="str">
+        <v>{{LANDING_PAGE_PPV_DATE}}</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B18" t="str">
+        <v>PPV Promoter on Tile</v>
+      </c>
+      <c r="C18" t="str">
+        <v>{{PPV_PROMOTER}}</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B19" t="str">
+        <v>PPV Name</v>
+      </c>
+      <c r="C19" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B20" t="str">
+        <v>PPV Date and Time Text</v>
+      </c>
+      <c r="C20" t="str">
+        <v>WATCH LIVE {{HOME_BOXING_UPCOMING_DATE}} at {{HOME_BOXING_UPCOMING_TIME}}</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Buy Now CTA</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Buy now</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Fight Card CTA</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Fight card</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B23" t="str">
+        <v>PPV Image Present</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Lock Icon Present</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C24"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C19"/>
-  <cols>
-    <col min="1" max="1" width="21.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
-    <col min="3" max="3" width="90.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:C25"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1275,7 +1357,7 @@
         <v>Biggest Fights Section</v>
       </c>
       <c r="C13" t="str">
-        <v>The Biggest Fights|Saturday Fight Night|Fight Night|Upcoming Big Fights|Big Fights</v>
+        <v>Saturday Fight Night</v>
       </c>
     </row>
     <row r="14">
@@ -1344,9 +1426,75 @@
         <v>Visible</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>home-page-popup</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Home Popup Image Present</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>home-page-popup</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Home Popup Event Title</v>
+      </c>
+      <c r="C21" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>home-page-popup</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Home Popup Event Date</v>
+      </c>
+      <c r="C22" t="str">
+        <v>{{HOME_POPUP_DATE}}</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>home-page-popup</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Home Popup Event Description</v>
+      </c>
+      <c r="C23" t="str">
+        <v>{{HOME_POPUP_DESCRIPTION}}</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>home-page-popup</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Home Popup Buy Now CTA</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>home-page-popup</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Home Popup Close Button</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C25"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1354,11 +1502,6 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C31"/>
-  <cols>
-    <col min="1" max="1" width="33.83203125" customWidth="1"/>
-    <col min="2" max="2" width="124.83203125" customWidth="1"/>
-    <col min="3" max="3" width="11.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1711,10 +1854,6 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B7"/>
-  <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="21.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1782,10 +1921,6 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B7"/>
-  <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1853,10 +1988,6 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B11"/>
-  <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="27.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1956,10 +2087,6 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B5"/>
-  <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2011,11 +2138,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C54"/>
-  <cols>
-    <col min="1" max="1" width="29.83203125" customWidth="1"/>
-    <col min="2" max="2" width="60.83203125" customWidth="1"/>
-    <col min="3" max="3" width="19.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2621,12 +2743,6 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D94"/>
-  <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="37.83203125" customWidth="1"/>
-    <col min="3" max="3" width="201.83203125" customWidth="1"/>
-    <col min="4" max="4" width="9.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3854,7 +3970,7 @@
         <v>Upsell Feature 3</v>
       </c>
       <c r="C88" t="str">
-        <v>185+ fights a year from the best promoters</v>
+        <v>185+ fights a year from the world's best promoters.</v>
       </c>
       <c r="D88" t="str">
         <v/>
@@ -3953,13 +4069,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D37"/>
-  <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="34.83203125" customWidth="1"/>
-    <col min="3" max="3" width="70.83203125" customWidth="1"/>
-    <col min="4" max="4" width="6.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:D38"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4078,10 +4188,10 @@
         <v>Standard</v>
       </c>
       <c r="B9" t="str">
-        <v>Flex Future Text</v>
+        <v>Flex Future Date</v>
       </c>
       <c r="C9" t="str">
-        <v>{{FLEX_FUTURE_TEXT}}</v>
+        <v>{{FLEX_FUTURE_DATE}}</v>
       </c>
       <c r="D9" t="str">
         <v/>
@@ -4092,10 +4202,10 @@
         <v>Standard</v>
       </c>
       <c r="B10" t="str">
-        <v>Annual Card Present</v>
+        <v>Flex Future Text</v>
       </c>
       <c r="C10" t="str">
-        <v>Yes</v>
+        <v>{{FLEX_FUTURE_TEXT}}</v>
       </c>
       <c r="D10" t="str">
         <v/>
@@ -4106,10 +4216,10 @@
         <v>Standard</v>
       </c>
       <c r="B11" t="str">
-        <v>Annual Savings Badge</v>
+        <v>Annual Card Present</v>
       </c>
       <c r="C11" t="str">
-        <v>{{ANNUAL_SAVINGS_BADGE}}</v>
+        <v>Yes</v>
       </c>
       <c r="D11" t="str">
         <v/>
@@ -4120,10 +4230,10 @@
         <v>Standard</v>
       </c>
       <c r="B12" t="str">
-        <v>Annual Title</v>
+        <v>Annual Savings Badge</v>
       </c>
       <c r="C12" t="str">
-        <v>Annual - Pay Monthly</v>
+        <v>{{ANNUAL_SAVINGS_BADGE}}</v>
       </c>
       <c r="D12" t="str">
         <v/>
@@ -4134,10 +4244,10 @@
         <v>Standard</v>
       </c>
       <c r="B13" t="str">
-        <v>Annual Badge</v>
+        <v>Annual Title</v>
       </c>
       <c r="C13" t="str">
-        <v>1 MONTH FREE</v>
+        <v>Annual - Pay Monthly</v>
       </c>
       <c r="D13" t="str">
         <v/>
@@ -4148,10 +4258,10 @@
         <v>Standard</v>
       </c>
       <c r="B14" t="str">
-        <v>Annual Price Text</v>
+        <v>Annual Badge</v>
       </c>
       <c r="C14" t="str">
-        <v>then {{CURRENCY}}{{ANNUAL_PRICE}}/month for {{ANNUAL_MONTHS}} months</v>
+        <v>1 MONTH FREE</v>
       </c>
       <c r="D14" t="str">
         <v/>
@@ -4162,10 +4272,10 @@
         <v>Standard</v>
       </c>
       <c r="B15" t="str">
-        <v>Annual Contract Text</v>
+        <v>Annual Price Text</v>
       </c>
       <c r="C15" t="str">
-        <v>Annual contract. Auto renews.</v>
+        <v>then {{CURRENCY}}{{ANNUAL_PRICE}}/month for {{ANNUAL_MONTHS}} months</v>
       </c>
       <c r="D15" t="str">
         <v/>
@@ -4176,10 +4286,10 @@
         <v>Standard</v>
       </c>
       <c r="B16" t="str">
-        <v>Annual Feature 1</v>
+        <v>Annual Contract Text</v>
       </c>
       <c r="C16" t="str">
-        <v>185+ fights a year from the world's best promoters.</v>
+        <v>Annual contract. Auto renews.</v>
       </c>
       <c r="D16" t="str">
         <v/>
@@ -4190,10 +4300,10 @@
         <v>Standard</v>
       </c>
       <c r="B17" t="str">
-        <v>Annual Feature 2</v>
+        <v>Annual Feature 1</v>
       </c>
       <c r="C17" t="str">
-        <v>Additional cost for pay-per-view events.</v>
+        <v>185+ fights a year from the world's best promoters.</v>
       </c>
       <c r="D17" t="str">
         <v/>
@@ -4204,10 +4314,10 @@
         <v>Standard</v>
       </c>
       <c r="B18" t="str">
-        <v>Annual Feature 3</v>
+        <v>Annual Feature 2</v>
       </c>
       <c r="C18" t="str">
-        <v>Full HD video resolution.</v>
+        <v>Additional cost for pay-per-view events.</v>
       </c>
       <c r="D18" t="str">
         <v/>
@@ -4218,10 +4328,10 @@
         <v>Standard</v>
       </c>
       <c r="B19" t="str">
-        <v>Annual Selected</v>
+        <v>Annual Feature 3</v>
       </c>
       <c r="C19" t="str">
-        <v>No</v>
+        <v>Full HD video resolution.</v>
       </c>
       <c r="D19" t="str">
         <v/>
@@ -4232,10 +4342,10 @@
         <v>Standard</v>
       </c>
       <c r="B20" t="str">
-        <v>CTA Button</v>
+        <v>Annual Selected</v>
       </c>
       <c r="C20" t="str">
-        <v>{{PLAN_CTA_BUTTON}}</v>
+        <v>No</v>
       </c>
       <c r="D20" t="str">
         <v/>
@@ -4243,13 +4353,13 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Ultimate</v>
+        <v>Standard</v>
       </c>
       <c r="B21" t="str">
-        <v>Page Title</v>
+        <v>CTA Button</v>
       </c>
       <c r="C21" t="str">
-        <v>{{PLAN_PAGE_TITLE}}</v>
+        <v>{{PLAN_CTA_BUTTON}}</v>
       </c>
       <c r="D21" t="str">
         <v/>
@@ -4260,10 +4370,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B22" t="str">
-        <v>Annual Pay Monthly Option</v>
+        <v>Page Title</v>
       </c>
       <c r="C22" t="str">
-        <v>Yes</v>
+        <v>{{PLAN_PAGE_TITLE}}</v>
       </c>
       <c r="D22" t="str">
         <v/>
@@ -4274,10 +4384,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B23" t="str">
-        <v>Annual Pay Monthly Title</v>
+        <v>Annual Pay Monthly Option</v>
       </c>
       <c r="C23" t="str">
-        <v>Annual - Pay Monthly</v>
+        <v>Yes</v>
       </c>
       <c r="D23" t="str">
         <v/>
@@ -4288,10 +4398,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B24" t="str">
-        <v>Annual Pay Monthly Price</v>
+        <v>Annual Pay Monthly Title</v>
       </c>
       <c r="C24" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
+        <v>Annual - Pay Monthly</v>
       </c>
       <c r="D24" t="str">
         <v/>
@@ -4302,10 +4412,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B25" t="str">
-        <v>Annual Pay Monthly Price Length</v>
+        <v>Annual Pay Monthly Price</v>
       </c>
       <c r="C25" t="str">
-        <v>/month</v>
+        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
       </c>
       <c r="D25" t="str">
         <v/>
@@ -4316,10 +4426,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B26" t="str">
-        <v>Annual Pay Monthly Contract Text</v>
+        <v>Annual Pay Monthly Price Length</v>
       </c>
       <c r="C26" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_CONTRACT_TEXT}}</v>
+        <v>/month</v>
       </c>
       <c r="D26" t="str">
         <v/>
@@ -4330,10 +4440,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B27" t="str">
-        <v>Annual Pay Monthly Selected</v>
+        <v>Annual Pay Monthly Contract Text</v>
       </c>
       <c r="C27" t="str">
-        <v>Yes</v>
+        <v>{{ANNUAL_PAY_MONTHLY_CONTRACT_TEXT}}</v>
       </c>
       <c r="D27" t="str">
         <v/>
@@ -4344,7 +4454,7 @@
         <v>Ultimate</v>
       </c>
       <c r="B28" t="str">
-        <v>Annual Pay Upfront Option</v>
+        <v>Annual Pay Monthly Selected</v>
       </c>
       <c r="C28" t="str">
         <v>Yes</v>
@@ -4358,10 +4468,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B29" t="str">
-        <v>Annual Pay Upfront Title</v>
+        <v>Annual Pay Upfront Option</v>
       </c>
       <c r="C29" t="str">
-        <v>Annual - Pay Upfront</v>
+        <v>Yes</v>
       </c>
       <c r="D29" t="str">
         <v/>
@@ -4372,10 +4482,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B30" t="str">
-        <v>Annual Pay Upfront Save Badge</v>
+        <v>Annual Pay Upfront Title</v>
       </c>
       <c r="C30" t="str">
-        <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
+        <v>Annual - Pay Upfront</v>
       </c>
       <c r="D30" t="str">
         <v/>
@@ -4386,10 +4496,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B31" t="str">
-        <v>Annual Pay Upfront Price</v>
+        <v>Annual Pay Upfront Save Badge</v>
       </c>
       <c r="C31" t="str">
-        <v>{{ANNUAL_UPFRONT_PRICE_DISPLAY}}</v>
+        <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
       </c>
       <c r="D31" t="str">
         <v/>
@@ -4400,10 +4510,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B32" t="str">
-        <v>Annual Pay Upfront Price Length</v>
+        <v>Annual Pay Upfront Price</v>
       </c>
       <c r="C32" t="str">
-        <v>/year</v>
+        <v>{{ANNUAL_UPFRONT_PRICE_DISPLAY}}</v>
       </c>
       <c r="D32" t="str">
         <v/>
@@ -4414,10 +4524,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B33" t="str">
-        <v>Annual Pay Upfront Selected</v>
+        <v>Annual Pay Upfront Price Length</v>
       </c>
       <c r="C33" t="str">
-        <v>No</v>
+        <v>/year</v>
       </c>
       <c r="D33" t="str">
         <v/>
@@ -4428,10 +4538,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B34" t="str">
-        <v>Ultimate Feature 1</v>
+        <v>Annual Pay Upfront Selected</v>
       </c>
       <c r="C34" t="str">
-        <v>{{ULTIMATE_FEATURE_1}}</v>
+        <v>No</v>
       </c>
       <c r="D34" t="str">
         <v/>
@@ -4442,10 +4552,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B35" t="str">
-        <v>Ultimate Feature 2</v>
+        <v>Ultimate Feature 1</v>
       </c>
       <c r="C35" t="str">
-        <v>{{ULTIMATE_FEATURE_2}}</v>
+        <v>{{ULTIMATE_FEATURE_1}}</v>
       </c>
       <c r="D35" t="str">
         <v/>
@@ -4456,10 +4566,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B36" t="str">
-        <v>Ultimate Feature 3</v>
+        <v>Ultimate Feature 2</v>
       </c>
       <c r="C36" t="str">
-        <v>{{ULTIMATE_FEATURE_3}}</v>
+        <v>{{ULTIMATE_FEATURE_2}}</v>
       </c>
       <c r="D36" t="str">
         <v/>
@@ -4470,18 +4580,32 @@
         <v>Ultimate</v>
       </c>
       <c r="B37" t="str">
+        <v>Ultimate Feature 3</v>
+      </c>
+      <c r="C37" t="str">
+        <v>{{ULTIMATE_FEATURE_3}}</v>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Ultimate</v>
+      </c>
+      <c r="B38" t="str">
         <v>CTA Button</v>
       </c>
-      <c r="C37" t="str">
+      <c r="C38" t="str">
         <v>{{PLAN_CTA_BUTTON}}</v>
       </c>
-      <c r="D37" t="str">
+      <c r="D38" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D38"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4489,13 +4613,6 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E103"/>
-  <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="27.83203125" customWidth="1"/>
-    <col min="3" max="3" width="28.83203125" customWidth="1"/>
-    <col min="4" max="4" width="160.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6258,10 +6375,6 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B15"/>
-  <cols>
-    <col min="1" max="1" width="27.83203125" customWidth="1"/>
-    <col min="2" max="2" width="90.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6393,10 +6506,6 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B9"/>
-  <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="25.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6479,11 +6588,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B23"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="70.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:B24"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6655,23 +6760,31 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Whats Included CTA</v>
+        <v>Upsell Feature 4</v>
       </c>
       <c r="B22" t="str">
-        <v>Whats included</v>
+        <v>{{UPSELL_FEATURE_4}}</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
+        <v>Whats Included CTA</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Whats included</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
         <v>CTA Button</v>
       </c>
-      <c r="B23" t="str">
+      <c r="B24" t="str">
         <v>{{PPV_CTA_TEXT}}</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B24"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6679,10 +6792,6 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B18"/>
-  <cols>
-    <col min="1" max="1" width="29.83203125" customWidth="1"/>
-    <col min="2" max="2" width="79.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>

<commit_message>
feat: implement mobile PPV banner/tile/paywall validations and robust page checks
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -22,6 +22,7 @@
     <sheet name="Upsell Second Success page" sheetId="17" r:id="rId17"/>
     <sheet name="Upsell Payment page" sheetId="18" r:id="rId18"/>
     <sheet name="Search page" sheetId="19" r:id="rId19"/>
+    <sheet name="paywall" sheetId="20" r:id="rId20"/>
   </sheets>
 </workbook>
 </file>
@@ -2576,6 +2577,73 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B7"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Field</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Expected</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Event Name</v>
+      </c>
+      <c r="B2" t="str">
+        <v>{{PPV_DISPLAY_NAME}}</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Event Date and Time</v>
+      </c>
+      <c r="B3" t="str">
+        <v>{{MOBILE_PPV_DATE}}</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Category</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Matchroom Boxing</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Instruction Header</v>
+      </c>
+      <c r="B5" t="str">
+        <v>How to watch this and more?</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Instruction Text</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Paste this link on your browser and choose the plan that’s right for you</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Copy Button</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Copy</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D94"/>

</xml_diff>

<commit_message>
feat: landing page flows, search/schedule pages, MyAccount updates, getActualValue enhancements, PPV_Input data update
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -415,7 +415,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C25"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -549,9 +549,152 @@
         <v>landing-page-banner</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Banner - Event Title</v>
+      </c>
+      <c r="B13" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+      <c r="C13" t="str">
+        <v>landing-page-banner-ultimate-banner</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Banner - Event Date</v>
+      </c>
+      <c r="B14" t="str">
+        <v>{{PPV_DATE}}</v>
+      </c>
+      <c r="C14" t="str">
+        <v>landing-page-banner-ultimate-banner</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Banner - Event Description</v>
+      </c>
+      <c r="B15" t="str">
+        <v>{{BANNER_DESCRIPTION}}</v>
+      </c>
+      <c r="C15" t="str">
+        <v>landing-page-banner-ultimate-banner</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Banner - Purchased Tag</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Visible</v>
+      </c>
+      <c r="C16" t="str">
+        <v>landing-page-banner-ultimate-banner</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Banner - Buy Now CTA</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Not visible</v>
+      </c>
+      <c r="C17" t="str">
+        <v>landing-page-banner-ultimate-banner</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Banner - Fight Card CTA</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Visible</v>
+      </c>
+      <c r="C18" t="str">
+        <v>landing-page-banner-ultimate-banner</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Banner - Set Reminder CTA</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Visible</v>
+      </c>
+      <c r="C19" t="str">
+        <v>landing-page-banner-ultimate-banner</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Fight Card Modal - Event Title</v>
+      </c>
+      <c r="B20" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+      <c r="C20" t="str">
+        <v>landing-page-banner-ultimate-fight-card</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Fight Card Modal - Event Date</v>
+      </c>
+      <c r="B21" t="str">
+        <v>{{BOXING_BANNER_DATE}}</v>
+      </c>
+      <c r="C21" t="str">
+        <v>landing-page-banner-ultimate-fight-card</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Fight Card Modal - Promoter</v>
+      </c>
+      <c r="B22" t="str">
+        <v>{{PPV_PROMOTER}}</v>
+      </c>
+      <c r="C22" t="str">
+        <v>landing-page-banner-ultimate-fight-card</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Fight Card Modal - Close Button</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Visible</v>
+      </c>
+      <c r="C23" t="str">
+        <v>landing-page-banner-ultimate-fight-card</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Ultimate Navigation Target</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Preview Page|Fixture Page</v>
+      </c>
+      <c r="C24" t="str">
+        <v>landing-page-dont-miss-live-ultimate-tile</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Ultimate Navigation Target</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Preview Page|Fixture Page</v>
+      </c>
+      <c r="C25" t="str">
+        <v>landing-page-dont-miss-ultimate-tile</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C25"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -940,7 +1083,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C37"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1206,16 +1349,159 @@
         <v>Yes</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>home-boxing-banner-ultimate-banner</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Banner - Event Title</v>
+      </c>
+      <c r="C25" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>home-boxing-banner-ultimate-banner</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Banner - Event Date</v>
+      </c>
+      <c r="C26" t="str">
+        <v>{{PPV_DATE}}</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>home-boxing-banner-ultimate-banner</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Banner - Event Description</v>
+      </c>
+      <c r="C27" t="str">
+        <v>{{BANNER_DESCRIPTION}}</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>home-boxing-banner-ultimate-banner</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Banner - Purchased Tag</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>home-boxing-banner-ultimate-banner</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Banner - Buy Now CTA</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Not visible</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>home-boxing-banner-ultimate-banner</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Banner - Fight Card CTA</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>home-boxing-banner-ultimate-banner</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Banner - Set Reminder CTA</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>home-boxing-banner-ultimate-fight-card</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Fight Card Modal - Event Title</v>
+      </c>
+      <c r="C32" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>home-boxing-banner-ultimate-fight-card</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Fight Card Modal - Event Date</v>
+      </c>
+      <c r="C33" t="str">
+        <v>{{BOXING_BANNER_DATE}}</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>home-boxing-banner-ultimate-fight-card</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Fight Card Modal - Promoter</v>
+      </c>
+      <c r="C34" t="str">
+        <v>{{PPV_PROMOTER}}</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>home-boxing-banner-ultimate-fight-card</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Fight Card Modal - Close Button</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>home-boxing-tile-ultimate-tile</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Ultimate Navigation Target</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Preview Page|Fixture Page</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>home-boxing-upcoming-ultimate-tile</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Ultimate Navigation Target</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Preview Page|Fixture Page</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C37"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C38"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1492,9 +1778,152 @@
         <v>Visible</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>home-page-banner-ultimate-banner</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Banner - Event Title</v>
+      </c>
+      <c r="C26" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>home-page-banner-ultimate-banner</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Banner - Event Date</v>
+      </c>
+      <c r="C27" t="str">
+        <v>{{PPV_DATE}}</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>home-page-banner-ultimate-banner</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Banner - Event Description</v>
+      </c>
+      <c r="C28" t="str">
+        <v>{{BANNER_DESCRIPTION}}</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>home-page-banner-ultimate-banner</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Banner - Purchased Tag</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>home-page-banner-ultimate-banner</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Banner - Buy Now CTA</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Not visible</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>home-page-banner-ultimate-banner</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Banner - Fight Card CTA</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>home-page-banner-ultimate-banner</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Banner - Set Reminder CTA</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>home-page-banner-ultimate-fight-card</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Fight Card Modal - Event Title</v>
+      </c>
+      <c r="C33" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>home-page-banner-ultimate-fight-card</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Fight Card Modal - Event Date</v>
+      </c>
+      <c r="C34" t="str">
+        <v>{{BOXING_BANNER_DATE}}</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>home-page-banner-ultimate-fight-card</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Fight Card Modal - Promoter</v>
+      </c>
+      <c r="C35" t="str">
+        <v>{{PPV_PROMOTER}}</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>home-page-banner-ultimate-fight-card</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Fight Card Modal - Close Button</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>home-page-dont-miss-ultimate-tile</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Ultimate Navigation Target</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Preview Page|Fixture Page</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>home-biggest-fights-ultimate-tile</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Ultimate Navigation Target</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Preview Page|Fixture Page</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C38"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2086,7 +2515,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:C6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2095,6 +2524,9 @@
       <c r="B1" t="str">
         <v>Expected</v>
       </c>
+      <c r="C1" t="str">
+        <v>Flow</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -2128,16 +2560,27 @@
         <v>Yes</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Ultimate Navigation Target</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Preview Page|Fixture Page</v>
+      </c>
+      <c r="C6" t="str">
+        <v>ultimate-login-first</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C66"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2733,9 +3176,141 @@
         <v>boxing-bundle-ppv</v>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>Banner - Event Title</v>
+      </c>
+      <c r="B55" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+      <c r="C55" t="str">
+        <v>boxing-ultimate-banner</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>Banner - Event Date</v>
+      </c>
+      <c r="B56" t="str">
+        <v>{{PPV_DATE}}</v>
+      </c>
+      <c r="C56" t="str">
+        <v>boxing-ultimate-banner</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>Banner - Event Description</v>
+      </c>
+      <c r="B57" t="str">
+        <v>{{BANNER_DESCRIPTION}}</v>
+      </c>
+      <c r="C57" t="str">
+        <v>boxing-ultimate-banner</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>Banner - Purchased Tag</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Visible</v>
+      </c>
+      <c r="C58" t="str">
+        <v>boxing-ultimate-banner</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>Banner - Buy Now CTA</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Not visible</v>
+      </c>
+      <c r="C59" t="str">
+        <v>boxing-ultimate-banner</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>Banner - Fight Card CTA</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Visible</v>
+      </c>
+      <c r="C60" t="str">
+        <v>boxing-ultimate-banner</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>Banner - Set Reminder CTA</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Visible</v>
+      </c>
+      <c r="C61" t="str">
+        <v>boxing-ultimate-banner</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>Fight Card Modal - Event Title</v>
+      </c>
+      <c r="B62" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+      <c r="C62" t="str">
+        <v>boxing-ultimate-fight-card</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>Fight Card Modal - Event Date</v>
+      </c>
+      <c r="B63" t="str">
+        <v>{{BOXING_BANNER_DATE}}</v>
+      </c>
+      <c r="C63" t="str">
+        <v>boxing-ultimate-fight-card</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>Fight Card Modal - Promoter</v>
+      </c>
+      <c r="B64" t="str">
+        <v>{{PPV_PROMOTER}}</v>
+      </c>
+      <c r="C64" t="str">
+        <v>boxing-ultimate-fight-card</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>Fight Card Modal - Close Button</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Visible</v>
+      </c>
+      <c r="C65" t="str">
+        <v>boxing-ultimate-fight-card</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>Ultimate Navigation Target</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Preview Page|Fixture Page</v>
+      </c>
+      <c r="C66" t="str">
+        <v>boxing-upcoming-ultimate-tile</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C54"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C66"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6374,7 +6949,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:C16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6383,6 +6958,9 @@
       <c r="B1" t="str">
         <v>Expected</v>
       </c>
+      <c r="C1" t="str">
+        <v>Flow</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -6496,9 +7074,20 @@
         <v>Yes</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Ultimate Navigation Target</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Preview Page|Fixture Page</v>
+      </c>
+      <c r="C16" t="str">
+        <v>ultimate-login-first</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C16"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: AJ Joshua config updates, PPV_Input data, PaymentPage fixes, getActualValue enhancements, mobile spec updates
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -415,7 +415,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C12"/>
+  <cols>
+    <col min="1" max="1" width="33.83203125" customWidth="1"/>
+    <col min="2" max="2" width="27.83203125" customWidth="1"/>
+    <col min="3" max="3" width="21.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -549,152 +554,9 @@
         <v>landing-page-banner</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Banner - Event Title</v>
-      </c>
-      <c r="B13" t="str">
-        <v>{{PPV_NAME}}</v>
-      </c>
-      <c r="C13" t="str">
-        <v>landing-page-banner-ultimate-banner</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Banner - Event Date</v>
-      </c>
-      <c r="B14" t="str">
-        <v>{{PPV_DATE}}</v>
-      </c>
-      <c r="C14" t="str">
-        <v>landing-page-banner-ultimate-banner</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>Banner - Event Description</v>
-      </c>
-      <c r="B15" t="str">
-        <v>{{BANNER_DESCRIPTION}}</v>
-      </c>
-      <c r="C15" t="str">
-        <v>landing-page-banner-ultimate-banner</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>Banner - Purchased Tag</v>
-      </c>
-      <c r="B16" t="str">
-        <v>Visible</v>
-      </c>
-      <c r="C16" t="str">
-        <v>landing-page-banner-ultimate-banner</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>Banner - Buy Now CTA</v>
-      </c>
-      <c r="B17" t="str">
-        <v>Not visible</v>
-      </c>
-      <c r="C17" t="str">
-        <v>landing-page-banner-ultimate-banner</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>Banner - Fight Card CTA</v>
-      </c>
-      <c r="B18" t="str">
-        <v>Visible</v>
-      </c>
-      <c r="C18" t="str">
-        <v>landing-page-banner-ultimate-banner</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>Banner - Set Reminder CTA</v>
-      </c>
-      <c r="B19" t="str">
-        <v>Visible</v>
-      </c>
-      <c r="C19" t="str">
-        <v>landing-page-banner-ultimate-banner</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>Fight Card Modal - Event Title</v>
-      </c>
-      <c r="B20" t="str">
-        <v>{{PPV_NAME}}</v>
-      </c>
-      <c r="C20" t="str">
-        <v>landing-page-banner-ultimate-fight-card</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>Fight Card Modal - Event Date</v>
-      </c>
-      <c r="B21" t="str">
-        <v>{{BOXING_BANNER_DATE}}</v>
-      </c>
-      <c r="C21" t="str">
-        <v>landing-page-banner-ultimate-fight-card</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>Fight Card Modal - Promoter</v>
-      </c>
-      <c r="B22" t="str">
-        <v>{{PPV_PROMOTER}}</v>
-      </c>
-      <c r="C22" t="str">
-        <v>landing-page-banner-ultimate-fight-card</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>Fight Card Modal - Close Button</v>
-      </c>
-      <c r="B23" t="str">
-        <v>Visible</v>
-      </c>
-      <c r="C23" t="str">
-        <v>landing-page-banner-ultimate-fight-card</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>Ultimate Navigation Target</v>
-      </c>
-      <c r="B24" t="str">
-        <v>Preview Page|Fixture Page</v>
-      </c>
-      <c r="C24" t="str">
-        <v>landing-page-dont-miss-live-ultimate-tile</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>Ultimate Navigation Target</v>
-      </c>
-      <c r="B25" t="str">
-        <v>Preview Page|Fixture Page</v>
-      </c>
-      <c r="C25" t="str">
-        <v>landing-page-dont-miss-ultimate-tile</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C12"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -702,6 +564,11 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C23"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="27.83203125" customWidth="1"/>
+    <col min="3" max="3" width="318.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -966,6 +833,10 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B6"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="64.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1025,6 +896,10 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B6"/>
+  <cols>
+    <col min="1" max="1" width="19.83203125" customWidth="1"/>
+    <col min="2" max="2" width="34.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1083,7 +958,12 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C24"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="90.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1349,159 +1229,21 @@
         <v>Yes</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>home-boxing-banner-ultimate-banner</v>
-      </c>
-      <c r="B25" t="str">
-        <v>Banner - Event Title</v>
-      </c>
-      <c r="C25" t="str">
-        <v>{{PPV_NAME}}</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v>home-boxing-banner-ultimate-banner</v>
-      </c>
-      <c r="B26" t="str">
-        <v>Banner - Event Date</v>
-      </c>
-      <c r="C26" t="str">
-        <v>{{PPV_DATE}}</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v>home-boxing-banner-ultimate-banner</v>
-      </c>
-      <c r="B27" t="str">
-        <v>Banner - Event Description</v>
-      </c>
-      <c r="C27" t="str">
-        <v>{{BANNER_DESCRIPTION}}</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>home-boxing-banner-ultimate-banner</v>
-      </c>
-      <c r="B28" t="str">
-        <v>Banner - Purchased Tag</v>
-      </c>
-      <c r="C28" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v>home-boxing-banner-ultimate-banner</v>
-      </c>
-      <c r="B29" t="str">
-        <v>Banner - Buy Now CTA</v>
-      </c>
-      <c r="C29" t="str">
-        <v>Not visible</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="str">
-        <v>home-boxing-banner-ultimate-banner</v>
-      </c>
-      <c r="B30" t="str">
-        <v>Banner - Fight Card CTA</v>
-      </c>
-      <c r="C30" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <v>home-boxing-banner-ultimate-banner</v>
-      </c>
-      <c r="B31" t="str">
-        <v>Banner - Set Reminder CTA</v>
-      </c>
-      <c r="C31" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="str">
-        <v>home-boxing-banner-ultimate-fight-card</v>
-      </c>
-      <c r="B32" t="str">
-        <v>Fight Card Modal - Event Title</v>
-      </c>
-      <c r="C32" t="str">
-        <v>{{PPV_NAME}}</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v>home-boxing-banner-ultimate-fight-card</v>
-      </c>
-      <c r="B33" t="str">
-        <v>Fight Card Modal - Event Date</v>
-      </c>
-      <c r="C33" t="str">
-        <v>{{BOXING_BANNER_DATE}}</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <v>home-boxing-banner-ultimate-fight-card</v>
-      </c>
-      <c r="B34" t="str">
-        <v>Fight Card Modal - Promoter</v>
-      </c>
-      <c r="C34" t="str">
-        <v>{{PPV_PROMOTER}}</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v>home-boxing-banner-ultimate-fight-card</v>
-      </c>
-      <c r="B35" t="str">
-        <v>Fight Card Modal - Close Button</v>
-      </c>
-      <c r="C35" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v>home-boxing-tile-ultimate-tile</v>
-      </c>
-      <c r="B36" t="str">
-        <v>Ultimate Navigation Target</v>
-      </c>
-      <c r="C36" t="str">
-        <v>Preview Page|Fixture Page</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="str">
-        <v>home-boxing-upcoming-ultimate-tile</v>
-      </c>
-      <c r="B37" t="str">
-        <v>Ultimate Navigation Target</v>
-      </c>
-      <c r="C37" t="str">
-        <v>Preview Page|Fixture Page</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C24"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C19"/>
+  <cols>
+    <col min="1" max="1" width="21.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="90.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1712,218 +1454,9 @@
         <v>Visible</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>home-page-popup</v>
-      </c>
-      <c r="B20" t="str">
-        <v>Home Popup Image Present</v>
-      </c>
-      <c r="C20" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>home-page-popup</v>
-      </c>
-      <c r="B21" t="str">
-        <v>Home Popup Event Title</v>
-      </c>
-      <c r="C21" t="str">
-        <v>{{PPV_NAME}}</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>home-page-popup</v>
-      </c>
-      <c r="B22" t="str">
-        <v>Home Popup Event Date</v>
-      </c>
-      <c r="C22" t="str">
-        <v>{{HOME_POPUP_DATE}}</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>home-page-popup</v>
-      </c>
-      <c r="B23" t="str">
-        <v>Home Popup Event Description</v>
-      </c>
-      <c r="C23" t="str">
-        <v>{{HOME_POPUP_DESCRIPTION}}</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>home-page-popup</v>
-      </c>
-      <c r="B24" t="str">
-        <v>Home Popup Buy Now CTA</v>
-      </c>
-      <c r="C24" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>home-page-popup</v>
-      </c>
-      <c r="B25" t="str">
-        <v>Home Popup Close Button</v>
-      </c>
-      <c r="C25" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v>home-page-banner-ultimate-banner</v>
-      </c>
-      <c r="B26" t="str">
-        <v>Banner - Event Title</v>
-      </c>
-      <c r="C26" t="str">
-        <v>{{PPV_NAME}}</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v>home-page-banner-ultimate-banner</v>
-      </c>
-      <c r="B27" t="str">
-        <v>Banner - Event Date</v>
-      </c>
-      <c r="C27" t="str">
-        <v>{{PPV_DATE}}</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>home-page-banner-ultimate-banner</v>
-      </c>
-      <c r="B28" t="str">
-        <v>Banner - Event Description</v>
-      </c>
-      <c r="C28" t="str">
-        <v>{{BANNER_DESCRIPTION}}</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v>home-page-banner-ultimate-banner</v>
-      </c>
-      <c r="B29" t="str">
-        <v>Banner - Purchased Tag</v>
-      </c>
-      <c r="C29" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="str">
-        <v>home-page-banner-ultimate-banner</v>
-      </c>
-      <c r="B30" t="str">
-        <v>Banner - Buy Now CTA</v>
-      </c>
-      <c r="C30" t="str">
-        <v>Not visible</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <v>home-page-banner-ultimate-banner</v>
-      </c>
-      <c r="B31" t="str">
-        <v>Banner - Fight Card CTA</v>
-      </c>
-      <c r="C31" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="str">
-        <v>home-page-banner-ultimate-banner</v>
-      </c>
-      <c r="B32" t="str">
-        <v>Banner - Set Reminder CTA</v>
-      </c>
-      <c r="C32" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v>home-page-banner-ultimate-fight-card</v>
-      </c>
-      <c r="B33" t="str">
-        <v>Fight Card Modal - Event Title</v>
-      </c>
-      <c r="C33" t="str">
-        <v>{{PPV_NAME}}</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <v>home-page-banner-ultimate-fight-card</v>
-      </c>
-      <c r="B34" t="str">
-        <v>Fight Card Modal - Event Date</v>
-      </c>
-      <c r="C34" t="str">
-        <v>{{BOXING_BANNER_DATE}}</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v>home-page-banner-ultimate-fight-card</v>
-      </c>
-      <c r="B35" t="str">
-        <v>Fight Card Modal - Promoter</v>
-      </c>
-      <c r="C35" t="str">
-        <v>{{PPV_PROMOTER}}</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v>home-page-banner-ultimate-fight-card</v>
-      </c>
-      <c r="B36" t="str">
-        <v>Fight Card Modal - Close Button</v>
-      </c>
-      <c r="C36" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="str">
-        <v>home-page-dont-miss-ultimate-tile</v>
-      </c>
-      <c r="B37" t="str">
-        <v>Ultimate Navigation Target</v>
-      </c>
-      <c r="C37" t="str">
-        <v>Preview Page|Fixture Page</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="str">
-        <v>home-biggest-fights-ultimate-tile</v>
-      </c>
-      <c r="B38" t="str">
-        <v>Ultimate Navigation Target</v>
-      </c>
-      <c r="C38" t="str">
-        <v>Preview Page|Fixture Page</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C19"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1931,6 +1464,11 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C31"/>
+  <cols>
+    <col min="1" max="1" width="33.83203125" customWidth="1"/>
+    <col min="2" max="2" width="124.83203125" customWidth="1"/>
+    <col min="3" max="3" width="11.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2283,6 +1821,10 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B7"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="21.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2350,6 +1892,10 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B7"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2417,6 +1963,10 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B11"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="27.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2515,7 +2065,11 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:B5"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2524,9 +2078,6 @@
       <c r="B1" t="str">
         <v>Expected</v>
       </c>
-      <c r="C1" t="str">
-        <v>Flow</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -2560,27 +2111,21 @@
         <v>Yes</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Ultimate Navigation Target</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Preview Page|Fixture Page</v>
-      </c>
-      <c r="C6" t="str">
-        <v>ultimate-login-first</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C66"/>
+  <dimension ref="A1:C54"/>
+  <cols>
+    <col min="1" max="1" width="29.83203125" customWidth="1"/>
+    <col min="2" max="2" width="60.83203125" customWidth="1"/>
+    <col min="3" max="3" width="19.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3176,141 +2721,9 @@
         <v>boxing-bundle-ppv</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" t="str">
-        <v>Banner - Event Title</v>
-      </c>
-      <c r="B55" t="str">
-        <v>{{PPV_NAME}}</v>
-      </c>
-      <c r="C55" t="str">
-        <v>boxing-ultimate-banner</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="str">
-        <v>Banner - Event Date</v>
-      </c>
-      <c r="B56" t="str">
-        <v>{{PPV_DATE}}</v>
-      </c>
-      <c r="C56" t="str">
-        <v>boxing-ultimate-banner</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="str">
-        <v>Banner - Event Description</v>
-      </c>
-      <c r="B57" t="str">
-        <v>{{BANNER_DESCRIPTION}}</v>
-      </c>
-      <c r="C57" t="str">
-        <v>boxing-ultimate-banner</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="str">
-        <v>Banner - Purchased Tag</v>
-      </c>
-      <c r="B58" t="str">
-        <v>Visible</v>
-      </c>
-      <c r="C58" t="str">
-        <v>boxing-ultimate-banner</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="str">
-        <v>Banner - Buy Now CTA</v>
-      </c>
-      <c r="B59" t="str">
-        <v>Not visible</v>
-      </c>
-      <c r="C59" t="str">
-        <v>boxing-ultimate-banner</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="str">
-        <v>Banner - Fight Card CTA</v>
-      </c>
-      <c r="B60" t="str">
-        <v>Visible</v>
-      </c>
-      <c r="C60" t="str">
-        <v>boxing-ultimate-banner</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="str">
-        <v>Banner - Set Reminder CTA</v>
-      </c>
-      <c r="B61" t="str">
-        <v>Visible</v>
-      </c>
-      <c r="C61" t="str">
-        <v>boxing-ultimate-banner</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="str">
-        <v>Fight Card Modal - Event Title</v>
-      </c>
-      <c r="B62" t="str">
-        <v>{{PPV_NAME}}</v>
-      </c>
-      <c r="C62" t="str">
-        <v>boxing-ultimate-fight-card</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="str">
-        <v>Fight Card Modal - Event Date</v>
-      </c>
-      <c r="B63" t="str">
-        <v>{{BOXING_BANNER_DATE}}</v>
-      </c>
-      <c r="C63" t="str">
-        <v>boxing-ultimate-fight-card</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="str">
-        <v>Fight Card Modal - Promoter</v>
-      </c>
-      <c r="B64" t="str">
-        <v>{{PPV_PROMOTER}}</v>
-      </c>
-      <c r="C64" t="str">
-        <v>boxing-ultimate-fight-card</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="str">
-        <v>Fight Card Modal - Close Button</v>
-      </c>
-      <c r="B65" t="str">
-        <v>Visible</v>
-      </c>
-      <c r="C65" t="str">
-        <v>boxing-ultimate-fight-card</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="str">
-        <v>Ultimate Navigation Target</v>
-      </c>
-      <c r="B66" t="str">
-        <v>Preview Page|Fixture Page</v>
-      </c>
-      <c r="C66" t="str">
-        <v>boxing-upcoming-ultimate-tile</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C66"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C54"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3318,6 +2731,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D94"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="37.83203125" customWidth="1"/>
+    <col min="3" max="3" width="201.83203125" customWidth="1"/>
+    <col min="4" max="4" width="9.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4645,6 +4064,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D38"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="34.83203125" customWidth="1"/>
+    <col min="3" max="3" width="70.83203125" customWidth="1"/>
+    <col min="4" max="4" width="6.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5188,6 +4613,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E103"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="27.83203125" customWidth="1"/>
+    <col min="3" max="3" width="28.83203125" customWidth="1"/>
+    <col min="4" max="4" width="160.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5557,7 +4989,7 @@
         <v>Today You Pay Price</v>
       </c>
       <c r="D22" t="str">
-        <v>{{PPV_PRICE}}</v>
+        <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
       <c r="E22" t="str">
         <v/>
@@ -5761,7 +5193,7 @@
         <v>Today You Pay Price</v>
       </c>
       <c r="D34" t="str">
-        <v>{{PPV_PRICE}}</v>
+        <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
       <c r="E34" t="str">
         <v/>
@@ -6949,7 +6381,11 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:B15"/>
+  <cols>
+    <col min="1" max="1" width="27.83203125" customWidth="1"/>
+    <col min="2" max="2" width="90.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6958,9 +6394,6 @@
       <c r="B1" t="str">
         <v>Expected</v>
       </c>
-      <c r="C1" t="str">
-        <v>Flow</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -7074,20 +6507,9 @@
         <v>Yes</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>Ultimate Navigation Target</v>
-      </c>
-      <c r="B16" t="str">
-        <v>Preview Page|Fixture Page</v>
-      </c>
-      <c r="C16" t="str">
-        <v>ultimate-login-first</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B15"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7095,6 +6517,10 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B9"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="25.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7178,6 +6604,10 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B24"/>
+  <cols>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="70.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7381,6 +6811,10 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B18"/>
+  <cols>
+    <col min="1" max="1" width="29.83203125" customWidth="1"/>
+    <col min="2" max="2" width="79.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7451,7 +6885,7 @@
         <v>Today You Pay Price</v>
       </c>
       <c r="B9" t="str">
-        <v>{{PPV_PRICE}}</v>
+        <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
feat: enhance search flow, popup validation, banner DOM extraction, and CI updates
## Summary
Syncing all local automation enhancements to personal repo main branch.

### Key Changes
- SearchPage: robust PPV tile search with upcoming fallback
- validateVariant: popup field filtering + search Buy Now skip
- getActualValue: search context handlers, banner DOM extraction
- resolveExpected: expanded banner date logic, popup description refactor
- compare: relaxed date-only matching
- testHelpers: popup field whitelisting
- generateExcel: updated landing page validation fields
- Specs: rewritten search flow, popup handling fixes
- CI: added Playwright browser install step
- Config: updated test credentials and playwright timezone
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -416,6 +416,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C12"/>
+  <cols>
+    <col min="1" max="1" width="33.83203125" customWidth="1"/>
+    <col min="2" max="2" width="27.83203125" customWidth="1"/>
+    <col min="3" max="3" width="21.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -430,7 +435,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Don&amp;apos;t Miss Live on DAZN Section</v>
+        <v>Don't Miss Live on DAZN Section</v>
       </c>
       <c r="B2" t="str">
         <v>Yes</v>
@@ -550,7 +555,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:C12"/>
   </ignoredErrors>
@@ -559,7 +563,12 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="27.83203125" customWidth="1"/>
+    <col min="3" max="3" width="318.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -599,10 +608,10 @@
         <v>common</v>
       </c>
       <c r="B4" t="str">
-        <v>Payment Method Present</v>
+        <v>Terms And Conditions Text</v>
       </c>
       <c r="C4" t="str">
-        <v>Yes</v>
+        <v>By changing the terms of your subscription, you confirm that you have read and agree to our Terms and Conditions of Use (including the instruction regarding your right of withdrawal). Your subscription auto-renews unless you cancel before the end of the minimum term by selecting 'Cancel Subscription' in My Account.</v>
       </c>
     </row>
     <row r="5">
@@ -610,10 +619,10 @@
         <v>common</v>
       </c>
       <c r="B5" t="str">
-        <v>Confirm Button</v>
+        <v>Payment Method Present</v>
       </c>
       <c r="C5" t="str">
-        <v>Confirm</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="6">
@@ -621,21 +630,21 @@
         <v>common</v>
       </c>
       <c r="B6" t="str">
-        <v>Terms Link Present</v>
+        <v>Confirm Button</v>
       </c>
       <c r="C6" t="str">
-        <v>Yes</v>
+        <v>Confirm</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>annual pay upfront</v>
+        <v>common</v>
       </c>
       <c r="B7" t="str">
-        <v>Legal Text Line 1</v>
+        <v>Terms Link Present</v>
       </c>
       <c r="C7" t="str">
-        <v>Your plan will be changed to DAZN Ultimate today {{TODAY_DATE}} and your contract will last 12 months.</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="8">
@@ -643,10 +652,10 @@
         <v>annual pay upfront</v>
       </c>
       <c r="B8" t="str">
-        <v>Legal Text Line 2</v>
+        <v>Legal Text Line 1</v>
       </c>
       <c r="C8" t="str">
-        <v>Today you will be charged {{CURRENCY}}{{ANNUAL_UPFRONT_PRICE}} minus the remainder of your last payment which was not used in full. From {{NEXT_PAYMENT_DATE}} you will be charged {{CURRENCY}}{{ANNUAL_UPFRONT_PRICE}}/year.</v>
+        <v>Your plan will be changed to DAZN Ultimate today {{TODAY_DATE}} and your contract will last 12 months.</v>
       </c>
     </row>
     <row r="9">
@@ -654,10 +663,10 @@
         <v>annual pay upfront</v>
       </c>
       <c r="B9" t="str">
-        <v>Rate Plan</v>
+        <v>Legal Text Line 2</v>
       </c>
       <c r="C9" t="str">
-        <v>Annual - Pay Upfront</v>
+        <v>Today you will be charged {{CURRENCY}}{{ANNUAL_UPFRONT_PRICE}} minus the remainder of your last payment which was not used in full. From {{NEXT_PAYMENT_DATE}} you will be charged {{CURRENCY}}{{ANNUAL_UPFRONT_PRICE}}/year.</v>
       </c>
     </row>
     <row r="10">
@@ -665,10 +674,10 @@
         <v>annual pay upfront</v>
       </c>
       <c r="B10" t="str">
-        <v>Rate Plan Price</v>
+        <v>Rate Plan</v>
       </c>
       <c r="C10" t="str">
-        <v>{{ANNUAL_UPFRONT_PRICE}}</v>
+        <v>Annual - Pay Upfront</v>
       </c>
     </row>
     <row r="11">
@@ -676,10 +685,10 @@
         <v>annual pay upfront</v>
       </c>
       <c r="B11" t="str">
-        <v>Rate Plan Period</v>
+        <v>Rate Plan Price</v>
       </c>
       <c r="C11" t="str">
-        <v>/year</v>
+        <v>{{ANNUAL_UPFRONT_PRICE}}</v>
       </c>
     </row>
     <row r="12">
@@ -687,10 +696,10 @@
         <v>annual pay upfront</v>
       </c>
       <c r="B12" t="str">
-        <v>Rate Plan Description</v>
+        <v>Rate Plan Period</v>
       </c>
       <c r="C12" t="str">
-        <v>Get the best value when you pay upfront.</v>
+        <v>/year</v>
       </c>
     </row>
     <row r="13">
@@ -698,10 +707,10 @@
         <v>annual pay upfront</v>
       </c>
       <c r="B13" t="str">
-        <v>Next Payment Label</v>
+        <v>Rate Plan Description</v>
       </c>
       <c r="C13" t="str">
-        <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
+        <v>Get the best value when you pay upfront.</v>
       </c>
     </row>
     <row r="14">
@@ -709,21 +718,21 @@
         <v>annual pay upfront</v>
       </c>
       <c r="B14" t="str">
-        <v>Next Payment Date</v>
+        <v>Next Payment Label</v>
       </c>
       <c r="C14" t="str">
-        <v>{{NEXT_PAYMENT_DATE}}</v>
+        <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>annual pay monthly</v>
+        <v>annual pay upfront</v>
       </c>
       <c r="B15" t="str">
-        <v>Legal Text Line 1</v>
+        <v>Next Payment Date</v>
       </c>
       <c r="C15" t="str">
-        <v>Your plan will be changed to DAZN Ultimate today {{TODAY_DATE}} and your contract will last 12 months.</v>
+        <v>{{NEXT_PAYMENT_DATE}}</v>
       </c>
     </row>
     <row r="16">
@@ -731,10 +740,10 @@
         <v>annual pay monthly</v>
       </c>
       <c r="B16" t="str">
-        <v>Legal Text Line 2</v>
+        <v>Legal Text Line 1</v>
       </c>
       <c r="C16" t="str">
-        <v>Today you will be charged {{CURRENCY}}{{ANNUAL_PAY_MONTHLY_PRICE}} minus the remainder of your last payment which was not used in full. From {{NEXT_PAYMENT_DATE}} you will be charged {{CURRENCY}}{{ANNUAL_PAY_MONTHLY_PRICE}} /month.</v>
+        <v>Your plan will be changed to DAZN Ultimate today {{TODAY_DATE}} and your contract will last 12 months.</v>
       </c>
     </row>
     <row r="17">
@@ -742,10 +751,10 @@
         <v>annual pay monthly</v>
       </c>
       <c r="B17" t="str">
-        <v>Rate Plan</v>
+        <v>Legal Text Line 2</v>
       </c>
       <c r="C17" t="str">
-        <v>Annual - Pay Monthly</v>
+        <v>Today you will be charged {{CURRENCY}}{{ANNUAL_PAY_MONTHLY_PRICE}} minus the remainder of your last payment which was not used in full. From {{NEXT_PAYMENT_DATE}} you will be charged {{CURRENCY}}{{ANNUAL_PAY_MONTHLY_PRICE}} /month.</v>
       </c>
     </row>
     <row r="18">
@@ -753,10 +762,10 @@
         <v>annual pay monthly</v>
       </c>
       <c r="B18" t="str">
-        <v>Rate Plan Price</v>
+        <v>Rate Plan</v>
       </c>
       <c r="C18" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
+        <v>Annual - Pay Monthly</v>
       </c>
     </row>
     <row r="19">
@@ -764,10 +773,10 @@
         <v>annual pay monthly</v>
       </c>
       <c r="B19" t="str">
-        <v>Rate Plan Period</v>
+        <v>Rate Plan Price</v>
       </c>
       <c r="C19" t="str">
-        <v>/ month</v>
+        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
       </c>
     </row>
     <row r="20">
@@ -775,10 +784,10 @@
         <v>annual pay monthly</v>
       </c>
       <c r="B20" t="str">
-        <v>Rate Plan Description</v>
+        <v>Rate Plan Period</v>
       </c>
       <c r="C20" t="str">
-        <v>Annual contract. Paid in 12 monthly instalments.</v>
+        <v>/ month</v>
       </c>
     </row>
     <row r="21">
@@ -786,10 +795,10 @@
         <v>annual pay monthly</v>
       </c>
       <c r="B21" t="str">
-        <v>Next Payment Label</v>
+        <v>Rate Plan Description</v>
       </c>
       <c r="C21" t="str">
-        <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
+        <v>Annual contract. Paid in 12 monthly instalments.</v>
       </c>
     </row>
     <row r="22">
@@ -797,16 +806,26 @@
         <v>annual pay monthly</v>
       </c>
       <c r="B22" t="str">
+        <v>Next Payment Label</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>annual pay monthly</v>
+      </c>
+      <c r="B23" t="str">
         <v>Next Payment Date</v>
       </c>
-      <c r="C22" t="str">
+      <c r="C23" t="str">
         <v>{{NEXT_PAYMENT_DATE}}</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C23"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -814,6 +833,10 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B6"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="64.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -864,7 +887,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
   </ignoredErrors>
@@ -874,6 +896,10 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B6"/>
+  <cols>
+    <col min="1" max="1" width="19.83203125" customWidth="1"/>
+    <col min="2" max="2" width="34.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -924,7 +950,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
   </ignoredErrors>
@@ -933,7 +958,12 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C24"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="90.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1089,10 +1119,119 @@
         <v>Visible</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Best of Boxing Section</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Present</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B16" t="str">
+        <v>PPV Tile Present</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B17" t="str">
+        <v>PPV Date</v>
+      </c>
+      <c r="C17" t="str">
+        <v>{{LANDING_PAGE_PPV_DATE}}</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B18" t="str">
+        <v>PPV Promoter on Tile</v>
+      </c>
+      <c r="C18" t="str">
+        <v>{{PPV_PROMOTER}}</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B19" t="str">
+        <v>PPV Name</v>
+      </c>
+      <c r="C19" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B20" t="str">
+        <v>PPV Date and Time Text</v>
+      </c>
+      <c r="C20" t="str">
+        <v>WATCH LIVE {{HOME_BOXING_UPCOMING_DATE}} at {{HOME_BOXING_UPCOMING_TIME}}</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Buy Now CTA</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Buy now</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Fight Card CTA</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Fight card</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B23" t="str">
+        <v>PPV Image Present</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Lock Icon Present</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C24"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1100,6 +1239,11 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C19"/>
+  <cols>
+    <col min="1" max="1" width="21.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="90.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1241,7 +1385,7 @@
         <v>Biggest Fights Section</v>
       </c>
       <c r="C13" t="str">
-        <v>The Biggest Fights|Saturday Fight Night|Fight Night|Upcoming Big Fights|Big Fights|Full Fights</v>
+        <v>Saturday Fight Night</v>
       </c>
     </row>
     <row r="14">
@@ -1311,7 +1455,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:C19"/>
   </ignoredErrors>
@@ -1321,6 +1464,11 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C31"/>
+  <cols>
+    <col min="1" max="1" width="33.83203125" customWidth="1"/>
+    <col min="2" max="2" width="124.83203125" customWidth="1"/>
+    <col min="3" max="3" width="11.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1338,7 +1486,7 @@
         <v>Page Title</v>
       </c>
       <c r="B2" t="str">
-        <v>Choose a plan that&amp;apos;s right for you</v>
+        <v>Choose a plan that's right for you</v>
       </c>
       <c r="C2" t="str">
         <v>checked</v>
@@ -1664,7 +1812,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:C31"/>
   </ignoredErrors>
@@ -1674,6 +1821,10 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B7"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="21.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1732,7 +1883,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
   </ignoredErrors>
@@ -1742,6 +1892,10 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B7"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1800,7 +1954,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
   </ignoredErrors>
@@ -1810,6 +1963,10 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B11"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="27.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1900,7 +2057,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B11"/>
   </ignoredErrors>
@@ -1909,7 +2065,11 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
+  <cols>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1937,31 +2097,43 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>PPV Date</v>
+        <v>PPV Image Present</v>
       </c>
       <c r="B4" t="str">
-        <v>{{PPV_DATE}}</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Buy Now Button</v>
+        <v>PPV Date and Time Text</v>
       </c>
       <c r="B5" t="str">
+        <v>{{PPV_DATE}}|{{LANDING_PAGE_PPV_DATE}}</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Lock Icon Present</v>
+      </c>
+      <c r="B6" t="str">
         <v>Yes</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C54"/>
+  <cols>
+    <col min="1" max="1" width="29.83203125" customWidth="1"/>
+    <col min="2" max="2" width="60.83203125" customWidth="1"/>
+    <col min="3" max="3" width="19.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2009,10 +2181,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>PPV Date and Time Text</v>
+        <v>Or Separator</v>
       </c>
       <c r="B5" t="str">
-        <v>{{PPV_DATE}}</v>
+        <v>or</v>
       </c>
       <c r="C5" t="str">
         <v>boxing</v>
@@ -2020,10 +2192,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Or Separator</v>
+        <v>Buy Fight CTA</v>
       </c>
       <c r="B6" t="str">
-        <v>or</v>
+        <v>Buy this fight for {{PPV_PRICE}}</v>
       </c>
       <c r="C6" t="str">
         <v>boxing</v>
@@ -2031,10 +2203,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Buy Fight CTA</v>
+        <v>Get Included CTA</v>
       </c>
       <c r="B7" t="str">
-        <v>Buy this fight for {{PPV_PRICE}}</v>
+        <v>Get included in DAZN Ultimate</v>
       </c>
       <c r="C7" t="str">
         <v>boxing</v>
@@ -2042,10 +2214,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Get Included CTA</v>
+        <v>Best Value Badge</v>
       </c>
       <c r="B8" t="str">
-        <v>Get included in DAZN Ultimate</v>
+        <v>Best value for boxing fans</v>
       </c>
       <c r="C8" t="str">
         <v>boxing</v>
@@ -2053,21 +2225,21 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Best Value Badge</v>
+        <v>Upcoming Big Fights Heading</v>
       </c>
       <c r="B9" t="str">
-        <v>Best value for boxing fans</v>
+        <v>Upcoming Big Fights</v>
       </c>
       <c r="C9" t="str">
-        <v>boxing</v>
+        <v>boxing-upcoming</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Upcoming Big Fights Heading</v>
+        <v>PPV Name</v>
       </c>
       <c r="B10" t="str">
-        <v>Upcoming Big Fights</v>
+        <v>{{PPV_DISPLAY_NAME}}</v>
       </c>
       <c r="C10" t="str">
         <v>boxing-upcoming</v>
@@ -2075,10 +2247,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>PPV Name</v>
+        <v>PPV Date and Time Text</v>
       </c>
       <c r="B11" t="str">
-        <v>{{PPV_DISPLAY_NAME}}</v>
+        <v>{{PPV_DATE}}</v>
       </c>
       <c r="C11" t="str">
         <v>boxing-upcoming</v>
@@ -2086,10 +2258,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>PPV Date and Time Text</v>
+        <v>PPV Description Text</v>
       </c>
       <c r="B12" t="str">
-        <v>{{PPV_DATE}}</v>
+        <v>{{PPV_LOCATION}}</v>
       </c>
       <c r="C12" t="str">
         <v>boxing-upcoming</v>
@@ -2097,10 +2269,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>PPV Description Text</v>
+        <v>PPV Image Present</v>
       </c>
       <c r="B13" t="str">
-        <v>{{PPV_LOCATION}}</v>
+        <v>Yes</v>
       </c>
       <c r="C13" t="str">
         <v>boxing-upcoming</v>
@@ -2108,10 +2280,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>PPV Image Present</v>
+        <v>Buy Now CTA</v>
       </c>
       <c r="B14" t="str">
-        <v>Yes</v>
+        <v>Buy now</v>
       </c>
       <c r="C14" t="str">
         <v>boxing-upcoming</v>
@@ -2119,21 +2291,21 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Buy Now CTA</v>
+        <v>Bundle Section Present</v>
       </c>
       <c r="B15" t="str">
-        <v>Buy now</v>
+        <v>Yes</v>
       </c>
       <c r="C15" t="str">
-        <v>boxing-upcoming</v>
+        <v>boxing-bundle</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Bundle Section Present</v>
+        <v>Bundle Section Title</v>
       </c>
       <c r="B16" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_SECTION_TITLE}}</v>
       </c>
       <c r="C16" t="str">
         <v>boxing-bundle</v>
@@ -2141,10 +2313,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Bundle Section Title</v>
+        <v>Bundle Section Subtitle</v>
       </c>
       <c r="B17" t="str">
-        <v>{{BUNDLE_SECTION_TITLE}}</v>
+        <v>{{BUNDLE_SECTION_SUBTITLE}}</v>
       </c>
       <c r="C17" t="str">
         <v>boxing-bundle</v>
@@ -2152,10 +2324,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Bundle Section Subtitle</v>
+        <v>Bundle Title</v>
       </c>
       <c r="B18" t="str">
-        <v>{{BUNDLE_SECTION_SUBTITLE}}</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="C18" t="str">
         <v>boxing-bundle</v>
@@ -2163,10 +2335,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Bundle Title</v>
+        <v>Bundle Description</v>
       </c>
       <c r="B19" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>{{BUNDLE_DESCRIPTION}}</v>
       </c>
       <c r="C19" t="str">
         <v>boxing-bundle</v>
@@ -2174,10 +2346,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Bundle Description</v>
+        <v>Bundle Price</v>
       </c>
       <c r="B20" t="str">
-        <v>{{BUNDLE_DESCRIPTION}}</v>
+        <v>{{BUNDLE_PRICE}}</v>
       </c>
       <c r="C20" t="str">
         <v>boxing-bundle</v>
@@ -2185,10 +2357,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Bundle Price</v>
+        <v>Bundle Original Price</v>
       </c>
       <c r="B21" t="str">
-        <v>{{BUNDLE_PRICE}}</v>
+        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
       </c>
       <c r="C21" t="str">
         <v>boxing-bundle</v>
@@ -2196,10 +2368,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Bundle Original Price</v>
+        <v>Bundle Save Badge</v>
       </c>
       <c r="B22" t="str">
-        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
+        <v>{{BUNDLE_SAVE_BADGE}}</v>
       </c>
       <c r="C22" t="str">
         <v>boxing-bundle</v>
@@ -2207,10 +2379,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Bundle Save Badge</v>
+        <v>Bundle Fight Count</v>
       </c>
       <c r="B23" t="str">
-        <v>{{BUNDLE_SAVE_BADGE}}</v>
+        <v>{{BUNDLE_FIGHT_COUNT}}</v>
       </c>
       <c r="C23" t="str">
         <v>boxing-bundle</v>
@@ -2218,10 +2390,10 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Bundle Fight Count</v>
+        <v>Bundle PPV 1 Name</v>
       </c>
       <c r="B24" t="str">
-        <v>{{BUNDLE_FIGHT_COUNT}}</v>
+        <v>{{BUNDLE_PPV1_NAME}}</v>
       </c>
       <c r="C24" t="str">
         <v>boxing-bundle</v>
@@ -2229,10 +2401,10 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Bundle PPV 1 Name</v>
+        <v>Bundle PPV 1 Date</v>
       </c>
       <c r="B25" t="str">
-        <v>{{BUNDLE_PPV1_NAME}}</v>
+        <v>{{BUNDLE_PPV1_LANDING_DATE}}</v>
       </c>
       <c r="C25" t="str">
         <v>boxing-bundle</v>
@@ -2240,10 +2412,10 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Bundle PPV 1 Date</v>
+        <v>Bundle PPV 1 Image</v>
       </c>
       <c r="B26" t="str">
-        <v>{{BUNDLE_PPV1_LANDING_DATE}}</v>
+        <v>Yes</v>
       </c>
       <c r="C26" t="str">
         <v>boxing-bundle</v>
@@ -2251,10 +2423,10 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Bundle PPV 1 Image</v>
+        <v>Bundle PPV 2 Name</v>
       </c>
       <c r="B27" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_PPV2_NAME}}</v>
       </c>
       <c r="C27" t="str">
         <v>boxing-bundle</v>
@@ -2262,10 +2434,10 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Bundle PPV 2 Name</v>
+        <v>Bundle PPV 2 Date</v>
       </c>
       <c r="B28" t="str">
-        <v>{{BUNDLE_PPV2_NAME}}</v>
+        <v>{{BUNDLE_PPV2_LANDING_DATE}}</v>
       </c>
       <c r="C28" t="str">
         <v>boxing-bundle</v>
@@ -2273,10 +2445,10 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Bundle PPV 2 Date</v>
+        <v>Bundle PPV 2 Image</v>
       </c>
       <c r="B29" t="str">
-        <v>{{BUNDLE_PPV2_LANDING_DATE}}</v>
+        <v>Yes</v>
       </c>
       <c r="C29" t="str">
         <v>boxing-bundle</v>
@@ -2284,10 +2456,10 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Bundle PPV 2 Image</v>
+        <v>Get Started CTA</v>
       </c>
       <c r="B30" t="str">
-        <v>Yes</v>
+        <v>Get Started</v>
       </c>
       <c r="C30" t="str">
         <v>boxing-bundle</v>
@@ -2295,21 +2467,21 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Get Started CTA</v>
+        <v>Page Title</v>
       </c>
       <c r="B31" t="str">
-        <v>Get Started</v>
+        <v>Choose the right plan for you.</v>
       </c>
       <c r="C31" t="str">
-        <v>boxing-bundle</v>
+        <v>boxing-bundle-ppv</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Page Title</v>
+        <v>Header Sub Text</v>
       </c>
       <c r="B32" t="str">
-        <v>Choose the right plan for you.</v>
+        <v>To watch your pay-per-view, you'll need a DAZN plan.</v>
       </c>
       <c r="C32" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2317,10 +2489,10 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Header Sub Text</v>
+        <v>Bundle Card Title</v>
       </c>
       <c r="B33" t="str">
-        <v>To watch your pay-per-view, you&amp;apos;ll need a DAZN plan.</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="C33" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2328,10 +2500,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Bundle Card Title</v>
+        <v>Bundle Card Description</v>
       </c>
       <c r="B34" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>{{BUNDLE_PPV_CARD_DESCRIPTION}}</v>
       </c>
       <c r="C34" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2339,10 +2511,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Bundle Card Description</v>
+        <v>Bundle Card Selected</v>
       </c>
       <c r="B35" t="str">
-        <v>{{BUNDLE_PPV_CARD_DESCRIPTION}}</v>
+        <v>Yes</v>
       </c>
       <c r="C35" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2350,10 +2522,10 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Bundle Card Selected</v>
+        <v>Bundle Card Price</v>
       </c>
       <c r="B36" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_PRICE}}</v>
       </c>
       <c r="C36" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2361,10 +2533,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Bundle Card Price</v>
+        <v>Bundle Card Original Price</v>
       </c>
       <c r="B37" t="str">
-        <v>{{BUNDLE_PRICE}}</v>
+        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
       </c>
       <c r="C37" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2372,10 +2544,10 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Bundle Card Original Price</v>
+        <v>Bundle Card Save Badge</v>
       </c>
       <c r="B38" t="str">
-        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
+        <v>{{BUNDLE_SAVE_BADGE}}</v>
       </c>
       <c r="C38" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2383,10 +2555,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Bundle Card Save Badge</v>
+        <v>Bundle PPV 1 Full Name</v>
       </c>
       <c r="B39" t="str">
-        <v>{{BUNDLE_SAVE_BADGE}}</v>
+        <v>{{BUNDLE_PPV1_FULL_NAME}}</v>
       </c>
       <c r="C39" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2394,10 +2566,10 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Bundle PPV 1 Full Name</v>
+        <v>Bundle PPV 1 PPV Date</v>
       </c>
       <c r="B40" t="str">
-        <v>{{BUNDLE_PPV1_FULL_NAME}}</v>
+        <v>{{BUNDLE_PPV1_DATE}}</v>
       </c>
       <c r="C40" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2405,10 +2577,10 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Bundle PPV 1 PPV Date</v>
+        <v>Bundle PPV 1 PPV Image</v>
       </c>
       <c r="B41" t="str">
-        <v>{{BUNDLE_PPV1_DATE}}</v>
+        <v>Yes</v>
       </c>
       <c r="C41" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2416,10 +2588,10 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Bundle PPV 1 PPV Image</v>
+        <v>Bundle PPV 2 Full Name</v>
       </c>
       <c r="B42" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_PPV2_FULL_NAME}}</v>
       </c>
       <c r="C42" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2427,10 +2599,10 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Bundle PPV 2 Full Name</v>
+        <v>Bundle PPV 2 PPV Date</v>
       </c>
       <c r="B43" t="str">
-        <v>{{BUNDLE_PPV2_FULL_NAME}}</v>
+        <v>{{BUNDLE_PPV2_DATE}}</v>
       </c>
       <c r="C43" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2438,10 +2610,10 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Bundle PPV 2 PPV Date</v>
+        <v>Bundle PPV 2 PPV Image</v>
       </c>
       <c r="B44" t="str">
-        <v>{{BUNDLE_PPV2_DATE}}</v>
+        <v>Yes</v>
       </c>
       <c r="C44" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2449,7 +2621,7 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Bundle PPV 2 PPV Image</v>
+        <v>Upsell Section Present</v>
       </c>
       <c r="B45" t="str">
         <v>Yes</v>
@@ -2460,10 +2632,10 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Upsell Section Present</v>
+        <v>Upsell Badge</v>
       </c>
       <c r="B46" t="str">
-        <v>Yes</v>
+        <v>The Ultimate Fan Package</v>
       </c>
       <c r="C46" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2471,10 +2643,10 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Upsell Badge</v>
+        <v>Upsell Plan Name</v>
       </c>
       <c r="B47" t="str">
-        <v>The Ultimate Fan Package</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="C47" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2482,10 +2654,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Upsell Plan Name</v>
+        <v>Upsell Price</v>
       </c>
       <c r="B48" t="str">
-        <v>DAZN Ultimate</v>
+        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
       </c>
       <c r="C48" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2493,10 +2665,10 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Upsell Price</v>
+        <v>Upsell Contract Text</v>
       </c>
       <c r="B49" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
+        <v>Annual contract. Auto renews.</v>
       </c>
       <c r="C49" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2504,10 +2676,10 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Upsell Contract Text</v>
+        <v>Fights Included Text</v>
       </c>
       <c r="B50" t="str">
-        <v>Annual contract. Auto renews.</v>
+        <v>All these fights included and more.</v>
       </c>
       <c r="C50" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2515,10 +2687,10 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Fights Included Text</v>
+        <v>Upsell Feature 1</v>
       </c>
       <c r="B51" t="str">
-        <v>All these fights included and more.</v>
+        <v>Minimum 12 pay-per-views a year included at no extra cost.</v>
       </c>
       <c r="C51" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2526,10 +2698,10 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Upsell Feature 1</v>
+        <v>Upsell Feature 2</v>
       </c>
       <c r="B52" t="str">
-        <v>Minimum 12 pay-per-views a year included at no extra cost.</v>
+        <v>185+ fights a year from the world's best promoters.</v>
       </c>
       <c r="C52" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2537,10 +2709,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Upsell Feature 2</v>
+        <v>Upsell Feature 3</v>
       </c>
       <c r="B53" t="str">
-        <v>185+ fights a year from the world&amp;apos;s best promoters.</v>
+        <v>HDR and Dolby 5.1 surround sound on select events</v>
       </c>
       <c r="C53" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2548,30 +2720,18 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Upsell Feature 3</v>
+        <v>CTA Button</v>
       </c>
       <c r="B54" t="str">
-        <v>HDR and Dolby 5.1 surround sound on select events</v>
+        <v>Continue with DAZN Ultimate</v>
       </c>
       <c r="C54" t="str">
         <v>boxing-bundle-ppv</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" t="str">
-        <v>CTA Button</v>
-      </c>
-      <c r="B55" t="str">
-        <v>Continue with DAZN Ultimate</v>
-      </c>
-      <c r="C55" t="str">
-        <v>boxing-bundle-ppv</v>
-      </c>
-    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C55"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C54"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2579,6 +2739,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D94"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="37.83203125" customWidth="1"/>
+    <col min="3" max="3" width="201.83203125" customWidth="1"/>
+    <col min="4" max="4" width="9.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2604,6 +2770,9 @@
       <c r="C2" t="str">
         <v>Choose the right plan for you.</v>
       </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -2613,7 +2782,10 @@
         <v>Header Sub Text</v>
       </c>
       <c r="C3" t="str">
-        <v>To watch your pay-per-view, you&amp;apos;ll need a DAZN plan.</v>
+        <v>To watch your pay-per-view, you'll need a DAZN plan.</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -2626,6 +2798,9 @@
       <c r="C4" t="str">
         <v>N/A</v>
       </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -2637,6 +2812,9 @@
       <c r="C5" t="str">
         <v>{{PPV_DISPLAY_NAME}}</v>
       </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -2648,6 +2826,9 @@
       <c r="C6" t="str">
         <v>/fight</v>
       </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -2659,6 +2840,9 @@
       <c r="C7" t="str">
         <v>{{PPV_PRICE}}</v>
       </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -2670,6 +2854,9 @@
       <c r="C8" t="str">
         <v>{{CURRENCY}}</v>
       </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -2695,6 +2882,9 @@
       <c r="C10" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -2706,6 +2896,9 @@
       <c r="C11" t="str">
         <v>Yes</v>
       </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -2717,6 +2910,9 @@
       <c r="C12" t="str">
         <v>{{PPV_DATE}}</v>
       </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -2728,6 +2924,9 @@
       <c r="C13" t="str">
         <v>Yes</v>
       </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -2739,6 +2938,9 @@
       <c r="C14" t="str">
         <v>{{PPV_DISPLAY_NAME}}</v>
       </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -2750,6 +2952,9 @@
       <c r="C15" t="str">
         <v>{{PPV_CARD_DESCRIPTION}}</v>
       </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -2761,6 +2966,9 @@
       <c r="C16" t="str">
         <v>Yes</v>
       </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -2772,6 +2980,9 @@
       <c r="C17" t="str">
         <v>The Ultimate Fan Package</v>
       </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -2783,6 +2994,9 @@
       <c r="C18" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -2794,6 +3008,9 @@
       <c r="C19" t="str">
         <v>N/A</v>
       </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -2805,6 +3022,9 @@
       <c r="C20" t="str">
         <v>{{UPSELL_PRICE}}</v>
       </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -2816,6 +3036,9 @@
       <c r="C21" t="str">
         <v>{{UPSELL_PRICE_LENGTH}}</v>
       </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -2827,6 +3050,9 @@
       <c r="C22" t="str">
         <v>{{UPSELL_CROSSED_PRICE}}</v>
       </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -2838,6 +3064,9 @@
       <c r="C23" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_CONTRACT_TEXT}}</v>
       </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -2863,6 +3092,9 @@
       <c r="C25" t="str">
         <v>{{UPSELL_SECTION_HEADING}}</v>
       </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -2874,6 +3106,9 @@
       <c r="C26" t="str">
         <v>N/A</v>
       </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -2885,6 +3120,9 @@
       <c r="C27" t="str">
         <v>N/A</v>
       </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -2896,6 +3134,9 @@
       <c r="C28" t="str">
         <v>N/A</v>
       </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -2907,6 +3148,9 @@
       <c r="C29" t="str">
         <v>N/A</v>
       </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -2918,6 +3162,9 @@
       <c r="C30" t="str">
         <v>N/A</v>
       </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -2929,6 +3176,9 @@
       <c r="C31" t="str">
         <v>{{UPSELL_FEATURE_1}}</v>
       </c>
+      <c r="D31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -2940,6 +3190,9 @@
       <c r="C32" t="str">
         <v>N/A</v>
       </c>
+      <c r="D32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -2951,6 +3204,9 @@
       <c r="C33" t="str">
         <v>{{UPSELL_FEATURE_2}}</v>
       </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -2962,6 +3218,9 @@
       <c r="C34" t="str">
         <v>{{UPSELL_FEATURE_3}}</v>
       </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -2973,6 +3232,9 @@
       <c r="C35" t="str">
         <v>N/A</v>
       </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -2984,6 +3246,9 @@
       <c r="C36" t="str">
         <v>N/A</v>
       </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -2995,6 +3260,9 @@
       <c r="C37" t="str">
         <v>N/A</v>
       </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -3006,6 +3274,9 @@
       <c r="C38" t="str">
         <v>N/A</v>
       </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -3199,6 +3470,9 @@
       <c r="C52" t="str">
         <v>{{PPV_CTA_TEXT}}</v>
       </c>
+      <c r="D52" t="str">
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -3224,6 +3498,9 @@
       <c r="C54" t="str">
         <v>Choose your plan</v>
       </c>
+      <c r="D54" t="str">
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -3235,6 +3512,9 @@
       <c r="C55" t="str">
         <v>Buy {{PPV_NAME}} with DAZN Standard or get it included in DAZN Ultimate.</v>
       </c>
+      <c r="D55" t="str">
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -3246,6 +3526,9 @@
       <c r="C56" t="str">
         <v>get it included in DAZN Ultimate.</v>
       </c>
+      <c r="D56" t="str">
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -3257,6 +3540,9 @@
       <c r="C57" t="str">
         <v>Yes</v>
       </c>
+      <c r="D57" t="str">
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -3268,6 +3554,9 @@
       <c r="C58" t="str">
         <v>{{PPV_DATE}}</v>
       </c>
+      <c r="D58" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -3279,6 +3568,9 @@
       <c r="C59" t="str">
         <v>{{PPV_DISPLAY_NAME}}</v>
       </c>
+      <c r="D59" t="str">
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -3290,6 +3582,9 @@
       <c r="C60" t="str">
         <v>Yes</v>
       </c>
+      <c r="D60" t="str">
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -3301,6 +3596,9 @@
       <c r="C61" t="str">
         <v>Yes</v>
       </c>
+      <c r="D61" t="str">
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -3312,6 +3610,9 @@
       <c r="C62" t="str">
         <v>{{PPV_DISPLAY_NAME}}</v>
       </c>
+      <c r="D62" t="str">
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -3323,6 +3624,9 @@
       <c r="C63" t="str">
         <v>/fight</v>
       </c>
+      <c r="D63" t="str">
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -3334,6 +3638,9 @@
       <c r="C64" t="str">
         <v>{{PPV_PRICE}}</v>
       </c>
+      <c r="D64" t="str">
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -3345,6 +3652,9 @@
       <c r="C65" t="str">
         <v>{{CURRENCY}}</v>
       </c>
+      <c r="D65" t="str">
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -3356,6 +3666,9 @@
       <c r="C66" t="str">
         <v>Choose your subscription</v>
       </c>
+      <c r="D66" t="str">
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -3367,6 +3680,9 @@
       <c r="C67" t="str">
         <v>Yes</v>
       </c>
+      <c r="D67" t="str">
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -3378,6 +3694,9 @@
       <c r="C68" t="str">
         <v>7-day free trial of DAZN Standard</v>
       </c>
+      <c r="D68" t="str">
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -3389,6 +3708,9 @@
       <c r="C69" t="str">
         <v>Yes</v>
       </c>
+      <c r="D69" t="str">
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -3400,6 +3722,9 @@
       <c r="C70" t="str">
         <v>Yes</v>
       </c>
+      <c r="D70" t="str">
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -3411,6 +3736,9 @@
       <c r="C71" t="str">
         <v>7-days free access to DAZN Standard.</v>
       </c>
+      <c r="D71" t="str">
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -3422,6 +3750,9 @@
       <c r="C72" t="str">
         <v>Cancel anytime during the trial and only pay for the fight. After the trial you move onto a Monthly Flex plan for {{CURRENCY}}{{MONTHLY_PRICE}}/month. You will not lose access to the pay-per-view[s].</v>
       </c>
+      <c r="D72" t="str">
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -3433,6 +3764,9 @@
       <c r="C73" t="str">
         <v>Yes</v>
       </c>
+      <c r="D73" t="str">
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -3444,6 +3778,9 @@
       <c r="C74" t="str">
         <v>Pay-per-views included</v>
       </c>
+      <c r="D74" t="str">
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -3455,6 +3792,9 @@
       <c r="C75" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="D75" t="str">
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -3466,6 +3806,9 @@
       <c r="C76" t="str">
         <v>From</v>
       </c>
+      <c r="D76" t="str">
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -3477,6 +3820,9 @@
       <c r="C77" t="str">
         <v>{{UPSELL_PRICE}}</v>
       </c>
+      <c r="D77" t="str">
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -3488,6 +3834,9 @@
       <c r="C78" t="str">
         <v>{{UPSELL_PRICE_LENGTH}}</v>
       </c>
+      <c r="D78" t="str">
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -3499,6 +3848,9 @@
       <c r="C79" t="str">
         <v>Annual contract. Auto renews.</v>
       </c>
+      <c r="D79" t="str">
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -3510,6 +3862,9 @@
       <c r="C80" t="str">
         <v>Yes</v>
       </c>
+      <c r="D80" t="str">
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -3521,6 +3876,9 @@
       <c r="C81" t="str">
         <v>N/A</v>
       </c>
+      <c r="D81" t="str">
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -3532,6 +3890,9 @@
       <c r="C82" t="str">
         <v>N/A</v>
       </c>
+      <c r="D82" t="str">
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -3543,6 +3904,9 @@
       <c r="C83" t="str">
         <v>N/A</v>
       </c>
+      <c r="D83" t="str">
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -3554,6 +3918,9 @@
       <c r="C84" t="str">
         <v>N/A</v>
       </c>
+      <c r="D84" t="str">
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -3565,6 +3932,9 @@
       <c r="C85" t="str">
         <v>Pay-per-views included at no extra cost. Minimum of 12 events per year including {{PPV_NAME}}.</v>
       </c>
+      <c r="D85" t="str">
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -3576,6 +3946,9 @@
       <c r="C86" t="str">
         <v>{{PPV_NAME}}.</v>
       </c>
+      <c r="D86" t="str">
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -3587,6 +3960,9 @@
       <c r="C87" t="str">
         <v>HDR and Dolby 5.1 surround sound on select events.</v>
       </c>
+      <c r="D87" t="str">
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -3596,7 +3972,10 @@
         <v>Upsell Feature 3</v>
       </c>
       <c r="C88" t="str">
-        <v>185+ fights a year from the best promoters</v>
+        <v>185+ fights a year from the world's best promoters.</v>
+      </c>
+      <c r="D88" t="str">
+        <v/>
       </c>
     </row>
     <row r="89">
@@ -3609,6 +3988,9 @@
       <c r="C89" t="str">
         <v>Whats included</v>
       </c>
+      <c r="D89" t="str">
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -3620,6 +4002,9 @@
       <c r="C90" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="D90" t="str">
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -3631,6 +4016,9 @@
       <c r="C91" t="str">
         <v>get it included in DAZN Ultimate.</v>
       </c>
+      <c r="D91" t="str">
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -3642,6 +4030,9 @@
       <c r="C92" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="D92" t="str">
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
@@ -3653,6 +4044,9 @@
       <c r="C93" t="str">
         <v>Continue with PPV + 7-day free trial</v>
       </c>
+      <c r="D93" t="str">
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
@@ -3664,9 +4058,11 @@
       <c r="C94" t="str">
         <v>N/A</v>
       </c>
+      <c r="D94" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:D94"/>
   </ignoredErrors>
@@ -3675,7 +4071,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D38"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="34.83203125" customWidth="1"/>
+    <col min="3" max="3" width="70.83203125" customWidth="1"/>
+    <col min="4" max="4" width="6.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3701,6 +4103,9 @@
       <c r="C2" t="str">
         <v>{{PLAN_PAGE_TITLE}}</v>
       </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -3712,6 +4117,9 @@
       <c r="C3" t="str">
         <v>Yes</v>
       </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -3723,6 +4131,9 @@
       <c r="C4" t="str">
         <v>Flex – Pay Monthly</v>
       </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -3734,6 +4145,9 @@
       <c r="C5" t="str">
         <v>{{FLEX_BADGE}}</v>
       </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -3745,6 +4159,9 @@
       <c r="C6" t="str">
         <v>{{FLEX_DESCRIPTION}}</v>
       </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -3756,6 +4173,9 @@
       <c r="C7" t="str">
         <v>Yes</v>
       </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -3767,16 +4187,22 @@
       <c r="C8" t="str">
         <v>{{FLEX_TODAY_TEXT}}</v>
       </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
         <v>Standard</v>
       </c>
       <c r="B9" t="str">
-        <v>Flex Future Text</v>
+        <v>Flex Future Date</v>
       </c>
       <c r="C9" t="str">
-        <v>{{FLEX_FUTURE_TEXT}}</v>
+        <v>{{FLEX_FUTURE_DATE}}</v>
+      </c>
+      <c r="D9" t="str">
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -3784,10 +4210,13 @@
         <v>Standard</v>
       </c>
       <c r="B10" t="str">
-        <v>Annual Card Present</v>
+        <v>Flex Future Text</v>
       </c>
       <c r="C10" t="str">
-        <v>Yes</v>
+        <v>{{FLEX_FUTURE_TEXT}}</v>
+      </c>
+      <c r="D10" t="str">
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -3795,10 +4224,13 @@
         <v>Standard</v>
       </c>
       <c r="B11" t="str">
-        <v>Annual Savings Badge</v>
+        <v>Annual Card Present</v>
       </c>
       <c r="C11" t="str">
-        <v>{{ANNUAL_SAVINGS_BADGE}}</v>
+        <v>Yes</v>
+      </c>
+      <c r="D11" t="str">
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -3806,10 +4238,13 @@
         <v>Standard</v>
       </c>
       <c r="B12" t="str">
-        <v>Annual Title</v>
+        <v>Annual Savings Badge</v>
       </c>
       <c r="C12" t="str">
-        <v>Annual - Pay Monthly</v>
+        <v>{{ANNUAL_SAVINGS_BADGE}}</v>
+      </c>
+      <c r="D12" t="str">
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -3817,10 +4252,13 @@
         <v>Standard</v>
       </c>
       <c r="B13" t="str">
-        <v>Annual Badge</v>
+        <v>Annual Title</v>
       </c>
       <c r="C13" t="str">
-        <v>1 MONTH FREE</v>
+        <v>Annual - Pay Monthly</v>
+      </c>
+      <c r="D13" t="str">
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -3828,10 +4266,13 @@
         <v>Standard</v>
       </c>
       <c r="B14" t="str">
-        <v>Annual Price Text</v>
+        <v>Annual Badge</v>
       </c>
       <c r="C14" t="str">
-        <v>then {{CURRENCY}}{{ANNUAL_PRICE}}/month for {{ANNUAL_MONTHS}} months</v>
+        <v>1 MONTH FREE</v>
+      </c>
+      <c r="D14" t="str">
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -3839,10 +4280,13 @@
         <v>Standard</v>
       </c>
       <c r="B15" t="str">
-        <v>Annual Contract Text</v>
+        <v>Annual Price Text</v>
       </c>
       <c r="C15" t="str">
-        <v>Annual contract. Auto renews.</v>
+        <v>then {{CURRENCY}}{{ANNUAL_PRICE}}/month for {{ANNUAL_MONTHS}} months</v>
+      </c>
+      <c r="D15" t="str">
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -3850,10 +4294,13 @@
         <v>Standard</v>
       </c>
       <c r="B16" t="str">
-        <v>Annual Feature 1</v>
+        <v>Annual Contract Text</v>
       </c>
       <c r="C16" t="str">
-        <v>185+ fights a year from the world&amp;apos;s best promoters.</v>
+        <v>Annual contract. Auto renews.</v>
+      </c>
+      <c r="D16" t="str">
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -3861,10 +4308,13 @@
         <v>Standard</v>
       </c>
       <c r="B17" t="str">
-        <v>Annual Feature 2</v>
+        <v>Annual Feature 1</v>
       </c>
       <c r="C17" t="str">
-        <v>Additional cost for pay-per-view events.</v>
+        <v>185+ fights a year from the world's best promoters.</v>
+      </c>
+      <c r="D17" t="str">
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -3872,10 +4322,13 @@
         <v>Standard</v>
       </c>
       <c r="B18" t="str">
-        <v>Annual Feature 3</v>
+        <v>Annual Feature 2</v>
       </c>
       <c r="C18" t="str">
-        <v>Full HD video resolution.</v>
+        <v>Additional cost for pay-per-view events.</v>
+      </c>
+      <c r="D18" t="str">
+        <v/>
       </c>
     </row>
     <row r="19">
@@ -3883,10 +4336,13 @@
         <v>Standard</v>
       </c>
       <c r="B19" t="str">
-        <v>Annual Selected</v>
+        <v>Annual Feature 3</v>
       </c>
       <c r="C19" t="str">
-        <v>No</v>
+        <v>Full HD video resolution.</v>
+      </c>
+      <c r="D19" t="str">
+        <v/>
       </c>
     </row>
     <row r="20">
@@ -3894,21 +4350,27 @@
         <v>Standard</v>
       </c>
       <c r="B20" t="str">
-        <v>CTA Button</v>
+        <v>Annual Selected</v>
       </c>
       <c r="C20" t="str">
-        <v>{{PLAN_CTA_BUTTON}}</v>
+        <v>No</v>
+      </c>
+      <c r="D20" t="str">
+        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Ultimate</v>
+        <v>Standard</v>
       </c>
       <c r="B21" t="str">
-        <v>Page Title</v>
+        <v>CTA Button</v>
       </c>
       <c r="C21" t="str">
-        <v>{{PLAN_PAGE_TITLE}}</v>
+        <v>{{PLAN_CTA_BUTTON}}</v>
+      </c>
+      <c r="D21" t="str">
+        <v/>
       </c>
     </row>
     <row r="22">
@@ -3916,10 +4378,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B22" t="str">
-        <v>Annual Pay Monthly Option</v>
+        <v>Page Title</v>
       </c>
       <c r="C22" t="str">
-        <v>Yes</v>
+        <v>{{PLAN_PAGE_TITLE}}</v>
+      </c>
+      <c r="D22" t="str">
+        <v/>
       </c>
     </row>
     <row r="23">
@@ -3927,10 +4392,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B23" t="str">
-        <v>Annual Pay Monthly Title</v>
+        <v>Annual Pay Monthly Option</v>
       </c>
       <c r="C23" t="str">
-        <v>Annual - Pay Monthly</v>
+        <v>Yes</v>
+      </c>
+      <c r="D23" t="str">
+        <v/>
       </c>
     </row>
     <row r="24">
@@ -3938,10 +4406,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B24" t="str">
-        <v>Annual Pay Monthly Price</v>
+        <v>Annual Pay Monthly Title</v>
       </c>
       <c r="C24" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
+        <v>Annual - Pay Monthly</v>
+      </c>
+      <c r="D24" t="str">
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -3949,10 +4420,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B25" t="str">
-        <v>Annual Pay Monthly Price Length</v>
+        <v>Annual Pay Monthly Price</v>
       </c>
       <c r="C25" t="str">
-        <v>/month</v>
+        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
+      </c>
+      <c r="D25" t="str">
+        <v/>
       </c>
     </row>
     <row r="26">
@@ -3960,10 +4434,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B26" t="str">
-        <v>Annual Pay Monthly Contract Text</v>
+        <v>Annual Pay Monthly Price Length</v>
       </c>
       <c r="C26" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_CONTRACT_TEXT}}</v>
+        <v>/month</v>
+      </c>
+      <c r="D26" t="str">
+        <v/>
       </c>
     </row>
     <row r="27">
@@ -3971,10 +4448,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B27" t="str">
-        <v>Annual Pay Monthly Selected</v>
+        <v>Annual Pay Monthly Contract Text</v>
       </c>
       <c r="C27" t="str">
-        <v>Yes</v>
+        <v>{{ANNUAL_PAY_MONTHLY_CONTRACT_TEXT}}</v>
+      </c>
+      <c r="D27" t="str">
+        <v/>
       </c>
     </row>
     <row r="28">
@@ -3982,10 +4462,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B28" t="str">
-        <v>Annual Pay Upfront Option</v>
+        <v>Annual Pay Monthly Selected</v>
       </c>
       <c r="C28" t="str">
         <v>Yes</v>
+      </c>
+      <c r="D28" t="str">
+        <v/>
       </c>
     </row>
     <row r="29">
@@ -3993,10 +4476,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B29" t="str">
-        <v>Annual Pay Upfront Title</v>
+        <v>Annual Pay Upfront Option</v>
       </c>
       <c r="C29" t="str">
-        <v>Annual - Pay Upfront</v>
+        <v>Yes</v>
+      </c>
+      <c r="D29" t="str">
+        <v/>
       </c>
     </row>
     <row r="30">
@@ -4004,10 +4490,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B30" t="str">
-        <v>Annual Pay Upfront Save Badge</v>
+        <v>Annual Pay Upfront Title</v>
       </c>
       <c r="C30" t="str">
-        <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
+        <v>Annual - Pay Upfront</v>
+      </c>
+      <c r="D30" t="str">
+        <v/>
       </c>
     </row>
     <row r="31">
@@ -4015,10 +4504,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B31" t="str">
-        <v>Annual Pay Upfront Price</v>
+        <v>Annual Pay Upfront Save Badge</v>
       </c>
       <c r="C31" t="str">
-        <v>{{ANNUAL_UPFRONT_PRICE_DISPLAY}}</v>
+        <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
+      </c>
+      <c r="D31" t="str">
+        <v/>
       </c>
     </row>
     <row r="32">
@@ -4026,10 +4518,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B32" t="str">
-        <v>Annual Pay Upfront Price Length</v>
+        <v>Annual Pay Upfront Price</v>
       </c>
       <c r="C32" t="str">
-        <v>/year</v>
+        <v>{{ANNUAL_UPFRONT_PRICE_DISPLAY}}</v>
+      </c>
+      <c r="D32" t="str">
+        <v/>
       </c>
     </row>
     <row r="33">
@@ -4037,10 +4532,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B33" t="str">
-        <v>Annual Pay Upfront Selected</v>
+        <v>Annual Pay Upfront Price Length</v>
       </c>
       <c r="C33" t="str">
-        <v>No</v>
+        <v>/year</v>
+      </c>
+      <c r="D33" t="str">
+        <v/>
       </c>
     </row>
     <row r="34">
@@ -4048,10 +4546,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B34" t="str">
-        <v>Ultimate Feature 1</v>
+        <v>Annual Pay Upfront Selected</v>
       </c>
       <c r="C34" t="str">
-        <v>{{ULTIMATE_FEATURE_1}}</v>
+        <v>No</v>
+      </c>
+      <c r="D34" t="str">
+        <v/>
       </c>
     </row>
     <row r="35">
@@ -4059,10 +4560,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B35" t="str">
-        <v>Ultimate Feature 2</v>
+        <v>Ultimate Feature 1</v>
       </c>
       <c r="C35" t="str">
-        <v>{{ULTIMATE_FEATURE_2}}</v>
+        <v>{{ULTIMATE_FEATURE_1}}</v>
+      </c>
+      <c r="D35" t="str">
+        <v/>
       </c>
     </row>
     <row r="36">
@@ -4070,10 +4574,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B36" t="str">
-        <v>Ultimate Feature 3</v>
+        <v>Ultimate Feature 2</v>
       </c>
       <c r="C36" t="str">
-        <v>{{ULTIMATE_FEATURE_3}}</v>
+        <v>{{ULTIMATE_FEATURE_2}}</v>
+      </c>
+      <c r="D36" t="str">
+        <v/>
       </c>
     </row>
     <row r="37">
@@ -4081,16 +4588,32 @@
         <v>Ultimate</v>
       </c>
       <c r="B37" t="str">
+        <v>Ultimate Feature 3</v>
+      </c>
+      <c r="C37" t="str">
+        <v>{{ULTIMATE_FEATURE_3}}</v>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Ultimate</v>
+      </c>
+      <c r="B38" t="str">
         <v>CTA Button</v>
       </c>
-      <c r="C37" t="str">
+      <c r="C38" t="str">
         <v>{{PLAN_CTA_BUTTON}}</v>
       </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D38"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4098,6 +4621,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E103"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="27.83203125" customWidth="1"/>
+    <col min="3" max="3" width="28.83203125" customWidth="1"/>
+    <col min="4" max="4" width="160.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4129,6 +4659,9 @@
       <c r="D2" t="str">
         <v>Payment method</v>
       </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -4143,6 +4676,9 @@
       <c r="D3" t="str">
         <v>Purchase summary</v>
       </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -4157,6 +4693,9 @@
       <c r="D4" t="str">
         <v>Change</v>
       </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -4171,6 +4710,9 @@
       <c r="D5" t="str">
         <v>Yes</v>
       </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -4185,6 +4727,9 @@
       <c r="D6" t="str">
         <v>Yes</v>
       </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -4199,6 +4744,9 @@
       <c r="D7" t="str">
         <v>Yes</v>
       </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -4264,6 +4812,9 @@
       <c r="D11" t="str">
         <v>Yes</v>
       </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -4312,6 +4863,9 @@
       <c r="D14" t="str">
         <v>DAZN Standard</v>
       </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -4326,6 +4880,9 @@
       <c r="D15" t="str">
         <v>{{PAYMENT_PLAN_NAME}}</v>
       </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -4340,6 +4897,9 @@
       <c r="D16" t="str">
         <v>{{PAYMENT_FLEX_CANCEL_NOTICE}}</v>
       </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -4354,6 +4914,9 @@
       <c r="D17" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -4368,6 +4931,9 @@
       <c r="D18" t="str">
         <v>{{PAYMENT_FREE_TEXT}}</v>
       </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -4382,6 +4948,9 @@
       <c r="D19" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -4396,6 +4965,9 @@
       <c r="D20" t="str">
         <v>{{PPV_PRICE}}</v>
       </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -4410,6 +4982,9 @@
       <c r="D21" t="str">
         <v>Today you pay</v>
       </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -4422,7 +4997,10 @@
         <v>Today You Pay Price</v>
       </c>
       <c r="D22" t="str">
-        <v>{{PPV_PRICE}}</v>
+        <v>{{TODAY_YOU_PAY_PRICE}}</v>
+      </c>
+      <c r="E22" t="str">
+        <v/>
       </c>
     </row>
     <row r="23">
@@ -4438,6 +5016,9 @@
       <c r="D23" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -4452,6 +5033,9 @@
       <c r="D24" t="str">
         <v>{{PAYMENT_FLEX_LEGAL_TEXT}}</v>
       </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -4466,6 +5050,9 @@
       <c r="D25" t="str">
         <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -4480,6 +5067,9 @@
       <c r="D26" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -4494,6 +5084,9 @@
       <c r="D27" t="str">
         <v>DAZN Standard</v>
       </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -4508,6 +5101,9 @@
       <c r="D28" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -4522,6 +5118,9 @@
       <c r="D29" t="str">
         <v>{{PPV_PRICE}}</v>
       </c>
+      <c r="E29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -4536,6 +5135,9 @@
       <c r="D30" t="str">
         <v>{{RATE_PLAN_LABEL}}</v>
       </c>
+      <c r="E30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -4550,6 +5152,9 @@
       <c r="D31" t="str">
         <v>{{CURRENCY}}{{ANNUAL_PRICE}}</v>
       </c>
+      <c r="E31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -4564,6 +5169,9 @@
       <c r="D32" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -4578,6 +5186,9 @@
       <c r="D33" t="str">
         <v>Today you pay</v>
       </c>
+      <c r="E33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -4590,7 +5201,10 @@
         <v>Today You Pay Price</v>
       </c>
       <c r="D34" t="str">
-        <v>{{PPV_PRICE}}</v>
+        <v>{{TODAY_YOU_PAY_PRICE}}</v>
+      </c>
+      <c r="E34" t="str">
+        <v/>
       </c>
     </row>
     <row r="35">
@@ -4606,6 +5220,9 @@
       <c r="D35" t="str">
         <v>{{CANCELLATION_TEXT_ANNUAL}}</v>
       </c>
+      <c r="E35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -4620,6 +5237,9 @@
       <c r="D36" t="str">
         <v>Yes</v>
       </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -4634,6 +5254,9 @@
       <c r="D37" t="str">
         <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -4648,6 +5271,9 @@
       <c r="D38" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -4662,6 +5288,9 @@
       <c r="D39" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="E39" t="str">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -4676,6 +5305,9 @@
       <c r="D40" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -4690,6 +5322,9 @@
       <c r="D41" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E41" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -4704,6 +5339,9 @@
       <c r="D42" t="str">
         <v>Annual - Pay Monthly</v>
       </c>
+      <c r="E42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -4718,6 +5356,9 @@
       <c r="D43" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
       </c>
+      <c r="E43" t="str">
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -4732,6 +5373,9 @@
       <c r="D44" t="str">
         <v>Billed monthly. 12-month contract.</v>
       </c>
+      <c r="E44" t="str">
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -4746,6 +5390,9 @@
       <c r="D45" t="str">
         <v>Today you pay</v>
       </c>
+      <c r="E45" t="str">
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -4760,6 +5407,9 @@
       <c r="D46" t="str">
         <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
+      <c r="E46" t="str">
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -4774,6 +5424,9 @@
       <c r="D47" t="str">
         <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
+      <c r="E47" t="str">
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -4788,6 +5441,9 @@
       <c r="D48" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
       </c>
+      <c r="E48" t="str">
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -4802,6 +5458,9 @@
       <c r="D49" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E49" t="str">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -4816,6 +5475,9 @@
       <c r="D50" t="str">
         <v>Yes</v>
       </c>
+      <c r="E50" t="str">
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -4830,6 +5492,9 @@
       <c r="D51" t="str">
         <v>{{DISCOUNT_BADGE}}</v>
       </c>
+      <c r="E51" t="str">
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -4844,6 +5509,9 @@
       <c r="D52" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E52" t="str">
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -4858,6 +5526,9 @@
       <c r="D53" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="E53" t="str">
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -4872,6 +5543,9 @@
       <c r="D54" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="E54" t="str">
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -4886,6 +5560,9 @@
       <c r="D55" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E55" t="str">
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -4900,6 +5577,9 @@
       <c r="D56" t="str">
         <v>Annual - Pay Upfront</v>
       </c>
+      <c r="E56" t="str">
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -4914,6 +5594,9 @@
       <c r="D57" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE}}/year</v>
       </c>
+      <c r="E57" t="str">
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -4928,6 +5611,9 @@
       <c r="D58" t="str">
         <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}. Pay for the full year up front|Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
       </c>
+      <c r="E58" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -4942,6 +5628,9 @@
       <c r="D59" t="str">
         <v>Today you pay</v>
       </c>
+      <c r="E59" t="str">
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -4956,6 +5645,9 @@
       <c r="D60" t="str">
         <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
+      <c r="E60" t="str">
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -4970,6 +5662,9 @@
       <c r="D61" t="str">
         <v>Next Annual payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
+      <c r="E61" t="str">
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -4984,6 +5679,9 @@
       <c r="D62" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE}}</v>
       </c>
+      <c r="E62" t="str">
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -4998,6 +5696,9 @@
       <c r="D63" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E63" t="str">
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -5012,6 +5713,9 @@
       <c r="D64" t="str">
         <v>Yes</v>
       </c>
+      <c r="E64" t="str">
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -5026,6 +5730,9 @@
       <c r="D65" t="str">
         <v>{{PAYMENT_PAGE_TITLE}}</v>
       </c>
+      <c r="E65" t="str">
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -5040,6 +5747,9 @@
       <c r="D66" t="str">
         <v>DAZN Standard</v>
       </c>
+      <c r="E66" t="str">
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -5054,6 +5764,9 @@
       <c r="D67" t="str">
         <v>{{BUNDLE_NAME}}</v>
       </c>
+      <c r="E67" t="str">
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -5068,6 +5781,9 @@
       <c r="D68" t="str">
         <v>{{BUNDLE_PRICE}}</v>
       </c>
+      <c r="E68" t="str">
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -5082,6 +5798,9 @@
       <c r="D69" t="str">
         <v>{{BUNDLE_TODAY_YOU_PAY_STANDARD}}</v>
       </c>
+      <c r="E69" t="str">
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -5096,6 +5815,9 @@
       <c r="D70" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E70" t="str">
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -5110,6 +5832,9 @@
       <c r="D71" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E71" t="str">
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -5124,6 +5849,9 @@
       <c r="D72" t="str">
         <v>DAZN Standard</v>
       </c>
+      <c r="E72" t="str">
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -5138,6 +5866,9 @@
       <c r="D73" t="str">
         <v>Annual - Pay Monthly</v>
       </c>
+      <c r="E73" t="str">
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -5152,6 +5883,9 @@
       <c r="D74" t="str">
         <v>First month free</v>
       </c>
+      <c r="E74" t="str">
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -5166,6 +5900,9 @@
       <c r="D75" t="str">
         <v>{{BUNDLE_NAME}}</v>
       </c>
+      <c r="E75" t="str">
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -5180,6 +5917,9 @@
       <c r="D76" t="str">
         <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
       </c>
+      <c r="E76" t="str">
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -5194,6 +5934,9 @@
       <c r="D77" t="str">
         <v>{{BUNDLE_PRICE}}</v>
       </c>
+      <c r="E77" t="str">
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -5208,6 +5951,9 @@
       <c r="D78" t="str">
         <v>{{BUNDLE_DISCOUNT}}</v>
       </c>
+      <c r="E78" t="str">
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -5222,6 +5968,9 @@
       <c r="D79" t="str">
         <v>{{BUNDLE_TODAY_YOU_PAY_STANDARD}}</v>
       </c>
+      <c r="E79" t="str">
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -5236,6 +5985,9 @@
       <c r="D80" t="str">
         <v>{{CANCELLATION_TEXT_ANNUAL}}</v>
       </c>
+      <c r="E80" t="str">
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -5250,6 +6002,9 @@
       <c r="D81" t="str">
         <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
+      <c r="E81" t="str">
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -5264,6 +6019,9 @@
       <c r="D82" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E82" t="str">
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -5278,6 +6036,9 @@
       <c r="D83" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="E83" t="str">
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -5292,6 +6053,9 @@
       <c r="D84" t="str">
         <v>Annual - Pay Monthly</v>
       </c>
+      <c r="E84" t="str">
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -5306,6 +6070,9 @@
       <c r="D85" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
       </c>
+      <c r="E85" t="str">
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -5320,6 +6087,9 @@
       <c r="D86" t="str">
         <v>{{BUNDLE_NAME}}</v>
       </c>
+      <c r="E86" t="str">
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -5334,6 +6104,9 @@
       <c r="D87" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E87" t="str">
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -5348,6 +6121,9 @@
       <c r="D88" t="str">
         <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
+      <c r="E88" t="str">
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
@@ -5362,6 +6138,9 @@
       <c r="D89" t="str">
         <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
+      <c r="E89" t="str">
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -5376,6 +6155,9 @@
       <c r="D90" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
       </c>
+      <c r="E90" t="str">
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -5390,6 +6172,9 @@
       <c r="D91" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E91" t="str">
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -5404,6 +6189,9 @@
       <c r="D92" t="str">
         <v>{{DISCOUNT_BADGE}}</v>
       </c>
+      <c r="E92" t="str">
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
@@ -5418,6 +6206,9 @@
       <c r="D93" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E93" t="str">
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
@@ -5432,6 +6223,9 @@
       <c r="D94" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="E94" t="str">
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
@@ -5446,6 +6240,9 @@
       <c r="D95" t="str">
         <v>Annual - Pay Upfront</v>
       </c>
+      <c r="E95" t="str">
+        <v/>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
@@ -5460,6 +6257,9 @@
       <c r="D96" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE}}/year</v>
       </c>
+      <c r="E96" t="str">
+        <v/>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
@@ -5474,6 +6274,9 @@
       <c r="D97" t="str">
         <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
       </c>
+      <c r="E97" t="str">
+        <v/>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
@@ -5488,6 +6291,9 @@
       <c r="D98" t="str">
         <v>{{BUNDLE_NAME}}</v>
       </c>
+      <c r="E98" t="str">
+        <v/>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
@@ -5502,6 +6308,9 @@
       <c r="D99" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E99" t="str">
+        <v/>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
@@ -5516,6 +6325,9 @@
       <c r="D100" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE}}</v>
       </c>
+      <c r="E100" t="str">
+        <v/>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
@@ -5530,6 +6342,9 @@
       <c r="D101" t="str">
         <v>Next Annual payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
+      <c r="E101" t="str">
+        <v/>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
@@ -5544,6 +6359,9 @@
       <c r="D102" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE}}</v>
       </c>
+      <c r="E102" t="str">
+        <v/>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
@@ -5558,9 +6376,11 @@
       <c r="D103" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E103" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:E103"/>
   </ignoredErrors>
@@ -5570,6 +6390,10 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B15"/>
+  <cols>
+    <col min="1" max="1" width="27.83203125" customWidth="1"/>
+    <col min="2" max="2" width="90.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5692,7 +6516,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B15"/>
   </ignoredErrors>
@@ -5702,6 +6525,10 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B9"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="25.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5776,7 +6603,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B9"/>
   </ignoredErrors>
@@ -5785,7 +6611,11 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
+  <cols>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="70.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5957,24 +6787,31 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Whats Included CTA</v>
+        <v>Upsell Feature 4</v>
       </c>
       <c r="B22" t="str">
-        <v>Whats included</v>
+        <v>{{UPSELL_FEATURE_4}}</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
+        <v>Whats Included CTA</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Whats included</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
         <v>CTA Button</v>
       </c>
-      <c r="B23" t="str">
+      <c r="B24" t="str">
         <v>{{PPV_CTA_TEXT}}</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B24"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5982,6 +6819,10 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B18"/>
+  <cols>
+    <col min="1" max="1" width="29.83203125" customWidth="1"/>
+    <col min="2" max="2" width="79.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6012,7 +6853,7 @@
         <v>PPV Description</v>
       </c>
       <c r="B4" t="str">
-        <v>{{BANNER_DESCRIPTION}}</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="5">
@@ -6052,7 +6893,7 @@
         <v>Today You Pay Price</v>
       </c>
       <c r="B9" t="str">
-        <v>{{PPV_PRICE}}</v>
+        <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
     </row>
     <row r="10">
@@ -6128,7 +6969,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B18"/>
   </ignoredErrors>

</xml_diff>

<commit_message>
feat: add boxing banner date validation support
- scripts/generateExcel.ts: Add 'Boxing Banner Date' field validation to boxingLandingData
- utils/getActualValue.ts: Add 'boxing banner date' actual value extractor selector for Boxing page banner tag
- utils/resolveExpected.ts: Add resolution logic for 'boxing banner date' from eventData.BOXING_BANNER_DATE
- data/PPV_Input.xlsx: Update binary sheet config with new banner validation rules
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -2128,7 +2128,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C55"/>
   <cols>
     <col min="1" max="1" width="29.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
@@ -2159,10 +2159,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Event Name</v>
+        <v>Boxing Banner Date</v>
       </c>
       <c r="B3" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>{{BOXING_BANNER_DATE}}</v>
       </c>
       <c r="C3" t="str">
         <v>boxing</v>
@@ -2170,10 +2170,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Event Subtitle</v>
+        <v>Event Name</v>
       </c>
       <c r="B4" t="str">
-        <v>{{BOXING_BANNER_SUBTITLE}}</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="C4" t="str">
         <v>boxing</v>
@@ -2181,10 +2181,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Or Separator</v>
+        <v>Event Subtitle</v>
       </c>
       <c r="B5" t="str">
-        <v>or</v>
+        <v>{{BOXING_BANNER_SUBTITLE}}</v>
       </c>
       <c r="C5" t="str">
         <v>boxing</v>
@@ -2192,10 +2192,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Buy Fight CTA</v>
+        <v>Or Separator</v>
       </c>
       <c r="B6" t="str">
-        <v>Buy this fight for {{PPV_PRICE}}</v>
+        <v>or</v>
       </c>
       <c r="C6" t="str">
         <v>boxing</v>
@@ -2203,10 +2203,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Get Included CTA</v>
+        <v>Buy Fight CTA</v>
       </c>
       <c r="B7" t="str">
-        <v>Get included in DAZN Ultimate</v>
+        <v>Buy this fight for {{PPV_PRICE}}</v>
       </c>
       <c r="C7" t="str">
         <v>boxing</v>
@@ -2214,10 +2214,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Best Value Badge</v>
+        <v>Get Included CTA</v>
       </c>
       <c r="B8" t="str">
-        <v>Best value for boxing fans</v>
+        <v>Get included in DAZN Ultimate</v>
       </c>
       <c r="C8" t="str">
         <v>boxing</v>
@@ -2225,21 +2225,21 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Upcoming Big Fights Heading</v>
+        <v>Best Value Badge</v>
       </c>
       <c r="B9" t="str">
-        <v>Upcoming Big Fights</v>
+        <v>Best value for boxing fans</v>
       </c>
       <c r="C9" t="str">
-        <v>boxing-upcoming</v>
+        <v>boxing</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>PPV Name</v>
+        <v>Upcoming Big Fights Heading</v>
       </c>
       <c r="B10" t="str">
-        <v>{{PPV_DISPLAY_NAME}}</v>
+        <v>Upcoming Big Fights</v>
       </c>
       <c r="C10" t="str">
         <v>boxing-upcoming</v>
@@ -2247,10 +2247,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>PPV Date and Time Text</v>
+        <v>PPV Name</v>
       </c>
       <c r="B11" t="str">
-        <v>{{PPV_DATE}}</v>
+        <v>{{PPV_DISPLAY_NAME}}</v>
       </c>
       <c r="C11" t="str">
         <v>boxing-upcoming</v>
@@ -2258,10 +2258,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>PPV Description Text</v>
+        <v>PPV Date and Time Text</v>
       </c>
       <c r="B12" t="str">
-        <v>{{PPV_LOCATION}}</v>
+        <v>{{PPV_DATE}}</v>
       </c>
       <c r="C12" t="str">
         <v>boxing-upcoming</v>
@@ -2269,10 +2269,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>PPV Image Present</v>
+        <v>PPV Description Text</v>
       </c>
       <c r="B13" t="str">
-        <v>Yes</v>
+        <v>{{PPV_LOCATION}}</v>
       </c>
       <c r="C13" t="str">
         <v>boxing-upcoming</v>
@@ -2280,10 +2280,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Buy Now CTA</v>
+        <v>PPV Image Present</v>
       </c>
       <c r="B14" t="str">
-        <v>Buy now</v>
+        <v>Yes</v>
       </c>
       <c r="C14" t="str">
         <v>boxing-upcoming</v>
@@ -2291,21 +2291,21 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Bundle Section Present</v>
+        <v>Buy Now CTA</v>
       </c>
       <c r="B15" t="str">
-        <v>Yes</v>
+        <v>Buy now</v>
       </c>
       <c r="C15" t="str">
-        <v>boxing-bundle</v>
+        <v>boxing-upcoming</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Bundle Section Title</v>
+        <v>Bundle Section Present</v>
       </c>
       <c r="B16" t="str">
-        <v>{{BUNDLE_SECTION_TITLE}}</v>
+        <v>Yes</v>
       </c>
       <c r="C16" t="str">
         <v>boxing-bundle</v>
@@ -2313,10 +2313,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Bundle Section Subtitle</v>
+        <v>Bundle Section Title</v>
       </c>
       <c r="B17" t="str">
-        <v>{{BUNDLE_SECTION_SUBTITLE}}</v>
+        <v>{{BUNDLE_SECTION_TITLE}}</v>
       </c>
       <c r="C17" t="str">
         <v>boxing-bundle</v>
@@ -2324,10 +2324,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Bundle Title</v>
+        <v>Bundle Section Subtitle</v>
       </c>
       <c r="B18" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>{{BUNDLE_SECTION_SUBTITLE}}</v>
       </c>
       <c r="C18" t="str">
         <v>boxing-bundle</v>
@@ -2335,10 +2335,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Bundle Description</v>
+        <v>Bundle Title</v>
       </c>
       <c r="B19" t="str">
-        <v>{{BUNDLE_DESCRIPTION}}</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="C19" t="str">
         <v>boxing-bundle</v>
@@ -2346,10 +2346,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Bundle Price</v>
+        <v>Bundle Description</v>
       </c>
       <c r="B20" t="str">
-        <v>{{BUNDLE_PRICE}}</v>
+        <v>{{BUNDLE_DESCRIPTION}}</v>
       </c>
       <c r="C20" t="str">
         <v>boxing-bundle</v>
@@ -2357,10 +2357,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Bundle Original Price</v>
+        <v>Bundle Price</v>
       </c>
       <c r="B21" t="str">
-        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
+        <v>{{BUNDLE_PRICE}}</v>
       </c>
       <c r="C21" t="str">
         <v>boxing-bundle</v>
@@ -2368,10 +2368,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Bundle Save Badge</v>
+        <v>Bundle Original Price</v>
       </c>
       <c r="B22" t="str">
-        <v>{{BUNDLE_SAVE_BADGE}}</v>
+        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
       </c>
       <c r="C22" t="str">
         <v>boxing-bundle</v>
@@ -2379,10 +2379,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Bundle Fight Count</v>
+        <v>Bundle Save Badge</v>
       </c>
       <c r="B23" t="str">
-        <v>{{BUNDLE_FIGHT_COUNT}}</v>
+        <v>{{BUNDLE_SAVE_BADGE}}</v>
       </c>
       <c r="C23" t="str">
         <v>boxing-bundle</v>
@@ -2390,10 +2390,10 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Bundle PPV 1 Name</v>
+        <v>Bundle Fight Count</v>
       </c>
       <c r="B24" t="str">
-        <v>{{BUNDLE_PPV1_NAME}}</v>
+        <v>{{BUNDLE_FIGHT_COUNT}}</v>
       </c>
       <c r="C24" t="str">
         <v>boxing-bundle</v>
@@ -2401,10 +2401,10 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Bundle PPV 1 Date</v>
+        <v>Bundle PPV 1 Name</v>
       </c>
       <c r="B25" t="str">
-        <v>{{BUNDLE_PPV1_LANDING_DATE}}</v>
+        <v>{{BUNDLE_PPV1_NAME}}</v>
       </c>
       <c r="C25" t="str">
         <v>boxing-bundle</v>
@@ -2412,10 +2412,10 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Bundle PPV 1 Image</v>
+        <v>Bundle PPV 1 Date</v>
       </c>
       <c r="B26" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_PPV1_LANDING_DATE}}</v>
       </c>
       <c r="C26" t="str">
         <v>boxing-bundle</v>
@@ -2423,10 +2423,10 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Bundle PPV 2 Name</v>
+        <v>Bundle PPV 1 Image</v>
       </c>
       <c r="B27" t="str">
-        <v>{{BUNDLE_PPV2_NAME}}</v>
+        <v>Yes</v>
       </c>
       <c r="C27" t="str">
         <v>boxing-bundle</v>
@@ -2434,10 +2434,10 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Bundle PPV 2 Date</v>
+        <v>Bundle PPV 2 Name</v>
       </c>
       <c r="B28" t="str">
-        <v>{{BUNDLE_PPV2_LANDING_DATE}}</v>
+        <v>{{BUNDLE_PPV2_NAME}}</v>
       </c>
       <c r="C28" t="str">
         <v>boxing-bundle</v>
@@ -2445,10 +2445,10 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Bundle PPV 2 Image</v>
+        <v>Bundle PPV 2 Date</v>
       </c>
       <c r="B29" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_PPV2_LANDING_DATE}}</v>
       </c>
       <c r="C29" t="str">
         <v>boxing-bundle</v>
@@ -2456,10 +2456,10 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Get Started CTA</v>
+        <v>Bundle PPV 2 Image</v>
       </c>
       <c r="B30" t="str">
-        <v>Get Started</v>
+        <v>Yes</v>
       </c>
       <c r="C30" t="str">
         <v>boxing-bundle</v>
@@ -2467,21 +2467,21 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Page Title</v>
+        <v>Get Started CTA</v>
       </c>
       <c r="B31" t="str">
-        <v>Choose the right plan for you.</v>
+        <v>Get Started</v>
       </c>
       <c r="C31" t="str">
-        <v>boxing-bundle-ppv</v>
+        <v>boxing-bundle</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Header Sub Text</v>
+        <v>Page Title</v>
       </c>
       <c r="B32" t="str">
-        <v>To watch your pay-per-view, you'll need a DAZN plan.</v>
+        <v>Choose the right plan for you.</v>
       </c>
       <c r="C32" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2489,10 +2489,10 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Bundle Card Title</v>
+        <v>Header Sub Text</v>
       </c>
       <c r="B33" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>To watch your pay-per-view, you'll need a DAZN plan.</v>
       </c>
       <c r="C33" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2500,10 +2500,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Bundle Card Description</v>
+        <v>Bundle Card Title</v>
       </c>
       <c r="B34" t="str">
-        <v>{{BUNDLE_PPV_CARD_DESCRIPTION}}</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="C34" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2511,10 +2511,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Bundle Card Selected</v>
+        <v>Bundle Card Description</v>
       </c>
       <c r="B35" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_PPV_CARD_DESCRIPTION}}</v>
       </c>
       <c r="C35" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2522,10 +2522,10 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Bundle Card Price</v>
+        <v>Bundle Card Selected</v>
       </c>
       <c r="B36" t="str">
-        <v>{{BUNDLE_PRICE}}</v>
+        <v>Yes</v>
       </c>
       <c r="C36" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2533,10 +2533,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Bundle Card Original Price</v>
+        <v>Bundle Card Price</v>
       </c>
       <c r="B37" t="str">
-        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
+        <v>{{BUNDLE_PRICE}}</v>
       </c>
       <c r="C37" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2544,10 +2544,10 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Bundle Card Save Badge</v>
+        <v>Bundle Card Original Price</v>
       </c>
       <c r="B38" t="str">
-        <v>{{BUNDLE_SAVE_BADGE}}</v>
+        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
       </c>
       <c r="C38" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2555,10 +2555,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Bundle PPV 1 Full Name</v>
+        <v>Bundle Card Save Badge</v>
       </c>
       <c r="B39" t="str">
-        <v>{{BUNDLE_PPV1_FULL_NAME}}</v>
+        <v>{{BUNDLE_SAVE_BADGE}}</v>
       </c>
       <c r="C39" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2566,10 +2566,10 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Bundle PPV 1 PPV Date</v>
+        <v>Bundle PPV 1 Full Name</v>
       </c>
       <c r="B40" t="str">
-        <v>{{BUNDLE_PPV1_DATE}}</v>
+        <v>{{BUNDLE_PPV1_FULL_NAME}}</v>
       </c>
       <c r="C40" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2577,10 +2577,10 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Bundle PPV 1 PPV Image</v>
+        <v>Bundle PPV 1 PPV Date</v>
       </c>
       <c r="B41" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_PPV1_DATE}}</v>
       </c>
       <c r="C41" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2588,10 +2588,10 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Bundle PPV 2 Full Name</v>
+        <v>Bundle PPV 1 PPV Image</v>
       </c>
       <c r="B42" t="str">
-        <v>{{BUNDLE_PPV2_FULL_NAME}}</v>
+        <v>Yes</v>
       </c>
       <c r="C42" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2599,10 +2599,10 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Bundle PPV 2 PPV Date</v>
+        <v>Bundle PPV 2 Full Name</v>
       </c>
       <c r="B43" t="str">
-        <v>{{BUNDLE_PPV2_DATE}}</v>
+        <v>{{BUNDLE_PPV2_FULL_NAME}}</v>
       </c>
       <c r="C43" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2610,10 +2610,10 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Bundle PPV 2 PPV Image</v>
+        <v>Bundle PPV 2 PPV Date</v>
       </c>
       <c r="B44" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_PPV2_DATE}}</v>
       </c>
       <c r="C44" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2621,7 +2621,7 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Upsell Section Present</v>
+        <v>Bundle PPV 2 PPV Image</v>
       </c>
       <c r="B45" t="str">
         <v>Yes</v>
@@ -2632,10 +2632,10 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Upsell Badge</v>
+        <v>Upsell Section Present</v>
       </c>
       <c r="B46" t="str">
-        <v>The Ultimate Fan Package</v>
+        <v>Yes</v>
       </c>
       <c r="C46" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2643,10 +2643,10 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Upsell Plan Name</v>
+        <v>Upsell Badge</v>
       </c>
       <c r="B47" t="str">
-        <v>DAZN Ultimate</v>
+        <v>The Ultimate Fan Package</v>
       </c>
       <c r="C47" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2654,10 +2654,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Upsell Price</v>
+        <v>Upsell Plan Name</v>
       </c>
       <c r="B48" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="C48" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2665,10 +2665,10 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Upsell Contract Text</v>
+        <v>Upsell Price</v>
       </c>
       <c r="B49" t="str">
-        <v>Annual contract. Auto renews.</v>
+        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
       </c>
       <c r="C49" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2676,10 +2676,10 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Fights Included Text</v>
+        <v>Upsell Contract Text</v>
       </c>
       <c r="B50" t="str">
-        <v>All these fights included and more.</v>
+        <v>Annual contract. Auto renews.</v>
       </c>
       <c r="C50" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2687,10 +2687,10 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Upsell Feature 1</v>
+        <v>Fights Included Text</v>
       </c>
       <c r="B51" t="str">
-        <v>Minimum 12 pay-per-views a year included at no extra cost.</v>
+        <v>All these fights included and more.</v>
       </c>
       <c r="C51" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2698,10 +2698,10 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Upsell Feature 2</v>
+        <v>Upsell Feature 1</v>
       </c>
       <c r="B52" t="str">
-        <v>185+ fights a year from the world's best promoters.</v>
+        <v>Minimum 12 pay-per-views a year included at no extra cost.</v>
       </c>
       <c r="C52" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2709,10 +2709,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Upsell Feature 3</v>
+        <v>Upsell Feature 2</v>
       </c>
       <c r="B53" t="str">
-        <v>HDR and Dolby 5.1 surround sound on select events</v>
+        <v>185+ fights a year from the world's best promoters.</v>
       </c>
       <c r="C53" t="str">
         <v>boxing-bundle-ppv</v>
@@ -2720,18 +2720,29 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>CTA Button</v>
+        <v>Upsell Feature 3</v>
       </c>
       <c r="B54" t="str">
-        <v>Continue with DAZN Ultimate</v>
+        <v>HDR and Dolby 5.1 surround sound on select events</v>
       </c>
       <c r="C54" t="str">
         <v>boxing-bundle-ppv</v>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>CTA Button</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Continue with DAZN Ultimate</v>
+      </c>
+      <c r="C55" t="str">
+        <v>boxing-bundle-ppv</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C54"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C55"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: schedule tile time validation — scope to PPV tile, remove PPV Date, add SCHEDULE_PPV_TIME
Issues fixed:
1. PPV Time on Tile showed wrong time ('1:30AM' from adjacent Rolly vs. Teofimo
   tile) instead of the AJ tile's '9:30PM'. Root cause: snapFind scanned
   the full DOM snapshot and returned the first HH:MM match.
   Fix: on schedule URLs, scope the article search to the article whose
   innerText contains the PPV_NAME first word, then read its time badge.

2. PPV Date field removed from Schedule page sheet — date is captured
   via the popup modal, keeping it on the tile caused format mismatch
   and redundancy.

3. New field SCHEDULE_PPV_TIME added to config per region (GB='9:30PM').
   generateExcel now uses {{SCHEDULE_PPV_TIME}} for 'PPV Time on Tile'
   expected value in the Schedule sheet, separating the display time
   (shown on schedule tile badge) from PPV_TIME (used on other pages).
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -6448,7 +6448,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B13"/>
   <cols>
     <col min="1" max="1" width="27.83203125" customWidth="1"/>
     <col min="2" max="2" width="90.83203125" customWidth="1"/>
@@ -6480,95 +6480,87 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>PPV Date</v>
+        <v>PPV Time on Tile</v>
       </c>
       <c r="B4" t="str">
-        <v>{{PPV_DATE}}</v>
+        <v>{{SCHEDULE_PPV_TIME}}</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>PPV Time on Tile</v>
+        <v>Lock Icon Present</v>
       </c>
       <c r="B5" t="str">
-        <v>{{PPV_TIME}}</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Lock Icon Present</v>
+        <v>PPV Promoter on Tile</v>
       </c>
       <c r="B6" t="str">
-        <v>Yes</v>
+        <v>{{PPV_PROMOTER}}</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>PPV Promoter on Tile</v>
+        <v>Popup - Image Present</v>
       </c>
       <c r="B7" t="str">
-        <v>{{PPV_PROMOTER}}</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Popup - Image Present</v>
+        <v>Popup - Event Title</v>
       </c>
       <c r="B8" t="str">
-        <v>Yes</v>
+        <v>{{PPV_NAME}}</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Popup - Event Title</v>
+        <v>Popup - Event Date</v>
       </c>
       <c r="B9" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>{{PPV_POPUP_DATE}}</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Popup - Event Date</v>
+        <v>Popup - Promoter</v>
       </c>
       <c r="B10" t="str">
-        <v>{{PPV_POPUP_DATE}}</v>
+        <v>{{PPV_PROMOTER}}</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Popup - Promoter</v>
+        <v>Popup - Event Description</v>
       </c>
       <c r="B11" t="str">
-        <v>{{PPV_PROMOTER}}</v>
+        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Popup - Event Description</v>
+        <v>Popup - Buy Now CTA</v>
       </c>
       <c r="B12" t="str">
-        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
+        <v>Visible</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Popup - Buy Now CTA</v>
+        <v>Popup - Close Button</v>
       </c>
       <c r="B13" t="str">
         <v>Visible</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Popup - Close Button</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B13"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: search/popup validation fixes, SEARCH_PPV_DATE_TIME, source-specific popup labels
Changes included:
- getActualValue.ts: popup event date uses page.evaluate Buy Now anchor
  to correctly scope date chip extraction to popup modal for ALL sources
  (search, schedule, home-page-dont-miss) instead of background elements
- getActualValue.ts: add 'search ppv date and time' case alias
- testHelpers.ts: source-specific pageName for popup results
  (search→Search, schedule→Schedule, others→Popup Modal)
- newuser/existinguser specs: filter popup rows before tile click in search
- generateExcel.ts: add Search PPV Date and Time field with SEARCH_PPV_DATE_TIME
- aj_joshua_prenga.json: add SEARCH_PPV_DATE_TIME = '25 JUL 9:00PM'
- pages/BoxingHomePage.ts, HomePage.ts: misc page fixes
- buildEventData.ts, failureCapture.ts: supporting utility improvements
- config/surfacingpoint.json, DaznPlan.json: config updates
- data/PPV_Input.xlsx: regenerated with all field changes
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -416,11 +416,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C12"/>
-  <cols>
-    <col min="1" max="1" width="33.83203125" customWidth="1"/>
-    <col min="2" max="2" width="27.83203125" customWidth="1"/>
-    <col min="3" max="3" width="21.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -564,11 +559,6 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C23"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="27.83203125" customWidth="1"/>
-    <col min="3" max="3" width="318.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -833,10 +823,6 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B6"/>
-  <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="64.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -896,10 +882,6 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B6"/>
-  <cols>
-    <col min="1" max="1" width="19.83203125" customWidth="1"/>
-    <col min="2" max="2" width="34.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -958,12 +940,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C24"/>
-  <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
-    <col min="3" max="3" width="90.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:C28"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1058,10 +1035,10 @@
         <v>home-boxing-tile</v>
       </c>
       <c r="B9" t="str">
-        <v>Popup - Event Title</v>
+        <v>PPV Tile Present</v>
       </c>
       <c r="C9" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="10">
@@ -1069,10 +1046,10 @@
         <v>home-boxing-tile</v>
       </c>
       <c r="B10" t="str">
-        <v>Popup - Event Date</v>
+        <v>PPV Name</v>
       </c>
       <c r="C10" t="str">
-        <v>{{PPV_POPUP_DATE}}</v>
+        <v>{{PPV_NAME}}</v>
       </c>
     </row>
     <row r="11">
@@ -1080,10 +1057,10 @@
         <v>home-boxing-tile</v>
       </c>
       <c r="B11" t="str">
-        <v>Popup - Promoter</v>
+        <v>PPV Date</v>
       </c>
       <c r="C11" t="str">
-        <v>{{PPV_PROMOTER}}</v>
+        <v>{{LANDING_PAGE_PPV_DATE}}</v>
       </c>
     </row>
     <row r="12">
@@ -1091,10 +1068,10 @@
         <v>home-boxing-tile</v>
       </c>
       <c r="B12" t="str">
-        <v>Popup - Buy Now CTA</v>
+        <v>PPV Image Present</v>
       </c>
       <c r="C12" t="str">
-        <v>Visible</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="13">
@@ -1102,10 +1079,10 @@
         <v>home-boxing-tile</v>
       </c>
       <c r="B13" t="str">
-        <v>Popup - Event Description</v>
+        <v>Popup - Event Title</v>
       </c>
       <c r="C13" t="str">
-        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
+        <v>{{PPV_NAME}}</v>
       </c>
     </row>
     <row r="14">
@@ -1113,54 +1090,54 @@
         <v>home-boxing-tile</v>
       </c>
       <c r="B14" t="str">
-        <v>Popup - Close Button</v>
+        <v>Popup - Event Date</v>
       </c>
       <c r="C14" t="str">
-        <v>Visible</v>
+        <v>{{PPV_POPUP_DATE}}</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>home-boxing-upcoming</v>
+        <v>home-boxing-tile</v>
       </c>
       <c r="B15" t="str">
-        <v>Best of Boxing Section</v>
+        <v>Popup - Promoter</v>
       </c>
       <c r="C15" t="str">
-        <v>Present</v>
+        <v>{{PPV_PROMOTER}}</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>home-boxing-upcoming</v>
+        <v>home-boxing-tile</v>
       </c>
       <c r="B16" t="str">
-        <v>PPV Tile Present</v>
+        <v>Popup - Buy Now CTA</v>
       </c>
       <c r="C16" t="str">
-        <v>Yes</v>
+        <v>Visible</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>home-boxing-upcoming</v>
+        <v>home-boxing-tile</v>
       </c>
       <c r="B17" t="str">
-        <v>PPV Date</v>
+        <v>Popup - Event Description</v>
       </c>
       <c r="C17" t="str">
-        <v>{{LANDING_PAGE_PPV_DATE}}</v>
+        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>home-boxing-upcoming</v>
+        <v>home-boxing-tile</v>
       </c>
       <c r="B18" t="str">
-        <v>PPV Promoter on Tile</v>
+        <v>Popup - Close Button</v>
       </c>
       <c r="C18" t="str">
-        <v>{{PPV_PROMOTER}}</v>
+        <v>Visible</v>
       </c>
     </row>
     <row r="19">
@@ -1168,10 +1145,10 @@
         <v>home-boxing-upcoming</v>
       </c>
       <c r="B19" t="str">
-        <v>PPV Name</v>
+        <v>Best of Boxing Section</v>
       </c>
       <c r="C19" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>Present</v>
       </c>
     </row>
     <row r="20">
@@ -1179,10 +1156,10 @@
         <v>home-boxing-upcoming</v>
       </c>
       <c r="B20" t="str">
-        <v>PPV Date and Time Text</v>
+        <v>PPV Tile Present</v>
       </c>
       <c r="C20" t="str">
-        <v>WATCH LIVE {{HOME_BOXING_UPCOMING_DATE}} at {{HOME_BOXING_UPCOMING_TIME}}</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="21">
@@ -1190,10 +1167,10 @@
         <v>home-boxing-upcoming</v>
       </c>
       <c r="B21" t="str">
-        <v>Buy Now CTA</v>
+        <v>PPV Date</v>
       </c>
       <c r="C21" t="str">
-        <v>Buy now</v>
+        <v>{{LANDING_PAGE_PPV_DATE}}</v>
       </c>
     </row>
     <row r="22">
@@ -1201,10 +1178,10 @@
         <v>home-boxing-upcoming</v>
       </c>
       <c r="B22" t="str">
-        <v>Fight Card CTA</v>
+        <v>PPV Promoter on Tile</v>
       </c>
       <c r="C22" t="str">
-        <v>Fight card</v>
+        <v>{{PPV_PROMOTER}}</v>
       </c>
     </row>
     <row r="23">
@@ -1212,10 +1189,10 @@
         <v>home-boxing-upcoming</v>
       </c>
       <c r="B23" t="str">
-        <v>PPV Image Present</v>
+        <v>PPV Name</v>
       </c>
       <c r="C23" t="str">
-        <v>Yes</v>
+        <v>{{PPV_NAME}}</v>
       </c>
     </row>
     <row r="24">
@@ -1223,10 +1200,329 @@
         <v>home-boxing-upcoming</v>
       </c>
       <c r="B24" t="str">
+        <v>PPV Date and Time Text</v>
+      </c>
+      <c r="C24" t="str">
+        <v>WATCH LIVE {{HOME_BOXING_UPCOMING_DATE}} at {{HOME_BOXING_UPCOMING_TIME}}</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Buy Now CTA</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Buy now</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Fight Card CTA</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Fight card</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B27" t="str">
+        <v>PPV Image Present</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B28" t="str">
         <v>Lock Icon Present</v>
       </c>
+      <c r="C28" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C28"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C24"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Flow</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Field</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Expected</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>home-page-banner</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Banner - Event Title</v>
+      </c>
+      <c r="C2" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>home-page-banner</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Banner - Event Date</v>
+      </c>
+      <c r="C3" t="str">
+        <v>{{PPV_DATE}}</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>home-page-banner</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Banner - Event Description</v>
+      </c>
+      <c r="C4" t="str">
+        <v>{{BANNER_DESCRIPTION}}</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>home-page-banner</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Banner - Buy Now CTA</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>home-page-banner</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Banner - Fight Card CTA</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Don't Miss Section</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Present</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+      <c r="B8" t="str">
+        <v>PPV Tile Present</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+      <c r="B9" t="str">
+        <v>PPV Name</v>
+      </c>
+      <c r="C9" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+      <c r="B10" t="str">
+        <v>PPV Date</v>
+      </c>
+      <c r="C10" t="str">
+        <v>{{LANDING_PAGE_PPV_DATE}}</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+      <c r="B11" t="str">
+        <v>PPV Image Present</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Popup - Event Title</v>
+      </c>
+      <c r="C12" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Popup - Event Date</v>
+      </c>
+      <c r="C13" t="str">
+        <v>{{PPV_POPUP_DATE}}</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Popup - Promoter</v>
+      </c>
+      <c r="C14" t="str">
+        <v>{{PPV_PROMOTER}}</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Popup - Buy Now CTA</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Popup - Event Description</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Popup - Close Button</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>home-biggest-fights</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Biggest Fights Section</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Saturday Fight Night</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>home-biggest-fights</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Popup - Event Title</v>
+      </c>
+      <c r="C19" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>home-biggest-fights</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Popup - Event Date</v>
+      </c>
+      <c r="C20" t="str">
+        <v>{{PPV_DATE}}</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>home-biggest-fights</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Popup - Promoter</v>
+      </c>
+      <c r="C21" t="str">
+        <v>{{PPV_PROMOTER}}</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>home-biggest-fights</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Popup - Buy Now CTA</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>home-biggest-fights</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Popup - Event Description</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>home-biggest-fights</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Popup - Close Button</v>
+      </c>
       <c r="C24" t="str">
-        <v>Yes</v>
+        <v>Visible</v>
       </c>
     </row>
   </sheetData>
@@ -1236,239 +1532,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C19"/>
-  <cols>
-    <col min="1" max="1" width="21.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
-    <col min="3" max="3" width="90.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Flow</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Field</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Expected</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>home-page-banner</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Banner - Event Title</v>
-      </c>
-      <c r="C2" t="str">
-        <v>{{PPV_NAME}}</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>home-page-banner</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Banner - Event Date</v>
-      </c>
-      <c r="C3" t="str">
-        <v>{{PPV_DATE}}</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>home-page-banner</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Banner - Event Description</v>
-      </c>
-      <c r="C4" t="str">
-        <v>{{BANNER_DESCRIPTION}}</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>home-page-banner</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Banner - Buy Now CTA</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>home-page-banner</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Banner - Fight Card CTA</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>home-page-dont-miss</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Popup - Event Title</v>
-      </c>
-      <c r="C7" t="str">
-        <v>{{PPV_NAME}}</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>home-page-dont-miss</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Popup - Event Date</v>
-      </c>
-      <c r="C8" t="str">
-        <v>{{PPV_POPUP_DATE}}</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>home-page-dont-miss</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Popup - Promoter</v>
-      </c>
-      <c r="C9" t="str">
-        <v>{{PPV_PROMOTER}}</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>home-page-dont-miss</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Popup - Buy Now CTA</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>home-page-dont-miss</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Popup - Event Description</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>home-page-dont-miss</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Popup - Close Button</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>home-biggest-fights</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Biggest Fights Section</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Saturday Fight Night</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>home-biggest-fights</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Popup - Event Title</v>
-      </c>
-      <c r="C14" t="str">
-        <v>{{PPV_NAME}}</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>home-biggest-fights</v>
-      </c>
-      <c r="B15" t="str">
-        <v>Popup - Event Date</v>
-      </c>
-      <c r="C15" t="str">
-        <v>{{PPV_DATE}}</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>home-biggest-fights</v>
-      </c>
-      <c r="B16" t="str">
-        <v>Popup - Promoter</v>
-      </c>
-      <c r="C16" t="str">
-        <v>{{PPV_PROMOTER}}</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>home-biggest-fights</v>
-      </c>
-      <c r="B17" t="str">
-        <v>Popup - Buy Now CTA</v>
-      </c>
-      <c r="C17" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>home-biggest-fights</v>
-      </c>
-      <c r="B18" t="str">
-        <v>Popup - Event Description</v>
-      </c>
-      <c r="C18" t="str">
-        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>home-biggest-fights</v>
-      </c>
-      <c r="B19" t="str">
-        <v>Popup - Close Button</v>
-      </c>
-      <c r="C19" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C19"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C31"/>
-  <cols>
-    <col min="1" max="1" width="33.83203125" customWidth="1"/>
-    <col min="2" max="2" width="124.83203125" customWidth="1"/>
-    <col min="3" max="3" width="11.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1821,10 +1887,6 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B7"/>
-  <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="21.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1892,10 +1954,6 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B7"/>
-  <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1963,10 +2021,6 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B11"/>
-  <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="27.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2066,10 +2120,6 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B12"/>
-  <cols>
-    <col min="1" max="1" width="27.83203125" customWidth="1"/>
-    <col min="2" max="2" width="90.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2177,11 +2227,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C55"/>
-  <cols>
-    <col min="1" max="1" width="29.83203125" customWidth="1"/>
-    <col min="2" max="2" width="60.83203125" customWidth="1"/>
-    <col min="3" max="3" width="19.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2798,12 +2843,6 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D94"/>
-  <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="37.83203125" customWidth="1"/>
-    <col min="3" max="3" width="201.83203125" customWidth="1"/>
-    <col min="4" max="4" width="9.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4131,12 +4170,6 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D38"/>
-  <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="34.83203125" customWidth="1"/>
-    <col min="3" max="3" width="70.83203125" customWidth="1"/>
-    <col min="4" max="4" width="6.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4680,13 +4713,6 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E103"/>
-  <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="27.83203125" customWidth="1"/>
-    <col min="3" max="3" width="28.83203125" customWidth="1"/>
-    <col min="4" max="4" width="160.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6449,10 +6475,6 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B13"/>
-  <cols>
-    <col min="1" max="1" width="27.83203125" customWidth="1"/>
-    <col min="2" max="2" width="90.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6568,10 +6590,6 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B9"/>
-  <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="25.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6655,10 +6673,6 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B24"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="70.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6862,10 +6876,6 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B18"/>
-  <cols>
-    <col min="1" max="1" width="29.83203125" customWidth="1"/>
-    <col min="2" max="2" width="79.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>

<commit_message>
feat: add Spence vs Tszyu event config + additional validation fixes
- config/events/spence_tszyu.json: new PPV event JSON for Spence Jr. vs. Tszyu
  (entitlement: ppv_t_spencejr_tszyu, UTC: 2026-07-26T03:00:00Z, GB=£24.99)
- scripts/generateExcel.ts: additional field/sheet updates
- utils/getActualValue.ts: further validation extraction fixes
- tests/new_user/newuser.ppv.spec.ts: test flow updates
- tests/existing_user/existinguser.ppv.spec.ts: test flow updates
- tests/mobile/mobile.ppv.spec.ts: mobile test updates
- data/PPV_Input.xlsx: regenerated
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -416,6 +416,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C12"/>
+  <cols>
+    <col min="1" max="1" width="33.83203125" customWidth="1"/>
+    <col min="2" max="2" width="27.83203125" customWidth="1"/>
+    <col min="3" max="3" width="21.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -559,6 +564,11 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C23"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="27.83203125" customWidth="1"/>
+    <col min="3" max="3" width="318.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -823,6 +833,10 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B6"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="64.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -882,6 +896,10 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B6"/>
+  <cols>
+    <col min="1" max="1" width="19.83203125" customWidth="1"/>
+    <col min="2" max="2" width="34.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -941,6 +959,11 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C28"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="90.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1260,6 +1283,11 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C24"/>
+  <cols>
+    <col min="1" max="1" width="21.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="90.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1535,6 +1563,11 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C31"/>
+  <cols>
+    <col min="1" max="1" width="33.83203125" customWidth="1"/>
+    <col min="2" max="2" width="124.83203125" customWidth="1"/>
+    <col min="3" max="3" width="11.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1887,6 +1920,10 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B7"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="21.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1954,6 +1991,10 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B7"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2021,6 +2062,10 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B11"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="27.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2120,6 +2165,10 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B12"/>
+  <cols>
+    <col min="1" max="1" width="27.83203125" customWidth="1"/>
+    <col min="2" max="2" width="90.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2227,6 +2276,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C55"/>
+  <cols>
+    <col min="1" max="1" width="29.83203125" customWidth="1"/>
+    <col min="2" max="2" width="60.83203125" customWidth="1"/>
+    <col min="3" max="3" width="19.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2843,6 +2897,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D94"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="37.83203125" customWidth="1"/>
+    <col min="3" max="3" width="201.83203125" customWidth="1"/>
+    <col min="4" max="4" width="9.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4169,7 +4229,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D44"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="34.83203125" customWidth="1"/>
+    <col min="3" max="3" width="70.83203125" customWidth="1"/>
+    <col min="4" max="4" width="24.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4484,13 +4550,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B23" t="str">
-        <v>Annual Pay Monthly Option</v>
+        <v>Ultimate Card Present</v>
       </c>
       <c r="C23" t="str">
         <v>Yes</v>
       </c>
       <c r="D23" t="str">
-        <v/>
+        <v>boxing-ultimate-direct</v>
       </c>
     </row>
     <row r="24">
@@ -4498,13 +4564,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B24" t="str">
-        <v>Annual Pay Monthly Title</v>
+        <v>Ultimate Badge</v>
       </c>
       <c r="C24" t="str">
-        <v>Annual - Pay Monthly</v>
+        <v>The Ultimate Fan Package</v>
       </c>
       <c r="D24" t="str">
-        <v/>
+        <v>boxing-ultimate-direct</v>
       </c>
     </row>
     <row r="25">
@@ -4512,13 +4578,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B25" t="str">
-        <v>Annual Pay Monthly Price</v>
+        <v>Ultimate Plan Name</v>
       </c>
       <c r="C25" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="D25" t="str">
-        <v/>
+        <v>boxing-ultimate-direct</v>
       </c>
     </row>
     <row r="26">
@@ -4526,13 +4592,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B26" t="str">
-        <v>Annual Pay Monthly Price Length</v>
+        <v>Ultimate Package Description</v>
       </c>
       <c r="C26" t="str">
-        <v>/month</v>
+        <v>All these fights and more this year. One unbeatable price.</v>
       </c>
       <c r="D26" t="str">
-        <v/>
+        <v>boxing-ultimate-direct</v>
       </c>
     </row>
     <row r="27">
@@ -4540,13 +4606,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B27" t="str">
-        <v>Annual Pay Monthly Contract Text</v>
+        <v>Ultimate Image Strip Present</v>
       </c>
       <c r="C27" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_CONTRACT_TEXT}}</v>
+        <v>Yes</v>
       </c>
       <c r="D27" t="str">
-        <v/>
+        <v>boxing-ultimate-direct</v>
       </c>
     </row>
     <row r="28">
@@ -4554,7 +4620,7 @@
         <v>Ultimate</v>
       </c>
       <c r="B28" t="str">
-        <v>Annual Pay Monthly Selected</v>
+        <v>Annual Pay Monthly Option</v>
       </c>
       <c r="C28" t="str">
         <v>Yes</v>
@@ -4568,10 +4634,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B29" t="str">
-        <v>Annual Pay Upfront Option</v>
+        <v>Annual Pay Monthly Title</v>
       </c>
       <c r="C29" t="str">
-        <v>Yes</v>
+        <v>Annual - Pay Monthly</v>
       </c>
       <c r="D29" t="str">
         <v/>
@@ -4582,10 +4648,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B30" t="str">
-        <v>Annual Pay Upfront Title</v>
+        <v>Annual Pay Monthly Price</v>
       </c>
       <c r="C30" t="str">
-        <v>Annual - Pay Upfront</v>
+        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
       </c>
       <c r="D30" t="str">
         <v/>
@@ -4596,10 +4662,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B31" t="str">
-        <v>Annual Pay Upfront Save Badge</v>
+        <v>Annual Pay Monthly Price Length</v>
       </c>
       <c r="C31" t="str">
-        <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
+        <v>/month</v>
       </c>
       <c r="D31" t="str">
         <v/>
@@ -4610,10 +4676,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B32" t="str">
-        <v>Annual Pay Upfront Price</v>
+        <v>Annual Pay Monthly Contract Text</v>
       </c>
       <c r="C32" t="str">
-        <v>{{ANNUAL_UPFRONT_PRICE_DISPLAY}}</v>
+        <v>{{ANNUAL_PAY_MONTHLY_CONTRACT_TEXT}}</v>
       </c>
       <c r="D32" t="str">
         <v/>
@@ -4624,10 +4690,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B33" t="str">
-        <v>Annual Pay Upfront Price Length</v>
+        <v>Annual Pay Monthly Selected</v>
       </c>
       <c r="C33" t="str">
-        <v>/year</v>
+        <v>Yes</v>
       </c>
       <c r="D33" t="str">
         <v/>
@@ -4638,10 +4704,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B34" t="str">
-        <v>Annual Pay Upfront Selected</v>
+        <v>Annual Pay Upfront Option</v>
       </c>
       <c r="C34" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="D34" t="str">
         <v/>
@@ -4652,10 +4718,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B35" t="str">
-        <v>Ultimate Feature 1</v>
+        <v>Annual Pay Upfront Title</v>
       </c>
       <c r="C35" t="str">
-        <v>{{ULTIMATE_FEATURE_1}}</v>
+        <v>Annual - Pay Upfront</v>
       </c>
       <c r="D35" t="str">
         <v/>
@@ -4666,10 +4732,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B36" t="str">
-        <v>Ultimate Feature 2</v>
+        <v>Annual Pay Upfront Save Badge</v>
       </c>
       <c r="C36" t="str">
-        <v>{{ULTIMATE_FEATURE_2}}</v>
+        <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
       </c>
       <c r="D36" t="str">
         <v/>
@@ -4680,10 +4746,10 @@
         <v>Ultimate</v>
       </c>
       <c r="B37" t="str">
-        <v>Ultimate Feature 3</v>
+        <v>Annual Pay Upfront Price</v>
       </c>
       <c r="C37" t="str">
-        <v>{{ULTIMATE_FEATURE_3}}</v>
+        <v>{{ANNUAL_UPFRONT_PRICE_DISPLAY}}</v>
       </c>
       <c r="D37" t="str">
         <v/>
@@ -4694,18 +4760,102 @@
         <v>Ultimate</v>
       </c>
       <c r="B38" t="str">
+        <v>Annual Pay Upfront Price Length</v>
+      </c>
+      <c r="C38" t="str">
+        <v>/year</v>
+      </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Ultimate</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Annual Pay Upfront Selected</v>
+      </c>
+      <c r="C39" t="str">
+        <v>No</v>
+      </c>
+      <c r="D39" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Ultimate</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Ultimate Feature 1</v>
+      </c>
+      <c r="C40" t="str">
+        <v>{{ULTIMATE_FEATURE_1}}</v>
+      </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Ultimate</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Ultimate Feature 2</v>
+      </c>
+      <c r="C41" t="str">
+        <v>{{ULTIMATE_FEATURE_2}}</v>
+      </c>
+      <c r="D41" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Ultimate</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Ultimate Feature 3</v>
+      </c>
+      <c r="C42" t="str">
+        <v>{{ULTIMATE_FEATURE_3}}</v>
+      </c>
+      <c r="D42" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>Ultimate</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Select How To Pay Heading</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Select how to pay</v>
+      </c>
+      <c r="D43" t="str">
+        <v>boxing-ultimate-direct</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>Ultimate</v>
+      </c>
+      <c r="B44" t="str">
         <v>CTA Button</v>
       </c>
-      <c r="C38" t="str">
+      <c r="C44" t="str">
         <v>{{PLAN_CTA_BUTTON}}</v>
       </c>
-      <c r="D38" t="str">
+      <c r="D44" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D44"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4713,6 +4863,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E103"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="27.83203125" customWidth="1"/>
+    <col min="3" max="3" width="28.83203125" customWidth="1"/>
+    <col min="4" max="4" width="160.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6475,6 +6632,10 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B13"/>
+  <cols>
+    <col min="1" max="1" width="27.83203125" customWidth="1"/>
+    <col min="2" max="2" width="90.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6590,6 +6751,10 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B9"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="25.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6673,6 +6838,10 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B24"/>
+  <cols>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="70.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6876,6 +7045,10 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B18"/>
+  <cols>
+    <col min="1" max="1" width="29.83203125" customWidth="1"/>
+    <col min="2" max="2" width="79.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>

<commit_message>
feat: home-page-popup validations, SearchPage fix, auth improvements and config updates
- scripts/generateExcel.ts: add home-page-popup validation rows (HOME_POPUP_DATE, HOME_POPUP_DESCRIPTION)
- config/events/aj_joshua_prenga.json: align HOME_POPUP_DESCRIPTION with BANNER_DESCRIPTION
- config/events/spence_tszyu.json: update event config fields
- auth/AuthenticationManager.ts: improve email auth reliability and error handling
- config/userstatus.json: update test credentials
- data/PPV_Input.xlsx: regenerated with home-page-popup rows
- pages/SearchPage.ts: restore complete file (fix truncation from upstream merge)
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -1282,7 +1282,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C29"/>
   <cols>
     <col min="1" max="1" width="21.83203125" customWidth="1"/>
     <col min="2" max="2" width="28.83203125" customWidth="1"/>
@@ -1553,9 +1553,64 @@
         <v>Visible</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>home-page-popup</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Popup - Image Present</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>home-page-popup</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Popup - Event Title</v>
+      </c>
+      <c r="C26" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>home-page-popup</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Popup - Event Date</v>
+      </c>
+      <c r="C27" t="str">
+        <v>{{HOME_POPUP_DATE}}</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>home-page-popup</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Popup - Event Description</v>
+      </c>
+      <c r="C28" t="str">
+        <v>{{HOME_POPUP_DESCRIPTION}}</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>home-page-popup</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Popup - Buy Now CTA</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C29"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add Android validation updates and supporting config changes
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -22,6 +22,7 @@
     <sheet name="Upsell Second Success page" sheetId="17" r:id="rId17"/>
     <sheet name="Upsell Payment page" sheetId="18" r:id="rId18"/>
     <sheet name="Search page" sheetId="19" r:id="rId19"/>
+    <sheet name="paywall" sheetId="20" r:id="rId20"/>
   </sheets>
 </workbook>
 </file>
@@ -416,11 +417,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C12"/>
-  <cols>
-    <col min="1" max="1" width="33.83203125" customWidth="1"/>
-    <col min="2" max="2" width="27.83203125" customWidth="1"/>
-    <col min="3" max="3" width="21.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -564,11 +560,6 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C23"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="27.83203125" customWidth="1"/>
-    <col min="3" max="3" width="318.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -833,10 +824,6 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B6"/>
-  <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="64.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -896,10 +883,6 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B6"/>
-  <cols>
-    <col min="1" max="1" width="19.83203125" customWidth="1"/>
-    <col min="2" max="2" width="34.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -959,11 +942,6 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C28"/>
-  <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
-    <col min="3" max="3" width="90.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1283,11 +1261,6 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C24"/>
-  <cols>
-    <col min="1" max="1" width="21.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
-    <col min="3" max="3" width="90.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1563,11 +1536,6 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C31"/>
-  <cols>
-    <col min="1" max="1" width="33.83203125" customWidth="1"/>
-    <col min="2" max="2" width="124.83203125" customWidth="1"/>
-    <col min="3" max="3" width="11.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1920,10 +1888,6 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B7"/>
-  <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="21.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1991,10 +1955,6 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B7"/>
-  <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2062,10 +2022,6 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B11"/>
-  <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="27.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2165,10 +2121,6 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B12"/>
-  <cols>
-    <col min="1" max="1" width="27.83203125" customWidth="1"/>
-    <col min="2" max="2" width="90.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2276,11 +2228,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C55"/>
-  <cols>
-    <col min="1" max="1" width="29.83203125" customWidth="1"/>
-    <col min="2" max="2" width="60.83203125" customWidth="1"/>
-    <col min="3" max="3" width="19.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2894,15 +2841,76 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B7"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Field</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Expected</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Page Title</v>
+      </c>
+      <c r="B2" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>PPV Name</v>
+      </c>
+      <c r="B3" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>PPV Date and Time</v>
+      </c>
+      <c r="B4" t="str">
+        <v>{{PPV_DATE}}</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Banner Image Present</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Buy Now Button</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Buy now</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>PPV Tile Present</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D94"/>
-  <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="37.83203125" customWidth="1"/>
-    <col min="3" max="3" width="201.83203125" customWidth="1"/>
-    <col min="4" max="4" width="9.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4230,12 +4238,6 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D44"/>
-  <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="34.83203125" customWidth="1"/>
-    <col min="3" max="3" width="70.83203125" customWidth="1"/>
-    <col min="4" max="4" width="24.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4863,13 +4865,6 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E103"/>
-  <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="27.83203125" customWidth="1"/>
-    <col min="3" max="3" width="28.83203125" customWidth="1"/>
-    <col min="4" max="4" width="160.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6632,10 +6627,6 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B13"/>
-  <cols>
-    <col min="1" max="1" width="27.83203125" customWidth="1"/>
-    <col min="2" max="2" width="90.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6751,10 +6742,6 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B9"/>
-  <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="25.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6838,10 +6825,6 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B24"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="70.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7045,10 +7028,6 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B18"/>
-  <cols>
-    <col min="1" max="1" width="29.83203125" customWidth="1"/>
-    <col min="2" max="2" width="79.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>

<commit_message>
fix: sync generateExcel.ts with manually edited PPV_Input.xlsx
- Landing page: use PPV_NAME/PPV_DATE/BANNER_DESCRIPTION instead of MOBILE_ variants;
  add Fight Card CTA; remove Copy rows
- Schedule page: replace 19 rows with 12 focused rows using SCHEDULE_PPV_TIME
  and PPV_POPUP_DATE; consistent Popup- field naming
- Home of Boxing: replace home-boxing-upcoming with correct 10-row structure
  (PPV tile, date, promoter, lock icon, WATCH LIVE date+time text)
- Home page: simplify banner (remove Banner Image Present, use direct vars);
  add tile validation rows to dont-miss; remove home-page-popup section
- Search page: add 6 popup validation rows; use SEARCH_PPV_DATE_TIME field
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -417,6 +417,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C12"/>
+  <cols>
+    <col min="1" max="1" width="33.83203125" customWidth="1"/>
+    <col min="2" max="2" width="27.83203125" customWidth="1"/>
+    <col min="3" max="3" width="21.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -560,6 +565,11 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C23"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="27.83203125" customWidth="1"/>
+    <col min="3" max="3" width="318.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -824,6 +834,10 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B6"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="64.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -883,6 +897,10 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B6"/>
+  <cols>
+    <col min="1" max="1" width="19.83203125" customWidth="1"/>
+    <col min="2" max="2" width="34.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -942,6 +960,11 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C28"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="90.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1261,6 +1284,11 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C24"/>
+  <cols>
+    <col min="1" max="1" width="21.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="90.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1536,6 +1564,11 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C31"/>
+  <cols>
+    <col min="1" max="1" width="33.83203125" customWidth="1"/>
+    <col min="2" max="2" width="124.83203125" customWidth="1"/>
+    <col min="3" max="3" width="11.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1888,6 +1921,10 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B7"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="21.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1955,6 +1992,10 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B7"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2022,6 +2063,10 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B11"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="27.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2121,6 +2166,10 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B12"/>
+  <cols>
+    <col min="1" max="1" width="27.83203125" customWidth="1"/>
+    <col min="2" max="2" width="90.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2228,6 +2277,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C55"/>
+  <cols>
+    <col min="1" max="1" width="29.83203125" customWidth="1"/>
+    <col min="2" max="2" width="60.83203125" customWidth="1"/>
+    <col min="3" max="3" width="19.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2844,6 +2898,10 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B7"/>
+  <cols>
+    <col min="1" max="1" width="21.83203125" customWidth="1"/>
+    <col min="2" max="2" width="74.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2855,50 +2913,50 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Page Title</v>
+        <v>Event Name</v>
       </c>
       <c r="B2" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>{{MOBILE_BANNER_TITLE}}</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>PPV Name</v>
+        <v>Event Date and Time</v>
       </c>
       <c r="B3" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>{{MOBILE_PPV_DATE}}</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>PPV Date and Time</v>
+        <v>Category</v>
       </c>
       <c r="B4" t="str">
-        <v>{{PPV_DATE}}</v>
+        <v>Matchroom Boxing</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Banner Image Present</v>
+        <v>Instruction Header</v>
       </c>
       <c r="B5" t="str">
-        <v>Yes</v>
+        <v>How to watch this and more?</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Buy Now Button</v>
+        <v>Instruction Text</v>
       </c>
       <c r="B6" t="str">
-        <v>Buy now</v>
+        <v>Paste this link on your browser and choose the plan that’s right for you</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>PPV Tile Present</v>
+        <v>Copy Button</v>
       </c>
       <c r="B7" t="str">
-        <v>Yes</v>
+        <v>Copy</v>
       </c>
     </row>
   </sheetData>
@@ -2911,6 +2969,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D94"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="37.83203125" customWidth="1"/>
+    <col min="3" max="3" width="201.83203125" customWidth="1"/>
+    <col min="4" max="4" width="9.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4238,6 +4302,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D44"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="34.83203125" customWidth="1"/>
+    <col min="3" max="3" width="70.83203125" customWidth="1"/>
+    <col min="4" max="4" width="24.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4865,6 +4935,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E103"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="27.83203125" customWidth="1"/>
+    <col min="3" max="3" width="28.83203125" customWidth="1"/>
+    <col min="4" max="4" width="160.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6627,6 +6704,10 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B13"/>
+  <cols>
+    <col min="1" max="1" width="27.83203125" customWidth="1"/>
+    <col min="2" max="2" width="90.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6742,6 +6823,10 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B9"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="25.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6825,6 +6910,10 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B24"/>
+  <cols>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="70.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7028,6 +7117,10 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B18"/>
+  <cols>
+    <col min="1" max="1" width="29.83203125" customWidth="1"/>
+    <col min="2" max="2" width="79.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>

<commit_message>
fix: additive sync — add xlsx-only fields to generateExcel.ts (keep all MOBILE_ fields)
Added fields from manually edited xlsx WITHOUT removing any existing mobile fields:
- Landing page: + Banner - Fight Card CTA (Visible)
- Schedule page: + PPV Time on Tile (SCHEDULE_PPV_TIME); + Popup- prefix rows
  alongside existing Popup rows (PPV_POPUP_DATE, consistent naming)
- Home of Boxing: + PPV Promoter on Tile, PPV Date and Time Text, Buy Now CTA,
  Fight Card CTA, Lock Icon Present to home-boxing-upcoming
- Home page: + Don't Miss Section, PPV Tile Present, PPV Name, PPV Date,
  PPV Image Present to home-page-dont-miss (tile rows before popup)
- Search page: + Search PPV Date and Time (SEARCH_PPV_DATE_TIME) + 6 Popup- rows
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -416,10 +416,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C15"/>
   <cols>
     <col min="1" max="1" width="33.83203125" customWidth="1"/>
-    <col min="2" max="2" width="27.83203125" customWidth="1"/>
+    <col min="2" max="2" width="99.83203125" customWidth="1"/>
     <col min="3" max="3" width="21.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -491,10 +491,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Banner - Event Title</v>
+        <v>Banner Image Present</v>
       </c>
       <c r="B7" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>Yes</v>
       </c>
       <c r="C7" t="str">
         <v>landing-page-banner</v>
@@ -502,10 +502,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Banner - Event Date</v>
+        <v>Banner - Event Title</v>
       </c>
       <c r="B8" t="str">
-        <v>{{PPV_DATE}}</v>
+        <v>{{MOBILE_BANNER_TITLE}}</v>
       </c>
       <c r="C8" t="str">
         <v>landing-page-banner</v>
@@ -513,10 +513,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Banner - Event Description</v>
+        <v>Banner - Buy Now CTA</v>
       </c>
       <c r="B9" t="str">
-        <v>{{BANNER_DESCRIPTION}}</v>
+        <v>Buy now</v>
       </c>
       <c r="C9" t="str">
         <v>landing-page-banner</v>
@@ -524,10 +524,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Banner Image Present</v>
+        <v>Banner - Event Description</v>
       </c>
       <c r="B10" t="str">
-        <v>Yes</v>
+        <v>{{MOBILE_BANNER_DESCRIPTION}}</v>
       </c>
       <c r="C10" t="str">
         <v>landing-page-banner</v>
@@ -535,10 +535,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Banner - Buy Now CTA</v>
+        <v>Banner - Event Date</v>
       </c>
       <c r="B11" t="str">
-        <v>Visible</v>
+        <v>{{MOBILE_BANNER_DATE_TIME}}</v>
       </c>
       <c r="C11" t="str">
         <v>landing-page-banner</v>
@@ -546,18 +546,51 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Banner - Fight Card CTA</v>
+        <v>Copy Description</v>
       </c>
       <c r="B12" t="str">
-        <v>Visible</v>
+        <v>Copy the link below and paste it in your browser. We'll take you back to the app when you finish.</v>
       </c>
       <c r="C12" t="str">
         <v>landing-page-banner</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Copy URL</v>
+      </c>
+      <c r="B13" t="str">
+        <v>https://dazn-direct-subscription-prod.s3.eu-</v>
+      </c>
+      <c r="C13" t="str">
+        <v>landing-page-banner</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Copy Button</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Copy</v>
+      </c>
+      <c r="C14" t="str">
+        <v>landing-page-banner</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Banner - Fight Card CTA</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Visible</v>
+      </c>
+      <c r="C15" t="str">
+        <v>landing-page-banner</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C15"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -959,7 +992,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C32"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="28.83203125" customWidth="1"/>
@@ -1169,10 +1202,10 @@
         <v>home-boxing-upcoming</v>
       </c>
       <c r="B19" t="str">
-        <v>Best of Boxing Section</v>
+        <v>PPV Image Present</v>
       </c>
       <c r="C19" t="str">
-        <v>Present</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="20">
@@ -1180,10 +1213,10 @@
         <v>home-boxing-upcoming</v>
       </c>
       <c r="B20" t="str">
-        <v>PPV Tile Present</v>
+        <v>PPV Title</v>
       </c>
       <c r="C20" t="str">
-        <v>Yes</v>
+        <v>{{MOBILE_BANNER_TITLE}}</v>
       </c>
     </row>
     <row r="21">
@@ -1191,10 +1224,10 @@
         <v>home-boxing-upcoming</v>
       </c>
       <c r="B21" t="str">
-        <v>PPV Date</v>
+        <v>Sponsor</v>
       </c>
       <c r="C21" t="str">
-        <v>{{LANDING_PAGE_PPV_DATE}}</v>
+        <v>Matchroom Boxing</v>
       </c>
     </row>
     <row r="22">
@@ -1202,10 +1235,10 @@
         <v>home-boxing-upcoming</v>
       </c>
       <c r="B22" t="str">
-        <v>PPV Promoter on Tile</v>
+        <v>Description</v>
       </c>
       <c r="C22" t="str">
-        <v>{{PPV_PROMOTER}}</v>
+        <v>WATCH LIVE {{MOBILE_SEARCH_PPV_DATE}}</v>
       </c>
     </row>
     <row r="23">
@@ -1213,10 +1246,10 @@
         <v>home-boxing-upcoming</v>
       </c>
       <c r="B23" t="str">
-        <v>PPV Name</v>
+        <v>Tile - Day</v>
       </c>
       <c r="C23" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>{{MOBILE_SCHEDULE_DAY}}</v>
       </c>
     </row>
     <row r="24">
@@ -1224,10 +1257,10 @@
         <v>home-boxing-upcoming</v>
       </c>
       <c r="B24" t="str">
-        <v>PPV Date and Time Text</v>
+        <v>Tile - Date</v>
       </c>
       <c r="C24" t="str">
-        <v>WATCH LIVE {{HOME_BOXING_UPCOMING_DATE}} at {{HOME_BOXING_UPCOMING_TIME}}</v>
+        <v>{{MOBILE_SCHEDULE_DATE}}</v>
       </c>
     </row>
     <row r="25">
@@ -1235,10 +1268,10 @@
         <v>home-boxing-upcoming</v>
       </c>
       <c r="B25" t="str">
-        <v>Buy Now CTA</v>
+        <v>Tile - Month</v>
       </c>
       <c r="C25" t="str">
-        <v>Buy now</v>
+        <v>{{MOBILE_SCHEDULE_MONTH}}</v>
       </c>
     </row>
     <row r="26">
@@ -1246,10 +1279,10 @@
         <v>home-boxing-upcoming</v>
       </c>
       <c r="B26" t="str">
-        <v>Fight Card CTA</v>
+        <v>Buy Now Button</v>
       </c>
       <c r="C26" t="str">
-        <v>Fight card</v>
+        <v>Buy now</v>
       </c>
     </row>
     <row r="27">
@@ -1257,10 +1290,10 @@
         <v>home-boxing-upcoming</v>
       </c>
       <c r="B27" t="str">
-        <v>PPV Image Present</v>
+        <v>Fight Card Button</v>
       </c>
       <c r="C27" t="str">
-        <v>Yes</v>
+        <v>Fight card</v>
       </c>
     </row>
     <row r="28">
@@ -1268,22 +1301,66 @@
         <v>home-boxing-upcoming</v>
       </c>
       <c r="B28" t="str">
+        <v>PPV Promoter on Tile</v>
+      </c>
+      <c r="C28" t="str">
+        <v>{{PPV_PROMOTER}}</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B29" t="str">
+        <v>PPV Date and Time Text</v>
+      </c>
+      <c r="C29" t="str">
+        <v>WATCH LIVE {{HOME_BOXING_UPCOMING_DATE}} at {{HOME_BOXING_UPCOMING_TIME}}</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Buy Now CTA</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Buy now</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Fight Card CTA</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Fight card</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>home-boxing-upcoming</v>
+      </c>
+      <c r="B32" t="str">
         <v>Lock Icon Present</v>
       </c>
-      <c r="C28" t="str">
+      <c r="C32" t="str">
         <v>Yes</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C32"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C30"/>
   <cols>
     <col min="1" max="1" width="21.83203125" customWidth="1"/>
     <col min="2" max="2" width="28.83203125" customWidth="1"/>
@@ -1306,10 +1383,10 @@
         <v>home-page-banner</v>
       </c>
       <c r="B2" t="str">
-        <v>Banner - Event Title</v>
+        <v>Banner Image Present</v>
       </c>
       <c r="C2" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="3">
@@ -1317,10 +1394,10 @@
         <v>home-page-banner</v>
       </c>
       <c r="B3" t="str">
-        <v>Banner - Event Date</v>
+        <v>Banner - Event Title</v>
       </c>
       <c r="C3" t="str">
-        <v>{{PPV_DATE}}</v>
+        <v>{{MOBILE_BANNER_TITLE}}</v>
       </c>
     </row>
     <row r="4">
@@ -1328,10 +1405,10 @@
         <v>home-page-banner</v>
       </c>
       <c r="B4" t="str">
-        <v>Banner - Event Description</v>
+        <v>Banner - Event Date</v>
       </c>
       <c r="C4" t="str">
-        <v>{{BANNER_DESCRIPTION}}</v>
+        <v>{{MOBILE_BANNER_DATE_TIME}}</v>
       </c>
     </row>
     <row r="5">
@@ -1339,10 +1416,10 @@
         <v>home-page-banner</v>
       </c>
       <c r="B5" t="str">
-        <v>Banner - Buy Now CTA</v>
+        <v>Banner - Event Description</v>
       </c>
       <c r="C5" t="str">
-        <v>Visible</v>
+        <v>{{MOBILE_BANNER_DESCRIPTION}}</v>
       </c>
     </row>
     <row r="6">
@@ -1350,21 +1427,21 @@
         <v>home-page-banner</v>
       </c>
       <c r="B6" t="str">
-        <v>Banner - Fight Card CTA</v>
+        <v>Banner - Buy Now CTA</v>
       </c>
       <c r="C6" t="str">
-        <v>Visible</v>
+        <v>Buy now</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>home-page-dont-miss</v>
+        <v>home-page-banner</v>
       </c>
       <c r="B7" t="str">
-        <v>Don't Miss Section</v>
+        <v>Banner - Fight Card CTA</v>
       </c>
       <c r="C7" t="str">
-        <v>Present</v>
+        <v>Fight Card</v>
       </c>
     </row>
     <row r="8">
@@ -1372,10 +1449,10 @@
         <v>home-page-dont-miss</v>
       </c>
       <c r="B8" t="str">
-        <v>PPV Tile Present</v>
+        <v>Don't Miss Section</v>
       </c>
       <c r="C8" t="str">
-        <v>Yes</v>
+        <v>Present</v>
       </c>
     </row>
     <row r="9">
@@ -1383,10 +1460,10 @@
         <v>home-page-dont-miss</v>
       </c>
       <c r="B9" t="str">
-        <v>PPV Name</v>
+        <v>PPV Tile Present</v>
       </c>
       <c r="C9" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="10">
@@ -1394,10 +1471,10 @@
         <v>home-page-dont-miss</v>
       </c>
       <c r="B10" t="str">
-        <v>PPV Date</v>
+        <v>PPV Name</v>
       </c>
       <c r="C10" t="str">
-        <v>{{LANDING_PAGE_PPV_DATE}}</v>
+        <v>{{PPV_NAME}}</v>
       </c>
     </row>
     <row r="11">
@@ -1405,10 +1482,10 @@
         <v>home-page-dont-miss</v>
       </c>
       <c r="B11" t="str">
-        <v>PPV Image Present</v>
+        <v>PPV Date</v>
       </c>
       <c r="C11" t="str">
-        <v>Yes</v>
+        <v>{{LANDING_PAGE_PPV_DATE}}</v>
       </c>
     </row>
     <row r="12">
@@ -1416,10 +1493,10 @@
         <v>home-page-dont-miss</v>
       </c>
       <c r="B12" t="str">
-        <v>Popup - Event Title</v>
+        <v>PPV Image Present</v>
       </c>
       <c r="C12" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="13">
@@ -1427,10 +1504,10 @@
         <v>home-page-dont-miss</v>
       </c>
       <c r="B13" t="str">
-        <v>Popup - Event Date</v>
+        <v>Popup - Event Title</v>
       </c>
       <c r="C13" t="str">
-        <v>{{PPV_POPUP_DATE}}</v>
+        <v>{{PPV_NAME}}</v>
       </c>
     </row>
     <row r="14">
@@ -1438,10 +1515,10 @@
         <v>home-page-dont-miss</v>
       </c>
       <c r="B14" t="str">
-        <v>Popup - Promoter</v>
+        <v>Popup - Event Date</v>
       </c>
       <c r="C14" t="str">
-        <v>{{PPV_PROMOTER}}</v>
+        <v>{{PPV_POPUP_DATE}}</v>
       </c>
     </row>
     <row r="15">
@@ -1449,10 +1526,10 @@
         <v>home-page-dont-miss</v>
       </c>
       <c r="B15" t="str">
-        <v>Popup - Buy Now CTA</v>
+        <v>Popup - Promoter</v>
       </c>
       <c r="C15" t="str">
-        <v>Visible</v>
+        <v>{{PPV_PROMOTER}}</v>
       </c>
     </row>
     <row r="16">
@@ -1460,10 +1537,10 @@
         <v>home-page-dont-miss</v>
       </c>
       <c r="B16" t="str">
-        <v>Popup - Event Description</v>
+        <v>Popup - Buy Now CTA</v>
       </c>
       <c r="C16" t="str">
-        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
+        <v>Visible</v>
       </c>
     </row>
     <row r="17">
@@ -1471,21 +1548,21 @@
         <v>home-page-dont-miss</v>
       </c>
       <c r="B17" t="str">
-        <v>Popup - Close Button</v>
+        <v>Popup - Event Description</v>
       </c>
       <c r="C17" t="str">
-        <v>Visible</v>
+        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>home-biggest-fights</v>
+        <v>home-page-dont-miss</v>
       </c>
       <c r="B18" t="str">
-        <v>Biggest Fights Section</v>
+        <v>Popup - Close Button</v>
       </c>
       <c r="C18" t="str">
-        <v>Saturday Fight Night</v>
+        <v>Visible</v>
       </c>
     </row>
     <row r="19">
@@ -1493,10 +1570,10 @@
         <v>home-biggest-fights</v>
       </c>
       <c r="B19" t="str">
-        <v>Popup - Event Title</v>
+        <v>Biggest Fights Section</v>
       </c>
       <c r="C19" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>Saturday Fight Night</v>
       </c>
     </row>
     <row r="20">
@@ -1504,10 +1581,10 @@
         <v>home-biggest-fights</v>
       </c>
       <c r="B20" t="str">
-        <v>Popup - Event Date</v>
+        <v>Popup - Event Title</v>
       </c>
       <c r="C20" t="str">
-        <v>{{PPV_DATE}}</v>
+        <v>{{PPV_NAME}}</v>
       </c>
     </row>
     <row r="21">
@@ -1515,10 +1592,10 @@
         <v>home-biggest-fights</v>
       </c>
       <c r="B21" t="str">
-        <v>Popup - Promoter</v>
+        <v>Popup - Event Date</v>
       </c>
       <c r="C21" t="str">
-        <v>{{PPV_PROMOTER}}</v>
+        <v>{{PPV_DATE}}</v>
       </c>
     </row>
     <row r="22">
@@ -1526,10 +1603,10 @@
         <v>home-biggest-fights</v>
       </c>
       <c r="B22" t="str">
-        <v>Popup - Buy Now CTA</v>
+        <v>Popup - Promoter</v>
       </c>
       <c r="C22" t="str">
-        <v>Visible</v>
+        <v>{{PPV_PROMOTER}}</v>
       </c>
     </row>
     <row r="23">
@@ -1537,10 +1614,10 @@
         <v>home-biggest-fights</v>
       </c>
       <c r="B23" t="str">
-        <v>Popup - Event Description</v>
+        <v>Popup - Buy Now CTA</v>
       </c>
       <c r="C23" t="str">
-        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
+        <v>Visible</v>
       </c>
     </row>
     <row r="24">
@@ -1548,15 +1625,81 @@
         <v>home-biggest-fights</v>
       </c>
       <c r="B24" t="str">
+        <v>Popup - Event Description</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>home-biggest-fights</v>
+      </c>
+      <c r="B25" t="str">
         <v>Popup - Close Button</v>
       </c>
-      <c r="C24" t="str">
+      <c r="C25" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>home-page-popup</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Popup - Image Present</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>home-page-popup</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Popup - Event Title</v>
+      </c>
+      <c r="C27" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>home-page-popup</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Popup - Event Date</v>
+      </c>
+      <c r="C28" t="str">
+        <v>{{HOME_POPUP_DATE}}</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>home-page-popup</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Popup - Event Description</v>
+      </c>
+      <c r="C29" t="str">
+        <v>{{HOME_POPUP_DESCRIPTION}}</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>home-page-popup</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Popup - Buy Now CTA</v>
+      </c>
+      <c r="C30" t="str">
         <v>Visible</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C30"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2165,7 +2308,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <cols>
     <col min="1" max="1" width="27.83203125" customWidth="1"/>
     <col min="2" max="2" width="90.83203125" customWidth="1"/>
@@ -2205,71 +2348,79 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Search PPV Date and Time</v>
+        <v>Lock Icon Present</v>
       </c>
       <c r="B5" t="str">
-        <v>{{SEARCH_PPV_DATE_TIME}}</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Lock Icon Present</v>
+        <v>PPV Description</v>
       </c>
       <c r="B6" t="str">
-        <v>Yes</v>
+        <v>WATCH LIVE {{MOBILE_SEARCH_PPV_DATE}}</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Popup - Event Title</v>
+        <v>Search PPV Date and Time</v>
       </c>
       <c r="B7" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>{{SEARCH_PPV_DATE_TIME}}</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Popup - Event Date</v>
+        <v>Popup - Event Title</v>
       </c>
       <c r="B8" t="str">
-        <v>{{PPV_POPUP_DATE}}</v>
+        <v>{{PPV_NAME}}</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Popup - Promoter</v>
+        <v>Popup - Event Date</v>
       </c>
       <c r="B9" t="str">
-        <v>{{PPV_PROMOTER}}</v>
+        <v>{{PPV_POPUP_DATE}}</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Popup - Buy Now CTA</v>
+        <v>Popup - Promoter</v>
       </c>
       <c r="B10" t="str">
-        <v>Visible</v>
+        <v>{{PPV_PROMOTER}}</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Popup - Event Description</v>
+        <v>Popup - Buy Now CTA</v>
       </c>
       <c r="B11" t="str">
-        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
+        <v>Visible</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
+        <v>Popup - Event Description</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
         <v>Popup - Close Button</v>
       </c>
-      <c r="B12" t="str">
+      <c r="B13" t="str">
         <v>Visible</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B13"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6703,7 +6854,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B28"/>
   <cols>
     <col min="1" max="1" width="27.83203125" customWidth="1"/>
     <col min="2" max="2" width="90.83203125" customWidth="1"/>
@@ -6743,7 +6894,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Lock Icon Present</v>
+        <v>PPV Image Present</v>
       </c>
       <c r="B5" t="str">
         <v>Yes</v>
@@ -6751,71 +6902,191 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>PPV Promoter on Tile</v>
+        <v>Lock Icon Present</v>
       </c>
       <c r="B6" t="str">
-        <v>{{PPV_PROMOTER}}</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Popup - Image Present</v>
+        <v>PPV Promoter on Tile</v>
       </c>
       <c r="B7" t="str">
-        <v>Yes</v>
+        <v>{{PPV_PROMOTER}}</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Popup - Event Title</v>
+        <v>Day</v>
       </c>
       <c r="B8" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>{{MOBILE_SCHEDULE_DAY}}</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Popup - Event Date</v>
+        <v>Month</v>
       </c>
       <c r="B9" t="str">
-        <v>{{PPV_POPUP_DATE}}</v>
+        <v>{{MOBILE_SCHEDULE_MONTH}}</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Popup - Promoter</v>
+        <v>Date</v>
       </c>
       <c r="B10" t="str">
-        <v>{{PPV_PROMOTER}}</v>
+        <v>{{MOBILE_SCHEDULE_DATE}}</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Popup - Event Description</v>
+        <v>Time</v>
       </c>
       <c r="B11" t="str">
-        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
+        <v>{{MOBILE_SCHEDULE_TIME}}</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Popup - Buy Now CTA</v>
+        <v>Bell Icon Present</v>
       </c>
       <c r="B12" t="str">
-        <v>Visible</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
+        <v>Three Dots Icon Present</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Popup Image Present</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Popup Date</v>
+      </c>
+      <c r="B15" t="str">
+        <v>{{PPV_DATE}}</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Popup PPV Name</v>
+      </c>
+      <c r="B16" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Popup Promoter</v>
+      </c>
+      <c r="B17" t="str">
+        <v>{{PPV_PROMOTER}}</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Popup Description</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Popup Buy Now CTA Present</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Popup Buy Now CTA Text</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Buy now</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Popup Close Button</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Popup - Image Present</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Popup - Event Title</v>
+      </c>
+      <c r="B23" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Popup - Event Date</v>
+      </c>
+      <c r="B24" t="str">
+        <v>{{PPV_POPUP_DATE}}</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Popup - Promoter</v>
+      </c>
+      <c r="B25" t="str">
+        <v>{{PPV_PROMOTER}}</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Popup - Event Description</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Popup - Buy Now CTA</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
         <v>Popup - Close Button</v>
       </c>
-      <c r="B13" t="str">
+      <c r="B28" t="str">
         <v>Visible</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B28"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: finalize AU timezone overrides, banner date regex, resolveExpected cleanup, and upstream XLSX sync
- config/events/aj_joshua_prenga.json: fix AU PPV_POPUP_DATE/SEARCH_PPV_DATE_TIME to '25 JUL 1:30PM'
  and SCHEDULE_PPV_TIME to '1:30PM' (correct AU local time for 19:00 UTC)
- data/PPV_Input.xlsx: sync with upstream (adds 6 home-page-popup validation rows:
  Image Present, Event Title, Event Date/HOME_POPUP_DATE, Description, Buy Now CTA, Close Button)
- utils/getActualValue.ts: extend banner/popup date regex to handle full month names
  (e.g. 'July' instead of 'Jul') and optional AM/PM suffix for broader DAZN UI coverage
- utils/resolveExpected.ts: remove deprecated 'banner - event date' and 'popup - event date'
  aliases that were causing resolution conflicts
- pages/LandingPage.ts: whitespace normalisation in catch blocks (no logic change)
- .env.template: update GOOGLE_EMAIL/GOOGLE_PASSWORD to working test credentials
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Gopi.Sanagapalli/Downloads/UAT-PPV-End-to-End-Automation-main/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Hari.Prasad/jobbot/dazn-tests/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{137EA7F4-FE94-4544-8C38-3152178CB07E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{335296E0-26D5-3646-AD36-FD28D6EFA861}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15940" firstSheet="5" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" firstSheet="8" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Landing page" sheetId="1" r:id="rId1"/>
@@ -2798,6 +2798,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="76.5" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -3131,6 +3136,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <ignoredErrors>
     <ignoredError sqref="A1:C24" numberStoredAsText="1"/>
   </ignoredErrors>

</xml_diff>

<commit_message>
feat: update event config, boxing home page, search page, and validation utils
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2005" uniqueCount="534">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2041" uniqueCount="538">
   <si>
     <t>Field</t>
   </si>
@@ -1145,6 +1145,9 @@
     <t>PPV Date</t>
   </si>
   <si>
+    <t>{{PPV_PAGE_DATE}}</t>
+  </si>
+  <si>
     <t>PPV Status</t>
   </si>
   <si>
@@ -1371,6 +1374,15 @@
   </si>
   <si>
     <t>home-boxing-upcoming-ultimate-tile</t>
+  </si>
+  <si>
+    <t>home-boxing-upcoming-ultimate-login-first</t>
+  </si>
+  <si>
+    <t>Purchased Tag</t>
+  </si>
+  <si>
+    <t>PPV Image Time</t>
   </si>
   <si>
     <t>home-page-banner</t>
@@ -2301,7 +2313,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B2" t="s">
         <v>91</v>
@@ -2312,32 +2324,32 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B3" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C3" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B4" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C4" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B5" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C5" t="s">
         <v>4</v>
@@ -2345,21 +2357,21 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B6" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C6" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B7" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C7" t="s">
         <v>4</v>
@@ -2367,29 +2379,29 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B8" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C8" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B9" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C9" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B10" t="s">
         <v>283</v>
@@ -2400,7 +2412,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B11" t="s">
         <v>330</v>
@@ -2411,10 +2423,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B12" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C12" t="s">
         <v>273</v>
@@ -2422,18 +2434,18 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B13" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C13" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B14" t="s">
         <v>332</v>
@@ -2444,40 +2456,40 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B15" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C15" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B16" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C16" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B17" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C17" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B18" t="s">
         <v>283</v>
@@ -2488,7 +2500,7 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B19" t="s">
         <v>330</v>
@@ -2499,29 +2511,29 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B20" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C20" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B21" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C21" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B22" t="s">
         <v>332</v>
@@ -2532,13 +2544,13 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>420</v>
+      </c>
+      <c r="B23" t="s">
+        <v>418</v>
+      </c>
+      <c r="C23" t="s">
         <v>419</v>
-      </c>
-      <c r="B23" t="s">
-        <v>417</v>
-      </c>
-      <c r="C23" t="s">
-        <v>418</v>
       </c>
     </row>
   </sheetData>
@@ -2564,20 +2576,20 @@
         <v>91</v>
       </c>
       <c r="B2" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B3" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
@@ -2585,15 +2597,15 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B5" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B6" t="s">
         <v>4</v>
@@ -2622,20 +2634,20 @@
         <v>91</v>
       </c>
       <c r="B2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B3" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
@@ -2643,15 +2655,15 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="B5" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B6" t="s">
         <v>4</v>
@@ -2664,7 +2676,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr defaultRowHeight="16" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -2680,18 +2692,18 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B2" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="C2" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
@@ -2702,7 +2714,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B4" t="s">
         <v>16</v>
@@ -2713,7 +2725,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B5" t="s">
         <v>18</v>
@@ -2724,7 +2736,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B6" t="s">
         <v>21</v>
@@ -2735,7 +2747,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B7" t="s">
         <v>23</v>
@@ -2746,18 +2758,18 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>438</v>
+      </c>
+      <c r="B8" t="s">
+        <v>436</v>
+      </c>
+      <c r="C8" t="s">
         <v>437</v>
-      </c>
-      <c r="B8" t="s">
-        <v>435</v>
-      </c>
-      <c r="C8" t="s">
-        <v>436</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B9" t="s">
         <v>6</v>
@@ -2768,7 +2780,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B10" t="s">
         <v>7</v>
@@ -2779,7 +2791,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B11" t="s">
         <v>369</v>
@@ -2790,7 +2802,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B12" t="s">
         <v>59</v>
@@ -2801,7 +2813,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B13" t="s">
         <v>355</v>
@@ -2812,7 +2824,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B14" t="s">
         <v>356</v>
@@ -2823,7 +2835,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B15" t="s">
         <v>358</v>
@@ -2834,7 +2846,7 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B16" t="s">
         <v>361</v>
@@ -2845,7 +2857,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B17" t="s">
         <v>359</v>
@@ -2856,7 +2868,7 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B18" t="s">
         <v>362</v>
@@ -2867,18 +2879,18 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B19" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="C19" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B20" t="s">
         <v>6</v>
@@ -2889,7 +2901,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B21" t="s">
         <v>369</v>
@@ -2900,7 +2912,7 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B22" t="s">
         <v>353</v>
@@ -2911,7 +2923,7 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B23" t="s">
         <v>7</v>
@@ -2922,18 +2934,18 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B24" t="s">
         <v>56</v>
       </c>
       <c r="C24" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B25" t="s">
         <v>60</v>
@@ -2944,18 +2956,18 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B26" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="C26" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B27" t="s">
         <v>59</v>
@@ -2966,7 +2978,7 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B28" t="s">
         <v>352</v>
@@ -2977,7 +2989,7 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="B29" t="s">
         <v>13</v>
@@ -2988,7 +3000,7 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="B30" t="s">
         <v>16</v>
@@ -2999,7 +3011,7 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="B31" t="s">
         <v>18</v>
@@ -3010,7 +3022,7 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="B32" t="s">
         <v>21</v>
@@ -3021,7 +3033,7 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="B33" t="s">
         <v>26</v>
@@ -3032,7 +3044,7 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="B34" t="s">
         <v>23</v>
@@ -3043,7 +3055,7 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="B35" t="s">
         <v>27</v>
@@ -3054,7 +3066,7 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="B36" t="s">
         <v>28</v>
@@ -3065,7 +3077,7 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="B37" t="s">
         <v>30</v>
@@ -3076,7 +3088,7 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="B38" t="s">
         <v>31</v>
@@ -3087,7 +3099,7 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="B39" t="s">
         <v>33</v>
@@ -3098,7 +3110,7 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="B40" t="s">
         <v>34</v>
@@ -3109,13 +3121,145 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="B41" t="s">
         <v>34</v>
       </c>
       <c r="C41" t="s">
         <v>35</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>447</v>
+      </c>
+      <c r="B42" t="s">
+        <v>436</v>
+      </c>
+      <c r="C42" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>447</v>
+      </c>
+      <c r="B43" t="s">
+        <v>6</v>
+      </c>
+      <c r="C43" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>447</v>
+      </c>
+      <c r="B44" t="s">
+        <v>369</v>
+      </c>
+      <c r="C44" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>447</v>
+      </c>
+      <c r="B45" t="s">
+        <v>353</v>
+      </c>
+      <c r="C45" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>447</v>
+      </c>
+      <c r="B46" t="s">
+        <v>7</v>
+      </c>
+      <c r="C46" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>447</v>
+      </c>
+      <c r="B47" t="s">
+        <v>56</v>
+      </c>
+      <c r="C47" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>447</v>
+      </c>
+      <c r="B48" t="s">
+        <v>60</v>
+      </c>
+      <c r="C48" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>447</v>
+      </c>
+      <c r="B49" t="s">
+        <v>441</v>
+      </c>
+      <c r="C49" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>447</v>
+      </c>
+      <c r="B50" t="s">
+        <v>59</v>
+      </c>
+      <c r="C50" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>447</v>
+      </c>
+      <c r="B51" t="s">
+        <v>352</v>
+      </c>
+      <c r="C51" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>447</v>
+      </c>
+      <c r="B52" t="s">
+        <v>448</v>
+      </c>
+      <c r="C52" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>447</v>
+      </c>
+      <c r="B53" t="s">
+        <v>449</v>
+      </c>
+      <c r="C53" t="s">
+        <v>351</v>
       </c>
     </row>
   </sheetData>
@@ -3146,7 +3290,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="B2" t="s">
         <v>13</v>
@@ -3157,7 +3301,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="B3" t="s">
         <v>16</v>
@@ -3168,7 +3312,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="B4" t="s">
         <v>18</v>
@@ -3179,7 +3323,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="B5" t="s">
         <v>21</v>
@@ -3190,7 +3334,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="B6" t="s">
         <v>23</v>
@@ -3201,18 +3345,18 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="B7" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="C7" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="B8" t="s">
         <v>6</v>
@@ -3223,7 +3367,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="B9" t="s">
         <v>7</v>
@@ -3234,7 +3378,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="B10" t="s">
         <v>369</v>
@@ -3245,7 +3389,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="B11" t="s">
         <v>59</v>
@@ -3256,7 +3400,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="B12" t="s">
         <v>355</v>
@@ -3267,7 +3411,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="B13" t="s">
         <v>356</v>
@@ -3278,7 +3422,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="B14" t="s">
         <v>358</v>
@@ -3289,7 +3433,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="B15" t="s">
         <v>361</v>
@@ -3300,7 +3444,7 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="B16" t="s">
         <v>359</v>
@@ -3311,7 +3455,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="B17" t="s">
         <v>362</v>
@@ -3322,18 +3466,18 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="B18" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="C18" t="s">
-        <v>451</v>
+        <v>455</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="B19" t="s">
         <v>355</v>
@@ -3344,7 +3488,7 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="B20" t="s">
         <v>356</v>
@@ -3355,7 +3499,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="B21" t="s">
         <v>358</v>
@@ -3366,7 +3510,7 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="B22" t="s">
         <v>361</v>
@@ -3377,7 +3521,7 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="B23" t="s">
         <v>359</v>
@@ -3388,7 +3532,7 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="B24" t="s">
         <v>362</v>
@@ -3399,7 +3543,7 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="B25" t="s">
         <v>354</v>
@@ -3410,7 +3554,7 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="B26" t="s">
         <v>355</v>
@@ -3421,29 +3565,29 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="B27" t="s">
         <v>356</v>
       </c>
       <c r="C27" t="s">
-        <v>453</v>
+        <v>457</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="B28" t="s">
         <v>359</v>
       </c>
       <c r="C28" t="s">
-        <v>454</v>
+        <v>458</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="B29" t="s">
         <v>361</v>
@@ -3454,7 +3598,7 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="B30" t="s">
         <v>362</v>
@@ -3465,7 +3609,7 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="B31" t="s">
         <v>13</v>
@@ -3476,7 +3620,7 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="B32" t="s">
         <v>16</v>
@@ -3487,7 +3631,7 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="B33" t="s">
         <v>18</v>
@@ -3498,7 +3642,7 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="B34" t="s">
         <v>21</v>
@@ -3509,7 +3653,7 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="B35" t="s">
         <v>26</v>
@@ -3520,7 +3664,7 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="B36" t="s">
         <v>23</v>
@@ -3531,7 +3675,7 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="B37" t="s">
         <v>27</v>
@@ -3542,7 +3686,7 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="B38" t="s">
         <v>28</v>
@@ -3553,7 +3697,7 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="B39" t="s">
         <v>30</v>
@@ -3564,7 +3708,7 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="B40" t="s">
         <v>31</v>
@@ -3575,7 +3719,7 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="B41" t="s">
         <v>33</v>
@@ -3586,7 +3730,7 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="B42" t="s">
         <v>34</v>
@@ -3597,7 +3741,7 @@
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
       <c r="B43" t="s">
         <v>34</v>
@@ -3608,7 +3752,7 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="B44" t="s">
         <v>34</v>
@@ -3636,7 +3780,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -3644,21 +3788,21 @@
         <v>91</v>
       </c>
       <c r="B2" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="C2" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="B3" t="s">
-        <v>464</v>
+        <v>468</v>
       </c>
       <c r="C3" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -3669,18 +3813,18 @@
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>465</v>
+        <v>469</v>
       </c>
       <c r="B5" t="s">
         <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -3691,7 +3835,7 @@
         <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -3699,32 +3843,32 @@
         <v>142</v>
       </c>
       <c r="B7" t="s">
+        <v>470</v>
+      </c>
+      <c r="C7" t="s">
         <v>466</v>
-      </c>
-      <c r="C7" t="s">
-        <v>462</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>467</v>
+        <v>471</v>
       </c>
       <c r="B8" t="s">
-        <v>468</v>
+        <v>472</v>
       </c>
       <c r="C8" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
       <c r="B9" t="s">
         <v>196</v>
       </c>
       <c r="C9" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -3735,7 +3879,7 @@
         <v>219</v>
       </c>
       <c r="C10" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -3743,10 +3887,10 @@
         <v>220</v>
       </c>
       <c r="B11" t="s">
-        <v>470</v>
+        <v>474</v>
       </c>
       <c r="C11" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -3754,10 +3898,10 @@
         <v>222</v>
       </c>
       <c r="B12" t="s">
-        <v>471</v>
+        <v>475</v>
       </c>
       <c r="C12" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -3765,10 +3909,10 @@
         <v>225</v>
       </c>
       <c r="B13" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="C13" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -3776,10 +3920,10 @@
         <v>227</v>
       </c>
       <c r="B14" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="C14" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -3787,10 +3931,10 @@
         <v>229</v>
       </c>
       <c r="B15" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="C15" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -3801,7 +3945,7 @@
         <v>235</v>
       </c>
       <c r="C16" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -3809,164 +3953,164 @@
         <v>236</v>
       </c>
       <c r="B17" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="C17" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="B18" t="s">
         <v>121</v>
       </c>
       <c r="C18" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
       <c r="B19" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
       <c r="C19" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>479</v>
+        <v>483</v>
       </c>
       <c r="B20" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
       <c r="C20" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="B21" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="C21" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
       <c r="B22" t="s">
-        <v>483</v>
+        <v>487</v>
       </c>
       <c r="C22" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
       <c r="B23" t="s">
-        <v>485</v>
+        <v>489</v>
       </c>
       <c r="C23" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
       <c r="B24" t="s">
         <v>219</v>
       </c>
       <c r="C24" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
       <c r="B25" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="C25" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>494</v>
+      </c>
+      <c r="B26" t="s">
+        <v>495</v>
+      </c>
+      <c r="C26" t="s">
         <v>490</v>
-      </c>
-      <c r="B26" t="s">
-        <v>491</v>
-      </c>
-      <c r="C26" t="s">
-        <v>486</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
       <c r="B27" t="s">
         <v>235</v>
       </c>
       <c r="C27" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>493</v>
+        <v>497</v>
       </c>
       <c r="B28" t="s">
         <v>267</v>
       </c>
       <c r="C28" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>494</v>
+        <v>498</v>
       </c>
       <c r="B29" t="s">
         <v>121</v>
       </c>
       <c r="C29" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>495</v>
+        <v>499</v>
       </c>
       <c r="B30" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
       <c r="C30" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>497</v>
+        <v>501</v>
       </c>
       <c r="B31" t="s">
         <v>269</v>
       </c>
       <c r="C31" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
     </row>
   </sheetData>
@@ -3989,23 +4133,23 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
       <c r="B2" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
       <c r="B3" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>502</v>
+        <v>506</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
@@ -4013,26 +4157,26 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="B5" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>505</v>
+        <v>509</v>
       </c>
       <c r="B6" t="s">
-        <v>506</v>
+        <v>510</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>507</v>
+        <v>511</v>
       </c>
       <c r="B7" t="s">
-        <v>508</v>
+        <v>512</v>
       </c>
     </row>
   </sheetData>
@@ -4055,31 +4199,31 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
       <c r="B2" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B3" t="s">
-        <v>511</v>
+        <v>515</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
       <c r="B4" t="s">
-        <v>513</v>
+        <v>517</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="B5" t="s">
         <v>4</v>
@@ -4087,18 +4231,18 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>515</v>
+        <v>519</v>
       </c>
       <c r="B6" t="s">
-        <v>516</v>
+        <v>520</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>517</v>
+        <v>521</v>
       </c>
       <c r="B7" t="s">
-        <v>518</v>
+        <v>522</v>
       </c>
     </row>
   </sheetData>
@@ -4124,7 +4268,7 @@
         <v>91</v>
       </c>
       <c r="B2" t="s">
-        <v>519</v>
+        <v>523</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -4137,10 +4281,10 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>520</v>
+        <v>524</v>
       </c>
       <c r="B4" t="s">
-        <v>521</v>
+        <v>525</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -4148,15 +4292,15 @@
         <v>142</v>
       </c>
       <c r="B5" t="s">
-        <v>522</v>
+        <v>526</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B6" t="s">
-        <v>523</v>
+        <v>527</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -4164,39 +4308,39 @@
         <v>314</v>
       </c>
       <c r="B7" t="s">
-        <v>524</v>
+        <v>528</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>525</v>
+        <v>529</v>
       </c>
       <c r="B8" t="s">
-        <v>526</v>
+        <v>530</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="B9" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B10" t="s">
-        <v>529</v>
+        <v>533</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>530</v>
+        <v>534</v>
       </c>
       <c r="B11" t="s">
-        <v>531</v>
+        <v>535</v>
       </c>
     </row>
   </sheetData>
@@ -4220,7 +4364,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -4228,7 +4372,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -4236,7 +4380,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>59</v>
       </c>
@@ -4244,15 +4388,15 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>532</v>
+        <v>536</v>
       </c>
       <c r="B5" t="s">
-        <v>533</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>352</v>
       </c>
@@ -4260,7 +4404,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>355</v>
       </c>
@@ -4268,7 +4412,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>356</v>
       </c>
@@ -4276,7 +4420,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>358</v>
       </c>
@@ -4284,7 +4428,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>361</v>
       </c>
@@ -4292,7 +4436,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>359</v>
       </c>
@@ -4300,7 +4444,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>362</v>
       </c>
@@ -4455,7 +4599,7 @@
         <v>56</v>
       </c>
       <c r="B12" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="C12" t="s">
         <v>54</v>
@@ -5102,7 +5246,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B4" t="s">
         <v>17</v>
@@ -8866,7 +9010,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -8874,7 +9018,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -8882,7 +9026,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>350</v>
       </c>
@@ -8890,7 +9034,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>352</v>
       </c>
@@ -8898,7 +9042,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>353</v>
       </c>
@@ -8906,7 +9050,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>354</v>
       </c>
@@ -8914,7 +9058,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>355</v>
       </c>
@@ -8922,7 +9066,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>356</v>
       </c>
@@ -8930,7 +9074,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>358</v>
       </c>
@@ -8938,7 +9082,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>359</v>
       </c>
@@ -8946,7 +9090,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>361</v>
       </c>
@@ -8954,7 +9098,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>362</v>
       </c>
@@ -9028,7 +9172,7 @@
         <v>369</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>370</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -9041,10 +9185,10 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B8" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -9078,12 +9222,12 @@
         <v>91</v>
       </c>
       <c r="B2" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B3" t="s">
         <v>14</v>
@@ -9094,12 +9238,12 @@
         <v>94</v>
       </c>
       <c r="B4" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B5" t="s">
         <v>4</v>
@@ -9107,7 +9251,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B6" t="s">
         <v>4</v>
@@ -9115,7 +9259,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B7" t="s">
         <v>143</v>
@@ -9131,7 +9275,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B9" t="s">
         <v>17</v>
@@ -9139,7 +9283,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B10" t="s">
         <v>4</v>
@@ -9147,7 +9291,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B11" t="s">
         <v>208</v>
@@ -9155,7 +9299,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B12" t="s">
         <v>154</v>
@@ -9163,15 +9307,15 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B13" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B14" t="s">
         <v>121</v>
@@ -9179,7 +9323,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="B15" t="s">
         <v>4</v>
@@ -9235,10 +9379,10 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B22" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -9277,7 +9421,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
@@ -9293,7 +9437,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
@@ -9309,7 +9453,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B6" t="s">
         <v>17</v>
@@ -9317,7 +9461,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
@@ -9341,7 +9485,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B10" t="s">
         <v>4</v>
@@ -9349,7 +9493,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B11" t="s">
         <v>4</v>
@@ -9357,7 +9501,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B12" t="s">
         <v>4</v>
@@ -9365,7 +9509,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B13" t="s">
         <v>4</v>
@@ -9373,7 +9517,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B14" t="s">
         <v>4</v>
@@ -9381,7 +9525,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B15" t="s">
         <v>4</v>
@@ -9389,7 +9533,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="B16" t="s">
         <v>4</v>
@@ -9397,18 +9541,18 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B17" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B18" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: update event times, add spence_tszyu config, boxing page and my account fixes
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2041" uniqueCount="538">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2038" uniqueCount="538">
   <si>
     <t>Field</t>
   </si>
@@ -4470,7 +4470,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C67"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr defaultRowHeight="16" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -5094,7 +5094,7 @@
         <v>16</v>
       </c>
       <c r="B57" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="C57" t="s">
         <v>132</v>
@@ -5124,7 +5124,7 @@
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B60" t="s">
         <v>22</v>
@@ -5135,7 +5135,7 @@
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B61" t="s">
         <v>22</v>
@@ -5146,21 +5146,21 @@
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B62" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="C62" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B63" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C63" t="s">
         <v>133</v>
@@ -5168,10 +5168,10 @@
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B64" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="C64" t="s">
         <v>133</v>
@@ -5179,10 +5179,10 @@
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B65" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="C65" t="s">
         <v>133</v>
@@ -5190,23 +5190,12 @@
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B66" t="s">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="C66" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>34</v>
-      </c>
-      <c r="B67" t="s">
-        <v>35</v>
-      </c>
-      <c r="C67" t="s">
         <v>134</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(ios): post-kickoff v3 — Safari page-ready wait, boxing feed wait, payment title fix, validation and flow improvements
Includes all local changes on top of upstream/main (PR #74 merged).
Conflicts with PR #74 base resolved by taking the local (more recent) versions.
TSC: clean (appium + root).
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -3926,7 +3926,7 @@
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C22"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4148,10 +4148,31 @@
         <v>home-boxing-upcoming</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Banner Description</v>
+      </c>
+      <c r="B21" t="str">
+        <v>{{MOBILE_BANNER_DESCRIPTION}}</v>
+      </c>
+      <c r="C21" t="str">
+        <v>home-boxing-banner</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Fight Card CTA</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Fight card</v>
+      </c>
+      <c r="C22" t="str">
+        <v>home-boxing-banner</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C22"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(CA): add Canada UFC PPV end-to-end automation, matrix & active ultimate purchase flow
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -701,7 +701,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C37"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -956,9 +956,163 @@
         <v>{{NEXT_PAYMENT_DATE}}</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>canada_popup</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Popup Title</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Get even more from your plan</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>canada_popup</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Popup Subtitle</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Upgrade to Ultimate for best quality streaming and more.</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>canada_popup</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Standard Streams</v>
+      </c>
+      <c r="C26" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>canada_popup</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Ultimate Streams</v>
+      </c>
+      <c r="C27" t="str">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>canada_popup</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Standard IP Locations</v>
+      </c>
+      <c r="C28" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>canada_popup</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Ultimate IP Locations</v>
+      </c>
+      <c r="C29" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>canada_popup</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Standard Multiview</v>
+      </c>
+      <c r="C30" t="str">
+        <v>✖</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>canada_popup</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Ultimate Multiview</v>
+      </c>
+      <c r="C31" t="str">
+        <v>✔</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>canada_popup</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Standard No Pre-Roll Ads</v>
+      </c>
+      <c r="C32" t="str">
+        <v>✖</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>canada_popup</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Ultimate No Pre-Roll Ads</v>
+      </c>
+      <c r="C33" t="str">
+        <v>✔</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>canada_popup</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Standard Downloads</v>
+      </c>
+      <c r="C34" t="str">
+        <v>✔</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>canada_popup</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Ultimate Downloads</v>
+      </c>
+      <c r="C35" t="str">
+        <v>✔</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>canada_popup</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Ultimate Action Button</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Continue with Ultimate</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>canada_popup</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Standard Action Button</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Continue with Standard</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C37"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3926,7 +4080,7 @@
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C19"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4007,7 +4161,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>PPV PROMOTER</v>
+        <v>Sponsor</v>
       </c>
       <c r="B8" t="str">
         <v>{{PPV_PROMOTER}}</v>
@@ -4021,7 +4175,7 @@
         <v>Description</v>
       </c>
       <c r="B9" t="str">
-        <v>WATCH LIVE {{MOBILE_SEARCH_PPV_DATE}} at {{PPV_TIME}}</v>
+        <v>WATCH LIVE {{MOBILE_SEARCH_PPV_DATE}}</v>
       </c>
       <c r="C9" t="str">
         <v>home-boxing-upcoming</v>
@@ -4137,21 +4291,10 @@
         <v>home-boxing-tile</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>PPV Time</v>
-      </c>
-      <c r="B20" t="str">
-        <v>{{PPV_TIME}}</v>
-      </c>
-      <c r="C20" t="str">
-        <v>home-boxing-upcoming</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C19"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4556,7 +4699,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D94"/>
+  <dimension ref="A1:D111"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4582,6 +4725,9 @@
       <c r="C2" t="str">
         <v>Choose the right plan for you.</v>
       </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -4593,6 +4739,9 @@
       <c r="C3" t="str">
         <v>To watch your pay-per-view, you'll need a DAZN plan.</v>
       </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -4604,6 +4753,9 @@
       <c r="C4" t="str">
         <v>N/A</v>
       </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -4615,6 +4767,9 @@
       <c r="C5" t="str">
         <v>{{PPV_DISPLAY_NAME}}</v>
       </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -4626,6 +4781,9 @@
       <c r="C6" t="str">
         <v>/fight</v>
       </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -4637,6 +4795,9 @@
       <c r="C7" t="str">
         <v>{{PPV_PRICE}}</v>
       </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -4648,6 +4809,9 @@
       <c r="C8" t="str">
         <v>{{CURRENCY}}</v>
       </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -4673,6 +4837,9 @@
       <c r="C10" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -4684,6 +4851,9 @@
       <c r="C11" t="str">
         <v>Yes</v>
       </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -4695,6 +4865,9 @@
       <c r="C12" t="str">
         <v>{{PPV_DATE}}</v>
       </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -4706,6 +4879,9 @@
       <c r="C13" t="str">
         <v>Yes</v>
       </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -4717,6 +4893,9 @@
       <c r="C14" t="str">
         <v>{{PPV_DISPLAY_NAME}}</v>
       </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -4728,6 +4907,9 @@
       <c r="C15" t="str">
         <v>{{PPV_CARD_DESCRIPTION}}</v>
       </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -4739,6 +4921,9 @@
       <c r="C16" t="str">
         <v>Yes</v>
       </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -4750,6 +4935,9 @@
       <c r="C17" t="str">
         <v>The Ultimate Fan Package</v>
       </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -4761,6 +4949,9 @@
       <c r="C18" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -4772,6 +4963,9 @@
       <c r="C19" t="str">
         <v>N/A</v>
       </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -4783,6 +4977,9 @@
       <c r="C20" t="str">
         <v>{{UPSELL_PRICE}}</v>
       </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -4794,6 +4991,9 @@
       <c r="C21" t="str">
         <v>{{UPSELL_PRICE_LENGTH}}</v>
       </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -4805,6 +5005,9 @@
       <c r="C22" t="str">
         <v>{{UPSELL_CROSSED_PRICE}}</v>
       </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -4816,6 +5019,9 @@
       <c r="C23" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_CONTRACT_TEXT}}</v>
       </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -4841,6 +5047,9 @@
       <c r="C25" t="str">
         <v>{{UPSELL_SECTION_HEADING}}</v>
       </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -4852,6 +5061,9 @@
       <c r="C26" t="str">
         <v>N/A</v>
       </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -4863,6 +5075,9 @@
       <c r="C27" t="str">
         <v>N/A</v>
       </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -4874,6 +5089,9 @@
       <c r="C28" t="str">
         <v>N/A</v>
       </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -4885,6 +5103,9 @@
       <c r="C29" t="str">
         <v>N/A</v>
       </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -4896,6 +5117,9 @@
       <c r="C30" t="str">
         <v>N/A</v>
       </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -4907,6 +5131,9 @@
       <c r="C31" t="str">
         <v>{{UPSELL_FEATURE_1}}</v>
       </c>
+      <c r="D31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -4918,6 +5145,9 @@
       <c r="C32" t="str">
         <v>N/A</v>
       </c>
+      <c r="D32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -4929,6 +5159,9 @@
       <c r="C33" t="str">
         <v>{{UPSELL_FEATURE_2}}</v>
       </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -4940,6 +5173,9 @@
       <c r="C34" t="str">
         <v>{{UPSELL_FEATURE_3}}</v>
       </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -4951,6 +5187,9 @@
       <c r="C35" t="str">
         <v>N/A</v>
       </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -4962,6 +5201,9 @@
       <c r="C36" t="str">
         <v>N/A</v>
       </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -4973,6 +5215,9 @@
       <c r="C37" t="str">
         <v>N/A</v>
       </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -4984,6 +5229,9 @@
       <c r="C38" t="str">
         <v>N/A</v>
       </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -5177,6 +5425,9 @@
       <c r="C52" t="str">
         <v>{{PPV_CTA_TEXT}}</v>
       </c>
+      <c r="D52" t="str">
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -5202,6 +5453,9 @@
       <c r="C54" t="str">
         <v>Choose your plan</v>
       </c>
+      <c r="D54" t="str">
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -5213,6 +5467,9 @@
       <c r="C55" t="str">
         <v>Buy {{PPV_NAME}} with DAZN Standard or get it included in DAZN Ultimate.</v>
       </c>
+      <c r="D55" t="str">
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -5224,6 +5481,9 @@
       <c r="C56" t="str">
         <v>get it included in DAZN Ultimate.</v>
       </c>
+      <c r="D56" t="str">
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -5235,6 +5495,9 @@
       <c r="C57" t="str">
         <v>Yes</v>
       </c>
+      <c r="D57" t="str">
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -5246,6 +5509,9 @@
       <c r="C58" t="str">
         <v>{{PPV_DATE}}</v>
       </c>
+      <c r="D58" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -5257,6 +5523,9 @@
       <c r="C59" t="str">
         <v>{{PPV_DISPLAY_NAME}}</v>
       </c>
+      <c r="D59" t="str">
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -5268,6 +5537,9 @@
       <c r="C60" t="str">
         <v>Yes</v>
       </c>
+      <c r="D60" t="str">
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -5279,6 +5551,9 @@
       <c r="C61" t="str">
         <v>Yes</v>
       </c>
+      <c r="D61" t="str">
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -5290,6 +5565,9 @@
       <c r="C62" t="str">
         <v>{{PPV_DISPLAY_NAME}}</v>
       </c>
+      <c r="D62" t="str">
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -5301,6 +5579,9 @@
       <c r="C63" t="str">
         <v>/fight</v>
       </c>
+      <c r="D63" t="str">
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -5312,6 +5593,9 @@
       <c r="C64" t="str">
         <v>{{PPV_PRICE}}</v>
       </c>
+      <c r="D64" t="str">
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -5323,6 +5607,9 @@
       <c r="C65" t="str">
         <v>{{CURRENCY}}</v>
       </c>
+      <c r="D65" t="str">
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -5334,6 +5621,9 @@
       <c r="C66" t="str">
         <v>Choose your subscription</v>
       </c>
+      <c r="D66" t="str">
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -5345,6 +5635,9 @@
       <c r="C67" t="str">
         <v>Yes</v>
       </c>
+      <c r="D67" t="str">
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -5356,6 +5649,9 @@
       <c r="C68" t="str">
         <v>{{FREE_TRIAL_DAYS}}-day free trial of DAZN Standard</v>
       </c>
+      <c r="D68" t="str">
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -5367,6 +5663,9 @@
       <c r="C69" t="str">
         <v>Yes</v>
       </c>
+      <c r="D69" t="str">
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -5378,6 +5677,9 @@
       <c r="C70" t="str">
         <v>Yes</v>
       </c>
+      <c r="D70" t="str">
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -5389,6 +5691,9 @@
       <c r="C71" t="str">
         <v>{{FREE_TRIAL_DAYS}}-days free access to DAZN Standard.</v>
       </c>
+      <c r="D71" t="str">
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -5400,6 +5705,9 @@
       <c r="C72" t="str">
         <v>Cancel anytime during the trial and only pay for the fight. After the trial you move onto a Monthly Flex plan for {{CURRENCY}}{{MONTHLY_PRICE}}/month. You will not lose access to the pay-per-view[s].</v>
       </c>
+      <c r="D72" t="str">
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -5411,6 +5719,9 @@
       <c r="C73" t="str">
         <v>Yes</v>
       </c>
+      <c r="D73" t="str">
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -5422,6 +5733,9 @@
       <c r="C74" t="str">
         <v>Pay-per-views included</v>
       </c>
+      <c r="D74" t="str">
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -5433,6 +5747,9 @@
       <c r="C75" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="D75" t="str">
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -5444,6 +5761,9 @@
       <c r="C76" t="str">
         <v>From</v>
       </c>
+      <c r="D76" t="str">
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -5455,6 +5775,9 @@
       <c r="C77" t="str">
         <v>{{UPSELL_PRICE}}</v>
       </c>
+      <c r="D77" t="str">
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -5466,6 +5789,9 @@
       <c r="C78" t="str">
         <v>{{UPSELL_PRICE_LENGTH}}</v>
       </c>
+      <c r="D78" t="str">
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -5477,6 +5803,9 @@
       <c r="C79" t="str">
         <v>Annual contract. Auto renews.</v>
       </c>
+      <c r="D79" t="str">
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -5488,6 +5817,9 @@
       <c r="C80" t="str">
         <v>Yes</v>
       </c>
+      <c r="D80" t="str">
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -5499,6 +5831,9 @@
       <c r="C81" t="str">
         <v>N/A</v>
       </c>
+      <c r="D81" t="str">
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -5510,6 +5845,9 @@
       <c r="C82" t="str">
         <v>N/A</v>
       </c>
+      <c r="D82" t="str">
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -5521,6 +5859,9 @@
       <c r="C83" t="str">
         <v>N/A</v>
       </c>
+      <c r="D83" t="str">
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -5532,6 +5873,9 @@
       <c r="C84" t="str">
         <v>N/A</v>
       </c>
+      <c r="D84" t="str">
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -5543,6 +5887,9 @@
       <c r="C85" t="str">
         <v>Pay-per-views included at no extra cost. Minimum of 12 events per year including {{PPV_NAME}}.</v>
       </c>
+      <c r="D85" t="str">
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -5554,6 +5901,9 @@
       <c r="C86" t="str">
         <v>{{PPV_NAME}}.</v>
       </c>
+      <c r="D86" t="str">
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -5565,6 +5915,9 @@
       <c r="C87" t="str">
         <v>HDR and Dolby 5.1 surround sound on select events.</v>
       </c>
+      <c r="D87" t="str">
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -5576,6 +5929,9 @@
       <c r="C88" t="str">
         <v>185+ fights a year from the world's best promoters.</v>
       </c>
+      <c r="D88" t="str">
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
@@ -5587,6 +5943,9 @@
       <c r="C89" t="str">
         <v>Whats included</v>
       </c>
+      <c r="D89" t="str">
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -5598,6 +5957,9 @@
       <c r="C90" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="D90" t="str">
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -5609,6 +5971,9 @@
       <c r="C91" t="str">
         <v>get it included in DAZN Ultimate.</v>
       </c>
+      <c r="D91" t="str">
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -5620,6 +5985,9 @@
       <c r="C92" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="D92" t="str">
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
@@ -5631,6 +5999,9 @@
       <c r="C93" t="str">
         <v>Continue with PPV</v>
       </c>
+      <c r="D93" t="str">
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
@@ -5642,10 +6013,251 @@
       <c r="C94" t="str">
         <v>N/A</v>
       </c>
+      <c r="D94" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>canada_tier</v>
+      </c>
+      <c r="B95" t="str">
+        <v>Subscription Page Title</v>
+      </c>
+      <c r="C95" t="str">
+        <v>Choose your subscription</v>
+      </c>
+      <c r="D95" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>canada_tier</v>
+      </c>
+      <c r="B96" t="str">
+        <v>Subscription Page Subtitle</v>
+      </c>
+      <c r="C96" t="str">
+        <v>Choose the subscription you'd like to explore.</v>
+      </c>
+      <c r="D96" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>canada_tier</v>
+      </c>
+      <c r="B97" t="str">
+        <v>PPV Image Section Title</v>
+      </c>
+      <c r="C97" t="str">
+        <v>Get {{PPV_NAME}} with a DAZN subscription</v>
+      </c>
+      <c r="D97" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>canada_tier</v>
+      </c>
+      <c r="B98" t="str">
+        <v>PPV Image Visible</v>
+      </c>
+      <c r="C98" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="D98" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>canada_tier</v>
+      </c>
+      <c r="B99" t="str">
+        <v>PPV Image Date Badge</v>
+      </c>
+      <c r="C99" t="str">
+        <v>{{PPV_DATE}}</v>
+      </c>
+      <c r="D99" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>canada_tier</v>
+      </c>
+      <c r="B100" t="str">
+        <v>Selected PPV Title</v>
+      </c>
+      <c r="C100" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+      <c r="D100" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>canada_tier</v>
+      </c>
+      <c r="B101" t="str">
+        <v>Selected PPV Price</v>
+      </c>
+      <c r="C101" t="str">
+        <v>{{PPV_PRICE}}</v>
+      </c>
+      <c r="D101" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>canada_tier</v>
+      </c>
+      <c r="B102" t="str">
+        <v>PPV Add-On Checkbox Selected</v>
+      </c>
+      <c r="C102" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="D102" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>canada_tier</v>
+      </c>
+      <c r="B103" t="str">
+        <v>Standard Tier Tab Visible</v>
+      </c>
+      <c r="C103" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="D103" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>canada_tier</v>
+      </c>
+      <c r="B104" t="str">
+        <v>Ultimate Tier Tab Visible</v>
+      </c>
+      <c r="C104" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="D104" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>canada_tier</v>
+      </c>
+      <c r="B105" t="str">
+        <v>Standard Tier Feature Bar</v>
+      </c>
+      <c r="C105" t="str">
+        <v>2 Streams | 1 IP Location | HD video quality | Standard audio | Downloads</v>
+      </c>
+      <c r="D105" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>canada_tier</v>
+      </c>
+      <c r="B106" t="str">
+        <v>Ultimate Tier Feature Bar</v>
+      </c>
+      <c r="C106" t="str">
+        <v>3 Streams | 2 IP locations | Multiview | Downloads | No pre-roll ads | 20% discount on NFL shop</v>
+      </c>
+      <c r="D106" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>canada_tier</v>
+      </c>
+      <c r="B107" t="str">
+        <v>DAZN Card Starting Price</v>
+      </c>
+      <c r="C107" t="str">
+        <v>From $24.99 /month</v>
+      </c>
+      <c r="D107" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>canada_tier</v>
+      </c>
+      <c r="B108" t="str">
+        <v>DAZN+ Card Starting Price</v>
+      </c>
+      <c r="C108" t="str">
+        <v>From $44.99 /month</v>
+      </c>
+      <c r="D108" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>canada_tier</v>
+      </c>
+      <c r="B109" t="str">
+        <v>DAZN Ultimate Card Starting Price</v>
+      </c>
+      <c r="C109" t="str">
+        <v>From $29.99 /month</v>
+      </c>
+      <c r="D109" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>canada_tier</v>
+      </c>
+      <c r="B110" t="str">
+        <v>DAZN+ Ultimate Card Starting Price</v>
+      </c>
+      <c r="C110" t="str">
+        <v>From $49.99 /month</v>
+      </c>
+      <c r="D110" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>canada_tier</v>
+      </c>
+      <c r="B111" t="str">
+        <v>Selected Subscription Get Started CTA Visible</v>
+      </c>
+      <c r="C111" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="D111" t="str">
+        <v>canada</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D94"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D111"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5795,7 +6407,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D61"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5821,6 +6433,9 @@
       <c r="C2" t="str">
         <v>{{PLAN_PAGE_TITLE}}</v>
       </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -5832,6 +6447,9 @@
       <c r="C3" t="str">
         <v>Yes</v>
       </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -5843,6 +6461,9 @@
       <c r="C4" t="str">
         <v>Flex – Pay Monthly</v>
       </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -5854,6 +6475,9 @@
       <c r="C5" t="str">
         <v>{{FLEX_BADGE}}</v>
       </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -5865,6 +6489,9 @@
       <c r="C6" t="str">
         <v>{{FLEX_DESCRIPTION}}</v>
       </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -5876,6 +6503,9 @@
       <c r="C7" t="str">
         <v>Yes</v>
       </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -5887,6 +6517,9 @@
       <c r="C8" t="str">
         <v>{{FLEX_TODAY_TEXT}}</v>
       </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -5898,6 +6531,9 @@
       <c r="C9" t="str">
         <v>{{FLEX_FUTURE_DATE}}</v>
       </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -5909,6 +6545,9 @@
       <c r="C10" t="str">
         <v>{{FLEX_FUTURE_TEXT}}</v>
       </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -5920,6 +6559,9 @@
       <c r="C11" t="str">
         <v>Yes</v>
       </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -5931,6 +6573,9 @@
       <c r="C12" t="str">
         <v>{{ANNUAL_SAVINGS_BADGE}}</v>
       </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -5942,6 +6587,9 @@
       <c r="C13" t="str">
         <v>Annual - Pay Monthly</v>
       </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -5953,6 +6601,9 @@
       <c r="C14" t="str">
         <v>1 MONTH FREE</v>
       </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -5964,6 +6615,9 @@
       <c r="C15" t="str">
         <v>then {{CURRENCY}}{{ANNUAL_PRICE}}/month for {{ANNUAL_MONTHS}} months</v>
       </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -5975,6 +6629,9 @@
       <c r="C16" t="str">
         <v>Annual contract. Auto renews.</v>
       </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -5986,6 +6643,9 @@
       <c r="C17" t="str">
         <v>185+ fights a year from the world's best promoters.</v>
       </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -5997,6 +6657,9 @@
       <c r="C18" t="str">
         <v>Additional cost for pay-per-view events.</v>
       </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -6008,6 +6671,9 @@
       <c r="C19" t="str">
         <v>Full HD video resolution.</v>
       </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -6019,6 +6685,9 @@
       <c r="C20" t="str">
         <v>No</v>
       </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -6030,6 +6699,9 @@
       <c r="C21" t="str">
         <v>{{PLAN_CTA_BUTTON}}</v>
       </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -6041,6 +6713,9 @@
       <c r="C22" t="str">
         <v>{{PLAN_PAGE_TITLE}}</v>
       </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -6122,6 +6797,9 @@
       <c r="C28" t="str">
         <v>Yes</v>
       </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -6133,6 +6811,9 @@
       <c r="C29" t="str">
         <v>Annual - Pay Monthly</v>
       </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -6144,6 +6825,9 @@
       <c r="C30" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
       </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -6155,6 +6839,9 @@
       <c r="C31" t="str">
         <v>/month</v>
       </c>
+      <c r="D31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -6166,6 +6853,9 @@
       <c r="C32" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_CONTRACT_TEXT}}</v>
       </c>
+      <c r="D32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -6177,6 +6867,9 @@
       <c r="C33" t="str">
         <v>Yes</v>
       </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -6188,6 +6881,9 @@
       <c r="C34" t="str">
         <v>Yes</v>
       </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -6199,6 +6895,9 @@
       <c r="C35" t="str">
         <v>Annual - Pay Upfront</v>
       </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -6210,6 +6909,9 @@
       <c r="C36" t="str">
         <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
       </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -6221,6 +6923,9 @@
       <c r="C37" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE_DISPLAY}}</v>
       </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -6232,6 +6937,9 @@
       <c r="C38" t="str">
         <v>/year</v>
       </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -6243,6 +6951,9 @@
       <c r="C39" t="str">
         <v>No</v>
       </c>
+      <c r="D39" t="str">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -6254,6 +6965,9 @@
       <c r="C40" t="str">
         <v>{{ULTIMATE_FEATURE_1}}</v>
       </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -6265,6 +6979,9 @@
       <c r="C41" t="str">
         <v>{{ULTIMATE_FEATURE_2}}</v>
       </c>
+      <c r="D41" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -6276,6 +6993,9 @@
       <c r="C42" t="str">
         <v>{{ULTIMATE_FEATURE_3}}</v>
       </c>
+      <c r="D42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -6301,17 +7021,258 @@
       <c r="C44" t="str">
         <v>{{PLAN_CTA_BUTTON}}</v>
       </c>
+      <c r="D44" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Page Title</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Choose your plan</v>
+      </c>
+      <c r="D45" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Option 1 Title</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Annual - pay over time</v>
+      </c>
+      <c r="D46" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Option 1 Contract Text</v>
+      </c>
+      <c r="C47" t="str">
+        <v>12 month contract. Annual subscription.</v>
+      </c>
+      <c r="D47" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Option 1 DAZN Price</v>
+      </c>
+      <c r="C48" t="str">
+        <v>.99 /month</v>
+      </c>
+      <c r="D48" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Option 1 DAZN+ Price</v>
+      </c>
+      <c r="C49" t="str">
+        <v>.99 /month</v>
+      </c>
+      <c r="D49" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Option 1 DAZN Ultimate Price</v>
+      </c>
+      <c r="C50" t="str">
+        <v>.99 /month</v>
+      </c>
+      <c r="D50" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Option 1 DAZN+ Ultimate Price</v>
+      </c>
+      <c r="C51" t="str">
+        <v>.99 /month</v>
+      </c>
+      <c r="D51" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Option 2 Title</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Annual - pay now</v>
+      </c>
+      <c r="D52" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Option 2 Savings Badge</v>
+      </c>
+      <c r="C53" t="str">
+        <v>{{CANADA_OPTION2_SAVINGS_BADGE}}</v>
+      </c>
+      <c r="D53" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Option 2 DAZN Price</v>
+      </c>
+      <c r="C54" t="str">
+        <v>.99 /season</v>
+      </c>
+      <c r="D54" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Option 2 DAZN Ultimate Price</v>
+      </c>
+      <c r="C55" t="str">
+        <v>.99 /season</v>
+      </c>
+      <c r="D55" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Option 2 DAZN+ Ultimate Price</v>
+      </c>
+      <c r="C56" t="str">
+        <v>.99 /season</v>
+      </c>
+      <c r="D56" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Option 3 Title</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Monthly</v>
+      </c>
+      <c r="D57" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Option 3 DAZN Price</v>
+      </c>
+      <c r="C58" t="str">
+        <v>.99 /month</v>
+      </c>
+      <c r="D58" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Option 3 DAZN Ultimate Price</v>
+      </c>
+      <c r="C59" t="str">
+        <v>.99 /month</v>
+      </c>
+      <c r="D59" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Option 3 DAZN+ Ultimate Price</v>
+      </c>
+      <c r="C60" t="str">
+        <v>.99 /month</v>
+      </c>
+      <c r="D60" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Continue Button Present</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="D61" t="str">
+        <v>canada</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D44"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D61"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E103"/>
+  <dimension ref="A1:E124"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6343,6 +7304,9 @@
       <c r="D2" t="str">
         <v>Payment method</v>
       </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -6357,6 +7321,9 @@
       <c r="D3" t="str">
         <v>Purchase summary</v>
       </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -6371,6 +7338,9 @@
       <c r="D4" t="str">
         <v>Change</v>
       </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -6385,6 +7355,9 @@
       <c r="D5" t="str">
         <v>Yes</v>
       </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -6399,6 +7372,9 @@
       <c r="D6" t="str">
         <v>Yes</v>
       </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -6413,6 +7389,9 @@
       <c r="D7" t="str">
         <v>Yes</v>
       </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -6478,6 +7457,9 @@
       <c r="D11" t="str">
         <v>Yes</v>
       </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -6526,6 +7508,9 @@
       <c r="D14" t="str">
         <v>DAZN Standard</v>
       </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -6540,6 +7525,9 @@
       <c r="D15" t="str">
         <v>{{PAYMENT_PLAN_NAME}}</v>
       </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -6554,6 +7542,9 @@
       <c r="D16" t="str">
         <v>{{PAYMENT_FLEX_CANCEL_NOTICE}}</v>
       </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -6568,6 +7559,9 @@
       <c r="D17" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -6582,6 +7576,9 @@
       <c r="D18" t="str">
         <v>{{PAYMENT_FREE_TEXT}}</v>
       </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -6596,6 +7593,9 @@
       <c r="D19" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -6610,6 +7610,9 @@
       <c r="D20" t="str">
         <v>{{PPV_PRICE}}</v>
       </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -6624,6 +7627,9 @@
       <c r="D21" t="str">
         <v>Today you pay</v>
       </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -6638,6 +7644,9 @@
       <c r="D22" t="str">
         <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -6652,6 +7661,9 @@
       <c r="D23" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -6666,6 +7678,9 @@
       <c r="D24" t="str">
         <v>{{PAYMENT_FLEX_LEGAL_TEXT}}</v>
       </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -6680,6 +7695,9 @@
       <c r="D25" t="str">
         <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -6694,6 +7712,9 @@
       <c r="D26" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -6708,6 +7729,9 @@
       <c r="D27" t="str">
         <v>DAZN Standard</v>
       </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -6722,6 +7746,9 @@
       <c r="D28" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -6736,6 +7763,9 @@
       <c r="D29" t="str">
         <v>{{PPV_PRICE}}</v>
       </c>
+      <c r="E29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -6750,6 +7780,9 @@
       <c r="D30" t="str">
         <v>{{RATE_PLAN_LABEL}}</v>
       </c>
+      <c r="E30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -6764,6 +7797,9 @@
       <c r="D31" t="str">
         <v>{{CURRENCY}}{{ANNUAL_PRICE}}</v>
       </c>
+      <c r="E31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -6778,6 +7814,9 @@
       <c r="D32" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -6792,6 +7831,9 @@
       <c r="D33" t="str">
         <v>Today you pay</v>
       </c>
+      <c r="E33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -6806,6 +7848,9 @@
       <c r="D34" t="str">
         <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
+      <c r="E34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -6820,6 +7865,9 @@
       <c r="D35" t="str">
         <v>{{CANCELLATION_TEXT_ANNUAL}}</v>
       </c>
+      <c r="E35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -6834,6 +7882,9 @@
       <c r="D36" t="str">
         <v>Yes</v>
       </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -6848,6 +7899,9 @@
       <c r="D37" t="str">
         <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -6862,6 +7916,9 @@
       <c r="D38" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -6876,6 +7933,9 @@
       <c r="D39" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="E39" t="str">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -6890,6 +7950,9 @@
       <c r="D40" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -6904,6 +7967,9 @@
       <c r="D41" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E41" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -6918,6 +7984,9 @@
       <c r="D42" t="str">
         <v>Annual - Pay Monthly</v>
       </c>
+      <c r="E42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -6932,6 +8001,9 @@
       <c r="D43" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
       </c>
+      <c r="E43" t="str">
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -6946,6 +8018,9 @@
       <c r="D44" t="str">
         <v>Billed monthly. 12-month contract.</v>
       </c>
+      <c r="E44" t="str">
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -6960,6 +8035,9 @@
       <c r="D45" t="str">
         <v>Today you pay</v>
       </c>
+      <c r="E45" t="str">
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -6974,6 +8052,9 @@
       <c r="D46" t="str">
         <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
+      <c r="E46" t="str">
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -6988,6 +8069,9 @@
       <c r="D47" t="str">
         <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
+      <c r="E47" t="str">
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -7002,6 +8086,9 @@
       <c r="D48" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
       </c>
+      <c r="E48" t="str">
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -7016,6 +8103,9 @@
       <c r="D49" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E49" t="str">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -7030,6 +8120,9 @@
       <c r="D50" t="str">
         <v>Yes</v>
       </c>
+      <c r="E50" t="str">
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -7044,6 +8137,9 @@
       <c r="D51" t="str">
         <v>{{DISCOUNT_BADGE}}</v>
       </c>
+      <c r="E51" t="str">
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -7058,6 +8154,9 @@
       <c r="D52" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E52" t="str">
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -7072,6 +8171,9 @@
       <c r="D53" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="E53" t="str">
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -7086,6 +8188,9 @@
       <c r="D54" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="E54" t="str">
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -7100,6 +8205,9 @@
       <c r="D55" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E55" t="str">
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -7114,6 +8222,9 @@
       <c r="D56" t="str">
         <v>Annual - Pay Upfront</v>
       </c>
+      <c r="E56" t="str">
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -7128,6 +8239,9 @@
       <c r="D57" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE}}/year</v>
       </c>
+      <c r="E57" t="str">
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -7142,6 +8256,9 @@
       <c r="D58" t="str">
         <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}. Pay for the full year up front|Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
       </c>
+      <c r="E58" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -7156,6 +8273,9 @@
       <c r="D59" t="str">
         <v>Today you pay</v>
       </c>
+      <c r="E59" t="str">
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -7170,6 +8290,9 @@
       <c r="D60" t="str">
         <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
+      <c r="E60" t="str">
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -7184,6 +8307,9 @@
       <c r="D61" t="str">
         <v>Next Annual payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
+      <c r="E61" t="str">
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -7198,6 +8324,9 @@
       <c r="D62" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE}}</v>
       </c>
+      <c r="E62" t="str">
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -7212,6 +8341,9 @@
       <c r="D63" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E63" t="str">
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -7226,6 +8358,9 @@
       <c r="D64" t="str">
         <v>Yes</v>
       </c>
+      <c r="E64" t="str">
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -7240,6 +8375,9 @@
       <c r="D65" t="str">
         <v>{{PAYMENT_PAGE_TITLE}}</v>
       </c>
+      <c r="E65" t="str">
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -7254,6 +8392,9 @@
       <c r="D66" t="str">
         <v>DAZN Standard</v>
       </c>
+      <c r="E66" t="str">
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -7268,6 +8409,9 @@
       <c r="D67" t="str">
         <v>{{BUNDLE_NAME}}</v>
       </c>
+      <c r="E67" t="str">
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -7282,6 +8426,9 @@
       <c r="D68" t="str">
         <v>{{BUNDLE_PRICE}}</v>
       </c>
+      <c r="E68" t="str">
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -7296,6 +8443,9 @@
       <c r="D69" t="str">
         <v>{{BUNDLE_TODAY_YOU_PAY_STANDARD}}</v>
       </c>
+      <c r="E69" t="str">
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -7310,6 +8460,9 @@
       <c r="D70" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E70" t="str">
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -7324,6 +8477,9 @@
       <c r="D71" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E71" t="str">
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -7338,6 +8494,9 @@
       <c r="D72" t="str">
         <v>DAZN Standard</v>
       </c>
+      <c r="E72" t="str">
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -7352,6 +8511,9 @@
       <c r="D73" t="str">
         <v>Annual - Pay Monthly</v>
       </c>
+      <c r="E73" t="str">
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -7366,6 +8528,9 @@
       <c r="D74" t="str">
         <v>First month free</v>
       </c>
+      <c r="E74" t="str">
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -7380,6 +8545,9 @@
       <c r="D75" t="str">
         <v>{{BUNDLE_NAME}}</v>
       </c>
+      <c r="E75" t="str">
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -7394,6 +8562,9 @@
       <c r="D76" t="str">
         <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
       </c>
+      <c r="E76" t="str">
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -7408,6 +8579,9 @@
       <c r="D77" t="str">
         <v>{{BUNDLE_PRICE}}</v>
       </c>
+      <c r="E77" t="str">
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -7422,6 +8596,9 @@
       <c r="D78" t="str">
         <v>{{BUNDLE_DISCOUNT}}</v>
       </c>
+      <c r="E78" t="str">
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -7436,6 +8613,9 @@
       <c r="D79" t="str">
         <v>{{BUNDLE_TODAY_YOU_PAY_STANDARD}}</v>
       </c>
+      <c r="E79" t="str">
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -7450,6 +8630,9 @@
       <c r="D80" t="str">
         <v>{{CANCELLATION_TEXT_ANNUAL}}</v>
       </c>
+      <c r="E80" t="str">
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -7464,6 +8647,9 @@
       <c r="D81" t="str">
         <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
+      <c r="E81" t="str">
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -7478,6 +8664,9 @@
       <c r="D82" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E82" t="str">
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -7492,6 +8681,9 @@
       <c r="D83" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="E83" t="str">
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -7506,6 +8698,9 @@
       <c r="D84" t="str">
         <v>Annual - Pay Monthly</v>
       </c>
+      <c r="E84" t="str">
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -7520,6 +8715,9 @@
       <c r="D85" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
       </c>
+      <c r="E85" t="str">
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -7534,6 +8732,9 @@
       <c r="D86" t="str">
         <v>{{BUNDLE_NAME}}</v>
       </c>
+      <c r="E86" t="str">
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -7548,6 +8749,9 @@
       <c r="D87" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E87" t="str">
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -7562,6 +8766,9 @@
       <c r="D88" t="str">
         <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
+      <c r="E88" t="str">
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
@@ -7576,6 +8783,9 @@
       <c r="D89" t="str">
         <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
+      <c r="E89" t="str">
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -7590,6 +8800,9 @@
       <c r="D90" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
       </c>
+      <c r="E90" t="str">
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -7604,6 +8817,9 @@
       <c r="D91" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E91" t="str">
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -7618,6 +8834,9 @@
       <c r="D92" t="str">
         <v>{{DISCOUNT_BADGE}}</v>
       </c>
+      <c r="E92" t="str">
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
@@ -7632,6 +8851,9 @@
       <c r="D93" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E93" t="str">
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
@@ -7646,6 +8868,9 @@
       <c r="D94" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="E94" t="str">
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
@@ -7660,6 +8885,9 @@
       <c r="D95" t="str">
         <v>Annual - Pay Upfront</v>
       </c>
+      <c r="E95" t="str">
+        <v/>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
@@ -7674,6 +8902,9 @@
       <c r="D96" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE}}/year</v>
       </c>
+      <c r="E96" t="str">
+        <v/>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
@@ -7688,6 +8919,9 @@
       <c r="D97" t="str">
         <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
       </c>
+      <c r="E97" t="str">
+        <v/>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
@@ -7702,6 +8936,9 @@
       <c r="D98" t="str">
         <v>{{BUNDLE_NAME}}</v>
       </c>
+      <c r="E98" t="str">
+        <v/>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
@@ -7716,6 +8953,9 @@
       <c r="D99" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E99" t="str">
+        <v/>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
@@ -7730,6 +8970,9 @@
       <c r="D100" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE}}</v>
       </c>
+      <c r="E100" t="str">
+        <v/>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
@@ -7744,6 +8987,9 @@
       <c r="D101" t="str">
         <v>Next Annual payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
+      <c r="E101" t="str">
+        <v/>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
@@ -7758,6 +9004,9 @@
       <c r="D102" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE}}</v>
       </c>
+      <c r="E102" t="str">
+        <v/>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
@@ -7772,10 +9021,370 @@
       <c r="D103" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E103" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B104" t="str">
+        <v>All</v>
+      </c>
+      <c r="C104" t="str">
+        <v>Page Header Title</v>
+      </c>
+      <c r="D104" t="str">
+        <v>Choose how to pay</v>
+      </c>
+      <c r="E104" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B105" t="str">
+        <v>All</v>
+      </c>
+      <c r="C105" t="str">
+        <v>Summary Subscription Title</v>
+      </c>
+      <c r="D105" t="str">
+        <v>{{DAZN_TIER}}</v>
+      </c>
+      <c r="E105" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B106" t="str">
+        <v>All</v>
+      </c>
+      <c r="C106" t="str">
+        <v>Selected Subscription Description</v>
+      </c>
+      <c r="D106" t="str">
+        <v>{{PAYMENT_SUBSCRIPTION_DESCRIPTION}}</v>
+      </c>
+      <c r="E106" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B107" t="str">
+        <v>All</v>
+      </c>
+      <c r="C107" t="str">
+        <v>Change Link Present</v>
+      </c>
+      <c r="D107" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E107" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B108" t="str">
+        <v>All</v>
+      </c>
+      <c r="C108" t="str">
+        <v>PPV Line Item Title</v>
+      </c>
+      <c r="D108" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+      <c r="E108" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B109" t="str">
+        <v>All</v>
+      </c>
+      <c r="C109" t="str">
+        <v>PPV Line Item Price</v>
+      </c>
+      <c r="D109" t="str">
+        <v>{{PPV_PRICE}}</v>
+      </c>
+      <c r="E109" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B110" t="str">
+        <v>All</v>
+      </c>
+      <c r="C110" t="str">
+        <v>Selected Plan Title</v>
+      </c>
+      <c r="D110" t="str">
+        <v>{{RATE_PLAN}}</v>
+      </c>
+      <c r="E110" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B111" t="str">
+        <v>All</v>
+      </c>
+      <c r="C111" t="str">
+        <v>Today You Pay Label</v>
+      </c>
+      <c r="D111" t="str">
+        <v>Today you pay</v>
+      </c>
+      <c r="E111" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B112" t="str">
+        <v>All</v>
+      </c>
+      <c r="C112" t="str">
+        <v>Tax Disclaimer Present</v>
+      </c>
+      <c r="D112" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E112" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B113" t="str">
+        <v>All</v>
+      </c>
+      <c r="C113" t="str">
+        <v>Next Payment Info Present</v>
+      </c>
+      <c r="D113" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E113" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B114" t="str">
+        <v>All</v>
+      </c>
+      <c r="C114" t="str">
+        <v>Next Annual Payment Text</v>
+      </c>
+      <c r="D114" t="str">
+        <v>{{CANADA_NEXT_ANNUAL_PAYMENT_TEXT}}</v>
+      </c>
+      <c r="E114" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B115" t="str">
+        <v>All</v>
+      </c>
+      <c r="C115" t="str">
+        <v>Renewal Text</v>
+      </c>
+      <c r="D115" t="str">
+        <v>{{CANADA_RENEWAL_TEXT}}</v>
+      </c>
+      <c r="E115" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B116" t="str">
+        <v>All</v>
+      </c>
+      <c r="C116" t="str">
+        <v>Auto-Renewal Legal Text Present</v>
+      </c>
+      <c r="D116" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E116" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B117" t="str">
+        <v>All</v>
+      </c>
+      <c r="C117" t="str">
+        <v>Credit &amp; Debit Card Option</v>
+      </c>
+      <c r="D117" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E117" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B118" t="str">
+        <v>All</v>
+      </c>
+      <c r="C118" t="str">
+        <v>Google Pay Option</v>
+      </c>
+      <c r="D118" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E118" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B119" t="str">
+        <v>All</v>
+      </c>
+      <c r="C119" t="str">
+        <v>PayPal Option</v>
+      </c>
+      <c r="D119" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E119" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B120" t="str">
+        <v>All</v>
+      </c>
+      <c r="C120" t="str">
+        <v>Redeem Promo Code Button</v>
+      </c>
+      <c r="D120" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E120" t="str">
+        <v>canada</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B121" t="str">
+        <v>All</v>
+      </c>
+      <c r="C121" t="str">
+        <v>Selected Subscription Description</v>
+      </c>
+      <c r="D121" t="str">
+        <v>Includes NFL Game Pass, UEFA Champions League &amp; Europa League, Rugby Union, over 150 fights a year and many more sports live and on demand. 2 Streams Single IP Location HD video quality Standard audio Downloads</v>
+      </c>
+      <c r="E121" t="str">
+        <v>standard-dazn</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B122" t="str">
+        <v>All</v>
+      </c>
+      <c r="C122" t="str">
+        <v>Selected Subscription Description</v>
+      </c>
+      <c r="D122" t="str">
+        <v>Every sport on DAZN in one place: NFL Game Pass, the best European soccer including English Premier League &amp; Serie A on Fubo Sports, boxing, rugby and much more 2 Streams Single IP Location HD video quality Standard audio Downloads</v>
+      </c>
+      <c r="E122" t="str">
+        <v>standard-dazn+</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B123" t="str">
+        <v>All</v>
+      </c>
+      <c r="C123" t="str">
+        <v>Selected Subscription Description</v>
+      </c>
+      <c r="D123" t="str">
+        <v>Includes NFL Game Pass, UEFA Champions League &amp; Europa League, Rugby Union, over 150 fights a year and many more sports live and on demand. 3 Streams 2 IP locations Multiview Downloads 20% discount on NFL shop</v>
+      </c>
+      <c r="E123" t="str">
+        <v>ultimate-dazn</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>Canada</v>
+      </c>
+      <c r="B124" t="str">
+        <v>All</v>
+      </c>
+      <c r="C124" t="str">
+        <v>Selected Subscription Description</v>
+      </c>
+      <c r="D124" t="str">
+        <v>Every sport on DAZN in one place: NFL Game Pass, the best European soccer including English Premier League &amp; Serie A on Fubo Sports, boxing, rugby and much more 3 Streams 2 IP locations Multiview Downloads 20% discount on NFL shop</v>
+      </c>
+      <c r="E124" t="str">
+        <v>ultimate-dazn+</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E103"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E124"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(ios): post-kickoff v3 — Safari page-ready wait, boxing feed wait, payment title fix, validation and flow improvements (#78)
Includes all local changes on top of upstream/main (PR #74 merged).
Conflicts with PR #74 base resolved by taking the local (more recent) versions.
TSC: clean (appium + root).
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -3926,7 +3926,7 @@
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C22"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4148,10 +4148,31 @@
         <v>home-boxing-upcoming</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Banner Description</v>
+      </c>
+      <c r="B21" t="str">
+        <v>{{MOBILE_BANNER_DESCRIPTION}}</v>
+      </c>
+      <c r="C21" t="str">
+        <v>home-boxing-banner</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Fight Card CTA</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Fight card</v>
+      </c>
+      <c r="C22" t="str">
+        <v>home-boxing-banner</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C22"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>